<commit_message>
Deploying to gh-pages from @ marcusburghardt/content@2217dbfaed772205b6bc8fbde79be820cd422e3a 🚀
</commit_message>
<xml_diff>
--- a/srg_mapping/srg-mapping-rhel9.xlsx
+++ b/srg_mapping/srg-mapping-rhel9.xlsx
@@ -544,7 +544,7 @@
     <row r="2" ht="130" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>AC-7 b,AC-7 a</t>
+          <t>AC-7 a,AC-7 b</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
@@ -628,7 +628,7 @@
     <row r="3" ht="130" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>AC-7 b,AC-7 a</t>
+          <t>AC-7 a,AC-7 b</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
@@ -713,7 +713,7 @@
     <row r="4" ht="130" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>AC-7 b,AC-7 a</t>
+          <t>AC-7 a,AC-7 b</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
@@ -785,7 +785,7 @@
     <row r="5" ht="130" customHeight="1">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>AC-7 b,AC-7 a</t>
+          <t>AC-7 a,AC-7 b</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
@@ -965,37 +965,37 @@
       <c r="Q6" s="2" t="n"/>
     </row>
     <row r="7" ht="130" customHeight="1">
-      <c r="A7" s="3" t="inlineStr">
+      <c r="A7" s="2" t="inlineStr">
         <is>
           <t>AU-5 a,AU-5 b</t>
         </is>
       </c>
-      <c r="B7" s="3" t="inlineStr">
+      <c r="B7" s="2" t="inlineStr">
         <is>
           <t>CCI-000139,CCI-000140</t>
         </is>
       </c>
-      <c r="C7" s="3" t="inlineStr">
+      <c r="C7" s="2" t="inlineStr">
         <is>
           <t>SRG-OS-000046-GPOS-00022,SRG-OS-000047-GPOS-00023</t>
         </is>
       </c>
-      <c r="D7" s="3" t="inlineStr">
+      <c r="D7" s="2" t="inlineStr">
         <is>
           <t>CCE-83709-6</t>
         </is>
       </c>
-      <c r="E7" s="3" t="inlineStr">
+      <c r="E7" s="2" t="inlineStr">
         <is>
           <t>The operating system must shut down by default upon audit failure (unless availability is an overriding concern).</t>
         </is>
       </c>
-      <c r="F7" s="3" t="inlineStr">
+      <c r="F7" s="2" t="inlineStr">
         <is>
           <t>Red Hat Enterprise Linux 9 must shut down by default upon audit failure (unless availability is an overriding concern).</t>
         </is>
       </c>
-      <c r="G7" s="3" t="inlineStr">
+      <c r="G7" s="2" t="inlineStr">
         <is>
           <t>It is critical that when the operating system is at risk of failing to process audit logs as required, it takes action to mitigate the failure. Audit processing failures include: software/hardware errors; failures in the audit capturing mechanisms; and audit storage capacity being reached or exceeded. Responses to audit failure depend upon the nature of the failure mode.
 When availability is an overriding concern, other approved actions in response to an audit failure are as follows: 
@@ -1003,7 +1003,7 @@
 2) If audit records are sent to a centralized collection server and communication with this server is lost or the server fails, the operating system must queue audit records locally until communication is restored or until the audit records are retrieved manually. Upon restoration of the connection to the centralized collection server, action should be taken to synchronize the local audit data with the collection server.</t>
         </is>
       </c>
-      <c r="H7" s="3" t="inlineStr">
+      <c r="H7" s="2" t="inlineStr">
         <is>
           <t>It is critical for the appropriate personnel to be aware if a system
 is at risk of failing to process audit logs as required. Without this
@@ -1014,17 +1014,17 @@
 exceeded.</t>
         </is>
       </c>
-      <c r="I7" s="3" t="inlineStr">
-        <is>
-          <t>Applicable - Configurable</t>
-        </is>
-      </c>
-      <c r="J7" s="3" t="inlineStr">
+      <c r="I7" s="2" t="inlineStr">
+        <is>
+          <t>Applicable - Configurable</t>
+        </is>
+      </c>
+      <c r="J7" s="2" t="inlineStr">
         <is>
           <t>Verify the operating system shuts down by default upon audit failure (unless availability is an overriding concern). If it does not, this is a finding.</t>
         </is>
       </c>
-      <c r="K7" s="3" t="inlineStr">
+      <c r="K7" s="2" t="inlineStr">
         <is>
           <t>To verify that the system will shutdown when "auditd" fails,
 run the following command:
@@ -1034,16 +1034,28 @@
 If the system is not configured to shutdown on auditd failures, then this is a finding.</t>
         </is>
       </c>
-      <c r="L7" s="3" t="n"/>
-      <c r="M7" s="3" t="inlineStr"/>
-      <c r="N7" s="3" t="inlineStr">
-        <is>
-          <t>CAT II</t>
-        </is>
-      </c>
-      <c r="O7" s="3" t="n"/>
-      <c r="P7" s="3" t="n"/>
-      <c r="Q7" s="3" t="n"/>
+      <c r="L7" s="2" t="n"/>
+      <c r="M7" s="2" t="inlineStr">
+        <is>
+          <t>Configure Red Hat Enterprise Linux 9 to shutdown when auditing failures occur.
+If the auditd daemon is configured to use the augenrules program to read
+audit rules during daemon startup (the default), add the following line to
+the bottom of "/etc/audit/rules.d/immutable.rules":
+-f 2
+If the auditd daemon is configured to use the auditctl utility to read
+audit rules during daemon startup, add the following line to the
+bottom of the /etc/audit/audit.rules file:
+-f 2</t>
+        </is>
+      </c>
+      <c r="N7" s="2" t="inlineStr">
+        <is>
+          <t>CAT II</t>
+        </is>
+      </c>
+      <c r="O7" s="2" t="n"/>
+      <c r="P7" s="2" t="n"/>
+      <c r="Q7" s="2" t="n"/>
     </row>
     <row r="8" ht="130" customHeight="1">
       <c r="A8" s="3" t="inlineStr">
@@ -1421,11 +1433,11 @@
       </c>
       <c r="K12" s="2" t="inlineStr">
         <is>
-          <t>For every temporary and emergency account, run the following command
+          <t>For every temporary account, run the following command
 to obtain its account aging and expiration information:
  $ sudo chage -l  USER  
 Verify each of these accounts has an expiration date set as documented.
-If any temporary or emergency accounts have no expiration date set or do not expire within a documented time frame, then this is a finding.</t>
+If any temporary accounts have no expiration date set or do not expire within a documented time frame, then this is a finding.</t>
         </is>
       </c>
       <c r="L12" s="2" t="n"/>
@@ -1449,7 +1461,7 @@
     <row r="13" ht="130" customHeight="1">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>AU-6 (4),AU-3,AU-7 (1),MA-4 (1) (a),AU-3 (1),AU-7 a,CM-6 b,AU-14 (1),CM-5 (1),AU-12 a</t>
+          <t>AU-3 (1),AU-14 (1),CM-5 (1),MA-4 (1) (a),AU-3,AU-6 (4),CM-6 b,AU-12 a,AU-7 a,AU-7 (1)</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
@@ -1534,7 +1546,7 @@
     <row r="14" ht="130" customHeight="1">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>CM-7 (5) (b),CM-7 (2)</t>
+          <t>CM-7 (2),CM-7 (5) (b)</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
@@ -1610,7 +1622,7 @@
     <row r="15" ht="130" customHeight="1">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>CM-7 (5) (b),CM-7 (2)</t>
+          <t>CM-7 (2),CM-7 (5) (b)</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
@@ -3252,7 +3264,7 @@
     <row r="37" ht="130" customHeight="1">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>AU-12 c,AU-3,MA-4 (1) (a),AU-3 (1),AU-14 (1),AU-12 a</t>
+          <t>AU-3 (1),MA-4 (1) (a),AU-3,AU-12 a,AU-14 (1),AU-12 c</t>
         </is>
       </c>
       <c r="B37" s="2" t="inlineStr">
@@ -3343,7 +3355,7 @@
     <row r="38" ht="130" customHeight="1">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>AU-4,AU-14 (1)</t>
+          <t>AU-14 (1),AU-4</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
@@ -3432,7 +3444,7 @@
     <row r="39" ht="130" customHeight="1">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>AU-3,AU-4 (1)</t>
+          <t>AU-4 (1),AU-3</t>
         </is>
       </c>
       <c r="B39" s="2" t="inlineStr">
@@ -3497,7 +3509,7 @@
       <c r="M39" s="2" t="inlineStr">
         <is>
           <t>Edit the file "/etc/audit/auditd.conf" and add or edit the following line:
-name_format=hostname</t>
+name_format = hostname</t>
         </is>
       </c>
       <c r="N39" s="2" t="inlineStr">
@@ -3826,7 +3838,7 @@
     <row r="44" ht="130" customHeight="1">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>CM-6 b,AU-4 (1),AU-6 (4)</t>
+          <t>AU-4 (1),CM-6 b,AU-6 (4)</t>
         </is>
       </c>
       <c r="B44" s="2" t="inlineStr">
@@ -3902,7 +3914,7 @@
     <row r="45" ht="130" customHeight="1">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>CM-6 b,AU-4 (1)</t>
+          <t>AU-4 (1),CM-6 b</t>
         </is>
       </c>
       <c r="B45" s="2" t="inlineStr">
@@ -3987,7 +3999,7 @@
     <row r="46" ht="130" customHeight="1">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>AU-8 b,AU-8 (1) (b),AU-8 (1) (a)</t>
+          <t>AU-8 b,AU-8 (1) (a),AU-8 (1) (b)</t>
         </is>
       </c>
       <c r="B46" s="2" t="inlineStr">
@@ -4312,7 +4324,7 @@
     <row r="50" ht="130" customHeight="1">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>SI-6 b,CM-3 (5),SI-6 d</t>
+          <t>SI-6 d,SI-6 b,CM-3 (5)</t>
         </is>
       </c>
       <c r="B50" s="2" t="inlineStr">
@@ -4404,7 +4416,7 @@
     <row r="51" ht="130" customHeight="1">
       <c r="A51" s="3" t="inlineStr">
         <is>
-          <t>CM-3 (5),SI-6 d</t>
+          <t>SI-6 d,CM-3 (5)</t>
         </is>
       </c>
       <c r="B51" s="3" t="inlineStr">
@@ -4488,7 +4500,7 @@
     <row r="52" ht="130" customHeight="1">
       <c r="A52" s="3" t="inlineStr">
         <is>
-          <t>AU-12 c,AU-3,MA-4 (1) (a),AU-3 (1),AU-12 a</t>
+          <t>AU-3 (1),MA-4 (1) (a),AU-3,AU-12 a,AU-12 c</t>
         </is>
       </c>
       <c r="B52" s="3" t="inlineStr">
@@ -4563,7 +4575,7 @@
     <row r="53" ht="130" customHeight="1">
       <c r="A53" s="3" t="inlineStr">
         <is>
-          <t>AU-12 c,AU-3,MA-4 (1) (a),AU-3 (1),AU-12 a</t>
+          <t>AU-3 (1),MA-4 (1) (a),AU-3,AU-12 a,AU-12 c</t>
         </is>
       </c>
       <c r="B53" s="3" t="inlineStr">
@@ -4638,7 +4650,7 @@
     <row r="54" ht="130" customHeight="1">
       <c r="A54" s="3" t="inlineStr">
         <is>
-          <t>AU-12 c,AU-3,MA-4 (1) (a),AU-3 (1),AU-12 a</t>
+          <t>AU-3 (1),MA-4 (1) (a),AU-3,AU-12 a,AU-12 c</t>
         </is>
       </c>
       <c r="B54" s="3" t="inlineStr">
@@ -4713,7 +4725,7 @@
     <row r="55" ht="130" customHeight="1">
       <c r="A55" s="3" t="inlineStr">
         <is>
-          <t>AU-12 c,AU-3,MA-4 (1) (a),AU-3 (1),AU-12 a</t>
+          <t>AU-3 (1),MA-4 (1) (a),AU-3,AU-12 a,AU-12 c</t>
         </is>
       </c>
       <c r="B55" s="3" t="inlineStr">
@@ -4788,7 +4800,7 @@
     <row r="56" ht="130" customHeight="1">
       <c r="A56" s="3" t="inlineStr">
         <is>
-          <t>AU-12 c,AU-3,MA-4 (1) (a),AU-3 (1),AU-12 a</t>
+          <t>AU-3 (1),MA-4 (1) (a),AU-3,AU-12 a,AU-12 c</t>
         </is>
       </c>
       <c r="B56" s="3" t="inlineStr">
@@ -4863,7 +4875,7 @@
     <row r="57" ht="130" customHeight="1">
       <c r="A57" s="3" t="inlineStr">
         <is>
-          <t>AU-12 c,AU-3,MA-4 (1) (a),AU-3 (1),AU-12 a</t>
+          <t>AU-3 (1),MA-4 (1) (a),AU-3,AU-12 a,AU-12 c</t>
         </is>
       </c>
       <c r="B57" s="3" t="inlineStr">
@@ -4938,7 +4950,7 @@
     <row r="58" ht="130" customHeight="1">
       <c r="A58" s="3" t="inlineStr">
         <is>
-          <t>AU-12 c,AU-3,MA-4 (1) (a),AU-3 (1),AU-12 a</t>
+          <t>AU-3 (1),MA-4 (1) (a),AU-3,AU-12 a,AU-12 c</t>
         </is>
       </c>
       <c r="B58" s="3" t="inlineStr">
@@ -5013,7 +5025,7 @@
     <row r="59" ht="130" customHeight="1">
       <c r="A59" s="3" t="inlineStr">
         <is>
-          <t>AU-12 c,AU-3,MA-4 (1) (a),AU-3 (1),AU-12 a</t>
+          <t>AU-3 (1),MA-4 (1) (a),AU-3,AU-12 a,AU-12 c</t>
         </is>
       </c>
       <c r="B59" s="3" t="inlineStr">
@@ -5088,7 +5100,7 @@
     <row r="60" ht="130" customHeight="1">
       <c r="A60" s="3" t="inlineStr">
         <is>
-          <t>AU-12 c,AU-3,MA-4 (1) (a),AU-3 (1),AU-12 a</t>
+          <t>AU-3 (1),MA-4 (1) (a),AU-3,AU-12 a,AU-12 c</t>
         </is>
       </c>
       <c r="B60" s="3" t="inlineStr">
@@ -5163,7 +5175,7 @@
     <row r="61" ht="130" customHeight="1">
       <c r="A61" s="2" t="inlineStr">
         <is>
-          <t>AU-12 c,CM-6 b,AU-8 b,AU-7 b,AU-7 a,AU-12 (3),CM-5 (1),AU-12 a</t>
+          <t>CM-5 (1),AU-7 b,AU-12 a,AU-8 b,AU-7 a,CM-6 b,AU-12 (3),AU-12 c</t>
         </is>
       </c>
       <c r="B61" s="2" t="inlineStr">
@@ -5237,7 +5249,7 @@
     <row r="62" ht="130" customHeight="1">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>AU-12 c,AU-3,AC-2 (4),MA-4 (1) (a),AU-3 (1),AU-12 a</t>
+          <t>AU-3 (1),MA-4 (1) (a),AU-3,AC-2 (4),AU-12 a,AU-12 c</t>
         </is>
       </c>
       <c r="B62" s="2" t="inlineStr">
@@ -5318,7 +5330,7 @@
     <row r="63" ht="130" customHeight="1">
       <c r="A63" s="2" t="inlineStr">
         <is>
-          <t>AU-12 c,AU-3,AC-2 (4),MA-4 (1) (a),AU-3 (1),AU-12 a</t>
+          <t>AU-3 (1),MA-4 (1) (a),AU-3,AC-2 (4),AU-12 a,AU-12 c</t>
         </is>
       </c>
       <c r="B63" s="2" t="inlineStr">
@@ -5399,7 +5411,7 @@
     <row r="64" ht="130" customHeight="1">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>AU-12 c,AU-3,AC-2 (4),MA-4 (1) (a),AU-3 (1),AU-12 a</t>
+          <t>AU-3 (1),MA-4 (1) (a),AU-3,AC-2 (4),AU-12 a,AU-12 c</t>
         </is>
       </c>
       <c r="B64" s="2" t="inlineStr">
@@ -5481,7 +5493,7 @@
     <row r="65" ht="130" customHeight="1">
       <c r="A65" s="2" t="inlineStr">
         <is>
-          <t>AU-12 c,AU-3,AC-2 (4),MA-4 (1) (a),AU-3 (1),AU-12 a</t>
+          <t>AU-3 (1),MA-4 (1) (a),AU-3,AC-2 (4),AU-12 a,AU-12 c</t>
         </is>
       </c>
       <c r="B65" s="2" t="inlineStr">
@@ -5563,7 +5575,7 @@
     <row r="66" ht="130" customHeight="1">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>AU-12 c,AU-3,AC-2 (4),MA-4 (1) (a),AU-3 (1),AU-12 a</t>
+          <t>AU-3 (1),MA-4 (1) (a),AU-3,AC-2 (4),AU-12 a,AU-12 c</t>
         </is>
       </c>
       <c r="B66" s="2" t="inlineStr">
@@ -5645,7 +5657,7 @@
     <row r="67" ht="130" customHeight="1">
       <c r="A67" s="2" t="inlineStr">
         <is>
-          <t>AU-12 c,AU-3,AC-2 (4),MA-4 (1) (a),AU-3 (1),AU-12 a</t>
+          <t>AU-3 (1),MA-4 (1) (a),AU-3,AC-2 (4),AU-12 a,AU-12 c</t>
         </is>
       </c>
       <c r="B67" s="2" t="inlineStr">
@@ -5727,7 +5739,7 @@
     <row r="68" ht="130" customHeight="1">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>AU-12 c,AU-3,AC-2 (4),MA-4 (1) (a),AU-3 (1),AU-12 a</t>
+          <t>AU-3 (1),MA-4 (1) (a),AU-3,AC-2 (4),AU-12 a,AU-12 c</t>
         </is>
       </c>
       <c r="B68" s="2" t="inlineStr">
@@ -6847,7 +6859,7 @@
     <row r="82" ht="130" customHeight="1">
       <c r="A82" s="3" t="inlineStr">
         <is>
-          <t>AU-12 c,AU-3,MA-4 (1) (a),AU-3 (1),AU-12 a</t>
+          <t>AU-3 (1),MA-4 (1) (a),AU-3,AU-12 a,AU-12 c</t>
         </is>
       </c>
       <c r="B82" s="3" t="inlineStr">
@@ -6921,7 +6933,7 @@
     <row r="83" ht="130" customHeight="1">
       <c r="A83" s="3" t="inlineStr">
         <is>
-          <t>AU-12 c,AU-3,MA-4 (1) (a),AU-3 (1),AU-12 a</t>
+          <t>AU-3 (1),MA-4 (1) (a),AU-3,AU-12 a,AU-12 c</t>
         </is>
       </c>
       <c r="B83" s="3" t="inlineStr">
@@ -6995,7 +7007,7 @@
     <row r="84" ht="130" customHeight="1">
       <c r="A84" s="3" t="inlineStr">
         <is>
-          <t>AU-12 c,AU-3,MA-4 (1) (a),AU-3 (1),AU-12 a</t>
+          <t>AU-3 (1),MA-4 (1) (a),AU-3,AU-12 a,AU-12 c</t>
         </is>
       </c>
       <c r="B84" s="3" t="inlineStr">
@@ -7069,7 +7081,7 @@
     <row r="85" ht="130" customHeight="1">
       <c r="A85" s="3" t="inlineStr">
         <is>
-          <t>AU-12 c,AU-3,MA-4 (1) (a),AU-3 (1),AU-12 a</t>
+          <t>AU-3 (1),MA-4 (1) (a),AU-3,AU-12 a,AU-12 c</t>
         </is>
       </c>
       <c r="B85" s="3" t="inlineStr">
@@ -7645,7 +7657,7 @@
     <row r="92" ht="130" customHeight="1">
       <c r="A92" s="3" t="inlineStr">
         <is>
-          <t>AU-12 c,AU-3,MA-4 (1) (a),AU-3 (1),AU-12 a</t>
+          <t>AU-3 (1),MA-4 (1) (a),AU-3,AU-12 a,AU-12 c</t>
         </is>
       </c>
       <c r="B92" s="3" t="inlineStr">
@@ -7720,7 +7732,7 @@
     <row r="93" ht="130" customHeight="1">
       <c r="A93" s="3" t="inlineStr">
         <is>
-          <t>AU-12 c,AU-3,MA-4 (1) (a),AU-3 (1),AU-12 a</t>
+          <t>AU-3 (1),MA-4 (1) (a),AU-3,AU-12 a,AU-12 c</t>
         </is>
       </c>
       <c r="B93" s="3" t="inlineStr">
@@ -7795,7 +7807,7 @@
     <row r="94" ht="130" customHeight="1">
       <c r="A94" s="3" t="inlineStr">
         <is>
-          <t>AU-12 c,AU-3,MA-4 (1) (a),AU-3 (1),AU-12 a</t>
+          <t>AU-3 (1),MA-4 (1) (a),AU-3,AU-12 a,AU-12 c</t>
         </is>
       </c>
       <c r="B94" s="3" t="inlineStr">
@@ -7870,7 +7882,7 @@
     <row r="95" ht="130" customHeight="1">
       <c r="A95" s="3" t="inlineStr">
         <is>
-          <t>AU-12 c,AU-3,MA-4 (1) (a),AU-3 (1),AU-12 a</t>
+          <t>AU-3 (1),MA-4 (1) (a),AU-3,AU-12 a,AU-12 c</t>
         </is>
       </c>
       <c r="B95" s="3" t="inlineStr">
@@ -7950,7 +7962,7 @@
     <row r="96" ht="130" customHeight="1">
       <c r="A96" s="2" t="inlineStr">
         <is>
-          <t>AU-12 c,AU-3,MA-4 (1) (a),AU-3 (1),AU-12 a</t>
+          <t>AU-3 (1),MA-4 (1) (a),AU-3,AU-12 a,AU-12 c</t>
         </is>
       </c>
       <c r="B96" s="2" t="inlineStr">
@@ -8032,7 +8044,7 @@
     <row r="97" ht="130" customHeight="1">
       <c r="A97" s="2" t="inlineStr">
         <is>
-          <t>AU-12 c,AU-3,MA-4 (1) (a),AU-3 (1),AU-12 a</t>
+          <t>AU-3 (1),MA-4 (1) (a),AU-3,AU-12 a,AU-12 c</t>
         </is>
       </c>
       <c r="B97" s="2" t="inlineStr">
@@ -8114,7 +8126,7 @@
     <row r="98" ht="130" customHeight="1">
       <c r="A98" s="2" t="inlineStr">
         <is>
-          <t>AU-12 c,AU-3,MA-4 (1) (a),AU-3 (1),AU-12 a</t>
+          <t>AU-3 (1),MA-4 (1) (a),AU-3,AU-12 a,AU-12 c</t>
         </is>
       </c>
       <c r="B98" s="2" t="inlineStr">
@@ -8196,7 +8208,7 @@
     <row r="99" ht="130" customHeight="1">
       <c r="A99" s="2" t="inlineStr">
         <is>
-          <t>AU-12 c,AU-3,MA-4 (1) (a),AU-3 (1),AU-12 a</t>
+          <t>AU-3 (1),MA-4 (1) (a),AU-3,AU-12 a,AU-12 c</t>
         </is>
       </c>
       <c r="B99" s="2" t="inlineStr">
@@ -8278,7 +8290,7 @@
     <row r="100" ht="130" customHeight="1">
       <c r="A100" s="2" t="inlineStr">
         <is>
-          <t>AU-12 c,AU-3,MA-4 (1) (a),AU-3 (1),AU-12 a</t>
+          <t>AU-3 (1),MA-4 (1) (a),AU-3,AU-12 a,AU-12 c</t>
         </is>
       </c>
       <c r="B100" s="2" t="inlineStr">
@@ -8360,7 +8372,7 @@
     <row r="101" ht="130" customHeight="1">
       <c r="A101" s="3" t="inlineStr">
         <is>
-          <t>AU-12 c,AU-3,MA-4 (1) (a),AU-3 (1),AU-12 a</t>
+          <t>AU-3 (1),MA-4 (1) (a),AU-3,AU-12 a,AU-12 c</t>
         </is>
       </c>
       <c r="B101" s="3" t="inlineStr">
@@ -8440,7 +8452,7 @@
     <row r="102" ht="130" customHeight="1">
       <c r="A102" s="3" t="inlineStr">
         <is>
-          <t>AU-12 c,AU-3,MA-4 (1) (a),AU-3 (1),AU-12 a</t>
+          <t>AU-3 (1),MA-4 (1) (a),AU-3,AU-12 a,AU-12 c</t>
         </is>
       </c>
       <c r="B102" s="3" t="inlineStr">
@@ -8520,7 +8532,7 @@
     <row r="103" ht="130" customHeight="1">
       <c r="A103" s="3" t="inlineStr">
         <is>
-          <t>AU-12 c,AU-3,MA-4 (1) (a),AU-3 (1),AU-12 a</t>
+          <t>AU-3 (1),MA-4 (1) (a),AU-3,AU-12 a,AU-12 c</t>
         </is>
       </c>
       <c r="B103" s="3" t="inlineStr">
@@ -8771,7 +8783,7 @@
     <row r="106" ht="130" customHeight="1">
       <c r="A106" s="2" t="inlineStr">
         <is>
-          <t>AC-6 (10),AC-11 b</t>
+          <t>AC-11 b,AC-6 (10)</t>
         </is>
       </c>
       <c r="B106" s="2" t="inlineStr">
@@ -9348,7 +9360,7 @@
     <row r="113" ht="130" customHeight="1">
       <c r="A113" s="2" t="inlineStr">
         <is>
-          <t>AC-17 (2),SC-13,SC-8,MA-4 c</t>
+          <t>AC-17 (2),SC-8,SC-13,MA-4 c</t>
         </is>
       </c>
       <c r="B113" s="2" t="inlineStr">
@@ -9430,7 +9442,7 @@
     <row r="114" ht="130" customHeight="1">
       <c r="A114" s="2" t="inlineStr">
         <is>
-          <t>AU-12 c,MA-4 (1) (a)</t>
+          <t>MA-4 (1) (a),AU-12 c</t>
         </is>
       </c>
       <c r="B114" s="2" t="inlineStr">
@@ -9508,7 +9520,7 @@
     <row r="115" ht="130" customHeight="1">
       <c r="A115" s="2" t="inlineStr">
         <is>
-          <t>AU-12 c,AU-3,MA-4 (1) (a),AU-3 (1),AU-12 a</t>
+          <t>AU-3 (1),MA-4 (1) (a),AU-3,AU-12 a,AU-12 c</t>
         </is>
       </c>
       <c r="B115" s="2" t="inlineStr">
@@ -9586,7 +9598,7 @@
     <row r="116" ht="130" customHeight="1">
       <c r="A116" s="2" t="inlineStr">
         <is>
-          <t>AU-12 c,MA-4 (1) (a)</t>
+          <t>MA-4 (1) (a),AU-12 c</t>
         </is>
       </c>
       <c r="B116" s="2" t="inlineStr">
@@ -9664,7 +9676,7 @@
     <row r="117" ht="130" customHeight="1">
       <c r="A117" s="3" t="inlineStr">
         <is>
-          <t>AU-12 c,AU-3,MA-4 (1) (a),AU-3 (1),AU-12 a</t>
+          <t>AU-3 (1),MA-4 (1) (a),AU-3,AU-12 a,AU-12 c</t>
         </is>
       </c>
       <c r="B117" s="3" t="inlineStr">
@@ -9744,7 +9756,7 @@
     <row r="118" ht="130" customHeight="1">
       <c r="A118" s="3" t="inlineStr">
         <is>
-          <t>AU-12 c,MA-4 (1) (a)</t>
+          <t>MA-4 (1) (a),AU-12 c</t>
         </is>
       </c>
       <c r="B118" s="3" t="inlineStr">
@@ -9813,7 +9825,7 @@
     <row r="119" ht="130" customHeight="1">
       <c r="A119" s="3" t="inlineStr">
         <is>
-          <t>AU-12 c,MA-4 (1) (a)</t>
+          <t>MA-4 (1) (a),AU-12 c</t>
         </is>
       </c>
       <c r="B119" s="3" t="inlineStr">
@@ -9882,7 +9894,7 @@
     <row r="120" ht="130" customHeight="1">
       <c r="A120" s="3" t="inlineStr">
         <is>
-          <t>AU-12 c,MA-4 (1) (a)</t>
+          <t>MA-4 (1) (a),AU-12 c</t>
         </is>
       </c>
       <c r="B120" s="3" t="inlineStr">
@@ -9951,7 +9963,7 @@
     <row r="121" ht="130" customHeight="1">
       <c r="A121" s="3" t="inlineStr">
         <is>
-          <t>AU-12 c,MA-4 (1) (a)</t>
+          <t>MA-4 (1) (a),AU-12 c</t>
         </is>
       </c>
       <c r="B121" s="3" t="inlineStr">
@@ -10020,7 +10032,7 @@
     <row r="122" ht="130" customHeight="1">
       <c r="A122" s="3" t="inlineStr">
         <is>
-          <t>AU-12 c,AU-3,MA-4 (1) (a),AU-3 (1),AU-12 a</t>
+          <t>AU-3 (1),MA-4 (1) (a),AU-3,AU-12 a,AU-12 c</t>
         </is>
       </c>
       <c r="B122" s="3" t="inlineStr">
@@ -10217,7 +10229,14 @@
 Techniques used to address this include protocols using nonces (e.g., numbers generated for a specific one-time use) or challenges (e.g., TLS, WS_Security). Additional techniques include time-synchronous or challenge-response one-time authenticators.</t>
         </is>
       </c>
-      <c r="H124" s="2" t="inlineStr"/>
+      <c r="H124" s="2" t="inlineStr">
+        <is>
+          <t>A replay attack may enable an unauthorized user to gain access to Red Hat Enterprise Linux 9. Authentication sessions between the authenticator and Red Hat Enterprise Linux 9 validating the user credentials must not be vulnerable to a replay attack.
+An authentication process resists replay attacks if it is impractical to achieve a successful authentication by recording and replaying a previous authentication message.
+A privileged account is any information system account with authorizations of a privileged user.
+Techniques used to address this include protocols using nonces (e.g., numbers generated for a specific one-time use) or challenges (e.g., TLS, WS_Security). Additional techniques include time-synchronous or challenge-response one-time authenticators.</t>
+        </is>
+      </c>
       <c r="I124" s="2" t="inlineStr">
         <is>
           <t>Applicable - Inherently Met</t>
@@ -10867,7 +10886,7 @@
     <row r="133" ht="130" customHeight="1">
       <c r="A133" s="2" t="inlineStr">
         <is>
-          <t>AC-6 (10),CM-6 b</t>
+          <t>CM-6 b,AC-6 (10)</t>
         </is>
       </c>
       <c r="B133" s="2" t="inlineStr">
@@ -10948,7 +10967,7 @@
     <row r="134" ht="130" customHeight="1">
       <c r="A134" s="2" t="inlineStr">
         <is>
-          <t>AC-6 (10),CM-6 b</t>
+          <t>CM-6 b,AC-6 (10)</t>
         </is>
       </c>
       <c r="B134" s="2" t="inlineStr">
@@ -11034,7 +11053,7 @@
     <row r="135" ht="130" customHeight="1">
       <c r="A135" s="2" t="inlineStr">
         <is>
-          <t>AC-6 (10),CM-6 b</t>
+          <t>CM-6 b,AC-6 (10)</t>
         </is>
       </c>
       <c r="B135" s="2" t="inlineStr">
@@ -11400,7 +11419,7 @@
     <row r="139" ht="130" customHeight="1">
       <c r="A139" s="3" t="inlineStr">
         <is>
-          <t>AU-12 c,MA-4 (1) (a)</t>
+          <t>MA-4 (1) (a),AU-12 c</t>
         </is>
       </c>
       <c r="B139" s="3" t="inlineStr">
@@ -11480,7 +11499,7 @@
     <row r="140" ht="130" customHeight="1">
       <c r="A140" s="3" t="inlineStr">
         <is>
-          <t>AU-12 c,AU-3,MA-4 (1) (a),AU-3 (1),AU-12 a</t>
+          <t>AU-3 (1),MA-4 (1) (a),AU-3,AU-12 a,AU-12 c</t>
         </is>
       </c>
       <c r="B140" s="3" t="inlineStr">
@@ -11560,7 +11579,7 @@
     <row r="141" ht="130" customHeight="1">
       <c r="A141" s="3" t="inlineStr">
         <is>
-          <t>AU-12 c,AU-3,MA-4 (1) (a),AU-3 (1),AU-12 a</t>
+          <t>AU-3 (1),MA-4 (1) (a),AU-3,AU-12 a,AU-12 c</t>
         </is>
       </c>
       <c r="B141" s="3" t="inlineStr">
@@ -11640,7 +11659,7 @@
     <row r="142" ht="130" customHeight="1">
       <c r="A142" s="3" t="inlineStr">
         <is>
-          <t>AU-12 c,AU-3,MA-4 (1) (a),AU-3 (1),AU-12 a</t>
+          <t>AU-3 (1),MA-4 (1) (a),AU-3,AU-12 a,AU-12 c</t>
         </is>
       </c>
       <c r="B142" s="3" t="inlineStr">
@@ -12262,7 +12281,7 @@
     <row r="150" ht="130" customHeight="1">
       <c r="A150" s="2" t="inlineStr">
         <is>
-          <t>AC-11 (1),AC-11 a</t>
+          <t>AC-11 a,AC-11 (1)</t>
         </is>
       </c>
       <c r="B150" s="2" t="inlineStr">
@@ -12423,7 +12442,7 @@
     <row r="152" ht="130" customHeight="1">
       <c r="A152" s="2" t="inlineStr">
         <is>
-          <t>CM-6 b,IA-7</t>
+          <t>IA-7,CM-6 b</t>
         </is>
       </c>
       <c r="B152" s="2" t="inlineStr">
@@ -12499,7 +12518,7 @@
     <row r="153" ht="130" customHeight="1">
       <c r="A153" s="2" t="inlineStr">
         <is>
-          <t>CM-6 b,IA-7</t>
+          <t>IA-7,CM-6 b</t>
         </is>
       </c>
       <c r="B153" s="2" t="inlineStr">
@@ -12584,7 +12603,7 @@
     <row r="154" ht="130" customHeight="1">
       <c r="A154" s="2" t="inlineStr">
         <is>
-          <t>CM-6 b,IA-7</t>
+          <t>IA-7,CM-6 b</t>
         </is>
       </c>
       <c r="B154" s="2" t="inlineStr">
@@ -12820,7 +12839,7 @@
     <row r="157" ht="130" customHeight="1">
       <c r="A157" s="3" t="inlineStr">
         <is>
-          <t>AU-12 c,AU-3,MA-4 (1) (a),AU-3 (1),AU-12 a</t>
+          <t>AU-3 (1),MA-4 (1) (a),AU-3,AU-12 a,AU-12 c</t>
         </is>
       </c>
       <c r="B157" s="3" t="inlineStr">
@@ -12897,7 +12916,7 @@
     <row r="158" ht="130" customHeight="1">
       <c r="A158" s="3" t="inlineStr">
         <is>
-          <t>AU-12 c,AU-3,MA-4 (1) (a),AU-12 a</t>
+          <t>MA-4 (1) (a),AU-3,AU-12 c,AU-12 a</t>
         </is>
       </c>
       <c r="B158" s="3" t="inlineStr">
@@ -12970,7 +12989,7 @@
     <row r="159" ht="130" customHeight="1">
       <c r="A159" s="3" t="inlineStr">
         <is>
-          <t>AU-12 c,AU-3,MA-4 (1) (a),AU-12 a</t>
+          <t>MA-4 (1) (a),AU-3,AU-12 c,AU-12 a</t>
         </is>
       </c>
       <c r="B159" s="3" t="inlineStr">
@@ -13043,7 +13062,7 @@
     <row r="160" ht="130" customHeight="1">
       <c r="A160" s="3" t="inlineStr">
         <is>
-          <t>AU-12 c,AU-3,MA-4 (1) (a),AU-3 (1),AU-12 a</t>
+          <t>AU-3 (1),MA-4 (1) (a),AU-3,AU-12 a,AU-12 c</t>
         </is>
       </c>
       <c r="B160" s="3" t="inlineStr">
@@ -13128,7 +13147,7 @@
     <row r="161" ht="130" customHeight="1">
       <c r="A161" s="3" t="inlineStr">
         <is>
-          <t>AU-12 c,AU-3,MA-4 (1) (a),AU-3 (1),AU-12 a</t>
+          <t>AU-3 (1),MA-4 (1) (a),AU-3,AU-12 a,AU-12 c</t>
         </is>
       </c>
       <c r="B161" s="3" t="inlineStr">
@@ -13203,7 +13222,7 @@
     <row r="162" ht="130" customHeight="1">
       <c r="A162" s="3" t="inlineStr">
         <is>
-          <t>AU-12 c,AU-3,MA-4 (1) (a),AU-3 (1),AU-12 a</t>
+          <t>AU-3 (1),MA-4 (1) (a),AU-3,AU-12 a,AU-12 c</t>
         </is>
       </c>
       <c r="B162" s="3" t="inlineStr">
@@ -13278,7 +13297,7 @@
     <row r="163" ht="130" customHeight="1">
       <c r="A163" s="3" t="inlineStr">
         <is>
-          <t>AU-12 c,AU-3,MA-4 (1) (a),AU-3 (1),AU-12 a</t>
+          <t>AU-3 (1),MA-4 (1) (a),AU-3,AU-12 a,AU-12 c</t>
         </is>
       </c>
       <c r="B163" s="3" t="inlineStr">
@@ -13353,7 +13372,7 @@
     <row r="164" ht="130" customHeight="1">
       <c r="A164" s="3" t="inlineStr">
         <is>
-          <t>AU-12 c,AU-3,MA-4 (1) (a),AU-3 (1),AU-12 a</t>
+          <t>AU-3 (1),MA-4 (1) (a),AU-3,AU-12 a,AU-12 c</t>
         </is>
       </c>
       <c r="B164" s="3" t="inlineStr">
@@ -13428,7 +13447,7 @@
     <row r="165" ht="130" customHeight="1">
       <c r="A165" s="3" t="inlineStr">
         <is>
-          <t>AU-12 c,MA-4 (1) (a)</t>
+          <t>MA-4 (1) (a),AU-12 c</t>
         </is>
       </c>
       <c r="B165" s="3" t="inlineStr">
@@ -13499,7 +13518,7 @@
     <row r="166" ht="130" customHeight="1">
       <c r="A166" s="3" t="inlineStr">
         <is>
-          <t>AU-12 c,MA-4 (1) (a)</t>
+          <t>MA-4 (1) (a),AU-12 c</t>
         </is>
       </c>
       <c r="B166" s="3" t="inlineStr">
@@ -13570,7 +13589,7 @@
     <row r="167" ht="130" customHeight="1">
       <c r="A167" s="3" t="inlineStr">
         <is>
-          <t>AU-12 c,MA-4 (1) (a)</t>
+          <t>MA-4 (1) (a),AU-12 c</t>
         </is>
       </c>
       <c r="B167" s="3" t="inlineStr">
@@ -13642,7 +13661,7 @@
     <row r="168" ht="130" customHeight="1">
       <c r="A168" s="3" t="inlineStr">
         <is>
-          <t>AU-12 c,MA-4 (1) (a)</t>
+          <t>MA-4 (1) (a),AU-12 c</t>
         </is>
       </c>
       <c r="B168" s="3" t="inlineStr">
@@ -13713,7 +13732,7 @@
     <row r="169" ht="130" customHeight="1">
       <c r="A169" s="3" t="inlineStr">
         <is>
-          <t>AU-12 c,MA-4 (1) (a)</t>
+          <t>MA-4 (1) (a),AU-12 c</t>
         </is>
       </c>
       <c r="B169" s="3" t="inlineStr">
@@ -13784,7 +13803,7 @@
     <row r="170" ht="130" customHeight="1">
       <c r="A170" s="3" t="inlineStr">
         <is>
-          <t>AU-12 c,MA-4 (1) (a)</t>
+          <t>MA-4 (1) (a),AU-12 c</t>
         </is>
       </c>
       <c r="B170" s="3" t="inlineStr">
@@ -13856,7 +13875,7 @@
     <row r="171" ht="130" customHeight="1">
       <c r="A171" s="3" t="inlineStr">
         <is>
-          <t>AU-12 c,AU-3,MA-4 (1) (a),AU-3 (1),AU-12 a</t>
+          <t>AU-3 (1),MA-4 (1) (a),AU-3,AU-12 a,AU-12 c</t>
         </is>
       </c>
       <c r="B171" s="3" t="inlineStr">
@@ -13931,7 +13950,7 @@
     <row r="172" ht="130" customHeight="1">
       <c r="A172" s="3" t="inlineStr">
         <is>
-          <t>AU-12 c,MA-4 (1) (a)</t>
+          <t>MA-4 (1) (a),AU-12 c</t>
         </is>
       </c>
       <c r="B172" s="3" t="inlineStr">
@@ -14002,7 +14021,7 @@
     <row r="173" ht="130" customHeight="1">
       <c r="A173" s="3" t="inlineStr">
         <is>
-          <t>AU-12 c,MA-4 (1) (a)</t>
+          <t>MA-4 (1) (a),AU-12 c</t>
         </is>
       </c>
       <c r="B173" s="3" t="inlineStr">
@@ -14073,7 +14092,7 @@
     <row r="174" ht="130" customHeight="1">
       <c r="A174" s="3" t="inlineStr">
         <is>
-          <t>AU-12 c,MA-4 (1) (a)</t>
+          <t>MA-4 (1) (a),AU-12 c</t>
         </is>
       </c>
       <c r="B174" s="3" t="inlineStr">
@@ -14145,7 +14164,7 @@
     <row r="175" ht="130" customHeight="1">
       <c r="A175" s="3" t="inlineStr">
         <is>
-          <t>AU-12 c,AU-3,MA-4 (1) (a),AU-3 (1),AU-12 a</t>
+          <t>AU-3 (1),MA-4 (1) (a),AU-3,AU-12 a,AU-12 c</t>
         </is>
       </c>
       <c r="B175" s="3" t="inlineStr">
@@ -14220,7 +14239,7 @@
     <row r="176" ht="130" customHeight="1">
       <c r="A176" s="3" t="inlineStr">
         <is>
-          <t>AU-12 c,AU-3,MA-4 (1) (a),AU-3 (1),AU-12 a</t>
+          <t>AU-3 (1),MA-4 (1) (a),AU-3,AU-12 a,AU-12 c</t>
         </is>
       </c>
       <c r="B176" s="3" t="inlineStr">
@@ -14302,7 +14321,7 @@
     <row r="177" ht="130" customHeight="1">
       <c r="A177" s="3" t="inlineStr">
         <is>
-          <t>AU-12 c,AU-3,MA-4 (1) (a),AU-3 (1),AU-12 a</t>
+          <t>AU-3 (1),MA-4 (1) (a),AU-3,AU-12 a,AU-12 c</t>
         </is>
       </c>
       <c r="B177" s="3" t="inlineStr">
@@ -14384,7 +14403,7 @@
     <row r="178" ht="130" customHeight="1">
       <c r="A178" s="3" t="inlineStr">
         <is>
-          <t>AU-12 c,AU-3,MA-4 (1) (a),AU-3 (1),AU-12 a</t>
+          <t>AU-3 (1),MA-4 (1) (a),AU-3,AU-12 a,AU-12 c</t>
         </is>
       </c>
       <c r="B178" s="3" t="inlineStr">
@@ -14466,7 +14485,7 @@
     <row r="179" ht="130" customHeight="1">
       <c r="A179" s="3" t="inlineStr">
         <is>
-          <t>AU-3,MA-4 (1) (a),AU-3 (1)</t>
+          <t>MA-4 (1) (a),AU-3,AU-3 (1)</t>
         </is>
       </c>
       <c r="B179" s="3" t="inlineStr">
@@ -14548,7 +14567,7 @@
     <row r="180" ht="130" customHeight="1">
       <c r="A180" s="3" t="inlineStr">
         <is>
-          <t>AU-12 c,AU-3,MA-4 (1) (a),AU-3 (1),AU-12 a</t>
+          <t>AU-3 (1),MA-4 (1) (a),AU-3,AU-12 a,AU-12 c</t>
         </is>
       </c>
       <c r="B180" s="3" t="inlineStr">
@@ -14630,7 +14649,7 @@
     <row r="181" ht="130" customHeight="1">
       <c r="A181" s="3" t="inlineStr">
         <is>
-          <t>AU-12 c,AU-3,MA-4 (1) (a),AU-3 (1),AU-12 a</t>
+          <t>AU-3 (1),MA-4 (1) (a),AU-3,AU-12 a,AU-12 c</t>
         </is>
       </c>
       <c r="B181" s="3" t="inlineStr">
@@ -14712,7 +14731,7 @@
     <row r="182" ht="130" customHeight="1">
       <c r="A182" s="3" t="inlineStr">
         <is>
-          <t>AU-12 c,AU-3,MA-4 (1) (a),AU-3 (1),AU-12 a</t>
+          <t>AU-3 (1),MA-4 (1) (a),AU-3,AU-12 a,AU-12 c</t>
         </is>
       </c>
       <c r="B182" s="3" t="inlineStr">
@@ -14794,7 +14813,7 @@
     <row r="183" ht="130" customHeight="1">
       <c r="A183" s="3" t="inlineStr">
         <is>
-          <t>AU-12 c,AU-3,MA-4 (1) (a),AU-3 (1),AU-12 a</t>
+          <t>AU-3 (1),MA-4 (1) (a),AU-3,AU-12 a,AU-12 c</t>
         </is>
       </c>
       <c r="B183" s="3" t="inlineStr">
@@ -14876,7 +14895,7 @@
     <row r="184" ht="130" customHeight="1">
       <c r="A184" s="3" t="inlineStr">
         <is>
-          <t>AU-12 c,AU-3,MA-4 (1) (a),AU-3 (1),AU-12 a</t>
+          <t>AU-3 (1),MA-4 (1) (a),AU-3,AU-12 a,AU-12 c</t>
         </is>
       </c>
       <c r="B184" s="3" t="inlineStr">
@@ -14958,7 +14977,7 @@
     <row r="185" ht="130" customHeight="1">
       <c r="A185" s="3" t="inlineStr">
         <is>
-          <t>AU-12 c,MA-4 (1) (a),AU-3 (1)</t>
+          <t>MA-4 (1) (a),AU-3 (1),AU-12 c</t>
         </is>
       </c>
       <c r="B185" s="3" t="inlineStr">
@@ -15036,7 +15055,7 @@
     <row r="186" ht="130" customHeight="1">
       <c r="A186" s="3" t="inlineStr">
         <is>
-          <t>AU-12 c,AU-3,MA-4 (1) (a),AU-3 (1),AU-12 a</t>
+          <t>AU-3 (1),MA-4 (1) (a),AU-3,AU-12 a,AU-12 c</t>
         </is>
       </c>
       <c r="B186" s="3" t="inlineStr">
@@ -15115,7 +15134,7 @@
     <row r="187" ht="130" customHeight="1">
       <c r="A187" s="3" t="inlineStr">
         <is>
-          <t>AU-12 c,AU-3,MA-4 (1) (a),AU-3 (1),AU-12 a</t>
+          <t>AU-3 (1),MA-4 (1) (a),AU-3,AU-12 a,AU-12 c</t>
         </is>
       </c>
       <c r="B187" s="3" t="inlineStr">
@@ -15197,7 +15216,7 @@
     <row r="188" ht="130" customHeight="1">
       <c r="A188" s="3" t="inlineStr">
         <is>
-          <t>AU-12 c,AU-3,MA-4 (1) (a),AU-3 (1),AU-12 a</t>
+          <t>AU-3 (1),MA-4 (1) (a),AU-3,AU-12 a,AU-12 c</t>
         </is>
       </c>
       <c r="B188" s="3" t="inlineStr">
@@ -15279,7 +15298,7 @@
     <row r="189" ht="130" customHeight="1">
       <c r="A189" s="3" t="inlineStr">
         <is>
-          <t>AU-12 c,AU-3,MA-4 (1) (a),AU-3 (1)</t>
+          <t>MA-4 (1) (a),AU-3,AU-3 (1),AU-12 c</t>
         </is>
       </c>
       <c r="B189" s="3" t="inlineStr">
@@ -15361,7 +15380,7 @@
     <row r="190" ht="130" customHeight="1">
       <c r="A190" s="3" t="inlineStr">
         <is>
-          <t>AU-12 c,AU-3,MA-4 (1) (a),AU-3 (1),AU-12 a</t>
+          <t>AU-3 (1),MA-4 (1) (a),AU-3,AU-12 a,AU-12 c</t>
         </is>
       </c>
       <c r="B190" s="3" t="inlineStr">
@@ -15443,7 +15462,7 @@
     <row r="191" ht="130" customHeight="1">
       <c r="A191" s="3" t="inlineStr">
         <is>
-          <t>AU-12 c,AU-3,MA-4 (1) (a),AU-3 (1),AU-12 a</t>
+          <t>AU-3 (1),MA-4 (1) (a),AU-3,AU-12 a,AU-12 c</t>
         </is>
       </c>
       <c r="B191" s="3" t="inlineStr">
@@ -15525,7 +15544,7 @@
     <row r="192" ht="130" customHeight="1">
       <c r="A192" s="3" t="inlineStr">
         <is>
-          <t>AU-12 c,AU-3,MA-4 (1) (a),AU-3 (1),AU-12 a</t>
+          <t>AU-3 (1),MA-4 (1) (a),AU-3,AU-12 a,AU-12 c</t>
         </is>
       </c>
       <c r="B192" s="3" t="inlineStr">
@@ -15607,7 +15626,7 @@
     <row r="193" ht="130" customHeight="1">
       <c r="A193" s="3" t="inlineStr">
         <is>
-          <t>AU-12 c,AU-3,MA-4 (1) (a),AU-3 (1),AU-12 a</t>
+          <t>AU-3 (1),MA-4 (1) (a),AU-3,AU-12 a,AU-12 c</t>
         </is>
       </c>
       <c r="B193" s="3" t="inlineStr">
@@ -15682,7 +15701,7 @@
     <row r="194" ht="130" customHeight="1">
       <c r="A194" s="3" t="inlineStr">
         <is>
-          <t>AU-12 c,AU-3,AC-2 (4),MA-4 (1) (a),AU-3 (1),AU-12 a</t>
+          <t>AU-3 (1),MA-4 (1) (a),AU-3,AC-2 (4),AU-12 a,AU-12 c</t>
         </is>
       </c>
       <c r="B194" s="3" t="inlineStr">
@@ -15755,7 +15774,7 @@
     <row r="195" ht="130" customHeight="1">
       <c r="A195" s="3" t="inlineStr">
         <is>
-          <t>AU-12 c,AU-3,AC-2 (4),MA-4 (1) (a),AU-3 (1)</t>
+          <t>AU-3 (1),MA-4 (1) (a),AU-3,AC-2 (4),AU-12 c</t>
         </is>
       </c>
       <c r="B195" s="3" t="inlineStr">
@@ -15832,7 +15851,7 @@
     <row r="196" ht="130" customHeight="1">
       <c r="A196" s="2" t="inlineStr">
         <is>
-          <t>IA-2 (1),IA-2 (2),IA-2 (3),IA-2 (4)</t>
+          <t>IA-2 (3),IA-2 (2),IA-2 (1),IA-2 (4)</t>
         </is>
       </c>
       <c r="B196" s="2" t="inlineStr">
@@ -15919,7 +15938,7 @@
     <row r="197" ht="130" customHeight="1">
       <c r="A197" s="2" t="inlineStr">
         <is>
-          <t>IA-2,IA-2 (4),IA-2 (2),IA-2 (5),IA-2 (3)</t>
+          <t>IA-2 (4),IA-2,IA-2 (2),IA-2 (3),IA-2 (5)</t>
         </is>
       </c>
       <c r="B197" s="2" t="inlineStr">
@@ -16008,7 +16027,7 @@
     <row r="198" ht="130" customHeight="1">
       <c r="A198" s="2" t="inlineStr">
         <is>
-          <t>IA-2,IA-2 (4),IA-2 (2),IA-2 (5),IA-2 (3)</t>
+          <t>IA-2 (4),IA-2,IA-2 (2),IA-2 (3),IA-2 (5)</t>
         </is>
       </c>
       <c r="B198" s="2" t="inlineStr">
@@ -16881,7 +16900,7 @@
     <row r="209" ht="130" customHeight="1">
       <c r="A209" s="2" t="inlineStr">
         <is>
-          <t>AC-11 (1),AC-11 a</t>
+          <t>AC-11 a,AC-11 (1)</t>
         </is>
       </c>
       <c r="B209" s="2" t="inlineStr">
@@ -16970,7 +16989,7 @@
     <row r="210" ht="130" customHeight="1">
       <c r="A210" s="2" t="inlineStr">
         <is>
-          <t>AC-11 (1),AC-11 a</t>
+          <t>AC-11 a,AC-11 (1)</t>
         </is>
       </c>
       <c r="B210" s="2" t="inlineStr">
@@ -17223,7 +17242,7 @@
     <row r="213" ht="130" customHeight="1">
       <c r="A213" s="2" t="inlineStr">
         <is>
-          <t>CM-6 b,CM-7 a,IA-5 (1) (c)</t>
+          <t>CM-7 a,CM-6 b,IA-5 (1) (c)</t>
         </is>
       </c>
       <c r="B213" s="2" t="inlineStr">
@@ -17381,37 +17400,37 @@
       <c r="Q214" s="3" t="n"/>
     </row>
     <row r="215" ht="130" customHeight="1">
-      <c r="A215" s="3" t="inlineStr">
+      <c r="A215" s="2" t="inlineStr">
         <is>
           <t>CM-6 b,AU-12 a</t>
         </is>
       </c>
-      <c r="B215" s="3" t="inlineStr">
+      <c r="B215" s="2" t="inlineStr">
         <is>
           <t>CCI-000366</t>
         </is>
       </c>
-      <c r="C215" s="3" t="inlineStr">
+      <c r="C215" s="2" t="inlineStr">
         <is>
           <t>SRG-OS-000062-GPOS-00031,SRG-OS-000480-GPOS-00227</t>
         </is>
       </c>
-      <c r="D215" s="3" t="inlineStr">
+      <c r="D215" s="2" t="inlineStr">
         <is>
           <t>CCE-83682-5</t>
         </is>
       </c>
-      <c r="E215" s="3" t="inlineStr">
+      <c r="E215" s="2" t="inlineStr">
         <is>
           <t>The operating system must provide audit record generation capability for DoD-defined auditable events for all operating system components.</t>
         </is>
       </c>
-      <c r="F215" s="3" t="inlineStr">
+      <c r="F215" s="2" t="inlineStr">
         <is>
           <t>Red Hat Enterprise Linux 9 must provide audit record generation capability for DoD-defined auditable events for all operating system components.</t>
         </is>
       </c>
-      <c r="G215" s="3" t="inlineStr">
+      <c r="G215" s="2" t="inlineStr">
         <is>
           <t>Without the capability to generate audit records, it would be difficult to establish, correlate, and investigate the events relating to an incident or identify those responsible for one.
 Audit records can be generated from various components within the information system (e.g., module or policy filter).
@@ -17423,18 +17442,18 @@
 4) All kernel module load, unload, and restart actions.</t>
         </is>
       </c>
-      <c r="H215" s="3" t="inlineStr">
+      <c r="H215" s="2" t="inlineStr">
         <is>
           <t>If option "local_events" isn't set to "yes" only events from
 network will be aggregated.</t>
         </is>
       </c>
-      <c r="I215" s="3" t="inlineStr">
-        <is>
-          <t>Applicable - Configurable</t>
-        </is>
-      </c>
-      <c r="J215" s="3" t="inlineStr">
+      <c r="I215" s="2" t="inlineStr">
+        <is>
+          <t>Applicable - Configurable</t>
+        </is>
+      </c>
+      <c r="J215" s="2" t="inlineStr">
         <is>
           <t>Verify the operating system provides audit record generation capability for DoD-defined auditable events for all operating system components. 
 DoD has defined the list of events for which the operating system will provide an audit record generation capability as the following: 
@@ -17445,7 +17464,7 @@
 If it does not, this is a finding.</t>
         </is>
       </c>
-      <c r="K215" s="3" t="inlineStr">
+      <c r="K215" s="2" t="inlineStr">
         <is>
           <t>To verify that Audit Daemon is configured to include local events, run the
 following command:
@@ -17455,21 +17474,26 @@
 If local_events isn't set to yes, then this is a finding.</t>
         </is>
       </c>
-      <c r="L215" s="3" t="n"/>
-      <c r="M215" s="3" t="inlineStr"/>
-      <c r="N215" s="3" t="inlineStr">
-        <is>
-          <t>CAT II</t>
-        </is>
-      </c>
-      <c r="O215" s="3" t="n"/>
-      <c r="P215" s="3" t="n"/>
-      <c r="Q215" s="3" t="n"/>
+      <c r="L215" s="2" t="n"/>
+      <c r="M215" s="2" t="inlineStr">
+        <is>
+          <t>Edit the file "/etc/audit/auditd.conf" and add or edit the following line:
+local_events = yes</t>
+        </is>
+      </c>
+      <c r="N215" s="2" t="inlineStr">
+        <is>
+          <t>CAT II</t>
+        </is>
+      </c>
+      <c r="O215" s="2" t="n"/>
+      <c r="P215" s="2" t="n"/>
+      <c r="Q215" s="2" t="n"/>
     </row>
     <row r="216" ht="130" customHeight="1">
       <c r="A216" s="2" t="inlineStr">
         <is>
-          <t>CM-6 b,SC-5 (2),SC-5</t>
+          <t>CM-6 b,SC-5,SC-5 (2)</t>
         </is>
       </c>
       <c r="B216" s="2" t="inlineStr">
@@ -17649,7 +17673,7 @@
     <row r="218" ht="130" customHeight="1">
       <c r="A218" s="2" t="inlineStr">
         <is>
-          <t>SI-16,CM-7 a</t>
+          <t>CM-7 a,SI-16</t>
         </is>
       </c>
       <c r="B218" s="2" t="inlineStr">
@@ -17741,7 +17765,7 @@
     <row r="219" ht="130" customHeight="1">
       <c r="A219" s="2" t="inlineStr">
         <is>
-          <t>CM-6 b,SI-16</t>
+          <t>SI-16,CM-6 b</t>
         </is>
       </c>
       <c r="B219" s="2" t="inlineStr">
@@ -17839,7 +17863,7 @@
     <row r="220" ht="130" customHeight="1">
       <c r="A220" s="2" t="inlineStr">
         <is>
-          <t>AU-3 (1),IA-2,IA-8</t>
+          <t>IA-2,AU-3 (1),IA-8</t>
         </is>
       </c>
       <c r="B220" s="2" t="inlineStr">
@@ -18074,43 +18098,43 @@
       <c r="Q222" s="2" t="n"/>
     </row>
     <row r="223" ht="130" customHeight="1">
-      <c r="A223" s="3" t="inlineStr">
+      <c r="A223" s="2" t="inlineStr">
         <is>
           <t>CM-5 (6)</t>
         </is>
       </c>
-      <c r="B223" s="3" t="inlineStr">
+      <c r="B223" s="2" t="inlineStr">
         <is>
           <t>CCI-001499</t>
         </is>
       </c>
-      <c r="C223" s="3" t="inlineStr">
+      <c r="C223" s="2" t="inlineStr">
         <is>
           <t>SRG-OS-000259-GPOS-00100</t>
         </is>
       </c>
-      <c r="D223" s="3" t="inlineStr">
+      <c r="D223" s="2" t="inlineStr">
         <is>
           <t>CCE-89858-5</t>
         </is>
       </c>
-      <c r="E223" s="3" t="inlineStr">
+      <c r="E223" s="2" t="inlineStr">
         <is>
           <t>The operating system must limit privileges to change software resident within software libraries.</t>
         </is>
       </c>
-      <c r="F223" s="3" t="inlineStr">
+      <c r="F223" s="2" t="inlineStr">
         <is>
           <t>Red Hat Enterprise Linux 9 must limit privileges to change software resident within software libraries.</t>
         </is>
       </c>
-      <c r="G223" s="3" t="inlineStr">
+      <c r="G223" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve"> If the operating system were to allow any user to make changes to software libraries, then those changes might be implemented without undergoing the appropriate testing and approvals that are part of a robust change management process.
 This requirement applies to operating systems with software libraries that are accessible and configurable, as in the case of interpreted languages. Software libraries also include privileged programs which execute with escalated privileges. Only qualified and authorized individuals shall be allowed to obtain access to information system components for purposes of initiating changes, including upgrades and modifications.</t>
         </is>
       </c>
-      <c r="H223" s="3" t="inlineStr">
+      <c r="H223" s="2" t="inlineStr">
         <is>
           <t>Files from shared library directories are loaded into the address
 space of processes (including privileged ones) or of the kernel itself at
@@ -18118,78 +18142,79 @@
 the integrity of the system.</t>
         </is>
       </c>
-      <c r="I223" s="3" t="inlineStr">
-        <is>
-          <t>Applicable - Configurable</t>
-        </is>
-      </c>
-      <c r="J223" s="3" t="inlineStr">
+      <c r="I223" s="2" t="inlineStr">
+        <is>
+          <t>Applicable - Configurable</t>
+        </is>
+      </c>
+      <c r="J223" s="2" t="inlineStr">
         <is>
           <t>Verify the operating system limits privileges to change software resident within software libraries. If it does not, this is a finding.</t>
         </is>
       </c>
-      <c r="K223" s="3" t="inlineStr">
-        <is>
-          <t>Shared libraries are stored in the following directories:
- /lib
-/lib64
-/usr/lib
-/usr/lib64 
-For each of these directories, run the following command to find files not
-owned by root:
- $ sudo find -L  $DIR  ! -user root -type d -exec chgrp root {} \; 
-If any of these directories are not group-owned by root, then this is a finding.</t>
-        </is>
-      </c>
-      <c r="L223" s="3" t="n"/>
-      <c r="M223" s="3" t="inlineStr"/>
-      <c r="N223" s="3" t="inlineStr">
-        <is>
-          <t>CAT II</t>
-        </is>
-      </c>
-      <c r="O223" s="3" t="n"/>
-      <c r="P223" s="3" t="n"/>
-      <c r="Q223" s="3" t="n"/>
+      <c r="K223" s="2" t="inlineStr">
+        <is>
+          <t>Verify the system-wide shared library directories are group-owned by "root" with the following command:
+$ sudo find /lib /lib64 /usr/lib /usr/lib64 ! -group root -type d -exec stat -c "%n %G" '{}' \;
+If any system-wide shared library directory is returned and is not group-owned by a required system account, this is a finding.
+If any system-wide shared library directory is returned and is not group-owned by a required system account, then this is a finding.</t>
+        </is>
+      </c>
+      <c r="L223" s="2" t="n"/>
+      <c r="M223" s="2" t="inlineStr">
+        <is>
+          <t>Configure the system-wide shared library directories (/lib, /lib64, /usr/lib and /usr/lib64) to be protected from unauthorized access.
+Run the following command, replacing "[DIRECTORY]" with any library directory not group-owned by "root".
+$ sudo chgrp root [DIRECTORY]</t>
+        </is>
+      </c>
+      <c r="N223" s="2" t="inlineStr">
+        <is>
+          <t>CAT II</t>
+        </is>
+      </c>
+      <c r="O223" s="2" t="n"/>
+      <c r="P223" s="2" t="n"/>
+      <c r="Q223" s="2" t="n"/>
     </row>
     <row r="224" ht="130" customHeight="1">
-      <c r="A224" s="3" t="inlineStr">
+      <c r="A224" s="2" t="inlineStr">
         <is>
           <t>CM-5 (6)</t>
         </is>
       </c>
-      <c r="B224" s="3" t="inlineStr">
+      <c r="B224" s="2" t="inlineStr">
         <is>
           <t>CCI-001499</t>
         </is>
       </c>
-      <c r="C224" s="3" t="inlineStr">
+      <c r="C224" s="2" t="inlineStr">
         <is>
           <t>SRG-OS-000259-GPOS-00100</t>
         </is>
       </c>
-      <c r="D224" s="3" t="inlineStr">
+      <c r="D224" s="2" t="inlineStr">
         <is>
           <t>CCE-89022-8</t>
         </is>
       </c>
-      <c r="E224" s="3" t="inlineStr">
+      <c r="E224" s="2" t="inlineStr">
         <is>
           <t>The operating system must limit privileges to change software resident within software libraries.</t>
         </is>
       </c>
-      <c r="F224" s="3" t="inlineStr">
+      <c r="F224" s="2" t="inlineStr">
         <is>
           <t>Red Hat Enterprise Linux 9 must limit privileges to change software resident within software libraries.</t>
         </is>
       </c>
-      <c r="G224" s="3" t="inlineStr">
+      <c r="G224" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve"> If the operating system were to allow any user to make changes to software libraries, then those changes might be implemented without undergoing the appropriate testing and approvals that are part of a robust change management process.
 This requirement applies to operating systems with software libraries that are accessible and configurable, as in the case of interpreted languages. Software libraries also include privileged programs which execute with escalated privileges. Only qualified and authorized individuals shall be allowed to obtain access to information system components for purposes of initiating changes, including upgrades and modifications.</t>
         </is>
       </c>
-      <c r="H224" s="3" t="inlineStr">
+      <c r="H224" s="2" t="inlineStr">
         <is>
           <t>Files from shared library directories are loaded into the address
 space of processes (including privileged ones) or of the kernel itself at
@@ -18197,78 +18222,78 @@
 the integrity of the system.</t>
         </is>
       </c>
-      <c r="I224" s="3" t="inlineStr">
-        <is>
-          <t>Applicable - Configurable</t>
-        </is>
-      </c>
-      <c r="J224" s="3" t="inlineStr">
+      <c r="I224" s="2" t="inlineStr">
+        <is>
+          <t>Applicable - Configurable</t>
+        </is>
+      </c>
+      <c r="J224" s="2" t="inlineStr">
         <is>
           <t>Verify the operating system limits privileges to change software resident within software libraries. If it does not, this is a finding.</t>
         </is>
       </c>
-      <c r="K224" s="3" t="inlineStr">
-        <is>
-          <t>Shared libraries are stored in the following directories:
- /lib
-/lib64
-/usr/lib
-/usr/lib64 
-For each of these directories, run the following command to find files not
-owned by root:
- $ sudo find -L  $DIR  ! -user root -type d -exec chown root {} \; 
-If any of these directories are not owned by root, then this is a finding.</t>
-        </is>
-      </c>
-      <c r="L224" s="3" t="n"/>
-      <c r="M224" s="3" t="inlineStr"/>
-      <c r="N224" s="3" t="inlineStr">
-        <is>
-          <t>CAT II</t>
-        </is>
-      </c>
-      <c r="O224" s="3" t="n"/>
-      <c r="P224" s="3" t="n"/>
-      <c r="Q224" s="3" t="n"/>
+      <c r="K224" s="2" t="inlineStr">
+        <is>
+          <t>Verify the system-wide shared library directories are owned by "root" with the following command:
+$ sudo find /lib /lib64 /usr/lib /usr/lib64 ! -user root -type d -exec stat -c "%n %U" '{}' \;
+If any system-wide shared library directory is not owned by root, then this is a finding.</t>
+        </is>
+      </c>
+      <c r="L224" s="2" t="n"/>
+      <c r="M224" s="2" t="inlineStr">
+        <is>
+          <t>Configure the system-wide shared library directories within (/lib, /lib64, /usr/lib and /usr/lib64) to be protected from unauthorized access.
+Run the following command, replacing "[DIRECTORY]" with any library directory not owned by "root".
+$ sudo chown root [DIRECTORY]</t>
+        </is>
+      </c>
+      <c r="N224" s="2" t="inlineStr">
+        <is>
+          <t>CAT II</t>
+        </is>
+      </c>
+      <c r="O224" s="2" t="n"/>
+      <c r="P224" s="2" t="n"/>
+      <c r="Q224" s="2" t="n"/>
     </row>
     <row r="225" ht="130" customHeight="1">
-      <c r="A225" s="3" t="inlineStr">
+      <c r="A225" s="2" t="inlineStr">
         <is>
           <t>CM-5 (6)</t>
         </is>
       </c>
-      <c r="B225" s="3" t="inlineStr">
+      <c r="B225" s="2" t="inlineStr">
         <is>
           <t>CCI-001499</t>
         </is>
       </c>
-      <c r="C225" s="3" t="inlineStr">
+      <c r="C225" s="2" t="inlineStr">
         <is>
           <t>SRG-OS-000259-GPOS-00100</t>
         </is>
       </c>
-      <c r="D225" s="3" t="inlineStr">
+      <c r="D225" s="2" t="inlineStr">
         <is>
           <t>CCE-89442-8</t>
         </is>
       </c>
-      <c r="E225" s="3" t="inlineStr">
+      <c r="E225" s="2" t="inlineStr">
         <is>
           <t>The operating system must limit privileges to change software resident within software libraries.</t>
         </is>
       </c>
-      <c r="F225" s="3" t="inlineStr">
+      <c r="F225" s="2" t="inlineStr">
         <is>
           <t>Red Hat Enterprise Linux 9 must limit privileges to change software resident within software libraries.</t>
         </is>
       </c>
-      <c r="G225" s="3" t="inlineStr">
+      <c r="G225" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve"> If the operating system were to allow any user to make changes to software libraries, then those changes might be implemented without undergoing the appropriate testing and approvals that are part of a robust change management process.
 This requirement applies to operating systems with software libraries that are accessible and configurable, as in the case of interpreted languages. Software libraries also include privileged programs which execute with escalated privileges. Only qualified and authorized individuals shall be allowed to obtain access to information system components for purposes of initiating changes, including upgrades and modifications.</t>
         </is>
       </c>
-      <c r="H225" s="3" t="inlineStr">
+      <c r="H225" s="2" t="inlineStr">
         <is>
           <t>If the operating system allows any user to make changes to software
 libraries, then those changes might be implemented without undergoing the
@@ -18282,398 +18307,389 @@
 of initiating changes, including upgrades and modifications.</t>
         </is>
       </c>
-      <c r="I225" s="3" t="inlineStr">
-        <is>
-          <t>Applicable - Configurable</t>
-        </is>
-      </c>
-      <c r="J225" s="3" t="inlineStr">
+      <c r="I225" s="2" t="inlineStr">
+        <is>
+          <t>Applicable - Configurable</t>
+        </is>
+      </c>
+      <c r="J225" s="2" t="inlineStr">
         <is>
           <t>Verify the operating system limits privileges to change software resident within software libraries. If it does not, this is a finding.</t>
         </is>
       </c>
-      <c r="K225" s="3" t="inlineStr">
-        <is>
-          <t>System commands are stored in the following directories:
- /bin
-/sbin
-/usr/bin
-/usr/sbin
-/usr/local/bin
-/usr/local/sbin 
-For each of these directories, run the following command to find files not
-owned by root group:
- $ sudo find -L  $DIR  ! -group root -type f \; 
-If any of these files are not owned by root group, then this is a finding.</t>
-        </is>
-      </c>
-      <c r="L225" s="3" t="n"/>
-      <c r="M225" s="3" t="inlineStr"/>
-      <c r="N225" s="3" t="inlineStr">
-        <is>
-          <t>CAT II</t>
-        </is>
-      </c>
-      <c r="O225" s="3" t="n"/>
-      <c r="P225" s="3" t="n"/>
-      <c r="Q225" s="3" t="n"/>
+      <c r="K225" s="2" t="inlineStr">
+        <is>
+          <t>Verify the system commands contained in the following directories are group-owned by "root", or a required system account, with the following command:
+$ sudo find -L /bin /sbin /usr/bin /usr/sbin /usr/local/bin /usr/local/sbin ! -group root -exec ls -l {} \;
+If any system commands are returned and is not group-owned by a required system account, then this is a finding.</t>
+        </is>
+      </c>
+      <c r="L225" s="2" t="n"/>
+      <c r="M225" s="2" t="inlineStr">
+        <is>
+          <t>Configure the system commands to be protected from unauthorized access.
+Run the following command, replacing "[FILE]" with any system command file not group-owned by "root" or a required system account.
+$ sudo chgrp root [FILE]</t>
+        </is>
+      </c>
+      <c r="N225" s="2" t="inlineStr">
+        <is>
+          <t>CAT II</t>
+        </is>
+      </c>
+      <c r="O225" s="2" t="n"/>
+      <c r="P225" s="2" t="n"/>
+      <c r="Q225" s="2" t="n"/>
     </row>
     <row r="226" ht="130" customHeight="1">
-      <c r="A226" s="3" t="inlineStr">
+      <c r="A226" s="2" t="inlineStr">
         <is>
           <t>CM-5 (6)</t>
         </is>
       </c>
-      <c r="B226" s="3" t="inlineStr">
+      <c r="B226" s="2" t="inlineStr">
         <is>
           <t>CCI-001499</t>
         </is>
       </c>
-      <c r="C226" s="3" t="inlineStr">
+      <c r="C226" s="2" t="inlineStr">
         <is>
           <t>SRG-OS-000259-GPOS-00100</t>
         </is>
       </c>
-      <c r="D226" s="3" t="inlineStr">
+      <c r="D226" s="2" t="inlineStr">
         <is>
           <t>CCE-83908-4</t>
         </is>
       </c>
-      <c r="E226" s="3" t="inlineStr">
+      <c r="E226" s="2" t="inlineStr">
         <is>
           <t>The operating system must limit privileges to change software resident within software libraries.</t>
         </is>
       </c>
-      <c r="F226" s="3" t="inlineStr">
+      <c r="F226" s="2" t="inlineStr">
         <is>
           <t>Red Hat Enterprise Linux 9 must limit privileges to change software resident within software libraries.</t>
         </is>
       </c>
-      <c r="G226" s="3" t="inlineStr">
+      <c r="G226" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve"> If the operating system were to allow any user to make changes to software libraries, then those changes might be implemented without undergoing the appropriate testing and approvals that are part of a robust change management process.
 This requirement applies to operating systems with software libraries that are accessible and configurable, as in the case of interpreted languages. Software libraries also include privileged programs which execute with escalated privileges. Only qualified and authorized individuals shall be allowed to obtain access to information system components for purposes of initiating changes, including upgrades and modifications.</t>
         </is>
       </c>
-      <c r="H226" s="3" t="inlineStr">
+      <c r="H226" s="2" t="inlineStr">
         <is>
           <t>System binaries are executed by privileged users as well as system services,
 and restrictive permissions are necessary to ensure that their
 execution of these programs cannot be co-opted.</t>
         </is>
       </c>
-      <c r="I226" s="3" t="inlineStr">
-        <is>
-          <t>Applicable - Configurable</t>
-        </is>
-      </c>
-      <c r="J226" s="3" t="inlineStr">
+      <c r="I226" s="2" t="inlineStr">
+        <is>
+          <t>Applicable - Configurable</t>
+        </is>
+      </c>
+      <c r="J226" s="2" t="inlineStr">
         <is>
           <t>Verify the operating system limits privileges to change software resident within software libraries. If it does not, this is a finding.</t>
         </is>
       </c>
-      <c r="K226" s="3" t="inlineStr">
-        <is>
-          <t>System executables are stored in the following directories by default:
- /bin
-/sbin
-/usr/bin
-/usr/libexec
-/usr/local/bin
-/usr/local/sbin
-/usr/sbin 
-To find system executables that are not owned by "root",
-run the following command for each directory  DIR  which contains system executables:
- $ sudo find  DIR/  \! -user root 
-If any system executables are found to not be owned by root, then this is a finding.</t>
-        </is>
-      </c>
-      <c r="L226" s="3" t="n"/>
-      <c r="M226" s="3" t="inlineStr"/>
-      <c r="N226" s="3" t="inlineStr">
-        <is>
-          <t>CAT II</t>
-        </is>
-      </c>
-      <c r="O226" s="3" t="n"/>
-      <c r="P226" s="3" t="n"/>
-      <c r="Q226" s="3" t="n"/>
+      <c r="K226" s="2" t="inlineStr">
+        <is>
+          <t>Verify the system commands contained in the following directories are owned by "root" with the following command:
+$ sudo find -L /bin /sbin /usr/bin /usr/sbin /usr/libexec /usr/local/bin /usr/local/sbin ! -user root -exec ls -l {} \;
+If any system commands are found to not be owned by root, then this is a finding.</t>
+        </is>
+      </c>
+      <c r="L226" s="2" t="n"/>
+      <c r="M226" s="2" t="inlineStr">
+        <is>
+          <t>Configure the system commands to be protected from unauthorized access.
+Run the following command, replacing "[FILE]" with any system command file not owned by "root".
+$ sudo chown root [FILE]</t>
+        </is>
+      </c>
+      <c r="N226" s="2" t="inlineStr">
+        <is>
+          <t>CAT II</t>
+        </is>
+      </c>
+      <c r="O226" s="2" t="n"/>
+      <c r="P226" s="2" t="n"/>
+      <c r="Q226" s="2" t="n"/>
     </row>
     <row r="227" ht="130" customHeight="1">
-      <c r="A227" s="3" t="inlineStr">
+      <c r="A227" s="2" t="inlineStr">
         <is>
           <t>CM-5 (6)</t>
         </is>
       </c>
-      <c r="B227" s="3" t="inlineStr">
+      <c r="B227" s="2" t="inlineStr">
         <is>
           <t>CCI-001499</t>
         </is>
       </c>
-      <c r="C227" s="3" t="inlineStr">
+      <c r="C227" s="2" t="inlineStr">
         <is>
           <t>SRG-OS-000259-GPOS-00100</t>
         </is>
       </c>
-      <c r="D227" s="3" t="inlineStr">
+      <c r="D227" s="2" t="inlineStr">
         <is>
           <t>CCE-83907-6</t>
         </is>
       </c>
-      <c r="E227" s="3" t="inlineStr">
+      <c r="E227" s="2" t="inlineStr">
         <is>
           <t>The operating system must limit privileges to change software resident within software libraries.</t>
         </is>
       </c>
-      <c r="F227" s="3" t="inlineStr">
+      <c r="F227" s="2" t="inlineStr">
         <is>
           <t>Red Hat Enterprise Linux 9 must limit privileges to change software resident within software libraries.</t>
         </is>
       </c>
-      <c r="G227" s="3" t="inlineStr">
+      <c r="G227" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve"> If the operating system were to allow any user to make changes to software libraries, then those changes might be implemented without undergoing the appropriate testing and approvals that are part of a robust change management process.
 This requirement applies to operating systems with software libraries that are accessible and configurable, as in the case of interpreted languages. Software libraries also include privileged programs which execute with escalated privileges. Only qualified and authorized individuals shall be allowed to obtain access to information system components for purposes of initiating changes, including upgrades and modifications.</t>
         </is>
       </c>
-      <c r="H227" s="3" t="inlineStr">
+      <c r="H227" s="2" t="inlineStr">
         <is>
           <t>Files from shared library directories are loaded into the address
 space of processes (including privileged ones) or of the kernel itself at
 runtime. Proper ownership is necessary to protect the integrity of the system.</t>
         </is>
       </c>
-      <c r="I227" s="3" t="inlineStr">
-        <is>
-          <t>Applicable - Configurable</t>
-        </is>
-      </c>
-      <c r="J227" s="3" t="inlineStr">
+      <c r="I227" s="2" t="inlineStr">
+        <is>
+          <t>Applicable - Configurable</t>
+        </is>
+      </c>
+      <c r="J227" s="2" t="inlineStr">
         <is>
           <t>Verify the operating system limits privileges to change software resident within software libraries. If it does not, this is a finding.</t>
         </is>
       </c>
-      <c r="K227" s="3" t="inlineStr">
-        <is>
-          <t>Shared libraries are stored in the following directories:
- /lib
-/lib64
-/usr/lib
-/usr/lib64 
-For each of these directories, run the following command to find files not
-owned by root:
- $ sudo find -L  $DIR  ! -user root -exec chown root {} \; 
-If any of these files are not owned by root, then this is a finding.</t>
-        </is>
-      </c>
-      <c r="L227" s="3" t="n"/>
-      <c r="M227" s="3" t="inlineStr"/>
-      <c r="N227" s="3" t="inlineStr">
-        <is>
-          <t>CAT II</t>
-        </is>
-      </c>
-      <c r="O227" s="3" t="n"/>
-      <c r="P227" s="3" t="n"/>
-      <c r="Q227" s="3" t="n"/>
+      <c r="K227" s="2" t="inlineStr">
+        <is>
+          <t>Verify the system-wide shared library files are owned by "root" with the following command:
+$ sudo find -L /lib /lib64 /usr/lib /usr/lib64 ! -user root -exec ls -l {} \;
+If any system wide shared library file is not owned by root, then this is a finding.</t>
+        </is>
+      </c>
+      <c r="L227" s="2" t="n"/>
+      <c r="M227" s="2" t="inlineStr">
+        <is>
+          <t>Configure the system-wide shared library files (/lib, /lib64, /usr/lib and /usr/lib64) to be protected from unauthorized access.
+Run the following command, replacing "[FILE]" with any library file not owned by "root".
+$ sudo chown root [FILE]</t>
+        </is>
+      </c>
+      <c r="N227" s="2" t="inlineStr">
+        <is>
+          <t>CAT II</t>
+        </is>
+      </c>
+      <c r="O227" s="2" t="n"/>
+      <c r="P227" s="2" t="n"/>
+      <c r="Q227" s="2" t="n"/>
     </row>
     <row r="228" ht="130" customHeight="1">
-      <c r="A228" s="3" t="inlineStr">
+      <c r="A228" s="2" t="inlineStr">
         <is>
           <t>CM-5 (6)</t>
         </is>
       </c>
-      <c r="B228" s="3" t="inlineStr">
+      <c r="B228" s="2" t="inlineStr">
         <is>
           <t>CCI-001499</t>
         </is>
       </c>
-      <c r="C228" s="3" t="inlineStr">
+      <c r="C228" s="2" t="inlineStr">
         <is>
           <t>SRG-OS-000259-GPOS-00100</t>
         </is>
       </c>
-      <c r="D228" s="3" t="inlineStr">
+      <c r="D228" s="2" t="inlineStr">
         <is>
           <t>CCE-83911-8</t>
         </is>
       </c>
-      <c r="E228" s="3" t="inlineStr">
+      <c r="E228" s="2" t="inlineStr">
         <is>
           <t>The operating system must limit privileges to change software resident within software libraries.</t>
         </is>
       </c>
-      <c r="F228" s="3" t="inlineStr">
+      <c r="F228" s="2" t="inlineStr">
         <is>
           <t>Red Hat Enterprise Linux 9 must limit privileges to change software resident within software libraries.</t>
         </is>
       </c>
-      <c r="G228" s="3" t="inlineStr">
+      <c r="G228" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve"> If the operating system were to allow any user to make changes to software libraries, then those changes might be implemented without undergoing the appropriate testing and approvals that are part of a robust change management process.
 This requirement applies to operating systems with software libraries that are accessible and configurable, as in the case of interpreted languages. Software libraries also include privileged programs which execute with escalated privileges. Only qualified and authorized individuals shall be allowed to obtain access to information system components for purposes of initiating changes, including upgrades and modifications.</t>
         </is>
       </c>
-      <c r="H228" s="3" t="inlineStr">
+      <c r="H228" s="2" t="inlineStr">
         <is>
           <t>System binaries are executed by privileged users, as well as system services,
 and restrictive permissions are necessary to ensure execution of these programs
 cannot be co-opted.</t>
         </is>
       </c>
-      <c r="I228" s="3" t="inlineStr">
-        <is>
-          <t>Applicable - Configurable</t>
-        </is>
-      </c>
-      <c r="J228" s="3" t="inlineStr">
+      <c r="I228" s="2" t="inlineStr">
+        <is>
+          <t>Applicable - Configurable</t>
+        </is>
+      </c>
+      <c r="J228" s="2" t="inlineStr">
         <is>
           <t>Verify the operating system limits privileges to change software resident within software libraries. If it does not, this is a finding.</t>
         </is>
       </c>
-      <c r="K228" s="3" t="inlineStr">
-        <is>
-          <t>System executables are stored in the following directories by default:
- /bin
-/sbin
-/usr/bin
-/usr/libexec
-/usr/local/bin
-/usr/local/sbin
-/usr/sbin 
-To find system executables that are group-writable or world-writable,
-run the following command for each directory  DIR  which contains system executables:
- $ sudo find -L  DIR  -perm /022 -type f 
-If any system executables are found to be group or world writable, then this is a finding.</t>
-        </is>
-      </c>
-      <c r="L228" s="3" t="n"/>
-      <c r="M228" s="3" t="inlineStr"/>
-      <c r="N228" s="3" t="inlineStr">
-        <is>
-          <t>CAT II</t>
-        </is>
-      </c>
-      <c r="O228" s="3" t="n"/>
-      <c r="P228" s="3" t="n"/>
-      <c r="Q228" s="3" t="n"/>
+      <c r="K228" s="2" t="inlineStr">
+        <is>
+          <t>Verify the system commands contained in the following directories have mode "755" or less permissive with the following command:
+$ sudo find -L /bin /sbin /usr/bin /usr/sbin /usr/libexec /usr/local/bin /usr/local/sbin -perm /022 -exec ls -l {} \;
+If any system commands are found to be group-writable or world-writable, then this is a finding.</t>
+        </is>
+      </c>
+      <c r="L228" s="2" t="n"/>
+      <c r="M228" s="2" t="inlineStr">
+        <is>
+          <t>Configure the system commands to be protected from unauthorized access.
+Run the following command, replacing "[FILE]" with any system command with a mode more permissive than "755".
+$ sudo chmod 755 [FILE]</t>
+        </is>
+      </c>
+      <c r="N228" s="2" t="inlineStr">
+        <is>
+          <t>CAT II</t>
+        </is>
+      </c>
+      <c r="O228" s="2" t="n"/>
+      <c r="P228" s="2" t="n"/>
+      <c r="Q228" s="2" t="n"/>
     </row>
     <row r="229" ht="130" customHeight="1">
-      <c r="A229" s="3" t="inlineStr">
+      <c r="A229" s="2" t="inlineStr">
         <is>
           <t>CM-5 (6)</t>
         </is>
       </c>
-      <c r="B229" s="3" t="inlineStr">
+      <c r="B229" s="2" t="inlineStr">
         <is>
           <t>CCI-001499</t>
         </is>
       </c>
-      <c r="C229" s="3" t="inlineStr">
+      <c r="C229" s="2" t="inlineStr">
         <is>
           <t>SRG-OS-000259-GPOS-00100</t>
         </is>
       </c>
-      <c r="D229" s="3" t="inlineStr">
+      <c r="D229" s="2" t="inlineStr">
         <is>
           <t>CCE-83909-2</t>
         </is>
       </c>
-      <c r="E229" s="3" t="inlineStr">
+      <c r="E229" s="2" t="inlineStr">
         <is>
           <t>The operating system must limit privileges to change software resident within software libraries.</t>
         </is>
       </c>
-      <c r="F229" s="3" t="inlineStr">
+      <c r="F229" s="2" t="inlineStr">
         <is>
           <t>Red Hat Enterprise Linux 9 must limit privileges to change software resident within software libraries.</t>
         </is>
       </c>
-      <c r="G229" s="3" t="inlineStr">
+      <c r="G229" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve"> If the operating system were to allow any user to make changes to software libraries, then those changes might be implemented without undergoing the appropriate testing and approvals that are part of a robust change management process.
 This requirement applies to operating systems with software libraries that are accessible and configurable, as in the case of interpreted languages. Software libraries also include privileged programs which execute with escalated privileges. Only qualified and authorized individuals shall be allowed to obtain access to information system components for purposes of initiating changes, including upgrades and modifications.</t>
         </is>
       </c>
-      <c r="H229" s="3" t="inlineStr">
+      <c r="H229" s="2" t="inlineStr">
         <is>
           <t>Files from shared library directories are loaded into the address
 space of processes (including privileged ones) or of the kernel itself at
 runtime. Restrictive permissions are necessary to protect the integrity of the system.</t>
         </is>
       </c>
-      <c r="I229" s="3" t="inlineStr">
-        <is>
-          <t>Applicable - Configurable</t>
-        </is>
-      </c>
-      <c r="J229" s="3" t="inlineStr">
+      <c r="I229" s="2" t="inlineStr">
+        <is>
+          <t>Applicable - Configurable</t>
+        </is>
+      </c>
+      <c r="J229" s="2" t="inlineStr">
         <is>
           <t>Verify the operating system limits privileges to change software resident within software libraries. If it does not, this is a finding.</t>
         </is>
       </c>
-      <c r="K229" s="3" t="inlineStr">
-        <is>
-          <t>Shared libraries are stored in the following directories:
- /lib
-/lib64
-/usr/lib
-/usr/lib64
-To find shared libraries that are group-writable or world-writable,
-run the following command for each directory  DIR  which contains shared libraries:
- $ sudo find -L  DIR  -perm /022 -type f 
-If any of these files are group-writable or world-writable, then this is a finding.</t>
-        </is>
-      </c>
-      <c r="L229" s="3" t="n"/>
-      <c r="M229" s="3" t="inlineStr"/>
-      <c r="N229" s="3" t="inlineStr">
-        <is>
-          <t>CAT II</t>
-        </is>
-      </c>
-      <c r="O229" s="3" t="n"/>
-      <c r="P229" s="3" t="n"/>
-      <c r="Q229" s="3" t="n"/>
+      <c r="K229" s="2" t="inlineStr">
+        <is>
+          <t>Verify the system-wide shared library files contained in the following directories have mode "755" or less permissive with the following command:
+$ sudo find -L /lib /lib64 /usr/lib /usr/lib64 -perm /022 -type f -exec ls -l {} \;
+If any system-wide shared library file is found to be group-writable or world-writable, then this is a finding.</t>
+        </is>
+      </c>
+      <c r="L229" s="2" t="n"/>
+      <c r="M229" s="2" t="inlineStr">
+        <is>
+          <t>Configure the library files to be protected from unauthorized access. Run the following command, replacing "[FILE]" with any library file with a mode more permissive than 755.
+$ sudo chmod 755 [FILE]</t>
+        </is>
+      </c>
+      <c r="N229" s="2" t="inlineStr">
+        <is>
+          <t>CAT II</t>
+        </is>
+      </c>
+      <c r="O229" s="2" t="n"/>
+      <c r="P229" s="2" t="n"/>
+      <c r="Q229" s="2" t="n"/>
     </row>
     <row r="230" ht="130" customHeight="1">
-      <c r="A230" s="3" t="inlineStr">
+      <c r="A230" s="2" t="inlineStr">
         <is>
           <t>CM-5 (6)</t>
         </is>
       </c>
-      <c r="B230" s="3" t="inlineStr">
+      <c r="B230" s="2" t="inlineStr">
         <is>
           <t>CCI-001499</t>
         </is>
       </c>
-      <c r="C230" s="3" t="inlineStr">
+      <c r="C230" s="2" t="inlineStr">
         <is>
           <t>SRG-OS-000259-GPOS-00100</t>
         </is>
       </c>
-      <c r="D230" s="3" t="inlineStr">
+      <c r="D230" s="2" t="inlineStr">
         <is>
           <t>CCE-87108-7</t>
         </is>
       </c>
-      <c r="E230" s="3" t="inlineStr">
+      <c r="E230" s="2" t="inlineStr">
         <is>
           <t>The operating system must limit privileges to change software resident within software libraries.</t>
         </is>
       </c>
-      <c r="F230" s="3" t="inlineStr">
+      <c r="F230" s="2" t="inlineStr">
         <is>
           <t>Red Hat Enterprise Linux 9 must limit privileges to change software resident within software libraries.</t>
         </is>
       </c>
-      <c r="G230" s="3" t="inlineStr">
+      <c r="G230" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve"> If the operating system were to allow any user to make changes to software libraries, then those changes might be implemented without undergoing the appropriate testing and approvals that are part of a robust change management process.
 This requirement applies to operating systems with software libraries that are accessible and configurable, as in the case of interpreted languages. Software libraries also include privileged programs which execute with escalated privileges. Only qualified and authorized individuals shall be allowed to obtain access to information system components for purposes of initiating changes, including upgrades and modifications.</t>
         </is>
       </c>
-      <c r="H230" s="3" t="inlineStr">
+      <c r="H230" s="2" t="inlineStr">
         <is>
           <t>If the operating system were to allow any user to make changes to software libraries,
 then those changes might be implemented without undergoing the appropriate testing and
@@ -18685,39 +18701,39 @@
 for purposes of initiating changes, including upgrades and modifications.</t>
         </is>
       </c>
-      <c r="I230" s="3" t="inlineStr">
-        <is>
-          <t>Applicable - Configurable</t>
-        </is>
-      </c>
-      <c r="J230" s="3" t="inlineStr">
+      <c r="I230" s="2" t="inlineStr">
+        <is>
+          <t>Applicable - Configurable</t>
+        </is>
+      </c>
+      <c r="J230" s="2" t="inlineStr">
         <is>
           <t>Verify the operating system limits privileges to change software resident within software libraries. If it does not, this is a finding.</t>
         </is>
       </c>
-      <c r="K230" s="3" t="inlineStr">
-        <is>
-          <t>System-wide library files are stored in the following directories:
- /lib
-/lib64
-/usr/lib
-/usr/lib64
-To find if system-wide library files stored in these directories are not group-owned by
-root run the following command for each directory  DIR :
- $ sudo find -L  DIR  ! -group root -type f  
-If system wide library files are not group-owned by root, then this is a finding.</t>
-        </is>
-      </c>
-      <c r="L230" s="3" t="n"/>
-      <c r="M230" s="3" t="inlineStr"/>
-      <c r="N230" s="3" t="inlineStr">
-        <is>
-          <t>CAT II</t>
-        </is>
-      </c>
-      <c r="O230" s="3" t="n"/>
-      <c r="P230" s="3" t="n"/>
-      <c r="Q230" s="3" t="n"/>
+      <c r="K230" s="2" t="inlineStr">
+        <is>
+          <t>Verify the system-wide shared library files are group-owned by "root" with the following command:
+$ sudo find -L /lib /lib64 /usr/lib /usr/lib64 ! -group root -exec ls -l {} \;
+If any system wide shared library file is returned and is not group-owned by a required system account, then this is a finding.</t>
+        </is>
+      </c>
+      <c r="L230" s="2" t="n"/>
+      <c r="M230" s="2" t="inlineStr">
+        <is>
+          <t>Configure the system-wide shared library files (/lib, /lib64, /usr/lib and /usr/lib64) to be protected from unauthorized access.
+Run the following command, replacing "[FILE]" with any library file not group-owned by "root".
+$ sudo chgrp root [FILE]</t>
+        </is>
+      </c>
+      <c r="N230" s="2" t="inlineStr">
+        <is>
+          <t>CAT II</t>
+        </is>
+      </c>
+      <c r="O230" s="2" t="n"/>
+      <c r="P230" s="2" t="n"/>
+      <c r="Q230" s="2" t="n"/>
     </row>
     <row r="231" ht="130" customHeight="1">
       <c r="A231" s="2" t="inlineStr">
@@ -18818,7 +18834,7 @@
     <row r="232" ht="130" customHeight="1">
       <c r="A232" s="2" t="inlineStr">
         <is>
-          <t>CM-6 b,SC-2,SI-16</t>
+          <t>SI-16,CM-6 b,SC-2</t>
         </is>
       </c>
       <c r="B232" s="2" t="inlineStr">
@@ -19164,7 +19180,7 @@
     <row r="236" ht="130" customHeight="1">
       <c r="A236" s="2" t="inlineStr">
         <is>
-          <t>AC-18 (1),CM-7 a</t>
+          <t>CM-7 a,AC-18 (1)</t>
         </is>
       </c>
       <c r="B236" s="2" t="inlineStr">
@@ -19246,61 +19262,61 @@
       <c r="Q236" s="2" t="n"/>
     </row>
     <row r="237" ht="130" customHeight="1">
-      <c r="A237" s="3" t="inlineStr">
+      <c r="A237" s="2" t="inlineStr">
         <is>
           <t>AU-6 (4)</t>
         </is>
       </c>
-      <c r="B237" s="3" t="inlineStr">
+      <c r="B237" s="2" t="inlineStr">
         <is>
           <t>CCI-000154</t>
         </is>
       </c>
-      <c r="C237" s="3" t="inlineStr">
+      <c r="C237" s="2" t="inlineStr">
         <is>
           <t>SRG-OS-000051-GPOS-00024</t>
         </is>
       </c>
-      <c r="D237" s="3" t="inlineStr">
+      <c r="D237" s="2" t="inlineStr">
         <is>
           <t>CCE-83704-7</t>
         </is>
       </c>
-      <c r="E237" s="3" t="inlineStr">
+      <c r="E237" s="2" t="inlineStr">
         <is>
           <t>The operating system must provide the capability to centrally review and analyze audit records from multiple components within the system.</t>
         </is>
       </c>
-      <c r="F237" s="3" t="inlineStr">
+      <c r="F237" s="2" t="inlineStr">
         <is>
           <t>Red Hat Enterprise Linux 9 must provide the capability to centrally review and analyze audit records from multiple components within the system.</t>
         </is>
       </c>
-      <c r="G237" s="3" t="inlineStr">
+      <c r="G237" s="2" t="inlineStr">
         <is>
           <t>Successful incident response and auditing relies on timely, accurate system information and analysis in order to allow the organization to identify and respond to potential incidents in a proficient manner. If the operating system does not provide the ability to centrally review the operating system logs, forensic analysis is negatively impacted.
 Segregation of logging data to multiple disparate computer systems is counterproductive and makes log analysis and log event alarming difficult to implement and manage, particularly when the system has multiple logging components writing to different locations or systems.
 To support the centralized capability, the operating system must be able to provide the information in a format that can be extracted and used, allowing the application performing the centralization of the log records to meet this requirement.</t>
         </is>
       </c>
-      <c r="H237" s="3" t="inlineStr">
+      <c r="H237" s="2" t="inlineStr">
         <is>
           <t>If option "freq" isn't set to "50", the flush to disk
 may happen after higher number of records, increasing the danger
 of audit loss.</t>
         </is>
       </c>
-      <c r="I237" s="3" t="inlineStr">
-        <is>
-          <t>Applicable - Configurable</t>
-        </is>
-      </c>
-      <c r="J237" s="3" t="inlineStr">
+      <c r="I237" s="2" t="inlineStr">
+        <is>
+          <t>Applicable - Configurable</t>
+        </is>
+      </c>
+      <c r="J237" s="2" t="inlineStr">
         <is>
           <t>Verify the operating system provides the capability to centrally review and analyze audit records from multiple components within the system. If it does not, this is a finding.</t>
         </is>
       </c>
-      <c r="K237" s="3" t="inlineStr">
+      <c r="K237" s="2" t="inlineStr">
         <is>
           <t>To verify that Audit Daemon is configured to flush to disk after
 every 50 records, run the following command:
@@ -19310,16 +19326,21 @@
 If freq isn't set to 50, then this is a finding.</t>
         </is>
       </c>
-      <c r="L237" s="3" t="n"/>
-      <c r="M237" s="3" t="inlineStr"/>
-      <c r="N237" s="3" t="inlineStr">
-        <is>
-          <t>CAT II</t>
-        </is>
-      </c>
-      <c r="O237" s="3" t="n"/>
-      <c r="P237" s="3" t="n"/>
-      <c r="Q237" s="3" t="n"/>
+      <c r="L237" s="2" t="n"/>
+      <c r="M237" s="2" t="inlineStr">
+        <is>
+          <t>Edit the file "/etc/audit/auditd.conf" and add or edit the following line:
+freq = 50</t>
+        </is>
+      </c>
+      <c r="N237" s="2" t="inlineStr">
+        <is>
+          <t>CAT II</t>
+        </is>
+      </c>
+      <c r="O237" s="2" t="n"/>
+      <c r="P237" s="2" t="n"/>
+      <c r="Q237" s="2" t="n"/>
     </row>
     <row r="238" ht="130" customHeight="1">
       <c r="A238" s="2" t="inlineStr">
@@ -20637,37 +20658,37 @@
       <c r="Q253" s="2" t="n"/>
     </row>
     <row r="254" ht="130" customHeight="1">
-      <c r="A254" s="3" t="inlineStr">
+      <c r="A254" s="2" t="inlineStr">
         <is>
           <t>IA-2 (12),IA-2 (11)</t>
         </is>
       </c>
-      <c r="B254" s="3" t="inlineStr">
+      <c r="B254" s="2" t="inlineStr">
         <is>
           <t>CCI-001954,CCI-001953</t>
         </is>
       </c>
-      <c r="C254" s="3" t="inlineStr">
+      <c r="C254" s="2" t="inlineStr">
         <is>
           <t>SRG-OS-000375-GPOS-00160,SRG-OS-000376-GPOS-00161</t>
         </is>
       </c>
-      <c r="D254" s="3" t="inlineStr">
+      <c r="D254" s="2" t="inlineStr">
         <is>
           <t>CCE-83595-9</t>
         </is>
       </c>
-      <c r="E254" s="3" t="inlineStr">
+      <c r="E254" s="2" t="inlineStr">
         <is>
           <t>The operating system must implement multifactor authentication for remote access to privileged accounts in such a way that one of the factors is provided by a device separate from the system gaining access.</t>
         </is>
       </c>
-      <c r="F254" s="3" t="inlineStr">
+      <c r="F254" s="2" t="inlineStr">
         <is>
           <t>Red Hat Enterprise Linux 9 must implement multifactor authentication for remote access to privileged accounts in such a way that one of the factors is provided by a device separate from the system gaining access.</t>
         </is>
       </c>
-      <c r="G254" s="3" t="inlineStr">
+      <c r="G254" s="2" t="inlineStr">
         <is>
           <t>Using an authentication device, such as a CAC or token that is separate from the information system, ensures that even if the information system is compromised, that compromise will not affect credentials stored on the authentication device.
 Multifactor solutions that require devices separate from information systems gaining access include, for example, hardware tokens providing time-based or challenge-response authenticators and smart cards such as the U.S. Government Personal Identity Verification card and the DoD Common Access Card.
@@ -20677,7 +20698,7 @@
 Requires further clarification from NIST.</t>
         </is>
       </c>
-      <c r="H254" s="3" t="inlineStr">
+      <c r="H254" s="2" t="inlineStr">
         <is>
           <t>Using an authentication device, such as a CAC or token that is separate from
 the information system, ensures that even if the information system is
@@ -20690,32 +20711,38 @@
 Access Card.</t>
         </is>
       </c>
-      <c r="I254" s="3" t="inlineStr">
-        <is>
-          <t>Applicable - Configurable</t>
-        </is>
-      </c>
-      <c r="J254" s="3" t="inlineStr">
+      <c r="I254" s="2" t="inlineStr">
+        <is>
+          <t>Applicable - Configurable</t>
+        </is>
+      </c>
+      <c r="J254" s="2" t="inlineStr">
         <is>
           <t>Verify the operating system implements multifactor authentication for remote access to privileged accounts in such a way that one of the factors is provided by a device separate from the system gaining access. If it does not, this is a finding.</t>
         </is>
       </c>
-      <c r="K254" s="3" t="inlineStr">
+      <c r="K254" s="2" t="inlineStr">
         <is>
           <t>Run the following command to determine if the  opensc  package is installed:  $ rpm -q opensc 
 If the package is not installed, then this is a finding.</t>
         </is>
       </c>
-      <c r="L254" s="3" t="n"/>
-      <c r="M254" s="3" t="inlineStr"/>
-      <c r="N254" s="3" t="inlineStr">
-        <is>
-          <t>CAT II</t>
-        </is>
-      </c>
-      <c r="O254" s="3" t="n"/>
-      <c r="P254" s="3" t="n"/>
-      <c r="Q254" s="3" t="n"/>
+      <c r="L254" s="2" t="n"/>
+      <c r="M254" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">
+The  opensc  package can be installed with the following command:
+$ sudo dnf install opensc </t>
+        </is>
+      </c>
+      <c r="N254" s="2" t="inlineStr">
+        <is>
+          <t>CAT II</t>
+        </is>
+      </c>
+      <c r="O254" s="2" t="n"/>
+      <c r="P254" s="2" t="n"/>
+      <c r="Q254" s="2" t="n"/>
     </row>
     <row r="255" ht="130" customHeight="1">
       <c r="A255" s="3" t="inlineStr">
@@ -21046,7 +21073,7 @@
     <row r="259" ht="130" customHeight="1">
       <c r="A259" s="3" t="inlineStr">
         <is>
-          <t>AC-6 (8),AC-6 (9)</t>
+          <t>AC-6 (9),AC-6 (8)</t>
         </is>
       </c>
       <c r="B259" s="3" t="inlineStr">
@@ -21126,7 +21153,7 @@
     <row r="260" ht="130" customHeight="1">
       <c r="A260" s="3" t="inlineStr">
         <is>
-          <t>CM-6 b,IA-2 (5)</t>
+          <t>IA-2 (5),CM-6 b</t>
         </is>
       </c>
       <c r="B260" s="3" t="inlineStr">
@@ -21592,7 +21619,7 @@
     <row r="266" ht="130" customHeight="1">
       <c r="A266" s="2" t="inlineStr">
         <is>
-          <t>AU-12 c,AU-9</t>
+          <t>AU-9,AU-12 c</t>
         </is>
       </c>
       <c r="B266" s="2" t="inlineStr">
@@ -22365,7 +22392,7 @@
     <row r="275" ht="130" customHeight="1">
       <c r="A275" s="3" t="inlineStr">
         <is>
-          <t>CM-6 b,CM-7 a</t>
+          <t>CM-7 a,CM-6 b</t>
         </is>
       </c>
       <c r="B275" s="3" t="inlineStr">
@@ -23361,7 +23388,7 @@
     <row r="288" ht="130" customHeight="1">
       <c r="A288" s="3" t="inlineStr">
         <is>
-          <t>CM-6 b,CM-7 a</t>
+          <t>CM-7 a,CM-6 b</t>
         </is>
       </c>
       <c r="B288" s="3" t="inlineStr">
@@ -23432,7 +23459,7 @@
     <row r="289" ht="130" customHeight="1">
       <c r="A289" s="3" t="inlineStr">
         <is>
-          <t>CM-6 b,CM-7 a</t>
+          <t>CM-7 a,CM-6 b</t>
         </is>
       </c>
       <c r="B289" s="3" t="inlineStr">
@@ -23504,7 +23531,7 @@
     <row r="290" ht="130" customHeight="1">
       <c r="A290" s="3" t="inlineStr">
         <is>
-          <t>CM-6 b,CM-7 a</t>
+          <t>CM-7 a,CM-6 b</t>
         </is>
       </c>
       <c r="B290" s="3" t="inlineStr">
@@ -23662,7 +23689,7 @@
     <row r="292" ht="130" customHeight="1">
       <c r="A292" s="3" t="inlineStr">
         <is>
-          <t>AU-12 c,AC-6 (9),AC-2 (4)</t>
+          <t>AC-6 (9),AC-2 (4),AU-12 c</t>
         </is>
       </c>
       <c r="B292" s="3" t="inlineStr">
@@ -23801,136 +23828,144 @@
       <c r="Q292" s="3" t="n"/>
     </row>
     <row r="293" ht="130" customHeight="1">
-      <c r="A293" s="3" t="inlineStr">
+      <c r="A293" s="2" t="inlineStr">
         <is>
           <t>AU-5 a</t>
         </is>
       </c>
-      <c r="B293" s="3" t="inlineStr">
+      <c r="B293" s="2" t="inlineStr">
         <is>
           <t>CCI-000139,CCI-000366</t>
         </is>
       </c>
-      <c r="C293" s="3" t="inlineStr">
+      <c r="C293" s="2" t="inlineStr">
         <is>
           <t>SRG-OS-000046-GPOS-00022</t>
         </is>
       </c>
-      <c r="D293" s="3" t="inlineStr">
+      <c r="D293" s="2" t="inlineStr">
         <is>
           <t>CCE-90826-9</t>
         </is>
       </c>
-      <c r="E293" s="3" t="inlineStr">
+      <c r="E293" s="2" t="inlineStr">
         <is>
           <t>The operating system must alert the ISSO and SA (at a minimum) in the event of an audit processing failure.</t>
         </is>
       </c>
-      <c r="F293" s="3" t="inlineStr">
+      <c r="F293" s="2" t="inlineStr">
         <is>
           <t>Red Hat Enterprise Linux 9 must alert the ISSO and SA (at a minimum) in the event of an audit processing failure.</t>
         </is>
       </c>
-      <c r="G293" s="3" t="inlineStr">
+      <c r="G293" s="2" t="inlineStr">
         <is>
           <t>It is critical for the appropriate personnel to be aware if a system is at risk of failing to process audit logs as required. Without this notification, the security personnel may be unaware of an impending failure of the audit capability, and system operation may be adversely affected.
 Audit processing failures include software/hardware errors, failures in the audit capturing mechanisms, and audit storage capacity being reached or exceeded.
 This requirement applies to each audit data storage repository (i.e., distinct information system component where audit records are stored), the centralized audit storage capacity of organizations (i.e., all audit data storage repositories combined), or both.</t>
         </is>
       </c>
-      <c r="H293" s="3" t="inlineStr">
+      <c r="H293" s="2" t="inlineStr">
         <is>
           <t>A number of system services utilize email messages sent to the root user to
 notify system administrators of active or impending issues.  These messages must
 be forwarded to at least one monitored email address.</t>
         </is>
       </c>
-      <c r="I293" s="3" t="inlineStr">
-        <is>
-          <t>Applicable - Configurable</t>
-        </is>
-      </c>
-      <c r="J293" s="3" t="inlineStr">
+      <c r="I293" s="2" t="inlineStr">
+        <is>
+          <t>Applicable - Configurable</t>
+        </is>
+      </c>
+      <c r="J293" s="2" t="inlineStr">
         <is>
           <t>Verify the operating system alerts the ISSO and SA (at a minimum) in the event of an audit processing failure. If it does not, this is a finding.</t>
         </is>
       </c>
-      <c r="K293" s="3" t="inlineStr">
+      <c r="K293" s="2" t="inlineStr">
         <is>
           <t>Find the list of alias maps used by the Postfix mail server:
  $ sudo postconf alias_maps 
 Query the Postfix alias maps for an alias for the  root  user:
  $ sudo postmap -q root hash:/etc/aliases 
 The output should return an alias.
-If it is not, then this is a finding.</t>
-        </is>
-      </c>
-      <c r="L293" s="3" t="n"/>
-      <c r="M293" s="3" t="inlineStr"/>
-      <c r="N293" s="3" t="inlineStr">
-        <is>
-          <t>CAT II</t>
-        </is>
-      </c>
-      <c r="O293" s="3" t="n"/>
-      <c r="P293" s="3" t="n"/>
-      <c r="Q293" s="3" t="n"/>
+If the alias is not set, then this is a finding.</t>
+        </is>
+      </c>
+      <c r="L293" s="2" t="n"/>
+      <c r="M293" s="2" t="inlineStr">
+        <is>
+          <t>Configure a valid email address as an alias for the root account.
+Append the following line to "/etc/aliases":
+root: system.administrator@mail.mil
+Then, run the following command:
+$ sudo newaliases</t>
+        </is>
+      </c>
+      <c r="N293" s="2" t="inlineStr">
+        <is>
+          <t>CAT II</t>
+        </is>
+      </c>
+      <c r="O293" s="2" t="n"/>
+      <c r="P293" s="2" t="n"/>
+      <c r="Q293" s="2" t="n"/>
     </row>
     <row r="294" ht="130" customHeight="1">
-      <c r="A294" s="3" t="inlineStr">
+      <c r="A294" s="2" t="inlineStr">
         <is>
           <t>AU-5 a,AU-5 (1)</t>
         </is>
       </c>
-      <c r="B294" s="3" t="inlineStr">
+      <c r="B294" s="2" t="inlineStr">
         <is>
           <t>CCI-000139,CCI-001855</t>
         </is>
       </c>
-      <c r="C294" s="3" t="inlineStr">
+      <c r="C294" s="2" t="inlineStr">
         <is>
           <t>SRG-OS-000046-GPOS-00022,SRG-OS-000343-GPOS-00134</t>
         </is>
       </c>
-      <c r="D294" s="3" t="inlineStr">
+      <c r="D294" s="2" t="inlineStr">
         <is>
           <t>CCE-83698-1</t>
         </is>
       </c>
-      <c r="E294" s="3" t="inlineStr">
+      <c r="E294" s="2" t="inlineStr">
         <is>
           <t>The operating system must alert the ISSO and SA (at a minimum) in the event of an audit processing failure.</t>
         </is>
       </c>
-      <c r="F294" s="3" t="inlineStr">
+      <c r="F294" s="2" t="inlineStr">
         <is>
           <t>Red Hat Enterprise Linux 9 must alert the ISSO and SA (at a minimum) in the event of an audit processing failure.</t>
         </is>
       </c>
-      <c r="G294" s="3" t="inlineStr">
+      <c r="G294" s="2" t="inlineStr">
         <is>
           <t>It is critical for the appropriate personnel to be aware if a system is at risk of failing to process audit logs as required. Without this notification, the security personnel may be unaware of an impending failure of the audit capability, and system operation may be adversely affected.
 Audit processing failures include software/hardware errors, failures in the audit capturing mechanisms, and audit storage capacity being reached or exceeded.
 This requirement applies to each audit data storage repository (i.e., distinct information system component where audit records are stored), the centralized audit storage capacity of organizations (i.e., all audit data storage repositories combined), or both.</t>
         </is>
       </c>
-      <c r="H294" s="3" t="inlineStr">
+      <c r="H294" s="2" t="inlineStr">
         <is>
           <t>Email sent to the root account is typically aliased to the
 administrators of the system, who can take appropriate action.</t>
         </is>
       </c>
-      <c r="I294" s="3" t="inlineStr">
-        <is>
-          <t>Applicable - Configurable</t>
-        </is>
-      </c>
-      <c r="J294" s="3" t="inlineStr">
+      <c r="I294" s="2" t="inlineStr">
+        <is>
+          <t>Applicable - Configurable</t>
+        </is>
+      </c>
+      <c r="J294" s="2" t="inlineStr">
         <is>
           <t>Verify the operating system alerts the ISSO and SA (at a minimum) in the event of an audit processing failure. If it does not, this is a finding.</t>
         </is>
       </c>
-      <c r="K294" s="3" t="inlineStr">
+      <c r="K294" s="2" t="inlineStr">
         <is>
           <t>Inspect "/etc/audit/auditd.conf" and locate the following line to
 determine if the system is configured to send email to an
@@ -23939,16 +23974,22 @@
 If auditd is not configured to send emails per identified actions, then this is a finding.</t>
         </is>
       </c>
-      <c r="L294" s="3" t="n"/>
-      <c r="M294" s="3" t="inlineStr"/>
-      <c r="N294" s="3" t="inlineStr">
-        <is>
-          <t>CAT II</t>
-        </is>
-      </c>
-      <c r="O294" s="3" t="n"/>
-      <c r="P294" s="3" t="n"/>
-      <c r="Q294" s="3" t="n"/>
+      <c r="L294" s="2" t="n"/>
+      <c r="M294" s="2" t="inlineStr">
+        <is>
+          <t>Configure "auditd" service to notify the SA and ISSO in the event of an audit processing failure.
+Edit the following line in "/etc/audit/auditd.conf" to ensure that administrators are notified via email for those situations:
+action_mail_acct = root</t>
+        </is>
+      </c>
+      <c r="N294" s="2" t="inlineStr">
+        <is>
+          <t>CAT II</t>
+        </is>
+      </c>
+      <c r="O294" s="2" t="n"/>
+      <c r="P294" s="2" t="n"/>
+      <c r="Q294" s="2" t="n"/>
     </row>
     <row r="295" ht="130" customHeight="1">
       <c r="A295" s="3" t="inlineStr">
@@ -29866,59 +29907,59 @@
       <c r="Q373" s="3" t="n"/>
     </row>
     <row r="374" ht="130" customHeight="1">
-      <c r="A374" s="3" t="inlineStr">
+      <c r="A374" s="2" t="inlineStr">
         <is>
           <t>CM-6 b,AU-3</t>
         </is>
       </c>
-      <c r="B374" s="3" t="inlineStr">
+      <c r="B374" s="2" t="inlineStr">
         <is>
           <t>CCI-000366</t>
         </is>
       </c>
-      <c r="C374" s="3" t="inlineStr">
+      <c r="C374" s="2" t="inlineStr">
         <is>
           <t>SRG-OS-000255-GPOS-00096,SRG-OS-000480-GPOS-00227</t>
         </is>
       </c>
-      <c r="D374" s="3" t="inlineStr">
+      <c r="D374" s="2" t="inlineStr">
         <is>
           <t>CCE-83696-5</t>
         </is>
       </c>
-      <c r="E374" s="3" t="inlineStr">
+      <c r="E374" s="2" t="inlineStr">
         <is>
           <t>The operating system must be configured in accordance with the security configuration settings based on DoD security configuration or implementation guidance, including STIGs, NSA configuration guides, CTOs, and DTMs.</t>
         </is>
       </c>
-      <c r="F374" s="3" t="inlineStr">
+      <c r="F374" s="2" t="inlineStr">
         <is>
           <t>Red Hat Enterprise Linux 9 must be configured in accordance with the security configuration settings based on DoD security configuration or implementation guidance, including STIGs, NSA configuration guides, CTOs, and DTMs.</t>
         </is>
       </c>
-      <c r="G374" s="3" t="inlineStr">
+      <c r="G374" s="2" t="inlineStr">
         <is>
           <t>Configuring the operating system to implement organization-wide security implementation guides and security checklists ensures compliance with federal standards and establishes a common security baseline across DoD that reflects the most restrictive security posture consistent with operational requirements.
 Configuration settings are the set of parameters that can be changed in hardware, software, or firmware components of the system that affect the security posture and/or functionality of the system. Security-related parameters are those parameters impacting the security state of the system, including the parameters required to satisfy other security control requirements. Security-related parameters include, for example: registry settings; account, file, directory permission settings; and settings for functions, ports, protocols, services, and remote connections.</t>
         </is>
       </c>
-      <c r="H374" s="3" t="inlineStr">
+      <c r="H374" s="2" t="inlineStr">
         <is>
           <t>If option "log_format" isn't set to "ENRICHED", the
 audit records will be stored in a format exactly as the kernel sends them.</t>
         </is>
       </c>
-      <c r="I374" s="3" t="inlineStr">
-        <is>
-          <t>Applicable - Configurable</t>
-        </is>
-      </c>
-      <c r="J374" s="3" t="inlineStr">
+      <c r="I374" s="2" t="inlineStr">
+        <is>
+          <t>Applicable - Configurable</t>
+        </is>
+      </c>
+      <c r="J374" s="2" t="inlineStr">
         <is>
           <t>Verify the operating system is configured in accordance with the security configuration settings based on DoD security configuration or implementation guidance, including STIGs, NSA configuration guides, CTOs, and DTMs. If it is not, this is a finding.</t>
         </is>
       </c>
-      <c r="K374" s="3" t="inlineStr">
+      <c r="K374" s="2" t="inlineStr">
         <is>
           <t>To verify that Audit Daemon is configured to resolve all uid, gid, syscall,
 architecture, and socket address information before writing the event to disk,
@@ -29929,71 +29970,76 @@
 If log_format isn't set to ENRICHED, then this is a finding.</t>
         </is>
       </c>
-      <c r="L374" s="3" t="n"/>
-      <c r="M374" s="3" t="inlineStr"/>
-      <c r="N374" s="3" t="inlineStr">
-        <is>
-          <t>CAT II</t>
-        </is>
-      </c>
-      <c r="O374" s="3" t="n"/>
-      <c r="P374" s="3" t="n"/>
-      <c r="Q374" s="3" t="n"/>
+      <c r="L374" s="2" t="n"/>
+      <c r="M374" s="2" t="inlineStr">
+        <is>
+          <t>Edit the file "/etc/audit/auditd.conf" and add or edit the following line:
+log_format = ENRICHED</t>
+        </is>
+      </c>
+      <c r="N374" s="2" t="inlineStr">
+        <is>
+          <t>CAT II</t>
+        </is>
+      </c>
+      <c r="O374" s="2" t="n"/>
+      <c r="P374" s="2" t="n"/>
+      <c r="Q374" s="2" t="n"/>
     </row>
     <row r="375" ht="130" customHeight="1">
-      <c r="A375" s="3" t="inlineStr">
+      <c r="A375" s="2" t="inlineStr">
         <is>
           <t>CM-6 b</t>
         </is>
       </c>
-      <c r="B375" s="3" t="inlineStr">
+      <c r="B375" s="2" t="inlineStr">
         <is>
           <t>CCI-000366</t>
         </is>
       </c>
-      <c r="C375" s="3" t="inlineStr">
+      <c r="C375" s="2" t="inlineStr">
         <is>
           <t>SRG-OS-000480-GPOS-00227</t>
         </is>
       </c>
-      <c r="D375" s="3" t="inlineStr">
+      <c r="D375" s="2" t="inlineStr">
         <is>
           <t>CCE-83705-4</t>
         </is>
       </c>
-      <c r="E375" s="3" t="inlineStr">
+      <c r="E375" s="2" t="inlineStr">
         <is>
           <t>The operating system must be configured in accordance with the security configuration settings based on DoD security configuration or implementation guidance, including STIGs, NSA configuration guides, CTOs, and DTMs.</t>
         </is>
       </c>
-      <c r="F375" s="3" t="inlineStr">
+      <c r="F375" s="2" t="inlineStr">
         <is>
           <t>Red Hat Enterprise Linux 9 must be configured in accordance with the security configuration settings based on DoD security configuration or implementation guidance, including STIGs, NSA configuration guides, CTOs, and DTMs.</t>
         </is>
       </c>
-      <c r="G375" s="3" t="inlineStr">
+      <c r="G375" s="2" t="inlineStr">
         <is>
           <t>Configuring the operating system to implement organization-wide security implementation guides and security checklists ensures compliance with federal standards and establishes a common security baseline across DoD that reflects the most restrictive security posture consistent with operational requirements.
 Configuration settings are the set of parameters that can be changed in hardware, software, or firmware components of the system that affect the security posture and/or functionality of the system. Security-related parameters are those parameters impacting the security state of the system, including the parameters required to satisfy other security control requirements. Security-related parameters include, for example: registry settings; account, file, directory permission settings; and settings for functions, ports, protocols, services, and remote connections.</t>
         </is>
       </c>
-      <c r="H375" s="3" t="inlineStr">
+      <c r="H375" s="2" t="inlineStr">
         <is>
           <t>If "write_logs" isn't set to "yes", the Audit logs will
 not be written to the disk.</t>
         </is>
       </c>
-      <c r="I375" s="3" t="inlineStr">
-        <is>
-          <t>Applicable - Configurable</t>
-        </is>
-      </c>
-      <c r="J375" s="3" t="inlineStr">
+      <c r="I375" s="2" t="inlineStr">
+        <is>
+          <t>Applicable - Configurable</t>
+        </is>
+      </c>
+      <c r="J375" s="2" t="inlineStr">
         <is>
           <t>Verify the operating system is configured in accordance with the security configuration settings based on DoD security configuration or implementation guidance, including STIGs, NSA configuration guides, CTOs, and DTMs. If it is not, this is a finding.</t>
         </is>
       </c>
-      <c r="K375" s="3" t="inlineStr">
+      <c r="K375" s="2" t="inlineStr">
         <is>
           <t>To verify that Audit Daemon is configured to write logs to the disk, run the
 following command:
@@ -30003,16 +30049,21 @@
 If write_logs isn't set to yes, then this is a finding.</t>
         </is>
       </c>
-      <c r="L375" s="3" t="n"/>
-      <c r="M375" s="3" t="inlineStr"/>
-      <c r="N375" s="3" t="inlineStr">
-        <is>
-          <t>CAT II</t>
-        </is>
-      </c>
-      <c r="O375" s="3" t="n"/>
-      <c r="P375" s="3" t="n"/>
-      <c r="Q375" s="3" t="n"/>
+      <c r="L375" s="2" t="n"/>
+      <c r="M375" s="2" t="inlineStr">
+        <is>
+          <t>Edit the file "/etc/audit/auditd.conf" and add or edit the following line:
+write_logs = yes</t>
+        </is>
+      </c>
+      <c r="N375" s="2" t="inlineStr">
+        <is>
+          <t>CAT II</t>
+        </is>
+      </c>
+      <c r="O375" s="2" t="n"/>
+      <c r="P375" s="2" t="n"/>
+      <c r="Q375" s="2" t="n"/>
     </row>
     <row r="376" ht="130" customHeight="1">
       <c r="A376" s="3" t="inlineStr">
@@ -30112,7 +30163,7 @@
     <row r="377" ht="130" customHeight="1">
       <c r="A377" s="2" t="inlineStr">
         <is>
-          <t>CM-6 b,SC-3</t>
+          <t>SC-3,CM-6 b</t>
         </is>
       </c>
       <c r="B377" s="2" t="inlineStr">
@@ -30506,7 +30557,7 @@
     <row r="382" ht="130" customHeight="1">
       <c r="A382" s="2" t="inlineStr">
         <is>
-          <t>CM-6 b,AC-17 (9),AC-17 (1),CM-7 b</t>
+          <t>AC-17 (1),CM-6 b,AC-17 (9),CM-7 b</t>
         </is>
       </c>
       <c r="B382" s="2" t="inlineStr">
@@ -30584,7 +30635,7 @@
     <row r="383" ht="130" customHeight="1">
       <c r="A383" s="2" t="inlineStr">
         <is>
-          <t>CM-6 b,AC-17 (1),CM-7 b</t>
+          <t>AC-17 (1),CM-6 b,CM-7 b</t>
         </is>
       </c>
       <c r="B383" s="2" t="inlineStr">
@@ -33858,7 +33909,7 @@
     <row r="422" ht="130" customHeight="1">
       <c r="A422" s="2" t="inlineStr">
         <is>
-          <t>CM-6 b,SC-3</t>
+          <t>SC-3,CM-6 b</t>
         </is>
       </c>
       <c r="B422" s="2" t="inlineStr">
@@ -34461,7 +34512,7 @@
     <row r="429" ht="130" customHeight="1">
       <c r="A429" s="2" t="inlineStr">
         <is>
-          <t>CM-6 b,SC-3</t>
+          <t>SC-3,CM-6 b</t>
         </is>
       </c>
       <c r="B429" s="2" t="inlineStr">
@@ -34913,7 +34964,7 @@
     <row r="435" ht="130" customHeight="1">
       <c r="A435" s="2" t="inlineStr">
         <is>
-          <t>AU-4,CM-6 b</t>
+          <t>CM-6 b,AU-4</t>
         </is>
       </c>
       <c r="B435" s="2" t="inlineStr">
@@ -36349,7 +36400,7 @@
     <row r="454" ht="130" customHeight="1">
       <c r="A454" s="3" t="inlineStr">
         <is>
-          <t>CM-6 b,SI-2 (2)</t>
+          <t>SI-2 (2),CM-6 b</t>
         </is>
       </c>
       <c r="B454" s="3" t="inlineStr">
@@ -36640,7 +36691,7 @@
     <row r="458" ht="130" customHeight="1">
       <c r="A458" s="3" t="inlineStr">
         <is>
-          <t>MA-4 (7),MA-4 e,SC-10,AC-12</t>
+          <t>MA-4 e,SC-10,MA-4 (7),AC-12</t>
         </is>
       </c>
       <c r="B458" s="3" t="inlineStr">
@@ -36870,7 +36921,7 @@
     <row r="461" ht="130" customHeight="1">
       <c r="A461" s="3" t="inlineStr">
         <is>
-          <t>SC-10,AC-11 a</t>
+          <t>AC-11 a,SC-10</t>
         </is>
       </c>
       <c r="B461" s="3" t="inlineStr">
@@ -39697,7 +39748,7 @@
     <row r="497" ht="130" customHeight="1">
       <c r="A497" s="2" t="inlineStr">
         <is>
-          <t>AU-4,AU-4 (1)</t>
+          <t>AU-4 (1),AU-4</t>
         </is>
       </c>
       <c r="B497" s="2" t="inlineStr">
@@ -39948,7 +39999,7 @@
     <row r="500" ht="130" customHeight="1">
       <c r="A500" s="2" t="inlineStr">
         <is>
-          <t>AC-8 c 1, AC-8 c 2, AC-8 c 3,AC-8 a</t>
+          <t>AC-8 a,AC-8 c 1, AC-8 c 2, AC-8 c 3</t>
         </is>
       </c>
       <c r="B500" s="2" t="inlineStr">
@@ -40050,7 +40101,7 @@
     <row r="501" ht="130" customHeight="1">
       <c r="A501" s="2" t="inlineStr">
         <is>
-          <t>AC-8 c 1, AC-8 c 2, AC-8 c 3,AC-8 a</t>
+          <t>AC-8 a,AC-8 c 1, AC-8 c 2, AC-8 c 3</t>
         </is>
       </c>
       <c r="B501" s="2" t="inlineStr">
@@ -40160,7 +40211,7 @@
     <row r="502" ht="130" customHeight="1">
       <c r="A502" s="2" t="inlineStr">
         <is>
-          <t>AC-8 c 1, AC-8 c 2, AC-8 c 3,AC-8 a</t>
+          <t>AC-8 a,AC-8 c 1, AC-8 c 2, AC-8 c 3</t>
         </is>
       </c>
       <c r="B502" s="2" t="inlineStr">
@@ -40271,7 +40322,7 @@
     <row r="503" ht="130" customHeight="1">
       <c r="A503" s="2" t="inlineStr">
         <is>
-          <t>AC-8 c 1, AC-8 c 2, AC-8 c 3,AC-8 a</t>
+          <t>AC-8 a,AC-8 c 1, AC-8 c 2, AC-8 c 3</t>
         </is>
       </c>
       <c r="B503" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Deploying to gh-pages from @ marcusburghardt/content@17099e6f580d9d46616de199c2893a2e8af2eff6 🚀
</commit_message>
<xml_diff>
--- a/srg_mapping/srg-mapping-rhel9.xlsx
+++ b/srg_mapping/srg-mapping-rhel9.xlsx
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q539"/>
+  <dimension ref="A1:Q538"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
@@ -544,7 +544,7 @@
     <row r="2" ht="130" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>AC-7 b,AC-7 a</t>
+          <t>AC-7 a,AC-7 b</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
@@ -628,7 +628,7 @@
     <row r="3" ht="130" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>AC-7 b,AC-7 a</t>
+          <t>AC-7 a,AC-7 b</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
@@ -713,7 +713,7 @@
     <row r="4" ht="130" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>AC-7 b,AC-7 a</t>
+          <t>AC-7 a,AC-7 b</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
@@ -785,7 +785,7 @@
     <row r="5" ht="130" customHeight="1">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>AC-7 b,AC-7 a</t>
+          <t>AC-7 a,AC-7 b</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
@@ -967,7 +967,7 @@
     <row r="7" ht="130" customHeight="1">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>AU-5 b,AU-5 a</t>
+          <t>AU-5 a,AU-5 b</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
@@ -1461,7 +1461,7 @@
     <row r="13" ht="130" customHeight="1">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>AU-7 (1),CM-5 (1),AU-3,AU-14 (1),AU-12 c,AU-12 a,AU-12 (3),AU-6 (4),AU-7 a,AU-3 (1),MA-4 (1) (a),AU-8 b,AU-7 b</t>
+          <t>AU-12 (3),AU-7 (1),AU-8 b,CM-5 (1),AU-3 (1),AU-14 (1),MA-4 (1) (a),AU-3,AU-7 a,AU-6 (4),AU-12 c,AU-7 b,AU-12 a</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
@@ -1522,7 +1522,7 @@
           <t xml:space="preserve">
 Run the following command to determine the current status of the
  auditd  service:
- $ systemctl is-active auditd 
+ $ sudo systemctl is-active auditd 
 If the service is running, it should return the following:  active 
 If the auditd service is not running, then this is a finding.</t>
         </is>
@@ -1546,7 +1546,7 @@
     <row r="14" ht="130" customHeight="1">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>AU-7 (1),CM-5 (1),AU-3,AU-14 (1),AU-12 c,AU-12 a,AU-12 (3),AU-6 (4),AU-7 a,AU-3 (1),MA-4 (1) (a),AU-8 b,AU-7 b</t>
+          <t>AU-12 (3),AU-7 (1),AU-8 b,CM-5 (1),AU-3 (1),AU-14 (1),MA-4 (1) (a),AU-3,AU-7 a,AU-6 (4),AU-12 c,AU-7 b,AU-12 a</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
@@ -1753,7 +1753,7 @@
           <t xml:space="preserve">
 Run the following command to determine the current status of the
  fapolicyd  service:
- $ systemctl is-active fapolicyd 
+ $ sudo systemctl is-active fapolicyd 
 If the service is running, it should return the following:  active 
 If the service is not enabled, then this is a finding.</t>
         </is>
@@ -3339,7 +3339,7 @@
     <row r="38" ht="130" customHeight="1">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>AU-3,AU-14 (1),AU-12 c,AU-12 a,AU-3 (1),MA-4 (1) (a)</t>
+          <t>AU-3 (1),AU-14 (1),MA-4 (1) (a),AU-3,AU-12 c,AU-12 a</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
@@ -3430,7 +3430,7 @@
     <row r="39" ht="130" customHeight="1">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>AU-14 (1),AU-4</t>
+          <t>AU-4,AU-14 (1)</t>
         </is>
       </c>
       <c r="B39" s="2" t="inlineStr">
@@ -3518,7 +3518,7 @@
     <row r="40" ht="130" customHeight="1">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>AU-3,AU-4 (1)</t>
+          <t>AU-4 (1),AU-3</t>
         </is>
       </c>
       <c r="B40" s="2" t="inlineStr">
@@ -3912,7 +3912,7 @@
     <row r="45" ht="130" customHeight="1">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>CM-6 b,AU-4 (1),AU-6 (4)</t>
+          <t>CM-6 b,AU-6 (4),AU-4 (1)</t>
         </is>
       </c>
       <c r="B45" s="2" t="inlineStr">
@@ -4073,7 +4073,7 @@
     <row r="47" ht="130" customHeight="1">
       <c r="A47" s="2" t="inlineStr">
         <is>
-          <t>AU-8 (1) (a),AU-8 (1) (b),AU-8 b</t>
+          <t>AU-8 b,AU-8 (1) (b),AU-8 (1) (a)</t>
         </is>
       </c>
       <c r="B47" s="2" t="inlineStr">
@@ -4314,7 +4314,7 @@
     <row r="50" ht="130" customHeight="1">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>IA-2 (12),IA-2 (11),IA-2 (1)</t>
+          <t>IA-2 (12),IA-2 (1),IA-2 (11)</t>
         </is>
       </c>
       <c r="B50" s="2" t="inlineStr">
@@ -4398,7 +4398,7 @@
     <row r="51" ht="130" customHeight="1">
       <c r="A51" s="2" t="inlineStr">
         <is>
-          <t>SI-6 b,SI-6 d,CM-3 (5)</t>
+          <t>CM-3 (5),SI-6 d,SI-6 b</t>
         </is>
       </c>
       <c r="B51" s="2" t="inlineStr">
@@ -4490,7 +4490,7 @@
     <row r="52" ht="130" customHeight="1">
       <c r="A52" s="3" t="inlineStr">
         <is>
-          <t>SI-6 d,CM-3 (5)</t>
+          <t>CM-3 (5),SI-6 d</t>
         </is>
       </c>
       <c r="B52" s="3" t="inlineStr">
@@ -4574,7 +4574,7 @@
     <row r="53" ht="130" customHeight="1">
       <c r="A53" s="3" t="inlineStr">
         <is>
-          <t>AU-3,AU-12 c,AU-12 a,AU-3 (1),MA-4 (1) (a)</t>
+          <t>AU-3 (1),MA-4 (1) (a),AU-3,AU-12 c,AU-12 a</t>
         </is>
       </c>
       <c r="B53" s="3" t="inlineStr">
@@ -4649,7 +4649,7 @@
     <row r="54" ht="130" customHeight="1">
       <c r="A54" s="3" t="inlineStr">
         <is>
-          <t>AU-3,AU-12 c,AU-12 a,AU-3 (1),MA-4 (1) (a)</t>
+          <t>AU-3 (1),MA-4 (1) (a),AU-3,AU-12 c,AU-12 a</t>
         </is>
       </c>
       <c r="B54" s="3" t="inlineStr">
@@ -4724,7 +4724,7 @@
     <row r="55" ht="130" customHeight="1">
       <c r="A55" s="3" t="inlineStr">
         <is>
-          <t>AU-3,AU-12 c,AU-12 a,AU-3 (1),MA-4 (1) (a)</t>
+          <t>AU-3 (1),MA-4 (1) (a),AU-3,AU-12 c,AU-12 a</t>
         </is>
       </c>
       <c r="B55" s="3" t="inlineStr">
@@ -4799,7 +4799,7 @@
     <row r="56" ht="130" customHeight="1">
       <c r="A56" s="3" t="inlineStr">
         <is>
-          <t>AU-3,AU-12 c,AU-12 a,AU-3 (1),MA-4 (1) (a)</t>
+          <t>AU-3 (1),MA-4 (1) (a),AU-3,AU-12 c,AU-12 a</t>
         </is>
       </c>
       <c r="B56" s="3" t="inlineStr">
@@ -4874,7 +4874,7 @@
     <row r="57" ht="130" customHeight="1">
       <c r="A57" s="3" t="inlineStr">
         <is>
-          <t>AU-3,AU-12 c,AU-12 a,AU-3 (1),MA-4 (1) (a)</t>
+          <t>AU-3 (1),MA-4 (1) (a),AU-3,AU-12 c,AU-12 a</t>
         </is>
       </c>
       <c r="B57" s="3" t="inlineStr">
@@ -4949,7 +4949,7 @@
     <row r="58" ht="130" customHeight="1">
       <c r="A58" s="3" t="inlineStr">
         <is>
-          <t>AU-3,AU-12 c,AU-12 a,AU-3 (1),MA-4 (1) (a)</t>
+          <t>AU-3 (1),MA-4 (1) (a),AU-3,AU-12 c,AU-12 a</t>
         </is>
       </c>
       <c r="B58" s="3" t="inlineStr">
@@ -5024,7 +5024,7 @@
     <row r="59" ht="130" customHeight="1">
       <c r="A59" s="3" t="inlineStr">
         <is>
-          <t>AU-3,AU-12 c,AU-12 a,AU-3 (1),MA-4 (1) (a)</t>
+          <t>AU-3 (1),MA-4 (1) (a),AU-3,AU-12 c,AU-12 a</t>
         </is>
       </c>
       <c r="B59" s="3" t="inlineStr">
@@ -5099,7 +5099,7 @@
     <row r="60" ht="130" customHeight="1">
       <c r="A60" s="3" t="inlineStr">
         <is>
-          <t>AU-3,AU-12 c,AU-12 a,AU-3 (1),MA-4 (1) (a)</t>
+          <t>AU-3 (1),MA-4 (1) (a),AU-3,AU-12 c,AU-12 a</t>
         </is>
       </c>
       <c r="B60" s="3" t="inlineStr">
@@ -5174,7 +5174,7 @@
     <row r="61" ht="130" customHeight="1">
       <c r="A61" s="3" t="inlineStr">
         <is>
-          <t>AU-3,AU-12 c,AU-12 a,AU-3 (1),MA-4 (1) (a)</t>
+          <t>AU-3 (1),MA-4 (1) (a),AU-3,AU-12 c,AU-12 a</t>
         </is>
       </c>
       <c r="B61" s="3" t="inlineStr">
@@ -5249,7 +5249,7 @@
     <row r="62" ht="130" customHeight="1">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>AU-3,AU-12 c,AU-12 a,AU-3 (1),MA-4 (1) (a),AC-2 (4)</t>
+          <t>AU-3 (1),MA-4 (1) (a),AU-3,AU-12 c,AC-2 (4),AU-12 a</t>
         </is>
       </c>
       <c r="B62" s="2" t="inlineStr">
@@ -5274,7 +5274,7 @@
       </c>
       <c r="F62" s="2" t="inlineStr">
         <is>
-          <t>Red Hat Enterprise Linux 9 Must Audit All Account Creations.</t>
+          <t xml:space="preserve"> Red Hat Enterprise Linux 9 must generate audit records for all account creations, modifications, disabling, and termination events that affect /etc/sudoers.</t>
         </is>
       </c>
       <c r="G62" s="2" t="inlineStr">
@@ -5330,7 +5330,7 @@
     <row r="63" ht="130" customHeight="1">
       <c r="A63" s="2" t="inlineStr">
         <is>
-          <t>AU-3,AU-12 c,AU-12 a,AU-3 (1),MA-4 (1) (a),AC-2 (4)</t>
+          <t>AU-3 (1),MA-4 (1) (a),AU-3,AU-12 c,AC-2 (4),AU-12 a</t>
         </is>
       </c>
       <c r="B63" s="2" t="inlineStr">
@@ -5355,7 +5355,7 @@
       </c>
       <c r="F63" s="2" t="inlineStr">
         <is>
-          <t>Red Hat Enterprise Linux 9 Must Audit All Account Creations.</t>
+          <t xml:space="preserve"> Red Hat Enterprise Linux 9 must generate audit records for all account creations, modifications, disabling, and termination events that affect /etc/sudoers.d/.</t>
         </is>
       </c>
       <c r="G63" s="2" t="inlineStr">
@@ -5411,7 +5411,7 @@
     <row r="64" ht="130" customHeight="1">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>AU-3,AU-12 c,AU-12 a,AU-3 (1),MA-4 (1) (a),AC-2 (4)</t>
+          <t>AU-3 (1),MA-4 (1) (a),AU-3,AU-12 c,AC-2 (4),AU-12 a</t>
         </is>
       </c>
       <c r="B64" s="2" t="inlineStr">
@@ -5436,7 +5436,7 @@
       </c>
       <c r="F64" s="2" t="inlineStr">
         <is>
-          <t>Red Hat Enterprise Linux 9 Must Audit All Account Creations.</t>
+          <t xml:space="preserve"> Red Hat Enterprise Linux 9 must generate audit records for all account creations, modifications, disabling, and termination events that affect /etc/group.</t>
         </is>
       </c>
       <c r="G64" s="2" t="inlineStr">
@@ -5493,7 +5493,7 @@
     <row r="65" ht="130" customHeight="1">
       <c r="A65" s="2" t="inlineStr">
         <is>
-          <t>AU-3,AU-12 c,AU-12 a,AU-3 (1),MA-4 (1) (a),AC-2 (4)</t>
+          <t>AU-3 (1),MA-4 (1) (a),AU-3,AU-12 c,AC-2 (4),AU-12 a</t>
         </is>
       </c>
       <c r="B65" s="2" t="inlineStr">
@@ -5518,7 +5518,7 @@
       </c>
       <c r="F65" s="2" t="inlineStr">
         <is>
-          <t>Red Hat Enterprise Linux 9 Must Audit All Account Creations.</t>
+          <t xml:space="preserve"> Red Hat Enterprise Linux 9 must generate audit records for all account creations, modifications, disabling, and termination events that affect /etc/gshadow.</t>
         </is>
       </c>
       <c r="G65" s="2" t="inlineStr">
@@ -5575,7 +5575,7 @@
     <row r="66" ht="130" customHeight="1">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>AU-3,AU-12 c,AU-12 a,AU-3 (1),MA-4 (1) (a),AC-2 (4)</t>
+          <t>AU-3 (1),MA-4 (1) (a),AU-3,AU-12 c,AC-2 (4),AU-12 a</t>
         </is>
       </c>
       <c r="B66" s="2" t="inlineStr">
@@ -5600,7 +5600,7 @@
       </c>
       <c r="F66" s="2" t="inlineStr">
         <is>
-          <t>Red Hat Enterprise Linux 9 Must Audit All Account Creations.</t>
+          <t xml:space="preserve"> Red Hat Enterprise Linux 9 must generate audit records for all account creations, modifications, disabling, and termination events that affect /etc/opasswd.</t>
         </is>
       </c>
       <c r="G66" s="2" t="inlineStr">
@@ -5657,7 +5657,7 @@
     <row r="67" ht="130" customHeight="1">
       <c r="A67" s="2" t="inlineStr">
         <is>
-          <t>AU-3,AU-12 c,AU-12 a,AU-3 (1),MA-4 (1) (a),AC-2 (4)</t>
+          <t>AU-3 (1),MA-4 (1) (a),AU-3,AU-12 c,AC-2 (4),AU-12 a</t>
         </is>
       </c>
       <c r="B67" s="2" t="inlineStr">
@@ -5682,7 +5682,7 @@
       </c>
       <c r="F67" s="2" t="inlineStr">
         <is>
-          <t>Red Hat Enterprise Linux 9 Must Audit All Account Creations.</t>
+          <t xml:space="preserve"> Red Hat Enterprise Linux 9 must generate audit records for all account creations, modifications, disabling, and termination events that affect /etc/passwd.</t>
         </is>
       </c>
       <c r="G67" s="2" t="inlineStr">
@@ -5739,7 +5739,7 @@
     <row r="68" ht="130" customHeight="1">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>AU-3,AU-12 c,AU-12 a,AU-3 (1),MA-4 (1) (a),AC-2 (4)</t>
+          <t>AU-3 (1),MA-4 (1) (a),AU-3,AU-12 c,AC-2 (4),AU-12 a</t>
         </is>
       </c>
       <c r="B68" s="2" t="inlineStr">
@@ -5764,7 +5764,7 @@
       </c>
       <c r="F68" s="2" t="inlineStr">
         <is>
-          <t>Red Hat Enterprise Linux 9 Must Audit All Account Creations.</t>
+          <t xml:space="preserve"> Red Hat Enterprise Linux 9 must generate audit records for all account creations, modifications, disabling, and termination events that affect /etc/shadow.</t>
         </is>
       </c>
       <c r="G68" s="2" t="inlineStr">
@@ -5821,7 +5821,7 @@
     <row r="69" ht="130" customHeight="1">
       <c r="A69" s="2" t="inlineStr">
         <is>
-          <t>SI-6 a,CM-3 (5)</t>
+          <t>CM-3 (5),SI-6 a</t>
         </is>
       </c>
       <c r="B69" s="2" t="inlineStr">
@@ -6859,7 +6859,7 @@
     <row r="82" ht="130" customHeight="1">
       <c r="A82" s="3" t="inlineStr">
         <is>
-          <t>AU-3,AU-12 c,AU-12 a,AU-3 (1),MA-4 (1) (a)</t>
+          <t>AU-3 (1),MA-4 (1) (a),AU-3,AU-12 c,AU-12 a</t>
         </is>
       </c>
       <c r="B82" s="3" t="inlineStr">
@@ -6933,7 +6933,7 @@
     <row r="83" ht="130" customHeight="1">
       <c r="A83" s="3" t="inlineStr">
         <is>
-          <t>AU-3,AU-12 c,AU-12 a,AU-3 (1),MA-4 (1) (a)</t>
+          <t>AU-3 (1),MA-4 (1) (a),AU-3,AU-12 c,AU-12 a</t>
         </is>
       </c>
       <c r="B83" s="3" t="inlineStr">
@@ -7007,7 +7007,7 @@
     <row r="84" ht="130" customHeight="1">
       <c r="A84" s="3" t="inlineStr">
         <is>
-          <t>AU-3,AU-12 c,AU-12 a,AU-3 (1),MA-4 (1) (a)</t>
+          <t>AU-3 (1),MA-4 (1) (a),AU-3,AU-12 c,AU-12 a</t>
         </is>
       </c>
       <c r="B84" s="3" t="inlineStr">
@@ -7081,7 +7081,7 @@
     <row r="85" ht="130" customHeight="1">
       <c r="A85" s="3" t="inlineStr">
         <is>
-          <t>AU-3,AU-12 c,AU-12 a,AU-3 (1),MA-4 (1) (a)</t>
+          <t>AU-3 (1),MA-4 (1) (a),AU-3,AU-12 c,AU-12 a</t>
         </is>
       </c>
       <c r="B85" s="3" t="inlineStr">
@@ -7161,7 +7161,7 @@
     <row r="86" ht="130" customHeight="1">
       <c r="A86" s="3" t="inlineStr">
         <is>
-          <t>MA-4 (6),SC-13</t>
+          <t>SC-13,MA-4 (6)</t>
         </is>
       </c>
       <c r="B86" s="3" t="inlineStr">
@@ -7322,7 +7322,7 @@
     <row r="88" ht="130" customHeight="1">
       <c r="A88" s="3" t="inlineStr">
         <is>
-          <t>MA-4 (6),SC-13</t>
+          <t>SC-13,MA-4 (6)</t>
         </is>
       </c>
       <c r="B88" s="3" t="inlineStr">
@@ -7657,7 +7657,7 @@
     <row r="92" ht="130" customHeight="1">
       <c r="A92" s="3" t="inlineStr">
         <is>
-          <t>AU-3,AU-12 c,AU-12 a,AU-3 (1),MA-4 (1) (a)</t>
+          <t>AU-3 (1),MA-4 (1) (a),AU-3,AU-12 c,AU-12 a</t>
         </is>
       </c>
       <c r="B92" s="3" t="inlineStr">
@@ -7732,7 +7732,7 @@
     <row r="93" ht="130" customHeight="1">
       <c r="A93" s="3" t="inlineStr">
         <is>
-          <t>AU-3,AU-12 c,AU-12 a,AU-3 (1),MA-4 (1) (a)</t>
+          <t>AU-3 (1),MA-4 (1) (a),AU-3,AU-12 c,AU-12 a</t>
         </is>
       </c>
       <c r="B93" s="3" t="inlineStr">
@@ -7807,7 +7807,7 @@
     <row r="94" ht="130" customHeight="1">
       <c r="A94" s="3" t="inlineStr">
         <is>
-          <t>AU-3,AU-12 c,AU-12 a,AU-3 (1),MA-4 (1) (a)</t>
+          <t>AU-3 (1),MA-4 (1) (a),AU-3,AU-12 c,AU-12 a</t>
         </is>
       </c>
       <c r="B94" s="3" t="inlineStr">
@@ -7882,7 +7882,7 @@
     <row r="95" ht="130" customHeight="1">
       <c r="A95" s="3" t="inlineStr">
         <is>
-          <t>AU-3,AU-12 c,AU-12 a,AU-3 (1),MA-4 (1) (a)</t>
+          <t>AU-3 (1),MA-4 (1) (a),AU-3,AU-12 c,AU-12 a</t>
         </is>
       </c>
       <c r="B95" s="3" t="inlineStr">
@@ -7962,7 +7962,7 @@
     <row r="96" ht="130" customHeight="1">
       <c r="A96" s="2" t="inlineStr">
         <is>
-          <t>AU-3,AU-12 c,AU-12 a,AU-3 (1),MA-4 (1) (a)</t>
+          <t>AU-3 (1),MA-4 (1) (a),AU-3,AU-12 c,AU-12 a</t>
         </is>
       </c>
       <c r="B96" s="2" t="inlineStr">
@@ -8044,7 +8044,7 @@
     <row r="97" ht="130" customHeight="1">
       <c r="A97" s="2" t="inlineStr">
         <is>
-          <t>AU-3,AU-12 c,AU-12 a,AU-3 (1),MA-4 (1) (a)</t>
+          <t>AU-3 (1),MA-4 (1) (a),AU-3,AU-12 c,AU-12 a</t>
         </is>
       </c>
       <c r="B97" s="2" t="inlineStr">
@@ -8126,7 +8126,7 @@
     <row r="98" ht="130" customHeight="1">
       <c r="A98" s="2" t="inlineStr">
         <is>
-          <t>AU-3,AU-12 c,AU-12 a,AU-3 (1),MA-4 (1) (a)</t>
+          <t>AU-3 (1),MA-4 (1) (a),AU-3,AU-12 c,AU-12 a</t>
         </is>
       </c>
       <c r="B98" s="2" t="inlineStr">
@@ -8208,7 +8208,7 @@
     <row r="99" ht="130" customHeight="1">
       <c r="A99" s="2" t="inlineStr">
         <is>
-          <t>AU-3,AU-12 c,AU-12 a,AU-3 (1),MA-4 (1) (a)</t>
+          <t>AU-3 (1),MA-4 (1) (a),AU-3,AU-12 c,AU-12 a</t>
         </is>
       </c>
       <c r="B99" s="2" t="inlineStr">
@@ -8290,7 +8290,7 @@
     <row r="100" ht="130" customHeight="1">
       <c r="A100" s="2" t="inlineStr">
         <is>
-          <t>AU-3,AU-12 c,AU-12 a,AU-3 (1),MA-4 (1) (a)</t>
+          <t>AU-3 (1),MA-4 (1) (a),AU-3,AU-12 c,AU-12 a</t>
         </is>
       </c>
       <c r="B100" s="2" t="inlineStr">
@@ -8372,7 +8372,7 @@
     <row r="101" ht="130" customHeight="1">
       <c r="A101" s="3" t="inlineStr">
         <is>
-          <t>AU-3,AU-12 c,AU-12 a,AU-3 (1),MA-4 (1) (a)</t>
+          <t>AU-3 (1),MA-4 (1) (a),AU-3,AU-12 c,AU-12 a</t>
         </is>
       </c>
       <c r="B101" s="3" t="inlineStr">
@@ -8452,7 +8452,7 @@
     <row r="102" ht="130" customHeight="1">
       <c r="A102" s="3" t="inlineStr">
         <is>
-          <t>AU-3,AU-12 c,AU-12 a,AU-3 (1),MA-4 (1) (a)</t>
+          <t>AU-3 (1),MA-4 (1) (a),AU-3,AU-12 c,AU-12 a</t>
         </is>
       </c>
       <c r="B102" s="3" t="inlineStr">
@@ -8532,7 +8532,7 @@
     <row r="103" ht="130" customHeight="1">
       <c r="A103" s="3" t="inlineStr">
         <is>
-          <t>AU-3,AU-12 c,AU-12 a,AU-3 (1),MA-4 (1) (a)</t>
+          <t>AU-3 (1),MA-4 (1) (a),AU-3,AU-12 c,AU-12 a</t>
         </is>
       </c>
       <c r="B103" s="3" t="inlineStr">
@@ -8783,7 +8783,7 @@
     <row r="106" ht="130" customHeight="1">
       <c r="A106" s="2" t="inlineStr">
         <is>
-          <t>AC-6 (10),AC-11 b</t>
+          <t>AC-11 b,AC-6 (10)</t>
         </is>
       </c>
       <c r="B106" s="2" t="inlineStr">
@@ -8862,7 +8862,7 @@
     <row r="107" ht="130" customHeight="1">
       <c r="A107" s="2" t="inlineStr">
         <is>
-          <t>AC-11 b,AC-11 a</t>
+          <t>AC-11 a,AC-11 b</t>
         </is>
       </c>
       <c r="B107" s="2" t="inlineStr">
@@ -8941,7 +8941,7 @@
     <row r="108" ht="130" customHeight="1">
       <c r="A108" s="2" t="inlineStr">
         <is>
-          <t>AC-11 b,AC-11 a</t>
+          <t>AC-11 a,AC-11 b</t>
         </is>
       </c>
       <c r="B108" s="2" t="inlineStr">
@@ -9028,7 +9028,7 @@
     <row r="109" ht="130" customHeight="1">
       <c r="A109" s="2" t="inlineStr">
         <is>
-          <t>AC-11 b,AC-11 a</t>
+          <t>AC-11 a,AC-11 b</t>
         </is>
       </c>
       <c r="B109" s="2" t="inlineStr">
@@ -9115,7 +9115,7 @@
     <row r="110" ht="130" customHeight="1">
       <c r="A110" s="3" t="inlineStr">
         <is>
-          <t>AC-11 b,AC-11 a</t>
+          <t>AC-11 a,AC-11 b</t>
         </is>
       </c>
       <c r="B110" s="3" t="inlineStr">
@@ -9360,7 +9360,7 @@
     <row r="113" ht="130" customHeight="1">
       <c r="A113" s="2" t="inlineStr">
         <is>
-          <t>AC-17 (2),SC-13,MA-4 c,SC-8</t>
+          <t>SC-8,AC-17 (2),SC-13,MA-4 c</t>
         </is>
       </c>
       <c r="B113" s="2" t="inlineStr">
@@ -9467,7 +9467,7 @@
       </c>
       <c r="F114" s="2" t="inlineStr">
         <is>
-          <t>Red Hat Enterprise Linux 9 Must Generate Audit Records When Concurrent Logons To The Same Account Occur From Different Sources.</t>
+          <t xml:space="preserve"> Red Hat Enterprise Linux 9 must generate audit records for all account creations, modifications, disabling, and termination events that affect /var/run/faillock.</t>
         </is>
       </c>
       <c r="G114" s="2" t="inlineStr">
@@ -9520,7 +9520,7 @@
     <row r="115" ht="130" customHeight="1">
       <c r="A115" s="2" t="inlineStr">
         <is>
-          <t>AU-3,AU-12 c,AU-12 a,AU-3 (1),MA-4 (1) (a)</t>
+          <t>AU-3 (1),MA-4 (1) (a),AU-3,AU-12 c,AU-12 a</t>
         </is>
       </c>
       <c r="B115" s="2" t="inlineStr">
@@ -9545,7 +9545,7 @@
       </c>
       <c r="F115" s="2" t="inlineStr">
         <is>
-          <t>Red Hat Enterprise Linux 9 Must Generate Audit Records When Concurrent Logons To The Same Account Occur From Different Sources.</t>
+          <t xml:space="preserve"> Red Hat Enterprise Linux 9 must generate audit records for all account creations, modifications, disabling, and termination events that affect /var/log/lastlog.</t>
         </is>
       </c>
       <c r="G115" s="2" t="inlineStr">
@@ -9623,7 +9623,7 @@
       </c>
       <c r="F116" s="2" t="inlineStr">
         <is>
-          <t>Red Hat Enterprise Linux 9 Must Generate Audit Records When Concurrent Logons To The Same Account Occur From Different Sources.</t>
+          <t xml:space="preserve"> Red Hat Enterprise Linux 9 must generate audit records for all account creations, modifications, disabling, and termination events that affect /var/log/tallylog.</t>
         </is>
       </c>
       <c r="G116" s="2" t="inlineStr">
@@ -9676,7 +9676,7 @@
     <row r="117" ht="130" customHeight="1">
       <c r="A117" s="3" t="inlineStr">
         <is>
-          <t>AU-3,AU-12 c,AU-12 a,AU-3 (1),MA-4 (1) (a)</t>
+          <t>AU-3 (1),MA-4 (1) (a),AU-3,AU-12 c,AU-12 a</t>
         </is>
       </c>
       <c r="B117" s="3" t="inlineStr">
@@ -10032,7 +10032,7 @@
     <row r="122" ht="130" customHeight="1">
       <c r="A122" s="3" t="inlineStr">
         <is>
-          <t>AU-3,AU-12 c,AU-12 a,AU-3 (1),MA-4 (1) (a)</t>
+          <t>AU-3 (1),MA-4 (1) (a),AU-3,AU-12 c,AU-12 a</t>
         </is>
       </c>
       <c r="B122" s="3" t="inlineStr">
@@ -10112,7 +10112,7 @@
     <row r="123" ht="130" customHeight="1">
       <c r="A123" s="2" t="inlineStr">
         <is>
-          <t>SC-28,SC-28 (1)</t>
+          <t>SC-28 (1),SC-28</t>
         </is>
       </c>
       <c r="B123" s="2" t="inlineStr">
@@ -10886,7 +10886,7 @@
     <row r="133" ht="130" customHeight="1">
       <c r="A133" s="2" t="inlineStr">
         <is>
-          <t>AC-6 (10),CM-6 b</t>
+          <t>CM-6 b,AC-6 (10)</t>
         </is>
       </c>
       <c r="B133" s="2" t="inlineStr">
@@ -10967,7 +10967,7 @@
     <row r="134" ht="130" customHeight="1">
       <c r="A134" s="2" t="inlineStr">
         <is>
-          <t>AC-6 (10),CM-6 b</t>
+          <t>CM-6 b,AC-6 (10)</t>
         </is>
       </c>
       <c r="B134" s="2" t="inlineStr">
@@ -11053,7 +11053,7 @@
     <row r="135" ht="130" customHeight="1">
       <c r="A135" s="2" t="inlineStr">
         <is>
-          <t>AC-6 (10),CM-6 b</t>
+          <t>CM-6 b,AC-6 (10)</t>
         </is>
       </c>
       <c r="B135" s="2" t="inlineStr">
@@ -11109,17 +11109,17 @@
           <t xml:space="preserve">
 To check that the  debug-shell  service is disabled in system boot configuration,
 run the following command:
- $ systemctl is-enabled  debug-shell  
+ $ sudo systemctl is-enabled  debug-shell  
 Output should indicate the  debug-shell  service has either not been installed,
 or has been disabled at all runlevels, as shown in the example below:
- $ systemctl is-enabled  debug-shell 
+ $ sudo systemctl is-enabled  debug-shell 
  disabled 
 Run the following command to verify  debug-shell  is not active (i.e. not running) through current runtime configuration:
- $ systemctl is-active debug-shell 
+ $ sudo systemctl is-active debug-shell 
 If the service is not running the command will return the following output:
  inactive 
 The service will also be masked, to check that the  debug-shell  is masked, run the following command:
- $ systemctl show  debug-shell  | grep "LoadState\|UnitFileState" 
+ $ sudo systemctl show  debug-shell  | grep "LoadState\|UnitFileState" 
 If the service is masked the command will return the following outputs:
  LoadState=masked 
  UnitFileState=masked 
@@ -11499,7 +11499,7 @@
     <row r="140" ht="130" customHeight="1">
       <c r="A140" s="3" t="inlineStr">
         <is>
-          <t>AU-3,AU-12 c,AU-12 a,AU-3 (1),MA-4 (1) (a)</t>
+          <t>AU-3 (1),MA-4 (1) (a),AU-3,AU-12 c,AU-12 a</t>
         </is>
       </c>
       <c r="B140" s="3" t="inlineStr">
@@ -11579,7 +11579,7 @@
     <row r="141" ht="130" customHeight="1">
       <c r="A141" s="3" t="inlineStr">
         <is>
-          <t>AU-3,AU-12 c,AU-12 a,AU-3 (1),MA-4 (1) (a)</t>
+          <t>AU-3 (1),MA-4 (1) (a),AU-3,AU-12 c,AU-12 a</t>
         </is>
       </c>
       <c r="B141" s="3" t="inlineStr">
@@ -11659,7 +11659,7 @@
     <row r="142" ht="130" customHeight="1">
       <c r="A142" s="3" t="inlineStr">
         <is>
-          <t>AU-3,AU-12 c,AU-12 a,AU-3 (1),MA-4 (1) (a)</t>
+          <t>AU-3 (1),MA-4 (1) (a),AU-3,AU-12 c,AU-12 a</t>
         </is>
       </c>
       <c r="B142" s="3" t="inlineStr">
@@ -11971,7 +11971,7 @@
     <row r="146" ht="130" customHeight="1">
       <c r="A146" s="2" t="inlineStr">
         <is>
-          <t>IA-5 (1) (c),IA-7</t>
+          <t>IA-7,IA-5 (1) (c)</t>
         </is>
       </c>
       <c r="B146" s="2" t="inlineStr">
@@ -12442,7 +12442,7 @@
     <row r="152" ht="130" customHeight="1">
       <c r="A152" s="2" t="inlineStr">
         <is>
-          <t>CM-6 b,IA-7</t>
+          <t>IA-7,CM-6 b</t>
         </is>
       </c>
       <c r="B152" s="2" t="inlineStr">
@@ -12518,7 +12518,7 @@
     <row r="153" ht="130" customHeight="1">
       <c r="A153" s="2" t="inlineStr">
         <is>
-          <t>CM-6 b,IA-7</t>
+          <t>IA-7,CM-6 b</t>
         </is>
       </c>
       <c r="B153" s="2" t="inlineStr">
@@ -12603,7 +12603,7 @@
     <row r="154" ht="130" customHeight="1">
       <c r="A154" s="2" t="inlineStr">
         <is>
-          <t>CM-6 b,IA-7</t>
+          <t>IA-7,CM-6 b</t>
         </is>
       </c>
       <c r="B154" s="2" t="inlineStr">
@@ -12839,7 +12839,7 @@
     <row r="157" ht="130" customHeight="1">
       <c r="A157" s="3" t="inlineStr">
         <is>
-          <t>AU-3,AU-12 c,AU-12 a,AU-3 (1),MA-4 (1) (a)</t>
+          <t>AU-3 (1),MA-4 (1) (a),AU-3,AU-12 c,AU-12 a</t>
         </is>
       </c>
       <c r="B157" s="3" t="inlineStr">
@@ -12916,7 +12916,7 @@
     <row r="158" ht="130" customHeight="1">
       <c r="A158" s="3" t="inlineStr">
         <is>
-          <t>AU-12 a,MA-4 (1) (a),AU-3,AU-12 c</t>
+          <t>MA-4 (1) (a),AU-12 a,AU-12 c,AU-3</t>
         </is>
       </c>
       <c r="B158" s="3" t="inlineStr">
@@ -12989,7 +12989,7 @@
     <row r="159" ht="130" customHeight="1">
       <c r="A159" s="3" t="inlineStr">
         <is>
-          <t>AU-12 a,MA-4 (1) (a),AU-3,AU-12 c</t>
+          <t>MA-4 (1) (a),AU-12 a,AU-12 c,AU-3</t>
         </is>
       </c>
       <c r="B159" s="3" t="inlineStr">
@@ -13062,7 +13062,7 @@
     <row r="160" ht="130" customHeight="1">
       <c r="A160" s="3" t="inlineStr">
         <is>
-          <t>AU-3,AU-12 c,AU-12 a,AU-3 (1),MA-4 (1) (a)</t>
+          <t>AU-3 (1),MA-4 (1) (a),AU-3,AU-12 c,AU-12 a</t>
         </is>
       </c>
       <c r="B160" s="3" t="inlineStr">
@@ -13147,7 +13147,7 @@
     <row r="161" ht="130" customHeight="1">
       <c r="A161" s="3" t="inlineStr">
         <is>
-          <t>AU-3,AU-12 c,AU-12 a,AU-3 (1),MA-4 (1) (a)</t>
+          <t>AU-3 (1),MA-4 (1) (a),AU-3,AU-12 c,AU-12 a</t>
         </is>
       </c>
       <c r="B161" s="3" t="inlineStr">
@@ -13222,7 +13222,7 @@
     <row r="162" ht="130" customHeight="1">
       <c r="A162" s="3" t="inlineStr">
         <is>
-          <t>AU-3,AU-12 c,AU-12 a,AU-3 (1),MA-4 (1) (a)</t>
+          <t>AU-3 (1),MA-4 (1) (a),AU-3,AU-12 c,AU-12 a</t>
         </is>
       </c>
       <c r="B162" s="3" t="inlineStr">
@@ -13297,7 +13297,7 @@
     <row r="163" ht="130" customHeight="1">
       <c r="A163" s="3" t="inlineStr">
         <is>
-          <t>AU-3,AU-12 c,AU-12 a,AU-3 (1),MA-4 (1) (a)</t>
+          <t>AU-3 (1),MA-4 (1) (a),AU-3,AU-12 c,AU-12 a</t>
         </is>
       </c>
       <c r="B163" s="3" t="inlineStr">
@@ -13372,7 +13372,7 @@
     <row r="164" ht="130" customHeight="1">
       <c r="A164" s="3" t="inlineStr">
         <is>
-          <t>AU-3,AU-12 c,AU-12 a,AU-3 (1),MA-4 (1) (a)</t>
+          <t>AU-3 (1),MA-4 (1) (a),AU-3,AU-12 c,AU-12 a</t>
         </is>
       </c>
       <c r="B164" s="3" t="inlineStr">
@@ -13875,7 +13875,7 @@
     <row r="171" ht="130" customHeight="1">
       <c r="A171" s="3" t="inlineStr">
         <is>
-          <t>AU-3,AU-12 c,AU-12 a,AU-3 (1),MA-4 (1) (a)</t>
+          <t>AU-3 (1),MA-4 (1) (a),AU-3,AU-12 c,AU-12 a</t>
         </is>
       </c>
       <c r="B171" s="3" t="inlineStr">
@@ -14164,7 +14164,7 @@
     <row r="175" ht="130" customHeight="1">
       <c r="A175" s="3" t="inlineStr">
         <is>
-          <t>AU-3,AU-12 c,AU-12 a,AU-3 (1),MA-4 (1) (a)</t>
+          <t>AU-3 (1),MA-4 (1) (a),AU-3,AU-12 c,AU-12 a</t>
         </is>
       </c>
       <c r="B175" s="3" t="inlineStr">
@@ -14239,7 +14239,7 @@
     <row r="176" ht="130" customHeight="1">
       <c r="A176" s="3" t="inlineStr">
         <is>
-          <t>AU-3,AU-12 c,AU-12 a,AU-3 (1),MA-4 (1) (a)</t>
+          <t>AU-3 (1),MA-4 (1) (a),AU-3,AU-12 c,AU-12 a</t>
         </is>
       </c>
       <c r="B176" s="3" t="inlineStr">
@@ -14321,7 +14321,7 @@
     <row r="177" ht="130" customHeight="1">
       <c r="A177" s="3" t="inlineStr">
         <is>
-          <t>AU-3,AU-12 c,AU-12 a,AU-3 (1),MA-4 (1) (a)</t>
+          <t>AU-3 (1),MA-4 (1) (a),AU-3,AU-12 c,AU-12 a</t>
         </is>
       </c>
       <c r="B177" s="3" t="inlineStr">
@@ -14403,7 +14403,7 @@
     <row r="178" ht="130" customHeight="1">
       <c r="A178" s="3" t="inlineStr">
         <is>
-          <t>AU-3,AU-12 c,AU-12 a,AU-3 (1),MA-4 (1) (a)</t>
+          <t>AU-3 (1),MA-4 (1) (a),AU-3,AU-12 c,AU-12 a</t>
         </is>
       </c>
       <c r="B178" s="3" t="inlineStr">
@@ -14567,7 +14567,7 @@
     <row r="180" ht="130" customHeight="1">
       <c r="A180" s="3" t="inlineStr">
         <is>
-          <t>AU-3,AU-12 c,AU-12 a,AU-3 (1),MA-4 (1) (a)</t>
+          <t>AU-3 (1),MA-4 (1) (a),AU-3,AU-12 c,AU-12 a</t>
         </is>
       </c>
       <c r="B180" s="3" t="inlineStr">
@@ -14649,7 +14649,7 @@
     <row r="181" ht="130" customHeight="1">
       <c r="A181" s="3" t="inlineStr">
         <is>
-          <t>AU-3,AU-12 c,AU-12 a,AU-3 (1),MA-4 (1) (a)</t>
+          <t>AU-3 (1),MA-4 (1) (a),AU-3,AU-12 c,AU-12 a</t>
         </is>
       </c>
       <c r="B181" s="3" t="inlineStr">
@@ -14731,7 +14731,7 @@
     <row r="182" ht="130" customHeight="1">
       <c r="A182" s="3" t="inlineStr">
         <is>
-          <t>AU-3,AU-12 c,AU-12 a,AU-3 (1),MA-4 (1) (a)</t>
+          <t>AU-3 (1),MA-4 (1) (a),AU-3,AU-12 c,AU-12 a</t>
         </is>
       </c>
       <c r="B182" s="3" t="inlineStr">
@@ -14813,7 +14813,7 @@
     <row r="183" ht="130" customHeight="1">
       <c r="A183" s="3" t="inlineStr">
         <is>
-          <t>AU-3,AU-12 c,AU-12 a,AU-3 (1),MA-4 (1) (a)</t>
+          <t>AU-3 (1),MA-4 (1) (a),AU-3,AU-12 c,AU-12 a</t>
         </is>
       </c>
       <c r="B183" s="3" t="inlineStr">
@@ -14895,7 +14895,7 @@
     <row r="184" ht="130" customHeight="1">
       <c r="A184" s="3" t="inlineStr">
         <is>
-          <t>AU-3,AU-12 c,AU-12 a,AU-3 (1),MA-4 (1) (a)</t>
+          <t>AU-3 (1),MA-4 (1) (a),AU-3,AU-12 c,AU-12 a</t>
         </is>
       </c>
       <c r="B184" s="3" t="inlineStr">
@@ -15055,7 +15055,7 @@
     <row r="186" ht="130" customHeight="1">
       <c r="A186" s="3" t="inlineStr">
         <is>
-          <t>AU-3,AU-12 c,AU-12 a,AU-3 (1),MA-4 (1) (a)</t>
+          <t>AU-3 (1),MA-4 (1) (a),AU-3,AU-12 c,AU-12 a</t>
         </is>
       </c>
       <c r="B186" s="3" t="inlineStr">
@@ -15134,7 +15134,7 @@
     <row r="187" ht="130" customHeight="1">
       <c r="A187" s="3" t="inlineStr">
         <is>
-          <t>AU-3,AU-12 c,AU-12 a,AU-3 (1),MA-4 (1) (a)</t>
+          <t>AU-3 (1),MA-4 (1) (a),AU-3,AU-12 c,AU-12 a</t>
         </is>
       </c>
       <c r="B187" s="3" t="inlineStr">
@@ -15216,7 +15216,7 @@
     <row r="188" ht="130" customHeight="1">
       <c r="A188" s="3" t="inlineStr">
         <is>
-          <t>AU-3,AU-12 c,AU-12 a,AU-3 (1),MA-4 (1) (a)</t>
+          <t>AU-3 (1),MA-4 (1) (a),AU-3,AU-12 c,AU-12 a</t>
         </is>
       </c>
       <c r="B188" s="3" t="inlineStr">
@@ -15298,7 +15298,7 @@
     <row r="189" ht="130" customHeight="1">
       <c r="A189" s="3" t="inlineStr">
         <is>
-          <t>AU-3 (1),MA-4 (1) (a),AU-3,AU-12 c</t>
+          <t>AU-3 (1),MA-4 (1) (a),AU-12 c,AU-3</t>
         </is>
       </c>
       <c r="B189" s="3" t="inlineStr">
@@ -15380,7 +15380,7 @@
     <row r="190" ht="130" customHeight="1">
       <c r="A190" s="3" t="inlineStr">
         <is>
-          <t>AU-3,AU-12 c,AU-12 a,AU-3 (1),MA-4 (1) (a)</t>
+          <t>AU-3 (1),MA-4 (1) (a),AU-3,AU-12 c,AU-12 a</t>
         </is>
       </c>
       <c r="B190" s="3" t="inlineStr">
@@ -15462,7 +15462,7 @@
     <row r="191" ht="130" customHeight="1">
       <c r="A191" s="3" t="inlineStr">
         <is>
-          <t>AU-3,AU-12 c,AU-12 a,AU-3 (1),MA-4 (1) (a)</t>
+          <t>AU-3 (1),MA-4 (1) (a),AU-3,AU-12 c,AU-12 a</t>
         </is>
       </c>
       <c r="B191" s="3" t="inlineStr">
@@ -15544,7 +15544,7 @@
     <row r="192" ht="130" customHeight="1">
       <c r="A192" s="3" t="inlineStr">
         <is>
-          <t>AU-3,AU-12 c,AU-12 a,AU-3 (1),MA-4 (1) (a)</t>
+          <t>AU-3 (1),MA-4 (1) (a),AU-3,AU-12 c,AU-12 a</t>
         </is>
       </c>
       <c r="B192" s="3" t="inlineStr">
@@ -15626,7 +15626,7 @@
     <row r="193" ht="130" customHeight="1">
       <c r="A193" s="3" t="inlineStr">
         <is>
-          <t>AU-3,AU-12 c,AU-12 a,AU-3 (1),MA-4 (1) (a)</t>
+          <t>AU-3 (1),MA-4 (1) (a),AU-3,AU-12 c,AU-12 a</t>
         </is>
       </c>
       <c r="B193" s="3" t="inlineStr">
@@ -15701,7 +15701,7 @@
     <row r="194" ht="130" customHeight="1">
       <c r="A194" s="2" t="inlineStr">
         <is>
-          <t>IA-2 (2),IA-2 (4),IA-2 (3),IA-2 (1)</t>
+          <t>IA-2 (3),IA-2 (1),IA-2 (4),IA-2 (2)</t>
         </is>
       </c>
       <c r="B194" s="2" t="inlineStr">
@@ -15788,7 +15788,7 @@
     <row r="195" ht="130" customHeight="1">
       <c r="A195" s="2" t="inlineStr">
         <is>
-          <t>IA-2,IA-2 (2),IA-2 (4),IA-2 (3),IA-2 (5)</t>
+          <t>IA-2 (2),IA-2,IA-2 (3),IA-2 (5),IA-2 (4)</t>
         </is>
       </c>
       <c r="B195" s="2" t="inlineStr">
@@ -15877,7 +15877,7 @@
     <row r="196" ht="130" customHeight="1">
       <c r="A196" s="2" t="inlineStr">
         <is>
-          <t>IA-2,IA-2 (2),IA-2 (4),IA-2 (3),IA-2 (5)</t>
+          <t>IA-2 (2),IA-2,IA-2 (3),IA-2 (5),IA-2 (4)</t>
         </is>
       </c>
       <c r="B196" s="2" t="inlineStr">
@@ -16501,7 +16501,7 @@
     <row r="204" ht="130" customHeight="1">
       <c r="A204" s="2" t="inlineStr">
         <is>
-          <t>SC-8 (1),SC-8 (2),SC-8</t>
+          <t>SC-8,SC-8 (2),SC-8 (1)</t>
         </is>
       </c>
       <c r="B204" s="2" t="inlineStr">
@@ -16578,7 +16578,7 @@
     <row r="205" ht="130" customHeight="1">
       <c r="A205" s="2" t="inlineStr">
         <is>
-          <t>SC-8 (1),SC-8 (2),SC-8</t>
+          <t>SC-8,SC-8 (2),SC-8 (1)</t>
         </is>
       </c>
       <c r="B205" s="2" t="inlineStr">
@@ -16640,7 +16640,7 @@
           <t xml:space="preserve">
 Run the following command to determine the current status of the
  sshd  service:
- $ systemctl is-active sshd 
+ $ sudo systemctl is-active sshd 
 If the service is running, it should return the following:  active 
 If sshd service is disabled, then this is a finding.</t>
         </is>
@@ -16664,7 +16664,7 @@
     <row r="206" ht="130" customHeight="1">
       <c r="A206" s="2" t="inlineStr">
         <is>
-          <t>SC-8 (1),SC-8,AC-18 (1)</t>
+          <t>SC-8,SC-8 (1),AC-18 (1)</t>
         </is>
       </c>
       <c r="B206" s="2" t="inlineStr">
@@ -17092,7 +17092,7 @@
     <row r="211" ht="130" customHeight="1">
       <c r="A211" s="2" t="inlineStr">
         <is>
-          <t>CM-6 b,IA-5 (1) (c),CM-7 a</t>
+          <t>IA-5 (1) (c),CM-6 b,CM-7 a</t>
         </is>
       </c>
       <c r="B211" s="2" t="inlineStr">
@@ -17343,7 +17343,7 @@
     <row r="214" ht="130" customHeight="1">
       <c r="A214" s="2" t="inlineStr">
         <is>
-          <t>CM-6 b,SC-5,SC-5 (2)</t>
+          <t>SC-5,CM-6 b,SC-5 (2)</t>
         </is>
       </c>
       <c r="B214" s="2" t="inlineStr">
@@ -17523,7 +17523,7 @@
     <row r="216" ht="130" customHeight="1">
       <c r="A216" s="2" t="inlineStr">
         <is>
-          <t>SI-16,CM-7 a</t>
+          <t>CM-7 a,SI-16</t>
         </is>
       </c>
       <c r="B216" s="2" t="inlineStr">
@@ -18684,7 +18684,7 @@
     <row r="230" ht="130" customHeight="1">
       <c r="A230" s="2" t="inlineStr">
         <is>
-          <t>SC-2,CM-6 b,SI-16</t>
+          <t>CM-6 b,SI-16,SC-2</t>
         </is>
       </c>
       <c r="B230" s="2" t="inlineStr">
@@ -19597,7 +19597,7 @@
     <row r="241" ht="130" customHeight="1">
       <c r="A241" s="2" t="inlineStr">
         <is>
-          <t>CM-6 b,IA-5 (1) (b),IA-5 (1) (a)</t>
+          <t>CM-6 b,IA-5 (1) (a),IA-5 (1) (b)</t>
         </is>
       </c>
       <c r="B241" s="2" t="inlineStr">
@@ -20421,7 +20421,7 @@
     <row r="251" ht="130" customHeight="1">
       <c r="A251" s="2" t="inlineStr">
         <is>
-          <t>IA-2 (11),IA-2 (1)</t>
+          <t>IA-2 (1),IA-2 (11)</t>
         </is>
       </c>
       <c r="B251" s="2" t="inlineStr">
@@ -20737,7 +20737,7 @@
           <t xml:space="preserve">
 Run the following command to determine the current status of the
  pcscd  service:
- $ systemctl is-active pcscd 
+ $ sudo systemctl is-active pcscd 
 If the service is running, it should return the following:  active 
 If the pcscd service is not enabled, then this is a finding.</t>
         </is>
@@ -21003,7 +21003,7 @@
     <row r="258" ht="130" customHeight="1">
       <c r="A258" s="3" t="inlineStr">
         <is>
-          <t>CM-6 b,IA-2 (5)</t>
+          <t>IA-2 (5),CM-6 b</t>
         </is>
       </c>
       <c r="B258" s="3" t="inlineStr">
@@ -22238,7 +22238,7 @@
     <row r="273" ht="130" customHeight="1">
       <c r="A273" s="3" t="inlineStr">
         <is>
-          <t>CM-6 b,CM-7 a</t>
+          <t>CM-7 a,CM-6 b</t>
         </is>
       </c>
       <c r="B273" s="3" t="inlineStr">
@@ -23234,7 +23234,7 @@
     <row r="286" ht="130" customHeight="1">
       <c r="A286" s="3" t="inlineStr">
         <is>
-          <t>CM-6 b,CM-7 a</t>
+          <t>CM-7 a,CM-6 b</t>
         </is>
       </c>
       <c r="B286" s="3" t="inlineStr">
@@ -23305,7 +23305,7 @@
     <row r="287" ht="130" customHeight="1">
       <c r="A287" s="3" t="inlineStr">
         <is>
-          <t>CM-6 b,CM-7 a</t>
+          <t>CM-7 a,CM-6 b</t>
         </is>
       </c>
       <c r="B287" s="3" t="inlineStr">
@@ -23377,7 +23377,7 @@
     <row r="288" ht="130" customHeight="1">
       <c r="A288" s="3" t="inlineStr">
         <is>
-          <t>CM-6 b,CM-7 a</t>
+          <t>CM-7 a,CM-6 b</t>
         </is>
       </c>
       <c r="B288" s="3" t="inlineStr">
@@ -23619,7 +23619,7 @@
     <row r="291" ht="130" customHeight="1">
       <c r="A291" s="2" t="inlineStr">
         <is>
-          <t>AU-5 (1),AU-5 a</t>
+          <t>AU-5 a,AU-5 (1)</t>
         </is>
       </c>
       <c r="B291" s="2" t="inlineStr">
@@ -24113,17 +24113,17 @@
           <t xml:space="preserve">
 To check that the  kdump  service is disabled in system boot configuration,
 run the following command:
- $ systemctl is-enabled  kdump  
+ $ sudo systemctl is-enabled  kdump  
 Output should indicate the  kdump  service has either not been installed,
 or has been disabled at all runlevels, as shown in the example below:
- $ systemctl is-enabled  kdump 
+ $ sudo systemctl is-enabled  kdump 
  disabled 
 Run the following command to verify  kdump  is not active (i.e. not running) through current runtime configuration:
- $ systemctl is-active kdump 
+ $ sudo systemctl is-active kdump 
 If the service is not running the command will return the following output:
  inactive 
 The service will also be masked, to check that the  kdump  is masked, run the following command:
- $ systemctl show  kdump  | grep "LoadState\|UnitFileState" 
+ $ sudo systemctl show  kdump  | grep "LoadState\|UnitFileState" 
 If the service is masked the command will return the following outputs:
  LoadState=masked 
  UnitFileState=masked 
@@ -26448,7 +26448,7 @@
           <t xml:space="preserve">
 Run the following command to determine the current status of the
  rngd  service:
- $ systemctl is-active rngd 
+ $ sudo systemctl is-active rngd 
 If the service is running, it should return the following:  active 
 If the service is not enabled, then this is a finding.</t>
         </is>
@@ -26987,7 +26987,7 @@
     <row r="336" ht="130" customHeight="1">
       <c r="A336" s="3" t="inlineStr">
         <is>
-          <t>CM-6 b,IA-5 (1) (c)</t>
+          <t>IA-5 (1) (c),CM-6 b</t>
         </is>
       </c>
       <c r="B336" s="3" t="inlineStr">
@@ -30243,7 +30243,7 @@
           <t xml:space="preserve">
 Run the following command to determine the current status of the
  rsyslog  service:
- $ systemctl is-active rsyslog 
+ $ sudo systemctl is-active rsyslog 
 If the service is running, it should return the following:  active 
 If , then this is a finding.</t>
         </is>
@@ -30262,7 +30262,7 @@
     <row r="379" ht="130" customHeight="1">
       <c r="A379" s="2" t="inlineStr">
         <is>
-          <t>CM-6 b,AC-17 (9),CM-7 b,AC-17 (1)</t>
+          <t>CM-7 b,CM-6 b,AC-17 (1),AC-17 (9)</t>
         </is>
       </c>
       <c r="B379" s="2" t="inlineStr">
@@ -30340,7 +30340,7 @@
     <row r="380" ht="130" customHeight="1">
       <c r="A380" s="2" t="inlineStr">
         <is>
-          <t>CM-6 b,CM-7 b,AC-17 (1)</t>
+          <t>CM-7 b,CM-6 b,AC-17 (1)</t>
         </is>
       </c>
       <c r="B380" s="2" t="inlineStr">
@@ -30396,7 +30396,7 @@
           <t xml:space="preserve">
 Run the following command to determine the current status of the
  firewalld  service:
- $ systemctl is-active firewalld 
+ $ sudo systemctl is-active firewalld 
 If the service is running, it should return the following:  active 
 If the service is not enabled, then this is a finding.</t>
         </is>
@@ -32978,17 +32978,17 @@
           <t xml:space="preserve">
 To check that the  autofs  service is disabled in system boot configuration,
 run the following command:
- $ systemctl is-enabled  autofs  
+ $ sudo systemctl is-enabled  autofs  
 Output should indicate the  autofs  service has either not been installed,
 or has been disabled at all runlevels, as shown in the example below:
- $ systemctl is-enabled  autofs 
+ $ sudo systemctl is-enabled  autofs 
  disabled 
 Run the following command to verify  autofs  is not active (i.e. not running) through current runtime configuration:
- $ systemctl is-active autofs 
+ $ sudo systemctl is-active autofs 
 If the service is not running the command will return the following output:
  inactive 
 The service will also be masked, to check that the  autofs  is masked, run the following command:
- $ systemctl show  autofs  | grep "LoadState\|UnitFileState" 
+ $ sudo systemctl show  autofs  | grep "LoadState\|UnitFileState" 
 If the service is masked the command will return the following outputs:
  LoadState=masked 
  UnitFileState=masked 
@@ -33795,7 +33795,7 @@
     <row r="421" ht="130" customHeight="1">
       <c r="A421" s="3" t="inlineStr">
         <is>
-          <t>SC-2,CM-6 b</t>
+          <t>CM-6 b,SC-2</t>
         </is>
       </c>
       <c r="B421" s="3" t="inlineStr">
@@ -33882,7 +33882,7 @@
     <row r="422" ht="130" customHeight="1">
       <c r="A422" s="3" t="inlineStr">
         <is>
-          <t>SC-2,CM-6 b</t>
+          <t>CM-6 b,SC-2</t>
         </is>
       </c>
       <c r="B422" s="3" t="inlineStr">
@@ -35458,7 +35458,7 @@
     <row r="442" ht="130" customHeight="1">
       <c r="A442" s="3" t="inlineStr">
         <is>
-          <t>CM-6 b,SI-2 (2)</t>
+          <t>SI-2 (2),CM-6 b</t>
         </is>
       </c>
       <c r="B442" s="3" t="inlineStr">
@@ -36105,7 +36105,7 @@
     <row r="451" ht="130" customHeight="1">
       <c r="A451" s="3" t="inlineStr">
         <is>
-          <t>CM-6 b,SI-2 (2)</t>
+          <t>SI-2 (2),CM-6 b</t>
         </is>
       </c>
       <c r="B451" s="3" t="inlineStr">
@@ -36396,7 +36396,7 @@
     <row r="455" ht="130" customHeight="1">
       <c r="A455" s="3" t="inlineStr">
         <is>
-          <t>MA-4 (7),MA-4 e,SC-10,AC-12</t>
+          <t>SC-10,MA-4 e,AC-12,MA-4 (7)</t>
         </is>
       </c>
       <c r="B455" s="3" t="inlineStr">
@@ -36626,7 +36626,7 @@
     <row r="458" ht="130" customHeight="1">
       <c r="A458" s="3" t="inlineStr">
         <is>
-          <t>AC-11 a,SC-10</t>
+          <t>SC-10,AC-11 a</t>
         </is>
       </c>
       <c r="B458" s="3" t="inlineStr">
@@ -36703,7 +36703,7 @@
     <row r="459" ht="130" customHeight="1">
       <c r="A459" s="2" t="inlineStr">
         <is>
-          <t>SC-8 (1),AC-17 (2),SC-8</t>
+          <t>SC-8,SC-8 (1),AC-17 (2)</t>
         </is>
       </c>
       <c r="B459" s="2" t="inlineStr">
@@ -37921,7 +37921,7 @@
           <t xml:space="preserve">
 Run the following command to determine the current status of the
  usbguard  service:
- $ systemctl is-active usbguard 
+ $ sudo systemctl is-active usbguard 
 If the service is running, it should return the following:  active 
 If the service is not enabled, then this is a finding.</t>
         </is>
@@ -38010,7 +38010,7 @@
     <row r="476" ht="130" customHeight="1">
       <c r="A476" s="2" t="inlineStr">
         <is>
-          <t>IA-3,CM-7 b</t>
+          <t>CM-7 b,IA-3</t>
         </is>
       </c>
       <c r="B476" s="2" t="inlineStr">
@@ -39453,7 +39453,7 @@
     <row r="494" ht="130" customHeight="1">
       <c r="A494" s="2" t="inlineStr">
         <is>
-          <t>AU-4 (1),AU-4</t>
+          <t>AU-4,AU-4 (1)</t>
         </is>
       </c>
       <c r="B494" s="2" t="inlineStr">
@@ -39704,7 +39704,7 @@
     <row r="497" ht="130" customHeight="1">
       <c r="A497" s="2" t="inlineStr">
         <is>
-          <t>AC-8 a,AC-8 c 1, AC-8 c 2, AC-8 c 3</t>
+          <t>AC-8 c 1, AC-8 c 2, AC-8 c 3,AC-8 a</t>
         </is>
       </c>
       <c r="B497" s="2" t="inlineStr">
@@ -39806,7 +39806,7 @@
     <row r="498" ht="130" customHeight="1">
       <c r="A498" s="2" t="inlineStr">
         <is>
-          <t>AC-8 a,AC-8 c 1, AC-8 c 2, AC-8 c 3</t>
+          <t>AC-8 c 1, AC-8 c 2, AC-8 c 3,AC-8 a</t>
         </is>
       </c>
       <c r="B498" s="2" t="inlineStr">
@@ -39916,7 +39916,7 @@
     <row r="499" ht="130" customHeight="1">
       <c r="A499" s="2" t="inlineStr">
         <is>
-          <t>AC-8 a,AC-8 c 1, AC-8 c 2, AC-8 c 3</t>
+          <t>AC-8 c 1, AC-8 c 2, AC-8 c 3,AC-8 a</t>
         </is>
       </c>
       <c r="B499" s="2" t="inlineStr">
@@ -40027,7 +40027,7 @@
     <row r="500" ht="130" customHeight="1">
       <c r="A500" s="2" t="inlineStr">
         <is>
-          <t>AC-8 a,AC-8 c 1, AC-8 c 2, AC-8 c 3</t>
+          <t>AC-8 c 1, AC-8 c 2, AC-8 c 3,AC-8 a</t>
         </is>
       </c>
       <c r="B500" s="2" t="inlineStr">
@@ -40455,119 +40455,44 @@
       </c>
     </row>
     <row r="505" ht="130" customHeight="1">
-      <c r="A505" s="3" t="inlineStr">
-        <is>
-          <t>AU-9</t>
-        </is>
-      </c>
-      <c r="B505" s="3" t="inlineStr">
-        <is>
-          <t>CCI-000162,CCI-000163,CCI-000164,CCI-001314</t>
-        </is>
-      </c>
-      <c r="C505" s="3" t="inlineStr">
-        <is>
-          <t>SRG-OS-000057-GPOS-00027,SRG-OS-000058-GPOS-00028,SRG-OS-000059-GPOS-00029</t>
-        </is>
-      </c>
-      <c r="D505" s="3" t="inlineStr">
-        <is>
-          <t>CCE-83726-0</t>
-        </is>
-      </c>
-      <c r="E505" s="3" t="inlineStr">
-        <is>
-          <t>The operating system must protect audit information from unauthorized deletion.</t>
-        </is>
-      </c>
-      <c r="F505" s="3" t="inlineStr">
-        <is>
-          <t>Red Hat Enterprise Linux 9 Must Protect Audit Information From Unauthorized Deletion.</t>
-        </is>
-      </c>
-      <c r="G505" s="3" t="inlineStr">
-        <is>
-          <t>If audit information were to become compromised, then forensic analysis and discovery of the true source of potentially malicious system activity is impossible to achieve.
-To ensure the veracity of audit information, the operating system must protect audit information from unauthorized deletion. This requirement can be achieved through multiple methods, which will depend upon system architecture and design.
-Audit information includes all information (e.g., audit records, audit settings, audit reports) needed to successfully audit information system activity.</t>
-        </is>
-      </c>
-      <c r="H505" s="3" t="inlineStr">
-        <is>
-          <t>Unauthorized disclosure of audit records can reveal system and configuration data to
-attackers, thus compromising its confidentiality.</t>
-        </is>
-      </c>
-      <c r="I505" s="3" t="inlineStr">
-        <is>
-          <t>Applicable - Configurable</t>
-        </is>
-      </c>
-      <c r="J505" s="3" t="inlineStr">
-        <is>
-          <t>Verify the operating system protects audit information from unauthorized deletion. If it does not, this is a finding.</t>
-        </is>
-      </c>
-      <c r="K505" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">
-To properly set the owner of  /var/log/audit , run the command:
- $ sudo chown root /var/log/audit  
-To properly set the owner of  /var/log/audit/* , run the command:
- $ sudo chown root /var/log/audit/*  
-If , then this is a finding.</t>
-        </is>
-      </c>
-      <c r="L505" s="3" t="n"/>
-      <c r="M505" s="3" t="inlineStr"/>
-      <c r="N505" s="3" t="inlineStr">
-        <is>
-          <t>CAT II</t>
-        </is>
-      </c>
-      <c r="O505" s="3" t="n"/>
-      <c r="P505" s="3" t="n"/>
-      <c r="Q505" s="3" t="n"/>
-    </row>
-    <row r="506" ht="130" customHeight="1">
-      <c r="A506" s="2" t="inlineStr">
+      <c r="A505" s="2" t="inlineStr">
         <is>
           <t>IA-5 (1) (a)</t>
         </is>
       </c>
-      <c r="B506" s="2" t="inlineStr">
+      <c r="B505" s="2" t="inlineStr">
         <is>
           <t>CCI-001619</t>
         </is>
       </c>
-      <c r="C506" s="2" t="inlineStr">
+      <c r="C505" s="2" t="inlineStr">
         <is>
           <t>SRG-OS-000266-GPOS-00101</t>
         </is>
       </c>
-      <c r="D506" s="2" t="inlineStr">
+      <c r="D505" s="2" t="inlineStr">
         <is>
           <t>CCE-83565-2</t>
         </is>
       </c>
-      <c r="E506" s="2" t="inlineStr">
+      <c r="E505" s="2" t="inlineStr">
         <is>
           <t>The operating system must enforce password complexity by requiring that at least one special character be used.</t>
         </is>
       </c>
-      <c r="F506" s="2" t="inlineStr">
+      <c r="F505" s="2" t="inlineStr">
         <is>
           <t>Red Hat Enterprise Linux 9 Must Enforce Password Complexity By Requiring That At Least One Special Character Be Used.</t>
         </is>
       </c>
-      <c r="G506" s="2" t="inlineStr">
+      <c r="G505" s="2" t="inlineStr">
         <is>
           <t>Use of a complex password helps to increase the time and resources required to compromise the password. Password complexity or strength is a measure of the effectiveness of a password in resisting attempts at guessing and brute-force attacks.
 Password complexity is one factor in determining how long it takes to crack a password. The more complex the password, the greater the number of possible combinations that need to be tested before the password is compromised.
 Special characters are those characters that are not alphanumeric. Examples include: ~ ! @ # $ % ^ *.</t>
         </is>
       </c>
-      <c r="H506" s="2" t="inlineStr">
+      <c r="H505" s="2" t="inlineStr">
         <is>
           <t>Use of a complex password helps to increase the time and resources required
 to compromise the password. Password complexity, or strength, is a measure of
@@ -40580,17 +40505,17 @@
 more difficult by ensuring a larger search space.</t>
         </is>
       </c>
-      <c r="I506" s="2" t="inlineStr">
-        <is>
-          <t>Applicable - Configurable</t>
-        </is>
-      </c>
-      <c r="J506" s="2" t="inlineStr">
+      <c r="I505" s="2" t="inlineStr">
+        <is>
+          <t>Applicable - Configurable</t>
+        </is>
+      </c>
+      <c r="J505" s="2" t="inlineStr">
         <is>
           <t>Verify the operating system enforces password complexity by requiring that at least one special character be used. If it does not, this is a finding.</t>
         </is>
       </c>
-      <c r="K506" s="2" t="inlineStr">
+      <c r="K505" s="2" t="inlineStr">
         <is>
           <t>To check how many special characters are required in a password, run the following command:
  $ grep ocredit /etc/security/pwquality.conf 
@@ -40599,74 +40524,74 @@
 If value of "ocredit" is a positive number or is commented out, then this is a finding.</t>
         </is>
       </c>
-      <c r="L506" s="2" t="n"/>
-      <c r="M506" s="2" t="inlineStr">
+      <c r="L505" s="2" t="n"/>
+      <c r="M505" s="2" t="inlineStr">
         <is>
           <t>Add or modify the "ocredit" option line in /etc/security/pwquality.conf to have the required
 value, like in the following example:
 ocredit = -1</t>
         </is>
       </c>
-      <c r="N506" s="2" t="inlineStr">
-        <is>
-          <t>CAT II</t>
-        </is>
-      </c>
-      <c r="O506" s="2" t="n"/>
-      <c r="P506" s="2" t="n"/>
-      <c r="Q506" s="2" t="n"/>
-    </row>
-    <row r="507" ht="130" customHeight="1">
-      <c r="A507" s="3" t="inlineStr">
+      <c r="N505" s="2" t="inlineStr">
+        <is>
+          <t>CAT II</t>
+        </is>
+      </c>
+      <c r="O505" s="2" t="n"/>
+      <c r="P505" s="2" t="n"/>
+      <c r="Q505" s="2" t="n"/>
+    </row>
+    <row r="506" ht="130" customHeight="1">
+      <c r="A506" s="3" t="inlineStr">
         <is>
           <t>AU-4 (1)</t>
         </is>
       </c>
-      <c r="B507" s="3" t="inlineStr">
+      <c r="B506" s="3" t="inlineStr">
         <is>
           <t>CCI-001851</t>
         </is>
       </c>
-      <c r="C507" s="3" t="inlineStr">
+      <c r="C506" s="3" t="inlineStr">
         <is>
           <t>SRG-OS-000342-GPOS-00133,SRG-OS-000479-GPOS-00224</t>
         </is>
       </c>
-      <c r="D507" s="3" t="inlineStr"/>
-      <c r="E507" s="3" t="inlineStr">
+      <c r="D506" s="3" t="inlineStr"/>
+      <c r="E506" s="3" t="inlineStr">
         <is>
           <t>The operating system must off-load audit records onto a different system or media from the system being audited.</t>
         </is>
       </c>
-      <c r="F507" s="3" t="inlineStr">
+      <c r="F506" s="3" t="inlineStr">
         <is>
           <t>Red Hat Enterprise Linux 9 Must Off-Load Audit Records Onto A Different System Or Media From The System Being Audited.</t>
         </is>
       </c>
-      <c r="G507" s="3" t="inlineStr">
+      <c r="G506" s="3" t="inlineStr">
         <is>
           <t>Information stored in one location is vulnerable to accidental or incidental deletion or alteration.
 Off-loading is a common process in information systems with limited audit storage capacity.</t>
         </is>
       </c>
-      <c r="H507" s="3" t="inlineStr">
+      <c r="H506" s="3" t="inlineStr">
         <is>
           <t>Information stored in one location is vulnerable to accidental or incidental
 deletion or alteration.Off-loading is a common process in information systems
 with limited audit storage capacity.</t>
         </is>
       </c>
-      <c r="I507" s="3" t="inlineStr">
-        <is>
-          <t>Applicable - Configurable</t>
-        </is>
-      </c>
-      <c r="J507" s="3" t="inlineStr">
+      <c r="I506" s="3" t="inlineStr">
+        <is>
+          <t>Applicable - Configurable</t>
+        </is>
+      </c>
+      <c r="J506" s="3" t="inlineStr">
         <is>
           <t>Verify the operating system off-loads audit records onto a different system or media from the system being audited. If it does not, this is a finding.</t>
         </is>
       </c>
-      <c r="K507" s="3" t="inlineStr">
+      <c r="K506" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">
 To verify the audispd plugin off-loads audit records onto a different system or
@@ -40677,67 +40602,67 @@
 If audispd is not sending logs to a remote system, then this is a finding.</t>
         </is>
       </c>
-      <c r="L507" s="3" t="n"/>
-      <c r="M507" s="3" t="inlineStr"/>
-      <c r="N507" s="3" t="inlineStr">
-        <is>
-          <t>CAT II</t>
-        </is>
-      </c>
-      <c r="O507" s="3" t="n"/>
-      <c r="P507" s="3" t="n"/>
-      <c r="Q507" s="3" t="n"/>
-    </row>
-    <row r="508" ht="130" customHeight="1">
-      <c r="A508" s="3" t="inlineStr">
+      <c r="L506" s="3" t="n"/>
+      <c r="M506" s="3" t="inlineStr"/>
+      <c r="N506" s="3" t="inlineStr">
+        <is>
+          <t>CAT II</t>
+        </is>
+      </c>
+      <c r="O506" s="3" t="n"/>
+      <c r="P506" s="3" t="n"/>
+      <c r="Q506" s="3" t="n"/>
+    </row>
+    <row r="507" ht="130" customHeight="1">
+      <c r="A507" s="3" t="inlineStr">
         <is>
           <t>AU-4 (1)</t>
         </is>
       </c>
-      <c r="B508" s="3" t="inlineStr">
+      <c r="B507" s="3" t="inlineStr">
         <is>
           <t>CCI-001851</t>
         </is>
       </c>
-      <c r="C508" s="3" t="inlineStr">
+      <c r="C507" s="3" t="inlineStr">
         <is>
           <t>SRG-OS-000342-GPOS-00133,SRG-OS-000479-GPOS-00224</t>
         </is>
       </c>
-      <c r="D508" s="3" t="inlineStr"/>
-      <c r="E508" s="3" t="inlineStr">
+      <c r="D507" s="3" t="inlineStr"/>
+      <c r="E507" s="3" t="inlineStr">
         <is>
           <t>The operating system must off-load audit records onto a different system or media from the system being audited.</t>
         </is>
       </c>
-      <c r="F508" s="3" t="inlineStr">
+      <c r="F507" s="3" t="inlineStr">
         <is>
           <t>Red Hat Enterprise Linux 9 Must Off-Load Audit Records Onto A Different System Or Media From The System Being Audited.</t>
         </is>
       </c>
-      <c r="G508" s="3" t="inlineStr">
+      <c r="G507" s="3" t="inlineStr">
         <is>
           <t>Information stored in one location is vulnerable to accidental or incidental deletion or alteration.
 Off-loading is a common process in information systems with limited audit storage capacity.</t>
         </is>
       </c>
-      <c r="H508" s="3" t="inlineStr">
+      <c r="H507" s="3" t="inlineStr">
         <is>
           <t>Taking appropriate action in case of a filled audit storage volume will
 minimize the possibility of losing audit records.</t>
         </is>
       </c>
-      <c r="I508" s="3" t="inlineStr">
-        <is>
-          <t>Applicable - Configurable</t>
-        </is>
-      </c>
-      <c r="J508" s="3" t="inlineStr">
+      <c r="I507" s="3" t="inlineStr">
+        <is>
+          <t>Applicable - Configurable</t>
+        </is>
+      </c>
+      <c r="J507" s="3" t="inlineStr">
         <is>
           <t>Verify the operating system off-loads audit records onto a different system or media from the system being audited. If it does not, this is a finding.</t>
         </is>
       </c>
-      <c r="K508" s="3" t="inlineStr">
+      <c r="K507" s="3" t="inlineStr">
         <is>
           <t>Inspect "/etc/audisp/audisp-remote.conf" and locate the following line to
 determine if the system is configured to either send to syslog, switch to single user mode,
@@ -40750,68 +40675,68 @@
 If the system is not configured to switch to single user mode for corrective action, then this is a finding.</t>
         </is>
       </c>
-      <c r="L508" s="3" t="n"/>
-      <c r="M508" s="3" t="inlineStr"/>
-      <c r="N508" s="3" t="inlineStr">
-        <is>
-          <t>CAT II</t>
-        </is>
-      </c>
-      <c r="O508" s="3" t="n"/>
-      <c r="P508" s="3" t="n"/>
-      <c r="Q508" s="3" t="n"/>
-    </row>
-    <row r="509" ht="130" customHeight="1">
-      <c r="A509" s="3" t="inlineStr">
+      <c r="L507" s="3" t="n"/>
+      <c r="M507" s="3" t="inlineStr"/>
+      <c r="N507" s="3" t="inlineStr">
+        <is>
+          <t>CAT II</t>
+        </is>
+      </c>
+      <c r="O507" s="3" t="n"/>
+      <c r="P507" s="3" t="n"/>
+      <c r="Q507" s="3" t="n"/>
+    </row>
+    <row r="508" ht="130" customHeight="1">
+      <c r="A508" s="3" t="inlineStr">
         <is>
           <t>AU-4 (1)</t>
         </is>
       </c>
-      <c r="B509" s="3" t="inlineStr">
+      <c r="B508" s="3" t="inlineStr">
         <is>
           <t>CCI-001851</t>
         </is>
       </c>
-      <c r="C509" s="3" t="inlineStr">
+      <c r="C508" s="3" t="inlineStr">
         <is>
           <t>SRG-OS-000342-GPOS-00133,SRG-OS-000479-GPOS-00224</t>
         </is>
       </c>
-      <c r="D509" s="3" t="inlineStr"/>
-      <c r="E509" s="3" t="inlineStr">
+      <c r="D508" s="3" t="inlineStr"/>
+      <c r="E508" s="3" t="inlineStr">
         <is>
           <t>The operating system must off-load audit records onto a different system or media from the system being audited.</t>
         </is>
       </c>
-      <c r="F509" s="3" t="inlineStr">
+      <c r="F508" s="3" t="inlineStr">
         <is>
           <t>Red Hat Enterprise Linux 9 Must Off-Load Audit Records Onto A Different System Or Media From The System Being Audited.</t>
         </is>
       </c>
-      <c r="G509" s="3" t="inlineStr">
+      <c r="G508" s="3" t="inlineStr">
         <is>
           <t>Information stored in one location is vulnerable to accidental or incidental deletion or alteration.
 Off-loading is a common process in information systems with limited audit storage capacity.</t>
         </is>
       </c>
-      <c r="H509" s="3" t="inlineStr">
+      <c r="H508" s="3" t="inlineStr">
         <is>
           <t>Information stored in one location is vulnerable to accidental or incidental deletion
 or alteration. Off-loading is a common process in information systems with limited
 audit storage capacity.</t>
         </is>
       </c>
-      <c r="I509" s="3" t="inlineStr">
-        <is>
-          <t>Applicable - Configurable</t>
-        </is>
-      </c>
-      <c r="J509" s="3" t="inlineStr">
+      <c r="I508" s="3" t="inlineStr">
+        <is>
+          <t>Applicable - Configurable</t>
+        </is>
+      </c>
+      <c r="J508" s="3" t="inlineStr">
         <is>
           <t>Verify the operating system off-loads audit records onto a different system or media from the system being audited. If it does not, this is a finding.</t>
         </is>
       </c>
-      <c r="K509" s="3" t="inlineStr">
+      <c r="K508" s="3" t="inlineStr">
         <is>
           <t>To verify the audispd plugin encrypts audit records off-loaded onto a different
 system or media from the system being audited, run the following command:
@@ -40821,67 +40746,67 @@
 If audispd is not encrypting audit records when sent over the network, then this is a finding.</t>
         </is>
       </c>
-      <c r="L509" s="3" t="n"/>
-      <c r="M509" s="3" t="inlineStr"/>
-      <c r="N509" s="3" t="inlineStr">
-        <is>
-          <t>CAT II</t>
-        </is>
-      </c>
-      <c r="O509" s="3" t="n"/>
-      <c r="P509" s="3" t="n"/>
-      <c r="Q509" s="3" t="n"/>
-    </row>
-    <row r="510" ht="130" customHeight="1">
-      <c r="A510" s="3" t="inlineStr">
+      <c r="L508" s="3" t="n"/>
+      <c r="M508" s="3" t="inlineStr"/>
+      <c r="N508" s="3" t="inlineStr">
+        <is>
+          <t>CAT II</t>
+        </is>
+      </c>
+      <c r="O508" s="3" t="n"/>
+      <c r="P508" s="3" t="n"/>
+      <c r="Q508" s="3" t="n"/>
+    </row>
+    <row r="509" ht="130" customHeight="1">
+      <c r="A509" s="3" t="inlineStr">
         <is>
           <t>AU-4 (1)</t>
         </is>
       </c>
-      <c r="B510" s="3" t="inlineStr">
+      <c r="B509" s="3" t="inlineStr">
         <is>
           <t>CCI-001851</t>
         </is>
       </c>
-      <c r="C510" s="3" t="inlineStr">
+      <c r="C509" s="3" t="inlineStr">
         <is>
           <t>SRG-OS-000342-GPOS-00133,SRG-OS-000479-GPOS-00224</t>
         </is>
       </c>
-      <c r="D510" s="3" t="inlineStr"/>
-      <c r="E510" s="3" t="inlineStr">
+      <c r="D509" s="3" t="inlineStr"/>
+      <c r="E509" s="3" t="inlineStr">
         <is>
           <t>The operating system must off-load audit records onto a different system or media from the system being audited.</t>
         </is>
       </c>
-      <c r="F510" s="3" t="inlineStr">
+      <c r="F509" s="3" t="inlineStr">
         <is>
           <t>Red Hat Enterprise Linux 9 Must Off-Load Audit Records Onto A Different System Or Media From The System Being Audited.</t>
         </is>
       </c>
-      <c r="G510" s="3" t="inlineStr">
+      <c r="G509" s="3" t="inlineStr">
         <is>
           <t>Information stored in one location is vulnerable to accidental or incidental deletion or alteration.
 Off-loading is a common process in information systems with limited audit storage capacity.</t>
         </is>
       </c>
-      <c r="H510" s="3" t="inlineStr">
+      <c r="H509" s="3" t="inlineStr">
         <is>
           <t>Taking appropriate action when there is an error sending audit records to a
 remote system will minimize the possibility of losing audit records.</t>
         </is>
       </c>
-      <c r="I510" s="3" t="inlineStr">
-        <is>
-          <t>Applicable - Configurable</t>
-        </is>
-      </c>
-      <c r="J510" s="3" t="inlineStr">
+      <c r="I509" s="3" t="inlineStr">
+        <is>
+          <t>Applicable - Configurable</t>
+        </is>
+      </c>
+      <c r="J509" s="3" t="inlineStr">
         <is>
           <t>Verify the operating system off-loads audit records onto a different system or media from the system being audited. If it does not, this is a finding.</t>
         </is>
       </c>
-      <c r="K510" s="3" t="inlineStr">
+      <c r="K509" s="3" t="inlineStr">
         <is>
           <t>Inspect "/etc/audisp/audisp-remote.conf" and locate the following line to
 determine if the system is configured to perform a correct action according to the policy:
@@ -40891,55 +40816,55 @@
 If the system is not configured to switch to single user mode for corrective action, then this is a finding.</t>
         </is>
       </c>
-      <c r="L510" s="3" t="n"/>
-      <c r="M510" s="3" t="inlineStr"/>
-      <c r="N510" s="3" t="inlineStr">
-        <is>
-          <t>CAT II</t>
-        </is>
-      </c>
-      <c r="O510" s="3" t="n"/>
-      <c r="P510" s="3" t="n"/>
-      <c r="Q510" s="3" t="n"/>
-    </row>
-    <row r="511" ht="130" customHeight="1">
-      <c r="A511" s="3" t="inlineStr">
+      <c r="L509" s="3" t="n"/>
+      <c r="M509" s="3" t="inlineStr"/>
+      <c r="N509" s="3" t="inlineStr">
+        <is>
+          <t>CAT II</t>
+        </is>
+      </c>
+      <c r="O509" s="3" t="n"/>
+      <c r="P509" s="3" t="n"/>
+      <c r="Q509" s="3" t="n"/>
+    </row>
+    <row r="510" ht="130" customHeight="1">
+      <c r="A510" s="3" t="inlineStr">
         <is>
           <t>AU-4 (1)</t>
         </is>
       </c>
-      <c r="B511" s="3" t="inlineStr">
+      <c r="B510" s="3" t="inlineStr">
         <is>
           <t>CCI-000136</t>
         </is>
       </c>
-      <c r="C511" s="3" t="inlineStr">
+      <c r="C510" s="3" t="inlineStr">
         <is>
           <t>SRG-OS-000479-GPOS-00224,SRG-OS-000342-GPOS-00133</t>
         </is>
       </c>
-      <c r="D511" s="3" t="inlineStr">
+      <c r="D510" s="3" t="inlineStr">
         <is>
           <t>CCE-83695-7</t>
         </is>
       </c>
-      <c r="E511" s="3" t="inlineStr">
+      <c r="E510" s="3" t="inlineStr">
         <is>
           <t>The operating system must off-load audit records onto a different system or media from the system being audited.</t>
         </is>
       </c>
-      <c r="F511" s="3" t="inlineStr">
+      <c r="F510" s="3" t="inlineStr">
         <is>
           <t>Red Hat Enterprise Linux 9 Must Off-Load Audit Records Onto A Different System Or Media From The System Being Audited.</t>
         </is>
       </c>
-      <c r="G511" s="3" t="inlineStr">
+      <c r="G510" s="3" t="inlineStr">
         <is>
           <t>Information stored in one location is vulnerable to accidental or incidental deletion or alteration.
 Off-loading is a common process in information systems with limited audit storage capacity.</t>
         </is>
       </c>
-      <c r="H511" s="3" t="inlineStr">
+      <c r="H510" s="3" t="inlineStr">
         <is>
           <t>The auditd service does not include the ability to send audit
 records to a centralized server for management directly. It does, however,
@@ -40947,17 +40872,17 @@
 to the local syslog server</t>
         </is>
       </c>
-      <c r="I511" s="3" t="inlineStr">
-        <is>
-          <t>Applicable - Configurable</t>
-        </is>
-      </c>
-      <c r="J511" s="3" t="inlineStr">
+      <c r="I510" s="3" t="inlineStr">
+        <is>
+          <t>Applicable - Configurable</t>
+        </is>
+      </c>
+      <c r="J510" s="3" t="inlineStr">
         <is>
           <t>Verify the operating system off-loads audit records onto a different system or media from the system being audited. If it does not, this is a finding.</t>
         </is>
       </c>
-      <c r="K511" s="3" t="inlineStr">
+      <c r="K510" s="3" t="inlineStr">
         <is>
           <t>To verify the audispd's syslog plugin is active, run the following command:
  $ sudo grep active /etc/audit/plugins.d/syslog.conf 
@@ -40965,6 +40890,77 @@
 If it is not activated, then this is a finding.</t>
         </is>
       </c>
+      <c r="L510" s="3" t="n"/>
+      <c r="M510" s="3" t="inlineStr"/>
+      <c r="N510" s="3" t="inlineStr">
+        <is>
+          <t>CAT II</t>
+        </is>
+      </c>
+      <c r="O510" s="3" t="n"/>
+      <c r="P510" s="3" t="n"/>
+      <c r="Q510" s="3" t="n"/>
+    </row>
+    <row r="511" ht="130" customHeight="1">
+      <c r="A511" s="3" t="inlineStr">
+        <is>
+          <t>AU-4 (1)</t>
+        </is>
+      </c>
+      <c r="B511" s="3" t="inlineStr">
+        <is>
+          <t>CCI-001851</t>
+        </is>
+      </c>
+      <c r="C511" s="3" t="inlineStr">
+        <is>
+          <t>SRG-OS-000342-GPOS-00133</t>
+        </is>
+      </c>
+      <c r="D511" s="3" t="inlineStr">
+        <is>
+          <t>CCE-83648-6</t>
+        </is>
+      </c>
+      <c r="E511" s="3" t="inlineStr">
+        <is>
+          <t>The operating system must off-load audit records onto a different system or media from the system being audited.</t>
+        </is>
+      </c>
+      <c r="F511" s="3" t="inlineStr">
+        <is>
+          <t>Red Hat Enterprise Linux 9 Must Off-Load Audit Records Onto A Different System Or Media From The System Being Audited.</t>
+        </is>
+      </c>
+      <c r="G511" s="3" t="inlineStr">
+        <is>
+          <t>Information stored in one location is vulnerable to accidental or incidental deletion or alteration.
+Off-loading is a common process in information systems with limited audit storage capacity.</t>
+        </is>
+      </c>
+      <c r="H511" s="3" t="inlineStr">
+        <is>
+          <t>"audispd-plugins" provides plugins for the real-time interface to the
+audit subsystem, "audispd". These plugins can do things like relay events
+to remote machines or analyze events for suspicious behavior.</t>
+        </is>
+      </c>
+      <c r="I511" s="3" t="inlineStr">
+        <is>
+          <t>Applicable - Configurable</t>
+        </is>
+      </c>
+      <c r="J511" s="3" t="inlineStr">
+        <is>
+          <t>Verify the operating system off-loads audit records onto a different system or media from the system being audited. If it does not, this is a finding.</t>
+        </is>
+      </c>
+      <c r="K511" s="3" t="inlineStr">
+        <is>
+          <t>Run the following command to determine if the  audispd-plugins  package is installed:  $ rpm -q audispd-plugins 
+If the package is not installed, then this is a finding.</t>
+        </is>
+      </c>
       <c r="L511" s="3" t="n"/>
       <c r="M511" s="3" t="inlineStr"/>
       <c r="N511" s="3" t="inlineStr">
@@ -40992,11 +40988,7 @@
           <t>SRG-OS-000342-GPOS-00133</t>
         </is>
       </c>
-      <c r="D512" s="3" t="inlineStr">
-        <is>
-          <t>CCE-83648-6</t>
-        </is>
-      </c>
+      <c r="D512" s="3" t="inlineStr"/>
       <c r="E512" s="3" t="inlineStr">
         <is>
           <t>The operating system must off-load audit records onto a different system or media from the system being audited.</t>
@@ -41015,9 +41007,7 @@
       </c>
       <c r="H512" s="3" t="inlineStr">
         <is>
-          <t>"audispd-plugins" provides plugins for the real-time interface to the
-audit subsystem, "audispd". These plugins can do things like relay events
-to remote machines or analyze events for suspicious behavior.</t>
+          <t>Information stored in one location is vulnerable to accidental or incidental deletion or alteration. Off-loading is a common process in information systems with limited audit storage capacity.</t>
         </is>
       </c>
       <c r="I512" s="3" t="inlineStr">
@@ -41032,7 +41022,7 @@
       </c>
       <c r="K512" s="3" t="inlineStr">
         <is>
-          <t>Run the following command to determine if the  audispd-plugins  package is installed:  $ rpm -q audispd-plugins 
+          <t xml:space="preserve">
 If the package is not installed, then this is a finding.</t>
         </is>
       </c>
@@ -41050,41 +41040,37 @@
     <row r="513" ht="130" customHeight="1">
       <c r="A513" s="3" t="inlineStr">
         <is>
-          <t>AU-4 (1)</t>
+          <t>AC-3 (4)</t>
         </is>
       </c>
       <c r="B513" s="3" t="inlineStr">
         <is>
-          <t>CCI-001851</t>
+          <t>CCI-002165</t>
         </is>
       </c>
       <c r="C513" s="3" t="inlineStr">
         <is>
-          <t>SRG-OS-000342-GPOS-00133</t>
+          <t>SRG-OS-000312-GPOS-00124</t>
         </is>
       </c>
       <c r="D513" s="3" t="inlineStr"/>
       <c r="E513" s="3" t="inlineStr">
         <is>
-          <t>The operating system must off-load audit records onto a different system or media from the system being audited.</t>
+          <t>The operating system must allow operating system admins to change security attributes on users, the operating system, or the operating systems components.</t>
         </is>
       </c>
       <c r="F513" s="3" t="inlineStr">
         <is>
-          <t>Red Hat Enterprise Linux 9 Must Off-Load Audit Records Onto A Different System Or Media From The System Being Audited.</t>
+          <t>Red Hat Enterprise Linux 9 must allow operating system admins to change security attributes on users, the operating system, or the operating systems components.</t>
         </is>
       </c>
       <c r="G513" s="3" t="inlineStr">
         <is>
-          <t>Information stored in one location is vulnerable to accidental or incidental deletion or alteration.
-Off-loading is a common process in information systems with limited audit storage capacity.</t>
-        </is>
-      </c>
-      <c r="H513" s="3" t="inlineStr">
-        <is>
-          <t>Information stored in one location is vulnerable to accidental or incidental deletion or alteration. Off-loading is a common process in information systems with limited audit storage capacity.</t>
-        </is>
-      </c>
+          <t>Discretionary Access Control (DAC) is based on the notion that individual users are "owners" of objects and therefore have discretion over who should be authorized to access the object and in which mode (e.g., read or write). Ownership is usually acquired as a consequence of creating the object or via specified ownership assignment. DAC allows the owner to determine who will have access to objects they control. An example of DAC includes user-controlled file permissions.
+When discretionary access control policies are implemented, subjects are not constrained with regard to what actions they can take with information for which they have already been granted access. Thus, subjects that have been granted access to information are not prevented from passing (i.e., the subjects have the discretion to pass) the information to other subjects or objects. A subject that is constrained in its operation by Mandatory Access Control policies is still able to operate under the less rigorous constraints of this requirement. Thus, while Mandatory Access Control imposes constraints preventing a subject from passing information to another subject operating at a different sensitivity level, this requirement permits the subject to pass the information to any subject at the same sensitivity level. The policy is bounded by the information system boundary. Once the information is passed outside the control of the information system, additional means may be required to ensure the constraints remain in effect. While the older, more traditional definitions of discretionary access control require identity-based access control, that limitation is not required for this use of discretionary access control.</t>
+        </is>
+      </c>
+      <c r="H513" s="3" t="inlineStr"/>
       <c r="I513" s="3" t="inlineStr">
         <is>
           <t>Applicable - Configurable</t>
@@ -41092,17 +41078,12 @@
       </c>
       <c r="J513" s="3" t="inlineStr">
         <is>
-          <t>Verify the operating system off-loads audit records onto a different system or media from the system being audited. If it does not, this is a finding.</t>
-        </is>
-      </c>
-      <c r="K513" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">
-If the package is not installed, then this is a finding.</t>
-        </is>
-      </c>
+          <t>Verify the operating system allows operating system admins to change security attributes on users, the operating system, or the operating system's components. If it does not, this is a finding.</t>
+        </is>
+      </c>
+      <c r="K513" s="3" t="n"/>
       <c r="L513" s="3" t="n"/>
-      <c r="M513" s="3" t="inlineStr"/>
+      <c r="M513" s="3" t="n"/>
       <c r="N513" s="3" t="inlineStr">
         <is>
           <t>CAT II</t>
@@ -41113,116 +41094,60 @@
       <c r="Q513" s="3" t="n"/>
     </row>
     <row r="514" ht="130" customHeight="1">
-      <c r="A514" s="3" t="inlineStr">
-        <is>
-          <t>AC-3 (4)</t>
-        </is>
-      </c>
-      <c r="B514" s="3" t="inlineStr">
-        <is>
-          <t>CCI-002165</t>
-        </is>
-      </c>
-      <c r="C514" s="3" t="inlineStr">
-        <is>
-          <t>SRG-OS-000312-GPOS-00124</t>
-        </is>
-      </c>
-      <c r="D514" s="3" t="inlineStr"/>
-      <c r="E514" s="3" t="inlineStr">
-        <is>
-          <t>The operating system must allow operating system admins to change security attributes on users, the operating system, or the operating systems components.</t>
-        </is>
-      </c>
-      <c r="F514" s="3" t="inlineStr">
-        <is>
-          <t>Red Hat Enterprise Linux 9 must allow operating system admins to change security attributes on users, the operating system, or the operating systems components.</t>
-        </is>
-      </c>
-      <c r="G514" s="3" t="inlineStr">
-        <is>
-          <t>Discretionary Access Control (DAC) is based on the notion that individual users are "owners" of objects and therefore have discretion over who should be authorized to access the object and in which mode (e.g., read or write). Ownership is usually acquired as a consequence of creating the object or via specified ownership assignment. DAC allows the owner to determine who will have access to objects they control. An example of DAC includes user-controlled file permissions.
-When discretionary access control policies are implemented, subjects are not constrained with regard to what actions they can take with information for which they have already been granted access. Thus, subjects that have been granted access to information are not prevented from passing (i.e., the subjects have the discretion to pass) the information to other subjects or objects. A subject that is constrained in its operation by Mandatory Access Control policies is still able to operate under the less rigorous constraints of this requirement. Thus, while Mandatory Access Control imposes constraints preventing a subject from passing information to another subject operating at a different sensitivity level, this requirement permits the subject to pass the information to any subject at the same sensitivity level. The policy is bounded by the information system boundary. Once the information is passed outside the control of the information system, additional means may be required to ensure the constraints remain in effect. While the older, more traditional definitions of discretionary access control require identity-based access control, that limitation is not required for this use of discretionary access control.</t>
-        </is>
-      </c>
-      <c r="H514" s="3" t="inlineStr"/>
-      <c r="I514" s="3" t="inlineStr">
-        <is>
-          <t>Applicable - Configurable</t>
-        </is>
-      </c>
-      <c r="J514" s="3" t="inlineStr">
-        <is>
-          <t>Verify the operating system allows operating system admins to change security attributes on users, the operating system, or the operating system's components. If it does not, this is a finding.</t>
-        </is>
-      </c>
-      <c r="K514" s="3" t="n"/>
-      <c r="L514" s="3" t="n"/>
-      <c r="M514" s="3" t="n"/>
-      <c r="N514" s="3" t="inlineStr">
-        <is>
-          <t>CAT II</t>
-        </is>
-      </c>
-      <c r="O514" s="3" t="n"/>
-      <c r="P514" s="3" t="n"/>
-      <c r="Q514" s="3" t="n"/>
-    </row>
-    <row r="515" ht="130" customHeight="1">
-      <c r="A515" s="2" t="inlineStr">
-        <is>
-          <t>SC-8 (2),SC-8</t>
-        </is>
-      </c>
-      <c r="B515" s="2" t="inlineStr">
+      <c r="A514" s="2" t="inlineStr">
+        <is>
+          <t>SC-8,SC-8 (2)</t>
+        </is>
+      </c>
+      <c r="B514" s="2" t="inlineStr">
         <is>
           <t>CCI-002422</t>
         </is>
       </c>
-      <c r="C515" s="2" t="inlineStr">
+      <c r="C514" s="2" t="inlineStr">
         <is>
           <t>SRG-OS-000423-GPOS-00187,SRG-OS-000426-GPOS-00190</t>
         </is>
       </c>
-      <c r="D515" s="2" t="inlineStr">
+      <c r="D514" s="2" t="inlineStr">
         <is>
           <t>CCE-83451-5</t>
         </is>
       </c>
-      <c r="E515" s="2" t="inlineStr">
+      <c r="E514" s="2" t="inlineStr">
         <is>
           <t>The operating system must maintain the confidentiality and integrity of information during reception.</t>
         </is>
       </c>
-      <c r="F515" s="2" t="inlineStr">
+      <c r="F514" s="2" t="inlineStr">
         <is>
           <t>Red Hat Enterprise Linux 9 Must Maintain The Confidentiality And Integrity Of Information During Reception.</t>
         </is>
       </c>
-      <c r="G515" s="2" t="inlineStr">
+      <c r="G514" s="2" t="inlineStr">
         <is>
           <t>Information can be either unintentionally or maliciously disclosed or modified during reception, including, for example, during aggregation, at protocol transformation points, and during packing/unpacking. These unauthorized disclosures or modifications compromise the confidentiality or integrity of the information.
 Ensuring the confidentiality of transmitted information requires the operating system to take measures in preparing information for transmission. This can be accomplished via access control and encryption.
 Use of this requirement will be limited to situations where the data owner has a strict requirement for ensuring data integrity and confidentiality is maintained at every step of the data transfer and handling process. When receiving data, operating systems need to leverage protection mechanisms such as TLS, SSL VPNs, or IPSec.</t>
         </is>
       </c>
-      <c r="H515" s="2" t="inlineStr">
+      <c r="H514" s="2" t="inlineStr">
         <is>
           <t>Overriding the system crypto policy makes the behavior of the BIND service violate expectations,
 and makes system configuration more fragmented.</t>
         </is>
       </c>
-      <c r="I515" s="2" t="inlineStr">
-        <is>
-          <t>Applicable - Configurable</t>
-        </is>
-      </c>
-      <c r="J515" s="2" t="inlineStr">
+      <c r="I514" s="2" t="inlineStr">
+        <is>
+          <t>Applicable - Configurable</t>
+        </is>
+      </c>
+      <c r="J514" s="2" t="inlineStr">
         <is>
           <t>Verify the operating system maintains the confidentiality and integrity of information during reception. If it does not, this is a finding.</t>
         </is>
       </c>
-      <c r="K515" s="2" t="inlineStr">
+      <c r="K514" s="2" t="inlineStr">
         <is>
           <t>To verify that BIND uses the system crypto policy, check out that the BIND config file
  /etc/named.conf  contains the  include "/etc/crypto-policies/back-ends/bind.config"; 
@@ -41233,60 +41158,60 @@
  include "/etc/crypto-policies/back-ends/bind.config";  directive, then this is a finding.</t>
         </is>
       </c>
-      <c r="L515" s="2" t="n"/>
-      <c r="M515" s="2" t="inlineStr">
+      <c r="L514" s="2" t="n"/>
+      <c r="M514" s="2" t="inlineStr">
         <is>
           <t>Configure BIND to use the system crypto policy.
 Add the following line to the "options" section in "/etc/named.conf":
 include "/etc/crypto-policies/back-ends/bind.config";</t>
         </is>
       </c>
-      <c r="N515" s="2" t="inlineStr">
-        <is>
-          <t>CAT II</t>
-        </is>
-      </c>
-      <c r="O515" s="2" t="n"/>
-      <c r="P515" s="2" t="n"/>
-      <c r="Q515" s="2" t="n"/>
-    </row>
-    <row r="516" ht="130" customHeight="1">
-      <c r="A516" s="2" t="inlineStr">
+      <c r="N514" s="2" t="inlineStr">
+        <is>
+          <t>CAT II</t>
+        </is>
+      </c>
+      <c r="O514" s="2" t="n"/>
+      <c r="P514" s="2" t="n"/>
+      <c r="Q514" s="2" t="n"/>
+    </row>
+    <row r="515" ht="130" customHeight="1">
+      <c r="A515" s="2" t="inlineStr">
         <is>
           <t>IA-5 (1) (d)</t>
         </is>
       </c>
-      <c r="B516" s="2" t="inlineStr">
+      <c r="B515" s="2" t="inlineStr">
         <is>
           <t>CCI-000199</t>
         </is>
       </c>
-      <c r="C516" s="2" t="inlineStr">
+      <c r="C515" s="2" t="inlineStr">
         <is>
           <t>SRG-OS-000076-GPOS-00044</t>
         </is>
       </c>
-      <c r="D516" s="2" t="inlineStr">
+      <c r="D515" s="2" t="inlineStr">
         <is>
           <t>CCE-83606-4</t>
         </is>
       </c>
-      <c r="E516" s="2" t="inlineStr">
+      <c r="E515" s="2" t="inlineStr">
         <is>
           <t>Operating systems must enforce a 60-day maximum password lifetime restriction.</t>
         </is>
       </c>
-      <c r="F516" s="2" t="inlineStr">
+      <c r="F515" s="2" t="inlineStr">
         <is>
           <t>Red Hat Enterprise Linux 9 user account passwords for new users or password changes must have a 60 day maximum password lifetime restriction in /etc/login.defs.</t>
         </is>
       </c>
-      <c r="G516" s="2" t="inlineStr">
+      <c r="G515" s="2" t="inlineStr">
         <is>
           <t>Any password, no matter how complex, can eventually be cracked. Therefore, passwords need to be changed periodically. If the operating system does not limit the lifetime of passwords and force users to change their passwords, there is the risk that the operating system passwords could be compromised.</t>
         </is>
       </c>
-      <c r="H516" s="2" t="inlineStr">
+      <c r="H515" s="2" t="inlineStr">
         <is>
           <t>Any password, no matter how complex, can eventually be cracked. Therefore, passwords
 need to be changed periodically. If the operating system does not limit the lifetime
@@ -41298,17 +41223,17 @@
 location subject to physical compromise.</t>
         </is>
       </c>
-      <c r="I516" s="2" t="inlineStr">
-        <is>
-          <t>Applicable - Configurable</t>
-        </is>
-      </c>
-      <c r="J516" s="2" t="inlineStr">
+      <c r="I515" s="2" t="inlineStr">
+        <is>
+          <t>Applicable - Configurable</t>
+        </is>
+      </c>
+      <c r="J515" s="2" t="inlineStr">
         <is>
           <t>Verify operating system enforces a 60-day maximum password lifetime restriction. If it does not, this is a finding.</t>
         </is>
       </c>
-      <c r="K516" s="2" t="inlineStr">
+      <c r="K515" s="2" t="inlineStr">
         <is>
           <t>To check the maximum password age, run the command:
  $ grep PASS_MAX_DAYS /etc/login.defs 
@@ -41316,60 +41241,60 @@
 If PASS_MAX_DAYS is not set equal to or greater than the required value, then this is a finding.</t>
         </is>
       </c>
-      <c r="L516" s="2" t="n"/>
-      <c r="M516" s="2" t="inlineStr">
+      <c r="L515" s="2" t="n"/>
+      <c r="M515" s="2" t="inlineStr">
         <is>
           <t>Configure Red Hat Enterprise Linux 9 to enforce a 60-day maximum password lifetime.
 Add, or modify the following line in the ""/etc/login.defs"" file:
 PASS_MAX_DAYS 60</t>
         </is>
       </c>
-      <c r="N516" s="2" t="inlineStr">
-        <is>
-          <t>CAT II</t>
-        </is>
-      </c>
-      <c r="O516" s="2" t="n"/>
-      <c r="P516" s="2" t="n"/>
-      <c r="Q516" s="2" t="n"/>
-    </row>
-    <row r="517" ht="130" customHeight="1">
-      <c r="A517" s="2" t="inlineStr">
+      <c r="N515" s="2" t="inlineStr">
+        <is>
+          <t>CAT II</t>
+        </is>
+      </c>
+      <c r="O515" s="2" t="n"/>
+      <c r="P515" s="2" t="n"/>
+      <c r="Q515" s="2" t="n"/>
+    </row>
+    <row r="516" ht="130" customHeight="1">
+      <c r="A516" s="2" t="inlineStr">
         <is>
           <t>IA-5 (1) (d)</t>
         </is>
       </c>
-      <c r="B517" s="2" t="inlineStr">
+      <c r="B516" s="2" t="inlineStr">
         <is>
           <t>CCI-000199</t>
         </is>
       </c>
-      <c r="C517" s="2" t="inlineStr">
+      <c r="C516" s="2" t="inlineStr">
         <is>
           <t>SRG-OS-000076-GPOS-00044</t>
         </is>
       </c>
-      <c r="D517" s="2" t="inlineStr">
+      <c r="D516" s="2" t="inlineStr">
         <is>
           <t>CCE-86031-2</t>
         </is>
       </c>
-      <c r="E517" s="2" t="inlineStr">
+      <c r="E516" s="2" t="inlineStr">
         <is>
           <t>Operating systems must enforce a 60-day maximum password lifetime restriction.</t>
         </is>
       </c>
-      <c r="F517" s="2" t="inlineStr">
+      <c r="F516" s="2" t="inlineStr">
         <is>
           <t>Red Hat Enterprise Linux 9 user account passwords must have a 60-day maximum password lifetime restriction.</t>
         </is>
       </c>
-      <c r="G517" s="2" t="inlineStr">
+      <c r="G516" s="2" t="inlineStr">
         <is>
           <t>Any password, no matter how complex, can eventually be cracked. Therefore, passwords need to be changed periodically. If the operating system does not limit the lifetime of passwords and force users to change their passwords, there is the risk that the operating system passwords could be compromised.</t>
         </is>
       </c>
-      <c r="H517" s="2" t="inlineStr">
+      <c r="H516" s="2" t="inlineStr">
         <is>
           <t>Any password, no matter how complex, can eventually be cracked. Therefore,
 passwords need to be changed periodically. If the operating system does
@@ -41378,17 +41303,17 @@
 compromised.</t>
         </is>
       </c>
-      <c r="I517" s="2" t="inlineStr">
-        <is>
-          <t>Applicable - Configurable</t>
-        </is>
-      </c>
-      <c r="J517" s="2" t="inlineStr">
+      <c r="I516" s="2" t="inlineStr">
+        <is>
+          <t>Applicable - Configurable</t>
+        </is>
+      </c>
+      <c r="J516" s="2" t="inlineStr">
         <is>
           <t>Verify operating system enforces a 60-day maximum password lifetime restriction. If it does not, this is a finding.</t>
         </is>
       </c>
-      <c r="K517" s="2" t="inlineStr">
+      <c r="K516" s="2" t="inlineStr">
         <is>
           <t>Check whether the maximum time period for existing passwords is restricted to 60 days with the following commands:
 $ sudo awk -F: '$5 &gt; 60 {print $1 "" "" $5}' /etc/shadow
@@ -41396,77 +41321,77 @@
 If any results are returned that are not associated with a system account, then this is a finding.</t>
         </is>
       </c>
-      <c r="L517" s="2" t="n"/>
-      <c r="M517" s="2" t="inlineStr">
+      <c r="L516" s="2" t="n"/>
+      <c r="M516" s="2" t="inlineStr">
         <is>
           <t>Configure non-compliant accounts to enforce a 60-day maximum password lifetime restriction.
 passwd -x 60 [user]</t>
         </is>
       </c>
-      <c r="N517" s="2" t="inlineStr">
-        <is>
-          <t>CAT II</t>
-        </is>
-      </c>
-      <c r="O517" s="2" t="n"/>
-      <c r="P517" s="2" t="n"/>
-      <c r="Q517" s="2" t="n"/>
-    </row>
-    <row r="518" ht="130" customHeight="1">
-      <c r="A518" s="2" t="inlineStr">
+      <c r="N516" s="2" t="inlineStr">
+        <is>
+          <t>CAT II</t>
+        </is>
+      </c>
+      <c r="O516" s="2" t="n"/>
+      <c r="P516" s="2" t="n"/>
+      <c r="Q516" s="2" t="n"/>
+    </row>
+    <row r="517" ht="130" customHeight="1">
+      <c r="A517" s="2" t="inlineStr">
         <is>
           <t>AU-9</t>
         </is>
       </c>
-      <c r="B518" s="2" t="inlineStr">
+      <c r="B517" s="2" t="inlineStr">
         <is>
           <t>CCI-001493</t>
         </is>
       </c>
-      <c r="C518" s="2" t="inlineStr">
+      <c r="C517" s="2" t="inlineStr">
         <is>
           <t>SRG-OS-000256-GPOS-00097</t>
         </is>
       </c>
-      <c r="D518" s="2" t="inlineStr">
+      <c r="D517" s="2" t="inlineStr">
         <is>
           <t>CCE-86228-4</t>
         </is>
       </c>
-      <c r="E518" s="2" t="inlineStr">
+      <c r="E517" s="2" t="inlineStr">
         <is>
           <t>The operating system must protect audit tools from unauthorized access.</t>
         </is>
       </c>
-      <c r="F518" s="2" t="inlineStr">
+      <c r="F517" s="2" t="inlineStr">
         <is>
           <t>Red Hat Enterprise Linux 9 Must Protect Audit Tools From Unauthorized Access.</t>
         </is>
       </c>
-      <c r="G518" s="2" t="inlineStr">
+      <c r="G517" s="2" t="inlineStr">
         <is>
           <t>Protecting audit information also includes identifying and protecting the tools used to view and manipulate log data. Therefore, protecting audit tools is necessary to prevent unauthorized operation on audit information.
 Operating systems providing tools to interface with audit information will leverage user permissions and roles identifying the user accessing the tools and the corresponding rights the user enjoys in order to make access decisions regarding the access to audit tools.
 Audit tools include, but are not limited to, vendor-provided and open source audit tools needed to successfully view and manipulate audit information system activity and records. Audit tools include custom queries and report generators.</t>
         </is>
       </c>
-      <c r="H518" s="2" t="inlineStr">
+      <c r="H517" s="2" t="inlineStr">
         <is>
           <t>Protecting audit information also includes identifying and protecting the tools used to view and manipulate log data.
 Therefore, protecting audit tools is necessary to prevent unauthorized operations on audit information.</t>
         </is>
       </c>
-      <c r="I518" s="2" t="inlineStr">
-        <is>
-          <t>Applicable - Configurable</t>
-        </is>
-      </c>
-      <c r="J518" s="2" t="inlineStr">
+      <c r="I517" s="2" t="inlineStr">
+        <is>
+          <t>Applicable - Configurable</t>
+        </is>
+      </c>
+      <c r="J517" s="2" t="inlineStr">
         <is>
           <t>Verify the operating system protects audit tools from unauthorized access. If it does not, this is a finding.</t>
         </is>
       </c>
-      <c r="K518" s="2" t="inlineStr">
+      <c r="K517" s="2" t="inlineStr">
         <is>
           <t>Verify the audit tools are protected from unauthorized access, deletion, or modification by checking the permissive mode.
 Check the octal permission of each audit tool by running the following command:
@@ -41474,78 +41399,78 @@
 If any of these files have more permissive permissions than 0755, then this is a finding.</t>
         </is>
       </c>
-      <c r="L518" s="2" t="n"/>
-      <c r="M518" s="2" t="inlineStr">
+      <c r="L517" s="2" t="n"/>
+      <c r="M517" s="2" t="inlineStr">
         <is>
           <t>Configure the audit tools to be owned by "root", by running the following command:
 $ sudo chmod 0755 [audit_tool]
 Replace "[audit_tool]" with each audit tool that has a more permissive mode than 0755.</t>
         </is>
       </c>
-      <c r="N518" s="2" t="inlineStr">
-        <is>
-          <t>CAT II</t>
-        </is>
-      </c>
-      <c r="O518" s="2" t="n"/>
-      <c r="P518" s="2" t="n"/>
-      <c r="Q518" s="2" t="n"/>
-    </row>
-    <row r="519" ht="130" customHeight="1">
-      <c r="A519" s="2" t="inlineStr">
+      <c r="N517" s="2" t="inlineStr">
+        <is>
+          <t>CAT II</t>
+        </is>
+      </c>
+      <c r="O517" s="2" t="n"/>
+      <c r="P517" s="2" t="n"/>
+      <c r="Q517" s="2" t="n"/>
+    </row>
+    <row r="518" ht="130" customHeight="1">
+      <c r="A518" s="2" t="inlineStr">
         <is>
           <t>AU-9</t>
         </is>
       </c>
-      <c r="B519" s="2" t="inlineStr">
+      <c r="B518" s="2" t="inlineStr">
         <is>
           <t>CCI-001493</t>
         </is>
       </c>
-      <c r="C519" s="2" t="inlineStr">
+      <c r="C518" s="2" t="inlineStr">
         <is>
           <t>SRG-OS-000256-GPOS-00097</t>
         </is>
       </c>
-      <c r="D519" s="2" t="inlineStr">
+      <c r="D518" s="2" t="inlineStr">
         <is>
           <t>CCE-86263-1</t>
         </is>
       </c>
-      <c r="E519" s="2" t="inlineStr">
+      <c r="E518" s="2" t="inlineStr">
         <is>
           <t>The operating system must protect audit tools from unauthorized access.</t>
         </is>
       </c>
-      <c r="F519" s="2" t="inlineStr">
+      <c r="F518" s="2" t="inlineStr">
         <is>
           <t>Red Hat Enterprise Linux 9 Must Protect Audit Tools From Unauthorized Access.</t>
         </is>
       </c>
-      <c r="G519" s="2" t="inlineStr">
+      <c r="G518" s="2" t="inlineStr">
         <is>
           <t>Protecting audit information also includes identifying and protecting the tools used to view and manipulate log data. Therefore, protecting audit tools is necessary to prevent unauthorized operation on audit information.
 Operating systems providing tools to interface with audit information will leverage user permissions and roles identifying the user accessing the tools and the corresponding rights the user enjoys in order to make access decisions regarding the access to audit tools.
 Audit tools include, but are not limited to, vendor-provided and open source audit tools needed to successfully view and manipulate audit information system activity and records. Audit tools include custom queries and report generators.</t>
         </is>
       </c>
-      <c r="H519" s="2" t="inlineStr">
+      <c r="H518" s="2" t="inlineStr">
         <is>
           <t>Protecting audit information also includes identifying and protecting the tools used to view and manipulate log data.
 Therefore, protecting audit tools is necessary to prevent unauthorized operations on audit information.</t>
         </is>
       </c>
-      <c r="I519" s="2" t="inlineStr">
-        <is>
-          <t>Applicable - Configurable</t>
-        </is>
-      </c>
-      <c r="J519" s="2" t="inlineStr">
+      <c r="I518" s="2" t="inlineStr">
+        <is>
+          <t>Applicable - Configurable</t>
+        </is>
+      </c>
+      <c r="J518" s="2" t="inlineStr">
         <is>
           <t>Verify the operating system protects audit tools from unauthorized access. If it does not, this is a finding.</t>
         </is>
       </c>
-      <c r="K519" s="2" t="inlineStr">
+      <c r="K518" s="2" t="inlineStr">
         <is>
           <t>Verify the audit tools are owned by "root" to prevent any unauthorized access, deletion, or modification.
 Check the owner of each audit tool by running the following command:
@@ -41560,78 +41485,78 @@
 If any audit tools are not owned by root, then this is a finding.</t>
         </is>
       </c>
-      <c r="L519" s="2" t="n"/>
-      <c r="M519" s="2" t="inlineStr">
+      <c r="L518" s="2" t="n"/>
+      <c r="M518" s="2" t="inlineStr">
         <is>
           <t>Configure the audit tools to be owned by "root", by running the following command:
 $ sudo chown root [audit_tool]
 Replace "[audit_tool]" with each audit tool not owned by "root".</t>
         </is>
       </c>
-      <c r="N519" s="2" t="inlineStr">
-        <is>
-          <t>CAT II</t>
-        </is>
-      </c>
-      <c r="O519" s="2" t="n"/>
-      <c r="P519" s="2" t="n"/>
-      <c r="Q519" s="2" t="n"/>
-    </row>
-    <row r="520" ht="130" customHeight="1">
-      <c r="A520" s="2" t="inlineStr">
+      <c r="N518" s="2" t="inlineStr">
+        <is>
+          <t>CAT II</t>
+        </is>
+      </c>
+      <c r="O518" s="2" t="n"/>
+      <c r="P518" s="2" t="n"/>
+      <c r="Q518" s="2" t="n"/>
+    </row>
+    <row r="519" ht="130" customHeight="1">
+      <c r="A519" s="2" t="inlineStr">
         <is>
           <t>AU-9</t>
         </is>
       </c>
-      <c r="B520" s="2" t="inlineStr">
+      <c r="B519" s="2" t="inlineStr">
         <is>
           <t>CCI-001493</t>
         </is>
       </c>
-      <c r="C520" s="2" t="inlineStr">
+      <c r="C519" s="2" t="inlineStr">
         <is>
           <t>SRG-OS-000256-GPOS-00097</t>
         </is>
       </c>
-      <c r="D520" s="2" t="inlineStr">
+      <c r="D519" s="2" t="inlineStr">
         <is>
           <t>CCE-86240-9</t>
         </is>
       </c>
-      <c r="E520" s="2" t="inlineStr">
+      <c r="E519" s="2" t="inlineStr">
         <is>
           <t>The operating system must protect audit tools from unauthorized access.</t>
         </is>
       </c>
-      <c r="F520" s="2" t="inlineStr">
+      <c r="F519" s="2" t="inlineStr">
         <is>
           <t>Red Hat Enterprise Linux 9 Must Protect Audit Tools From Unauthorized Access.</t>
         </is>
       </c>
-      <c r="G520" s="2" t="inlineStr">
+      <c r="G519" s="2" t="inlineStr">
         <is>
           <t>Protecting audit information also includes identifying and protecting the tools used to view and manipulate log data. Therefore, protecting audit tools is necessary to prevent unauthorized operation on audit information.
 Operating systems providing tools to interface with audit information will leverage user permissions and roles identifying the user accessing the tools and the corresponding rights the user enjoys in order to make access decisions regarding the access to audit tools.
 Audit tools include, but are not limited to, vendor-provided and open source audit tools needed to successfully view and manipulate audit information system activity and records. Audit tools include custom queries and report generators.</t>
         </is>
       </c>
-      <c r="H520" s="2" t="inlineStr">
+      <c r="H519" s="2" t="inlineStr">
         <is>
           <t>Protecting audit information also includes identifying and protecting the tools used to view and manipulate log data.
 Therefore, protecting audit tools is necessary to prevent unauthorized operations on audit information.</t>
         </is>
       </c>
-      <c r="I520" s="2" t="inlineStr">
-        <is>
-          <t>Applicable - Configurable</t>
-        </is>
-      </c>
-      <c r="J520" s="2" t="inlineStr">
+      <c r="I519" s="2" t="inlineStr">
+        <is>
+          <t>Applicable - Configurable</t>
+        </is>
+      </c>
+      <c r="J519" s="2" t="inlineStr">
         <is>
           <t>Verify the operating system protects audit tools from unauthorized access. If it does not, this is a finding.</t>
         </is>
       </c>
-      <c r="K520" s="2" t="inlineStr">
+      <c r="K519" s="2" t="inlineStr">
         <is>
           <t>Verify the audit tools are group-owned by "root" to prevent any unauthorized access, deletion, or modification.
 Check the group-owner of each audit tool by running the following command:
@@ -41646,140 +41571,140 @@
 If any audit tools are not group-owned by root, then this is a finding.</t>
         </is>
       </c>
-      <c r="L520" s="2" t="n"/>
-      <c r="M520" s="2" t="inlineStr">
+      <c r="L519" s="2" t="n"/>
+      <c r="M519" s="2" t="inlineStr">
         <is>
           <t>Configure the audit tools to be group-owned by "root", by running the following command:
 $ sudo chgrp root [audit_tool]
 Replace "[audit_tool]" with each audit tool not group-owned by "root".</t>
         </is>
       </c>
+      <c r="N519" s="2" t="inlineStr">
+        <is>
+          <t>CAT II</t>
+        </is>
+      </c>
+      <c r="O519" s="2" t="n"/>
+      <c r="P519" s="2" t="n"/>
+      <c r="Q519" s="2" t="n"/>
+    </row>
+    <row r="520" ht="130" customHeight="1">
+      <c r="A520" s="2" t="inlineStr">
+        <is>
+          <t>SI-2 (2)</t>
+        </is>
+      </c>
+      <c r="B520" s="2" t="inlineStr">
+        <is>
+          <t>CCI-001233</t>
+        </is>
+      </c>
+      <c r="C520" s="2" t="inlineStr">
+        <is>
+          <t>SRG-OS-000191-GPOS-00080</t>
+        </is>
+      </c>
+      <c r="D520" s="2" t="inlineStr"/>
+      <c r="E520" s="2" t="inlineStr">
+        <is>
+          <t>The operating system must employ automated mechanisms to determine the state of system components with regard to flaw remediation using the following frequency: continuously, where Endpoint Security Solution (ESS) is used; 30 days, for any additional internal network scans not covered by ESS; and annually, for external scans by Computer Network Defense Service Provider (CNDSP).</t>
+        </is>
+      </c>
+      <c r="F520" s="2" t="inlineStr">
+        <is>
+          <t>Red Hat Enterprise Linux 9 must employ automated mechanisms to determine the state of system components with regard to flaw remediation using the following frequency: continuously, where ESS is used; 30 days, for any additional internal network scans not cover</t>
+        </is>
+      </c>
+      <c r="G520" s="2" t="inlineStr">
+        <is>
+          <t>Without the use of automated mechanisms to scan for security flaws on a continuous and/or periodic basis, the operating system or other system components may remain vulnerable to the exploits presented by undetected software flaws.
+To support this requirement, the operating system may have an integrated solution incorporating continuous scanning using ESS and periodic scanning using other tools, as specified in the requirement.</t>
+        </is>
+      </c>
+      <c r="H520" s="2" t="inlineStr">
+        <is>
+          <t>Without the use of automated mechanisms to scan for security flaws on a continuous and/or periodic basis, the operating system or other system components may remain vulnerable to the exploits presented by undetected software flaws.
+To support this requirement, the operating system may gihave an integrated solution incorporating continuous scanning using ESS and periodic scanning using other tools, as specified in the requirement.</t>
+        </is>
+      </c>
+      <c r="I520" s="2" t="inlineStr">
+        <is>
+          <t>Applicable - Does Not Meet</t>
+        </is>
+      </c>
+      <c r="J520" s="2" t="inlineStr">
+        <is>
+          <t>Verify the operating system employs automated mechanisms to determine the state of system components with regard to flaw remediation using the following frequency: continuously, where ESS is used; 30 days, for any additional internal network scans not covered by ESS; and annually, for external scans by CNDSP.
+If it does not, this is a finding.</t>
+        </is>
+      </c>
+      <c r="K520" s="2" t="inlineStr">
+        <is>
+          <t>Red Hat Enterprise Linux 9 supports this requirement and cannot be configured to be out of compliance.</t>
+        </is>
+      </c>
+      <c r="L520" s="2" t="n"/>
+      <c r="M520" s="2" t="inlineStr">
+        <is>
+          <t>This requirement is a permanent finding and cannot be fixed. An appropriate mitigation for the system must be implemented, but this finding cannot be considered fixed.</t>
+        </is>
+      </c>
       <c r="N520" s="2" t="inlineStr">
         <is>
           <t>CAT II</t>
         </is>
       </c>
-      <c r="O520" s="2" t="n"/>
+      <c r="O520" s="2" t="inlineStr">
+        <is>
+          <t>A third-party software will be needed to meet this requirement e.g. McAfee policy auditor.
+Although the listed mitigation is supporting the security function, it is not sufficient to reduce the residual risk of this requirement.</t>
+        </is>
+      </c>
       <c r="P520" s="2" t="n"/>
-      <c r="Q520" s="2" t="n"/>
+      <c r="Q520" s="2" t="inlineStr">
+        <is>
+          <t>Red Hat Enterprise Linux 9 does not have configuration options to meet this requirement.</t>
+        </is>
+      </c>
     </row>
     <row r="521" ht="130" customHeight="1">
       <c r="A521" s="2" t="inlineStr">
         <is>
-          <t>SI-2 (2)</t>
+          <t>IA-5 (1) (a)</t>
         </is>
       </c>
       <c r="B521" s="2" t="inlineStr">
         <is>
-          <t>CCI-001233</t>
+          <t>CCI-000194</t>
         </is>
       </c>
       <c r="C521" s="2" t="inlineStr">
         <is>
-          <t>SRG-OS-000191-GPOS-00080</t>
-        </is>
-      </c>
-      <c r="D521" s="2" t="inlineStr"/>
+          <t>SRG-OS-000071-GPOS-00039</t>
+        </is>
+      </c>
+      <c r="D521" s="2" t="inlineStr">
+        <is>
+          <t>CCE-83566-0</t>
+        </is>
+      </c>
       <c r="E521" s="2" t="inlineStr">
         <is>
-          <t>The operating system must employ automated mechanisms to determine the state of system components with regard to flaw remediation using the following frequency: continuously, where Endpoint Security Solution (ESS) is used; 30 days, for any additional internal network scans not covered by ESS; and annually, for external scans by Computer Network Defense Service Provider (CNDSP).</t>
+          <t>The operating system must enforce password complexity by requiring that at least one numeric character be used.</t>
         </is>
       </c>
       <c r="F521" s="2" t="inlineStr">
         <is>
-          <t>Red Hat Enterprise Linux 9 must employ automated mechanisms to determine the state of system components with regard to flaw remediation using the following frequency: continuously, where ESS is used; 30 days, for any additional internal network scans not cover</t>
+          <t>Red Hat Enterprise Linux 9 Must Enforce Password Complexity By Requiring That At Least One Numeric Character Be Used.</t>
         </is>
       </c>
       <c r="G521" s="2" t="inlineStr">
-        <is>
-          <t>Without the use of automated mechanisms to scan for security flaws on a continuous and/or periodic basis, the operating system or other system components may remain vulnerable to the exploits presented by undetected software flaws.
-To support this requirement, the operating system may have an integrated solution incorporating continuous scanning using ESS and periodic scanning using other tools, as specified in the requirement.</t>
-        </is>
-      </c>
-      <c r="H521" s="2" t="inlineStr">
-        <is>
-          <t>Without the use of automated mechanisms to scan for security flaws on a continuous and/or periodic basis, the operating system or other system components may remain vulnerable to the exploits presented by undetected software flaws.
-To support this requirement, the operating system may gihave an integrated solution incorporating continuous scanning using ESS and periodic scanning using other tools, as specified in the requirement.</t>
-        </is>
-      </c>
-      <c r="I521" s="2" t="inlineStr">
-        <is>
-          <t>Applicable - Does Not Meet</t>
-        </is>
-      </c>
-      <c r="J521" s="2" t="inlineStr">
-        <is>
-          <t>Verify the operating system employs automated mechanisms to determine the state of system components with regard to flaw remediation using the following frequency: continuously, where ESS is used; 30 days, for any additional internal network scans not covered by ESS; and annually, for external scans by CNDSP.
-If it does not, this is a finding.</t>
-        </is>
-      </c>
-      <c r="K521" s="2" t="inlineStr">
-        <is>
-          <t>Red Hat Enterprise Linux 9 supports this requirement and cannot be configured to be out of compliance.</t>
-        </is>
-      </c>
-      <c r="L521" s="2" t="n"/>
-      <c r="M521" s="2" t="inlineStr">
-        <is>
-          <t>This requirement is a permanent finding and cannot be fixed. An appropriate mitigation for the system must be implemented, but this finding cannot be considered fixed.</t>
-        </is>
-      </c>
-      <c r="N521" s="2" t="inlineStr">
-        <is>
-          <t>CAT II</t>
-        </is>
-      </c>
-      <c r="O521" s="2" t="inlineStr">
-        <is>
-          <t>A third-party software will be needed to meet this requirement e.g. McAfee policy auditor.
-Although the listed mitigation is supporting the security function, it is not sufficient to reduce the residual risk of this requirement.</t>
-        </is>
-      </c>
-      <c r="P521" s="2" t="n"/>
-      <c r="Q521" s="2" t="inlineStr">
-        <is>
-          <t>Red Hat Enterprise Linux 9 does not have configuration options to meet this requirement.</t>
-        </is>
-      </c>
-    </row>
-    <row r="522" ht="130" customHeight="1">
-      <c r="A522" s="2" t="inlineStr">
-        <is>
-          <t>IA-5 (1) (a)</t>
-        </is>
-      </c>
-      <c r="B522" s="2" t="inlineStr">
-        <is>
-          <t>CCI-000194</t>
-        </is>
-      </c>
-      <c r="C522" s="2" t="inlineStr">
-        <is>
-          <t>SRG-OS-000071-GPOS-00039</t>
-        </is>
-      </c>
-      <c r="D522" s="2" t="inlineStr">
-        <is>
-          <t>CCE-83566-0</t>
-        </is>
-      </c>
-      <c r="E522" s="2" t="inlineStr">
-        <is>
-          <t>The operating system must enforce password complexity by requiring that at least one numeric character be used.</t>
-        </is>
-      </c>
-      <c r="F522" s="2" t="inlineStr">
-        <is>
-          <t>Red Hat Enterprise Linux 9 Must Enforce Password Complexity By Requiring That At Least One Numeric Character Be Used.</t>
-        </is>
-      </c>
-      <c r="G522" s="2" t="inlineStr">
         <is>
           <t>Use of a complex password helps to increase the time and resources required to compromise the password. Password complexity, or strength, is a measure of the effectiveness of a password in resisting attempts at guessing and brute-force attacks.
 Password complexity is one factor of several that determines how long it takes to crack a password. The more complex the password, the greater the number of possible combinations that need to be tested before the password is compromised.</t>
         </is>
       </c>
-      <c r="H522" s="2" t="inlineStr">
+      <c r="H521" s="2" t="inlineStr">
         <is>
           <t>Use of a complex password helps to increase the time and resources required
 to compromise the password. Password complexity, or strength, is a measure of
@@ -41792,17 +41717,17 @@
 search space.</t>
         </is>
       </c>
-      <c r="I522" s="2" t="inlineStr">
-        <is>
-          <t>Applicable - Configurable</t>
-        </is>
-      </c>
-      <c r="J522" s="2" t="inlineStr">
+      <c r="I521" s="2" t="inlineStr">
+        <is>
+          <t>Applicable - Configurable</t>
+        </is>
+      </c>
+      <c r="J521" s="2" t="inlineStr">
         <is>
           <t>Verify the operating system enforces password complexity by requiring that at least one numeric character be used. If it does not, this is a finding.</t>
         </is>
       </c>
-      <c r="K522" s="2" t="inlineStr">
+      <c r="K521" s="2" t="inlineStr">
         <is>
           <t>To check how many digits are required in a password, run the following command:
  $ grep dcredit /etc/security/pwquality.conf 
@@ -41810,58 +41735,58 @@
 If dcredit is not found or not equal to or less than the required value, then this is a finding.</t>
         </is>
       </c>
-      <c r="L522" s="2" t="n"/>
-      <c r="M522" s="2" t="inlineStr">
+      <c r="L521" s="2" t="n"/>
+      <c r="M521" s="2" t="inlineStr">
         <is>
           <t>Configure the operating system to enforce password complexity by requiring that at least numeric character be used by setting the "dcredit" option.
 Add the following line to "/etc/security/pwquality.conf" (or modify the line to have the required value):
 dcredit = -1</t>
         </is>
       </c>
-      <c r="N522" s="2" t="inlineStr">
-        <is>
-          <t>CAT II</t>
-        </is>
-      </c>
-      <c r="O522" s="2" t="n"/>
-      <c r="P522" s="2" t="n"/>
-      <c r="Q522" s="2" t="n"/>
-    </row>
-    <row r="523" ht="130" customHeight="1">
-      <c r="A523" s="3" t="inlineStr">
+      <c r="N521" s="2" t="inlineStr">
+        <is>
+          <t>CAT II</t>
+        </is>
+      </c>
+      <c r="O521" s="2" t="n"/>
+      <c r="P521" s="2" t="n"/>
+      <c r="Q521" s="2" t="n"/>
+    </row>
+    <row r="522" ht="130" customHeight="1">
+      <c r="A522" s="3" t="inlineStr">
         <is>
           <t>AC-17 (9)</t>
         </is>
       </c>
-      <c r="B523" s="3" t="inlineStr">
+      <c r="B522" s="3" t="inlineStr">
         <is>
           <t>CCI-002322</t>
         </is>
       </c>
-      <c r="C523" s="3" t="inlineStr">
+      <c r="C522" s="3" t="inlineStr">
         <is>
           <t>SRG-OS-000298-GPOS-00116</t>
         </is>
       </c>
-      <c r="D523" s="3" t="inlineStr"/>
-      <c r="E523" s="3" t="inlineStr">
+      <c r="D522" s="3" t="inlineStr"/>
+      <c r="E522" s="3" t="inlineStr">
         <is>
           <t>The operating system must provide the capability to immediately disconnect or disable remote access to the operating system.</t>
         </is>
       </c>
-      <c r="F523" s="3" t="inlineStr">
+      <c r="F522" s="3" t="inlineStr">
         <is>
           <t>Red Hat Enterprise Linux 9 must provide the capability to immediately disconnect or disable remote access to the operating system.</t>
         </is>
       </c>
-      <c r="G523" s="3" t="inlineStr">
+      <c r="G522" s="3" t="inlineStr">
         <is>
           <t>Without the ability to immediately disconnect or disable remote access, an attack or other compromise taking place would not be immediately stopped.
 Operating system remote access functionality must have the capability to immediately disconnect current users remotely accessing the information system and/or disable further remote access. The speed of disconnect or disablement varies based on the criticality of missions functions and the need to eliminate immediate or future remote access to organizational information systems.
 The remote access functionality (e.g., RDP) may implement features such as automatic disconnect (or user-initiated disconnect) in case of adverse information based on an indicator of compromise or attack.</t>
         </is>
       </c>
-      <c r="H523" s="3" t="inlineStr">
+      <c r="H522" s="3" t="inlineStr">
         <is>
           <t>Without the ability to immediately disconnect or disable remote access, an attack or other compromise taking place would not be immediately stopped.
 Red Hat Enterprise Linux 9 remote access functionality must have the capability to immediately disconnect current users remotely accessing the information system and/or disable further remote access.
@@ -41869,70 +41794,70 @@
 The remote access functionality (e.g., RDP) may implement features such as automatic disconnect (or user-initiated disconnect) in case of adverse information based on an indicator of compromise or attack.</t>
         </is>
       </c>
-      <c r="I523" s="3" t="inlineStr">
+      <c r="I522" s="3" t="inlineStr">
         <is>
           <t>Applicable - Inherently Met</t>
         </is>
       </c>
-      <c r="J523" s="3" t="inlineStr">
+      <c r="J522" s="3" t="inlineStr">
         <is>
           <t>Verify the operating system provides the capability to immediately disconnect or disable remote access to the operating system. If it does not, this is a finding.</t>
         </is>
       </c>
-      <c r="K523" s="3" t="inlineStr">
+      <c r="K522" s="3" t="inlineStr">
         <is>
           <t>Red Hat Enterprise Linux 9 supports this requirement and cannot be configured to be out of compliance.
 Red Hat Enterprise Linux 9 inherently meets this requirement.</t>
         </is>
       </c>
-      <c r="L523" s="3" t="n"/>
-      <c r="M523" s="3" t="n"/>
-      <c r="N523" s="3" t="inlineStr">
-        <is>
-          <t>CAT II</t>
-        </is>
-      </c>
-      <c r="O523" s="3" t="n"/>
-      <c r="P523" s="3" t="inlineStr">
+      <c r="L522" s="3" t="n"/>
+      <c r="M522" s="3" t="n"/>
+      <c r="N522" s="3" t="inlineStr">
+        <is>
+          <t>CAT II</t>
+        </is>
+      </c>
+      <c r="O522" s="3" t="n"/>
+      <c r="P522" s="3" t="inlineStr">
         <is>
           <t>The admin can shutdown networking to the host by port, NIC, or the entire network as desired.</t>
         </is>
       </c>
-      <c r="Q523" s="3" t="inlineStr">
+      <c r="Q522" s="3" t="inlineStr">
         <is>
           <t>The use of the "exit" command will end any communication session on the system. This is part of the kernel and cannot be removed without recompiling.
 The admin can shutdown networking to the host by port, NIC, or the entire network as desired.</t>
         </is>
       </c>
     </row>
-    <row r="524" ht="130" customHeight="1">
-      <c r="A524" s="2" t="inlineStr">
+    <row r="523" ht="130" customHeight="1">
+      <c r="A523" s="2" t="inlineStr">
         <is>
           <t>IA-2 (9)</t>
         </is>
       </c>
-      <c r="B524" s="2" t="inlineStr">
+      <c r="B523" s="2" t="inlineStr">
         <is>
           <t>CCI-001942</t>
         </is>
       </c>
-      <c r="C524" s="2" t="inlineStr">
+      <c r="C523" s="2" t="inlineStr">
         <is>
           <t>SRG-OS-000113-GPOS-00058</t>
         </is>
       </c>
-      <c r="D524" s="2" t="inlineStr"/>
-      <c r="E524" s="2" t="inlineStr">
+      <c r="D523" s="2" t="inlineStr"/>
+      <c r="E523" s="2" t="inlineStr">
         <is>
           <t>The operating system must implement replay-resistant authentication mechanisms for network access to non-privileged accounts.</t>
         </is>
       </c>
-      <c r="F524" s="2" t="inlineStr">
+      <c r="F523" s="2" t="inlineStr">
         <is>
           <t>Red Hat Enterprise Linux 9 system must implement replay-resistant authentication mechanisms for network access to non-privileged accounts.</t>
         </is>
       </c>
-      <c r="G524" s="2" t="inlineStr">
+      <c r="G523" s="2" t="inlineStr">
         <is>
           <t>A replay attack may enable an unauthorized user to gain access to the operating system. Authentication sessions between the authenticator and the operating system validating the user credentials must not be vulnerable to a replay attack.
 An authentication process resists replay attacks if it is impractical to achieve a successful authentication by recording and replaying a previous authentication message.
@@ -41940,76 +41865,76 @@
 Techniques used to address this include protocols using nonces (e.g., numbers generated for a specific one-time use) or challenges (e.g., TLS, WS_Security). Additional techniques include time-synchronous or challenge-response one-time authenticators.</t>
         </is>
       </c>
-      <c r="H524" s="2" t="inlineStr"/>
-      <c r="I524" s="2" t="inlineStr">
+      <c r="H523" s="2" t="inlineStr"/>
+      <c r="I523" s="2" t="inlineStr">
         <is>
           <t>Applicable - Inherently Met</t>
         </is>
       </c>
-      <c r="J524" s="2" t="inlineStr">
+      <c r="J523" s="2" t="inlineStr">
         <is>
           <t>Verify the operating system implements replay-resistant authentication mechanisms for network access to non-privileged accounts. If it does not, this is a finding.</t>
         </is>
       </c>
-      <c r="K524" s="2" t="inlineStr">
+      <c r="K523" s="2" t="inlineStr">
         <is>
           <t>Red Hat Enterprise Linux 9 supports this requirement and cannot be configured to be out of compliance.
 Red Hat Enterprise Linux 9 inherently meets this requirement.</t>
         </is>
       </c>
-      <c r="L524" s="2" t="n"/>
-      <c r="M524" s="2" t="inlineStr">
+      <c r="L523" s="2" t="n"/>
+      <c r="M523" s="2" t="inlineStr">
         <is>
           <t>Red Hat Enterprise Linux 9 inherently meets this requirement.
 No fix is required.</t>
         </is>
       </c>
-      <c r="N524" s="2" t="inlineStr">
-        <is>
-          <t>CAT II</t>
-        </is>
-      </c>
-      <c r="O524" s="2" t="n"/>
-      <c r="P524" s="2" t="inlineStr">
+      <c r="N523" s="2" t="inlineStr">
+        <is>
+          <t>CAT II</t>
+        </is>
+      </c>
+      <c r="O523" s="2" t="n"/>
+      <c r="P523" s="2" t="inlineStr">
         <is>
           <t>The release notes of OpenSSH 7.6 states "OpenSSH is a 100% complete SSH protocol 2.0 implementation and includes sftp client and server support."
 https://www.openssh.com/txt/release-7.6</t>
         </is>
       </c>
-      <c r="Q524" s="2" t="inlineStr">
+      <c r="Q523" s="2" t="inlineStr">
         <is>
           <t>The OpenSSH package in Red Hat Enterprise Linux 9 is version 8.7, which is newer than 7.6 which only supports SSH protocol 2.0 which is restraint to replay attacks.</t>
         </is>
       </c>
     </row>
-    <row r="525" ht="130" customHeight="1">
-      <c r="A525" s="3" t="inlineStr">
+    <row r="524" ht="130" customHeight="1">
+      <c r="A524" s="3" t="inlineStr">
         <is>
           <t>IA-3 (1)</t>
         </is>
       </c>
-      <c r="B525" s="3" t="inlineStr">
+      <c r="B524" s="3" t="inlineStr">
         <is>
           <t>CCI-001967</t>
         </is>
       </c>
-      <c r="C525" s="3" t="inlineStr">
+      <c r="C524" s="3" t="inlineStr">
         <is>
           <t>SRG-OS-000379-GPOS-00164</t>
         </is>
       </c>
-      <c r="D525" s="3" t="inlineStr"/>
-      <c r="E525" s="3" t="inlineStr">
+      <c r="D524" s="3" t="inlineStr"/>
+      <c r="E524" s="3" t="inlineStr">
         <is>
           <t>The operating system must authenticate all endpoint devices before establishing a local, remote, and/or network connection using bidirectional authentication that is cryptographically based.</t>
         </is>
       </c>
-      <c r="F525" s="3" t="inlineStr">
+      <c r="F524" s="3" t="inlineStr">
         <is>
           <t>Red Hat Enterprise Linux 9 must authenticate all endpoint devices before establishing a local, remote, and/or network connection using bidirectional authentication that is cryptographically based.</t>
         </is>
       </c>
-      <c r="G525" s="3" t="inlineStr">
+      <c r="G524" s="3" t="inlineStr">
         <is>
           <t>Without authenticating devices, unidentified or unknown devices may be introduced, thereby facilitating malicious activity. Bidirectional authentication provides stronger safeguards to validate the identity of other devices for connections that are of greater risk.
 Bidirectional authentication solutions include, but are not limited to, IEEE 802.1x and Extensible Authentication Protocol [EAP], RADIUS server with EAP-Transport Layer Security [TLS] authentication, Kerberos, and SSL mutual authentication.
@@ -42017,63 +41942,63 @@
 Because of the challenges of applying this requirement on a large scale, organizations are encouraged to only apply this requirement to those limited number (and type) of devices that truly need to support this capability.</t>
         </is>
       </c>
-      <c r="H525" s="3" t="inlineStr"/>
-      <c r="I525" s="3" t="inlineStr">
-        <is>
-          <t>Applicable - Configurable</t>
-        </is>
-      </c>
-      <c r="J525" s="3" t="inlineStr">
+      <c r="H524" s="3" t="inlineStr"/>
+      <c r="I524" s="3" t="inlineStr">
+        <is>
+          <t>Applicable - Configurable</t>
+        </is>
+      </c>
+      <c r="J524" s="3" t="inlineStr">
         <is>
           <t>Verify the operating system authenticates all endpoint devices before establishing a local, remote, and/or network connection using bidirectional authentication that is cryptographically based. If it does not, this is a finding.</t>
         </is>
       </c>
-      <c r="K525" s="3" t="n"/>
-      <c r="L525" s="3" t="n"/>
-      <c r="M525" s="3" t="n"/>
-      <c r="N525" s="3" t="inlineStr">
-        <is>
-          <t>CAT II</t>
-        </is>
-      </c>
-      <c r="O525" s="3" t="n"/>
-      <c r="P525" s="3" t="n"/>
-      <c r="Q525" s="3" t="n"/>
-    </row>
-    <row r="526" ht="130" customHeight="1">
-      <c r="A526" s="2" t="inlineStr">
+      <c r="K524" s="3" t="n"/>
+      <c r="L524" s="3" t="n"/>
+      <c r="M524" s="3" t="n"/>
+      <c r="N524" s="3" t="inlineStr">
+        <is>
+          <t>CAT II</t>
+        </is>
+      </c>
+      <c r="O524" s="3" t="n"/>
+      <c r="P524" s="3" t="n"/>
+      <c r="Q524" s="3" t="n"/>
+    </row>
+    <row r="525" ht="130" customHeight="1">
+      <c r="A525" s="2" t="inlineStr">
         <is>
           <t>AU-5 (2)</t>
         </is>
       </c>
-      <c r="B526" s="2" t="inlineStr">
+      <c r="B525" s="2" t="inlineStr">
         <is>
           <t>CCI-001858</t>
         </is>
       </c>
-      <c r="C526" s="2" t="inlineStr">
+      <c r="C525" s="2" t="inlineStr">
         <is>
           <t>SRG-OS-000344-GPOS-00135</t>
         </is>
       </c>
-      <c r="D526" s="2" t="inlineStr"/>
-      <c r="E526" s="2" t="inlineStr">
+      <c r="D525" s="2" t="inlineStr"/>
+      <c r="E525" s="2" t="inlineStr">
         <is>
           <t>The operating system must provide an immediate real-time alert to the SA and ISSO, at a minimum, of all audit failure events requiring real-time alerts.</t>
         </is>
       </c>
-      <c r="F526" s="2" t="inlineStr">
+      <c r="F525" s="2" t="inlineStr">
         <is>
           <t>Red Hat Enterprise Linux 9 must provide an immediate real-time alert to the SA and ISSO, at a minimum, of all audit failure events requiring real-time alerts.</t>
         </is>
       </c>
-      <c r="G526" s="2" t="inlineStr">
+      <c r="G525" s="2" t="inlineStr">
         <is>
           <t>It is critical for the appropriate personnel to be aware if a system is at risk of failing to process audit logs as required. Without a real-time alert, security personnel may be unaware of an impending failure of the audit capability and system operation may be adversely affected.
 Alerts provide organizations with urgent messages. Real-time alerts provide these messages immediately (i.e., the time from event detection to alert occurs in seconds or less).</t>
         </is>
       </c>
-      <c r="H526" s="2" t="inlineStr">
+      <c r="H525" s="2" t="inlineStr">
         <is>
           <t>It is critical for the appropriate personnel to be aware if a system is at risk of failing to process audit logs as required.
 Without a real-time alert, security personnel may be unaware of an impending failure of the audit capability and system operation may be adversely affected.
@@ -42081,184 +42006,262 @@
 Real-time alerts provide these messages immediately (i.e., the time from event detection to alert occurs in seconds or less).</t>
         </is>
       </c>
-      <c r="I526" s="2" t="inlineStr">
+      <c r="I525" s="2" t="inlineStr">
         <is>
           <t>Applicable - Does Not Meet</t>
         </is>
       </c>
-      <c r="J526" s="2" t="inlineStr">
+      <c r="J525" s="2" t="inlineStr">
         <is>
           <t>Verify the operating system provides an immediate real-time alert to the SA and ISSO, at a minimum, of all audit failure events requiring real-time alerts. If it does not, this is a finding.</t>
         </is>
       </c>
-      <c r="K526" s="2" t="inlineStr">
+      <c r="K525" s="2" t="inlineStr">
         <is>
           <t>Red Hat Enterprise Linux 9 does not support this requirement.
 This is an applicable-does not meet finding.</t>
         </is>
       </c>
-      <c r="L526" s="2" t="n"/>
-      <c r="M526" s="2" t="inlineStr">
+      <c r="L525" s="2" t="n"/>
+      <c r="M525" s="2" t="inlineStr">
         <is>
           <t>This requirement is a permanent finding and cannot be fixed. An appropriate mitigation for the system must be implemented, but this finding cannot be considered fixed.</t>
         </is>
       </c>
-      <c r="N526" s="2" t="inlineStr">
-        <is>
-          <t>CAT II</t>
-        </is>
-      </c>
-      <c r="O526" s="2" t="inlineStr">
+      <c r="N525" s="2" t="inlineStr">
+        <is>
+          <t>CAT II</t>
+        </is>
+      </c>
+      <c r="O525" s="2" t="inlineStr">
         <is>
           <t>Mitigate with third-party software.
 Although the listed mitigation is supporting the security function, it is not sufficient to reduce the residual risk of this requirement.</t>
         </is>
       </c>
-      <c r="P526" s="2" t="n"/>
-      <c r="Q526" s="2" t="inlineStr">
+      <c r="P525" s="2" t="n"/>
+      <c r="Q525" s="2" t="inlineStr">
         <is>
           <t>Notification when accounts are created/modified/deleted must be provided by a third party application that will communicate that an audit record of these actions has been created.</t>
         </is>
       </c>
     </row>
-    <row r="527" ht="130" customHeight="1">
-      <c r="A527" s="3" t="inlineStr">
+    <row r="526" ht="130" customHeight="1">
+      <c r="A526" s="3" t="inlineStr">
         <is>
           <t>AU-8 b</t>
         </is>
       </c>
-      <c r="B527" s="3" t="inlineStr">
+      <c r="B526" s="3" t="inlineStr">
         <is>
           <t>CCI-001889</t>
         </is>
       </c>
-      <c r="C527" s="3" t="inlineStr">
+      <c r="C526" s="3" t="inlineStr">
         <is>
           <t>SRG-OS-000358-GPOS-00145</t>
         </is>
       </c>
-      <c r="D527" s="3" t="inlineStr"/>
-      <c r="E527" s="3" t="inlineStr">
+      <c r="D526" s="3" t="inlineStr"/>
+      <c r="E526" s="3" t="inlineStr">
         <is>
           <t>The operating system must record time stamps for audit records that meet a minimum granularity of one second for a minimum degree of precision.</t>
         </is>
       </c>
-      <c r="F527" s="3" t="inlineStr">
+      <c r="F526" s="3" t="inlineStr">
         <is>
           <t>Red Hat Enterprise Linux 9 must record time stamps for audit records that meet a minimum granularity of one second for a minimum degree of precision.</t>
         </is>
       </c>
-      <c r="G527" s="3" t="inlineStr">
+      <c r="G526" s="3" t="inlineStr">
         <is>
           <t>Without sufficient granularity of time stamps, it is not possible to adequately determine the chronological order of records.
 Time stamps generated by the operating system include date and time. Granularity of time measurements refers to the degree of synchronization between information system clocks and reference clocks.</t>
         </is>
       </c>
-      <c r="H527" s="3" t="inlineStr">
+      <c r="H526" s="3" t="inlineStr">
         <is>
           <t>Without sufficient granularity of time stamps, it is not possible to adequately determine the chronological order of records.
 Time stamps generated by the operating system include date and time.
 Granularity of time measurements refers to the degree of synchronization between information system clocks and reference clocks.</t>
         </is>
       </c>
-      <c r="I527" s="3" t="inlineStr">
+      <c r="I526" s="3" t="inlineStr">
         <is>
           <t>Applicable - Inherently Met</t>
         </is>
       </c>
-      <c r="J527" s="3" t="inlineStr">
+      <c r="J526" s="3" t="inlineStr">
         <is>
           <t>Verify the operating system records time stamps for audit records that meet a minimum granularity of one second for a minimum degree of precision. If it does not, this is a finding.</t>
         </is>
       </c>
-      <c r="K527" s="3" t="inlineStr">
+      <c r="K526" s="3" t="inlineStr">
         <is>
           <t>Red Hat Enterprise Linux 9 supports this requirement and cannot be configured to be out of compliance.
 Red Hat Enterprise Linux 9 inherently meets this requirement.</t>
         </is>
       </c>
-      <c r="L527" s="3" t="n"/>
-      <c r="M527" s="3" t="n"/>
-      <c r="N527" s="3" t="inlineStr">
-        <is>
-          <t>CAT II</t>
-        </is>
-      </c>
-      <c r="O527" s="3" t="n"/>
-      <c r="P527" s="3" t="inlineStr">
+      <c r="L526" s="3" t="n"/>
+      <c r="M526" s="3" t="n"/>
+      <c r="N526" s="3" t="inlineStr">
+        <is>
+          <t>CAT II</t>
+        </is>
+      </c>
+      <c r="O526" s="3" t="n"/>
+      <c r="P526" s="3" t="inlineStr">
         <is>
           <t>Linux kernel audit subsystem always adds a timestamp to each audit buffer used to contain the entire audit log data.
 Function kernel/audit.c:audit_log_start() calls kernel/audit.c:audit_get_stamp() to fetch the timestamp and formats the message into the audit log buffer.</t>
         </is>
       </c>
-      <c r="Q527" s="3" t="inlineStr">
+      <c r="Q526" s="3" t="inlineStr">
         <is>
           <t>The Red Hat Enterprise Linux 9 clock is part of the Linux kernel and is driven by a timer interrupt.
 The "ntp_adjtime" only allows for two modes of operation: "ntp_adjtime" or "adj_nano".</t>
         </is>
       </c>
     </row>
-    <row r="528" ht="130" customHeight="1">
-      <c r="A528" s="2" t="inlineStr">
+    <row r="527" ht="130" customHeight="1">
+      <c r="A527" s="2" t="inlineStr">
         <is>
           <t>SI-11 a</t>
         </is>
       </c>
-      <c r="B528" s="2" t="inlineStr">
+      <c r="B527" s="2" t="inlineStr">
         <is>
           <t>CCI-001312</t>
         </is>
       </c>
-      <c r="C528" s="2" t="inlineStr">
+      <c r="C527" s="2" t="inlineStr">
         <is>
           <t>SRG-OS-000205-GPOS-00083</t>
         </is>
       </c>
-      <c r="D528" s="2" t="inlineStr"/>
-      <c r="E528" s="2" t="inlineStr">
+      <c r="D527" s="2" t="inlineStr"/>
+      <c r="E527" s="2" t="inlineStr">
         <is>
           <t>The operating system must generate error messages that provide information necessary for corrective actions without revealing information that could be exploited by adversaries.</t>
         </is>
       </c>
-      <c r="F528" s="2" t="inlineStr">
+      <c r="F527" s="2" t="inlineStr">
         <is>
           <t>Red Hat Enterprise Linux 9 must generate error messages that provide information necessary for corrective actions without revealing information that could be exploited by adversaries.</t>
         </is>
       </c>
-      <c r="G528" s="2" t="inlineStr">
+      <c r="G527" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve"> Any operating system providing too much information in error messages risks compromising the data and security of the structure, and content of error messages needs to be carefully considered by the organization.
 Organizations carefully consider the structure/content of error messages. The extent to which information systems are able to identify and handle error conditions is guided by organizational policy and operational requirements. Information that could be exploited by adversaries includes, for example, erroneous logon attempts with passwords entered by mistake as the username, mission/business information that can be derived from (if not stated explicitly by) information recorded, and personal information, such as account numbers, social security numbers, and credit card numbers.</t>
         </is>
       </c>
-      <c r="H528" s="2" t="inlineStr">
+      <c r="H527" s="2" t="inlineStr">
         <is>
           <t>Any operating system providing too much information in error messages risks compromising the data and security of the structure, and content of error messages needs to be carefully considered by the organization.
 Organizations carefully consider the structure/content of error messages. The extent to which information systems are able to identify and handle error conditions is guided by organizational policy and operational requirements.
 Information that could be exploited by adversaries includes, for example, erroneous logon attempts with passwords entered by mistake as the username, mission/business information that can be derived from (if not stated explicitly by) information recorded, and personal information, such as account numbers, social security numbers, and credit card numbers.</t>
         </is>
       </c>
-      <c r="I528" s="2" t="inlineStr">
+      <c r="I527" s="2" t="inlineStr">
         <is>
           <t>Applicable - Inherently Met</t>
         </is>
       </c>
-      <c r="J528" s="2" t="inlineStr">
+      <c r="J527" s="2" t="inlineStr">
         <is>
           <t>Verify the operating system generates error messages that provide information necessary for corrective actions without revealing information that could be exploited by adversaries. If it does not, this is a finding.</t>
         </is>
       </c>
-      <c r="K528" s="2" t="inlineStr">
+      <c r="K527" s="2" t="inlineStr">
         <is>
           <t>Red Hat Enterprise Linux 9 supports this requirement and cannot be configured to be out of compliance.
 Red Hat Enterprise Linux 9 inherently meets this requirement.</t>
         </is>
       </c>
+      <c r="L527" s="2" t="n"/>
+      <c r="M527" s="2" t="inlineStr">
+        <is>
+          <t>Red Hat Enterprise Linux 9 inherently meets this requirement.
+No fix is required.</t>
+        </is>
+      </c>
+      <c r="N527" s="2" t="inlineStr">
+        <is>
+          <t>CAT II</t>
+        </is>
+      </c>
+      <c r="O527" s="2" t="n"/>
+      <c r="P527" s="2" t="inlineStr">
+        <is>
+          <t>Common Criteria evaluation.</t>
+        </is>
+      </c>
+      <c r="Q527" s="2" t="inlineStr">
+        <is>
+          <t>Red Hat Enterprise Linux 9 is secure in the event of a failure.
+Authentication and authorizations are still necessary to access the system.</t>
+        </is>
+      </c>
+    </row>
+    <row r="528" ht="130" customHeight="1">
+      <c r="A528" s="2" t="inlineStr">
+        <is>
+          <t>SC-23 (5)</t>
+        </is>
+      </c>
+      <c r="B528" s="2" t="inlineStr">
+        <is>
+          <t>CCI-002470</t>
+        </is>
+      </c>
+      <c r="C528" s="2" t="inlineStr">
+        <is>
+          <t>SRG-OS-000403-GPOS-00182</t>
+        </is>
+      </c>
+      <c r="D528" s="2" t="inlineStr"/>
+      <c r="E528" s="2" t="inlineStr">
+        <is>
+          <t>The operating system must only allow the use of DoD PKI-established certificate authorities for authentication in the establishment of protected sessions to the operating system.</t>
+        </is>
+      </c>
+      <c r="F528" s="2" t="inlineStr">
+        <is>
+          <t>Red Hat Enterprise Linux 9 must only allow the use of DoD PKI-established certificate authorities for authentication in the establishment of protected sessions to Red Hat Enterprise Linux 9.</t>
+        </is>
+      </c>
+      <c r="G528" s="2" t="inlineStr">
+        <is>
+          <t>Untrusted Certificate Authorities (CA) can issue certificates, but they may be issued by organizations or individuals that seek to compromise DoD systems or by organizations with insufficient security controls. If the CA used for verifying the certificate is not a DoD-approved CA, trust of this CA has not been established.
+The DoD will only accept PKI-certificates obtained from a DoD-approved internal or external certificate authority. Reliance on CAs for the establishment of secure sessions includes, for example, the use of SSL/TLS certificates.</t>
+        </is>
+      </c>
+      <c r="H528" s="2" t="inlineStr">
+        <is>
+          <t>Untrusted Certificate Authorities (CA) can issue certificates, but they may be issued by organizations or individuals that seek to compromise DoD systems or by organizations with insufficient security controls. If the CA used for verifying the certificate is not a DoD-approved CA, trust of this CA has not been established.
+The DoD will only accept PKI-certificates obtained from a DoD-approved internal or external certificate authority. Reliance on CAs for the establishment of secure sessions includes, for example, the use of SSL/TLS certificates.</t>
+        </is>
+      </c>
+      <c r="I528" s="2" t="inlineStr">
+        <is>
+          <t>Applicable - Does Not Meet</t>
+        </is>
+      </c>
+      <c r="J528" s="2" t="inlineStr">
+        <is>
+          <t>Verify the operating system only allows the use of DoD PKI-established certificate authorities for verification of the establishment of protected sessions. If it does not, this is a finding.</t>
+        </is>
+      </c>
+      <c r="K528" s="2" t="inlineStr">
+        <is>
+          <t>Red Hat Enterprise Linux 9 does not support this requirement. This is an applicable-does not meet finding.</t>
+        </is>
+      </c>
       <c r="L528" s="2" t="n"/>
       <c r="M528" s="2" t="inlineStr">
         <is>
-          <t>Red Hat Enterprise Linux 9 inherently meets this requirement.
-No fix is required.</t>
+          <t>This requirement is a permanent finding and cannot be fixed. An appropriate mitigation for the system must be implemented, but this finding cannot be considered fixed.</t>
         </is>
       </c>
       <c r="N528" s="2" t="inlineStr">
@@ -42266,153 +42269,75 @@
           <t>CAT II</t>
         </is>
       </c>
-      <c r="O528" s="2" t="n"/>
-      <c r="P528" s="2" t="inlineStr">
-        <is>
-          <t>Common Criteria evaluation.</t>
-        </is>
-      </c>
+      <c r="O528" s="2" t="inlineStr">
+        <is>
+          <t>This item can be mitigated by installing an additional packages/software that is not included in the default install of Red Hat Enterprise Linux 9.
+Although the listed mitigation is supporting the security function, it is not sufficient to reduce the residual risk of this requirement.</t>
+        </is>
+      </c>
+      <c r="P528" s="2" t="n"/>
       <c r="Q528" s="2" t="inlineStr">
         <is>
-          <t>Red Hat Enterprise Linux 9 is secure in the event of a failure.
-Authentication and authorizations are still necessary to access the system.</t>
+          <t>This is a procedural-only requirement that is not enforced by the OS.</t>
         </is>
       </c>
     </row>
     <row r="529" ht="130" customHeight="1">
       <c r="A529" s="2" t="inlineStr">
         <is>
-          <t>SC-23 (5)</t>
+          <t>SC-8,AC-17 (2)</t>
         </is>
       </c>
       <c r="B529" s="2" t="inlineStr">
         <is>
-          <t>CCI-002470</t>
+          <t>CCI-001453</t>
         </is>
       </c>
       <c r="C529" s="2" t="inlineStr">
         <is>
-          <t>SRG-OS-000403-GPOS-00182</t>
-        </is>
-      </c>
-      <c r="D529" s="2" t="inlineStr"/>
+          <t>SRG-OS-000250-GPOS-00093,SRG-OS-000423-GPOS-00187</t>
+        </is>
+      </c>
+      <c r="D529" s="2" t="inlineStr">
+        <is>
+          <t>CCE-86860-4</t>
+        </is>
+      </c>
       <c r="E529" s="2" t="inlineStr">
         <is>
-          <t>The operating system must only allow the use of DoD PKI-established certificate authorities for authentication in the establishment of protected sessions to the operating system.</t>
+          <t>The operating system must protect the confidentiality and integrity of transmitted information.</t>
         </is>
       </c>
       <c r="F529" s="2" t="inlineStr">
         <is>
-          <t>Red Hat Enterprise Linux 9 must only allow the use of DoD PKI-established certificate authorities for authentication in the establishment of protected sessions to Red Hat Enterprise Linux 9.</t>
+          <t>Red Hat Enterprise Linux 9 Must Protect The Confidentiality And Integrity Of Transmitted Information.</t>
         </is>
       </c>
       <c r="G529" s="2" t="inlineStr">
-        <is>
-          <t>Untrusted Certificate Authorities (CA) can issue certificates, but they may be issued by organizations or individuals that seek to compromise DoD systems or by organizations with insufficient security controls. If the CA used for verifying the certificate is not a DoD-approved CA, trust of this CA has not been established.
-The DoD will only accept PKI-certificates obtained from a DoD-approved internal or external certificate authority. Reliance on CAs for the establishment of secure sessions includes, for example, the use of SSL/TLS certificates.</t>
-        </is>
-      </c>
-      <c r="H529" s="2" t="inlineStr">
-        <is>
-          <t>Untrusted Certificate Authorities (CA) can issue certificates, but they may be issued by organizations or individuals that seek to compromise DoD systems or by organizations with insufficient security controls. If the CA used for verifying the certificate is not a DoD-approved CA, trust of this CA has not been established.
-The DoD will only accept PKI-certificates obtained from a DoD-approved internal or external certificate authority. Reliance on CAs for the establishment of secure sessions includes, for example, the use of SSL/TLS certificates.</t>
-        </is>
-      </c>
-      <c r="I529" s="2" t="inlineStr">
-        <is>
-          <t>Applicable - Does Not Meet</t>
-        </is>
-      </c>
-      <c r="J529" s="2" t="inlineStr">
-        <is>
-          <t>Verify the operating system only allows the use of DoD PKI-established certificate authorities for verification of the establishment of protected sessions. If it does not, this is a finding.</t>
-        </is>
-      </c>
-      <c r="K529" s="2" t="inlineStr">
-        <is>
-          <t>Red Hat Enterprise Linux 9 does not support this requirement. This is an applicable-does not meet finding.</t>
-        </is>
-      </c>
-      <c r="L529" s="2" t="n"/>
-      <c r="M529" s="2" t="inlineStr">
-        <is>
-          <t>This requirement is a permanent finding and cannot be fixed. An appropriate mitigation for the system must be implemented, but this finding cannot be considered fixed.</t>
-        </is>
-      </c>
-      <c r="N529" s="2" t="inlineStr">
-        <is>
-          <t>CAT II</t>
-        </is>
-      </c>
-      <c r="O529" s="2" t="inlineStr">
-        <is>
-          <t>This item can be mitigated by installing an additional packages/software that is not included in the default install of Red Hat Enterprise Linux 9.
-Although the listed mitigation is supporting the security function, it is not sufficient to reduce the residual risk of this requirement.</t>
-        </is>
-      </c>
-      <c r="P529" s="2" t="n"/>
-      <c r="Q529" s="2" t="inlineStr">
-        <is>
-          <t>This is a procedural-only requirement that is not enforced by the OS.</t>
-        </is>
-      </c>
-    </row>
-    <row r="530" ht="130" customHeight="1">
-      <c r="A530" s="2" t="inlineStr">
-        <is>
-          <t>AC-17 (2),SC-8</t>
-        </is>
-      </c>
-      <c r="B530" s="2" t="inlineStr">
-        <is>
-          <t>CCI-001453</t>
-        </is>
-      </c>
-      <c r="C530" s="2" t="inlineStr">
-        <is>
-          <t>SRG-OS-000250-GPOS-00093,SRG-OS-000423-GPOS-00187</t>
-        </is>
-      </c>
-      <c r="D530" s="2" t="inlineStr">
-        <is>
-          <t>CCE-86860-4</t>
-        </is>
-      </c>
-      <c r="E530" s="2" t="inlineStr">
-        <is>
-          <t>The operating system must protect the confidentiality and integrity of transmitted information.</t>
-        </is>
-      </c>
-      <c r="F530" s="2" t="inlineStr">
-        <is>
-          <t>Red Hat Enterprise Linux 9 Must Protect The Confidentiality And Integrity Of Transmitted Information.</t>
-        </is>
-      </c>
-      <c r="G530" s="2" t="inlineStr">
         <is>
           <t>Without protection of the transmitted information, confidentiality and integrity may be compromised because unprotected communications can be intercepted and either read or altered. 
 This requirement applies to both internal and external networks and all types of information system components from which information can be transmitted (e.g., servers, mobile devices, notebook computers, printers, copiers, scanners, and facsimile machines). Communication paths outside the physical protection of a controlled boundary are exposed to the possibility of interception and modification. 
 Protecting the confidentiality and integrity of organizational information can be accomplished by physical means (e.g., employing physical distribution systems) or by logical means (e.g., employing cryptographic techniques). If physical means of protection are employed, then logical means (cryptography) do not have to be employed, and vice versa.</t>
         </is>
       </c>
-      <c r="H530" s="2" t="inlineStr">
+      <c r="H529" s="2" t="inlineStr">
         <is>
           <t>Overriding the system crypto policy makes the behavior of the GnuTLS
 library violate expectations, and makes system configuration more
 fragmented.</t>
         </is>
       </c>
-      <c r="I530" s="2" t="inlineStr">
-        <is>
-          <t>Applicable - Configurable</t>
-        </is>
-      </c>
-      <c r="J530" s="2" t="inlineStr">
+      <c r="I529" s="2" t="inlineStr">
+        <is>
+          <t>Applicable - Configurable</t>
+        </is>
+      </c>
+      <c r="J529" s="2" t="inlineStr">
         <is>
           <t>Verify the operating system protects the confidentiality and integrity of transmitted information. If it does not, this is a finding.</t>
         </is>
       </c>
-      <c r="K530" s="2" t="inlineStr">
+      <c r="K529" s="2" t="inlineStr">
         <is>
           <t>To verify if GnuTLS uses defined DoD-approved TLS Crypto Policy, run:
  $ sudo grep
@@ -42421,62 +42346,62 @@
 If cryptographic policy for gnutls is not configured or is configured incorrectly, then this is a finding.</t>
         </is>
       </c>
-      <c r="L530" s="2" t="n"/>
-      <c r="M530" s="2" t="inlineStr">
+      <c r="L529" s="2" t="n"/>
+      <c r="M529" s="2" t="inlineStr">
         <is>
           <t>Configure the Red Hat Enterprise Linux 9 GnuTLS library to use only DoD-approved encryption by adding the following line to "/etc/crypto-policies/back-ends/gnutls.config":
 +VERS-ALL:-VERS-DTLS0.9:-VERS-SSL3.0:-VERS-TLS1.0:-VERS-TLS1.1:-VERS-DTLS1.0
 A reboot is required for the changes to take effect.</t>
         </is>
       </c>
-      <c r="N530" s="2" t="inlineStr">
-        <is>
-          <t>CAT II</t>
-        </is>
-      </c>
-      <c r="O530" s="2" t="n"/>
-      <c r="P530" s="2" t="n"/>
-      <c r="Q530" s="2" t="n"/>
-    </row>
-    <row r="531" ht="130" customHeight="1">
-      <c r="A531" s="2" t="inlineStr">
+      <c r="N529" s="2" t="inlineStr">
+        <is>
+          <t>CAT II</t>
+        </is>
+      </c>
+      <c r="O529" s="2" t="n"/>
+      <c r="P529" s="2" t="n"/>
+      <c r="Q529" s="2" t="n"/>
+    </row>
+    <row r="530" ht="130" customHeight="1">
+      <c r="A530" s="2" t="inlineStr">
         <is>
           <t>MA-4 c</t>
         </is>
       </c>
-      <c r="B531" s="2" t="inlineStr">
+      <c r="B530" s="2" t="inlineStr">
         <is>
           <t>CCI-000877</t>
         </is>
       </c>
-      <c r="C531" s="2" t="inlineStr">
+      <c r="C530" s="2" t="inlineStr">
         <is>
           <t>SRG-OS-000125-GPOS-00065</t>
         </is>
       </c>
-      <c r="D531" s="2" t="inlineStr">
+      <c r="D530" s="2" t="inlineStr">
         <is>
           <t>CCE-86722-6</t>
         </is>
       </c>
-      <c r="E531" s="2" t="inlineStr">
+      <c r="E530" s="2" t="inlineStr">
         <is>
           <t>The operating system must employ strong authenticators in the establishment of nonlocal maintenance and diagnostic sessions.</t>
         </is>
       </c>
-      <c r="F531" s="2" t="inlineStr">
+      <c r="F530" s="2" t="inlineStr">
         <is>
           <t>Red Hat Enterprise Linux 9 Must Employ Strong Authenticators In The Establishment Of Nonlocal Maintenance And Diagnostic Sessions.</t>
         </is>
       </c>
-      <c r="G531" s="2" t="inlineStr">
+      <c r="G530" s="2" t="inlineStr">
         <is>
           <t>If maintenance tools are used by unauthorized personnel, they may accidentally or intentionally damage or compromise the system. The act of managing systems and applications includes the ability to access sensitive application information, such as system configuration details, diagnostic information, user information, and potentially sensitive application data.
 Some maintenance and test tools are either standalone devices with their own operating systems or are applications bundled with an operating system.
 Nonlocal maintenance and diagnostic activities are those activities conducted by individuals communicating through a network, either an external network (e.g., the Internet) or an internal network. Local maintenance and diagnostic activities are those activities carried out by individuals physically present at the information system or information system component and not communicating across a network connection. Typically, strong authentication requires authenticators that are resistant to replay attacks and employ multifactor authentication. Strong authenticators include, for example, PKI where certificates are stored on a token protected by a password, passphrase, or biometric.</t>
         </is>
       </c>
-      <c r="H531" s="2" t="inlineStr">
+      <c r="H530" s="2" t="inlineStr">
         <is>
           <t>When UsePAM is set to yes, PAM runs through account and session types properly. This is
 important if you want to restrict access to services based off of IP, time or other factors of
@@ -42484,17 +42409,17 @@
 on login or disallow access to the server.</t>
         </is>
       </c>
-      <c r="I531" s="2" t="inlineStr">
-        <is>
-          <t>Applicable - Configurable</t>
-        </is>
-      </c>
-      <c r="J531" s="2" t="inlineStr">
+      <c r="I530" s="2" t="inlineStr">
+        <is>
+          <t>Applicable - Configurable</t>
+        </is>
+      </c>
+      <c r="J530" s="2" t="inlineStr">
         <is>
           <t>Verify the operating system employs strong authenticators in the establishment of nonlocal maintenance and diagnostic sessions. If it does not, this is a finding.</t>
         </is>
       </c>
-      <c r="K531" s="2" t="inlineStr">
+      <c r="K530" s="2" t="inlineStr">
         <is>
           <t>To determine how the SSH daemon's "UsePAM" option is set, run the following command:
  $ sudo grep -i UsePAM /etc/ssh/sshd_config.d/00-complianceascode-hardening.conf 
@@ -42502,8 +42427,8 @@
 If the required value is not set, then this is a finding.</t>
         </is>
       </c>
-      <c r="L531" s="2" t="n"/>
-      <c r="M531" s="2" t="inlineStr">
+      <c r="L530" s="2" t="n"/>
+      <c r="M530" s="2" t="inlineStr">
         <is>
           <t>To configure the system add or modify the following line in "/etc/ssh/sshd_config".
 UsePAM yes
@@ -42511,52 +42436,52 @@
 $ sudo systemctl restart sshd.service</t>
         </is>
       </c>
-      <c r="N531" s="2" t="inlineStr">
-        <is>
-          <t>CAT II</t>
-        </is>
-      </c>
-      <c r="O531" s="2" t="n"/>
-      <c r="P531" s="2" t="n"/>
-      <c r="Q531" s="2" t="n"/>
-    </row>
-    <row r="532" ht="130" customHeight="1">
-      <c r="A532" s="3" t="inlineStr">
+      <c r="N530" s="2" t="inlineStr">
+        <is>
+          <t>CAT II</t>
+        </is>
+      </c>
+      <c r="O530" s="2" t="n"/>
+      <c r="P530" s="2" t="n"/>
+      <c r="Q530" s="2" t="n"/>
+    </row>
+    <row r="531" ht="130" customHeight="1">
+      <c r="A531" s="3" t="inlineStr">
         <is>
           <t>SC-13</t>
         </is>
       </c>
-      <c r="B532" s="3" t="inlineStr">
+      <c r="B531" s="3" t="inlineStr">
         <is>
           <t>CCI-000068,CCI-000803,CCI-002450</t>
         </is>
       </c>
-      <c r="C532" s="3" t="inlineStr">
+      <c r="C531" s="3" t="inlineStr">
         <is>
           <t>SRG-OS-000478-GPOS-00223</t>
         </is>
       </c>
-      <c r="D532" s="3" t="inlineStr">
+      <c r="D531" s="3" t="inlineStr">
         <is>
           <t>CCE-86547-7</t>
         </is>
       </c>
-      <c r="E532" s="3" t="inlineStr">
+      <c r="E531" s="3" t="inlineStr">
         <is>
           <t>The operating system must implement NIST FIPS-validated cryptography for the following: to provision digital signatures, to generate cryptographic hashes, and to protect unclassified information requiring confidentiality and cryptographic protection in accordance with applicable federal laws, Executive Orders, directives, policies, regulations, and standards.</t>
         </is>
       </c>
-      <c r="F532" s="3" t="inlineStr">
+      <c r="F531" s="3" t="inlineStr">
         <is>
           <t>Red Hat Enterprise Linux 9 Must Implement Nist Fips-Validated Cryptography For The Following: To Provision Digital Signatures, To Generate Cryptographic Hashes, And To Protect Unclassified Information Requiring Confidentiality And Cryptographic Protection In Accordance With Applicable Federal Laws, Executive Orders, Directives, Policies, Regulations, And Standards.</t>
         </is>
       </c>
-      <c r="G532" s="3" t="inlineStr">
+      <c r="G531" s="3" t="inlineStr">
         <is>
           <t>Use of weak or untested encryption algorithms undermines the purposes of utilizing encryption to protect data. The operating system must implement cryptographic modules adhering to the higher standards approved by the federal government since this provides assurance they have been tested and validated.</t>
         </is>
       </c>
-      <c r="H532" s="3" t="inlineStr">
+      <c r="H531" s="3" t="inlineStr">
         <is>
           <t>Use of weak or untested encryption algorithms undermines the purposes of utilizing encryption to
 protect data. The operating system must implement cryptographic modules adhering to the higher
@@ -42564,17 +42489,17 @@
 and validated.</t>
         </is>
       </c>
-      <c r="I532" s="3" t="inlineStr">
-        <is>
-          <t>Applicable - Configurable</t>
-        </is>
-      </c>
-      <c r="J532" s="3" t="inlineStr">
+      <c r="I531" s="3" t="inlineStr">
+        <is>
+          <t>Applicable - Configurable</t>
+        </is>
+      </c>
+      <c r="J531" s="3" t="inlineStr">
         <is>
           <t>Verify the operating system implements NIST FIPS-validated cryptography for the following: to provision digital signatures, to generate cryptographic hashes, and to protect unclassified information requiring confidentiality and cryptographic protection in accordance with applicable federal laws, Executive Orders, directives, policies, regulations, and standards. If it does not, this is a finding.</t>
         </is>
       </c>
-      <c r="K532" s="3" t="inlineStr">
+      <c r="K531" s="3" t="inlineStr">
         <is>
           <t>To verify that the Dracut FIPS module is enabled, run the following command:
 "grep "add_dracutmodules" /etc/dracut.conf.d/40-fips.conf"
@@ -42583,72 +42508,72 @@
 If the Dracut FIPS module is not enabled, then this is a finding.</t>
         </is>
       </c>
-      <c r="L532" s="3" t="n"/>
-      <c r="M532" s="3" t="inlineStr"/>
-      <c r="N532" s="3" t="inlineStr">
-        <is>
-          <t>CAT II</t>
-        </is>
-      </c>
-      <c r="O532" s="3" t="n"/>
-      <c r="P532" s="3" t="n"/>
-      <c r="Q532" s="3" t="n"/>
-    </row>
-    <row r="533" ht="130" customHeight="1">
-      <c r="A533" s="3" t="inlineStr">
+      <c r="L531" s="3" t="n"/>
+      <c r="M531" s="3" t="inlineStr"/>
+      <c r="N531" s="3" t="inlineStr">
+        <is>
+          <t>CAT II</t>
+        </is>
+      </c>
+      <c r="O531" s="3" t="n"/>
+      <c r="P531" s="3" t="n"/>
+      <c r="Q531" s="3" t="n"/>
+    </row>
+    <row r="532" ht="130" customHeight="1">
+      <c r="A532" s="3" t="inlineStr">
         <is>
           <t>AC-17 (2)</t>
         </is>
       </c>
-      <c r="B533" s="3" t="inlineStr">
+      <c r="B532" s="3" t="inlineStr">
         <is>
           <t>CCI-001453</t>
         </is>
       </c>
-      <c r="C533" s="3" t="inlineStr">
+      <c r="C532" s="3" t="inlineStr">
         <is>
           <t>SRG-OS-000250-GPOS-00093</t>
         </is>
       </c>
-      <c r="D533" s="3" t="inlineStr">
+      <c r="D532" s="3" t="inlineStr">
         <is>
           <t>CCE-83452-3</t>
         </is>
       </c>
-      <c r="E533" s="3" t="inlineStr">
+      <c r="E532" s="3" t="inlineStr">
         <is>
           <t>The operating system must implement cryptography to protect the integrity of remote access sessions.</t>
         </is>
       </c>
-      <c r="F533" s="3" t="inlineStr">
+      <c r="F532" s="3" t="inlineStr">
         <is>
           <t>Red Hat Enterprise Linux 9 Must Implement Cryptography To Protect The Integrity Of Remote Access Sessions.</t>
         </is>
       </c>
-      <c r="G533" s="3" t="inlineStr">
+      <c r="G532" s="3" t="inlineStr">
         <is>
           <t>Without cryptographic integrity protections, information can be altered by unauthorized users without detection.
 Remote access (e.g., RDP) is access to DoD nonpublic information systems by an authorized user (or an information system) communicating through an external, non-organization-controlled network. Remote access methods include, for example, dial-up, broadband, and wireless.
 Cryptographic mechanisms used for protecting the integrity of information include, for example, signed hash functions using asymmetric cryptography enabling distribution of the public key to verify the hash information while maintaining the confidentiality of the secret key used to generate the hash.</t>
         </is>
       </c>
-      <c r="H533" s="3" t="inlineStr">
+      <c r="H532" s="3" t="inlineStr">
         <is>
           <t>Overriding the system crypto policy makes the behavior of the Java runtime violates expectations,
 and makes system configuration more fragmented.</t>
         </is>
       </c>
-      <c r="I533" s="3" t="inlineStr">
-        <is>
-          <t>Applicable - Configurable</t>
-        </is>
-      </c>
-      <c r="J533" s="3" t="inlineStr">
+      <c r="I532" s="3" t="inlineStr">
+        <is>
+          <t>Applicable - Configurable</t>
+        </is>
+      </c>
+      <c r="J532" s="3" t="inlineStr">
         <is>
           <t>Verify the operating system implements cryptography to protect the integrity of remote access sessions. If it does not, this is a finding.</t>
         </is>
       </c>
-      <c r="K533" s="3" t="inlineStr">
+      <c r="K532" s="3" t="inlineStr">
         <is>
           <t>To verify that OpenSSL uses the system crypto policy, check out that the OpenSSL config file
  /etc/pki/tls/openssl.cnf  contains the  [ crypto_policy ]  section with the
@@ -42658,72 +42583,72 @@
 or that the section doesn't have the  .include /etc/crypto-policies/back-ends/opensslcnf.config  directive, then this is a finding.</t>
         </is>
       </c>
-      <c r="L533" s="3" t="n"/>
-      <c r="M533" s="3" t="inlineStr"/>
-      <c r="N533" s="3" t="inlineStr">
-        <is>
-          <t>CAT II</t>
-        </is>
-      </c>
-      <c r="O533" s="3" t="n"/>
-      <c r="P533" s="3" t="n"/>
-      <c r="Q533" s="3" t="n"/>
-    </row>
-    <row r="534" ht="130" customHeight="1">
-      <c r="A534" s="3" t="inlineStr">
+      <c r="L532" s="3" t="n"/>
+      <c r="M532" s="3" t="inlineStr"/>
+      <c r="N532" s="3" t="inlineStr">
+        <is>
+          <t>CAT II</t>
+        </is>
+      </c>
+      <c r="O532" s="3" t="n"/>
+      <c r="P532" s="3" t="n"/>
+      <c r="Q532" s="3" t="n"/>
+    </row>
+    <row r="533" ht="130" customHeight="1">
+      <c r="A533" s="3" t="inlineStr">
         <is>
           <t>AC-17 (2)</t>
         </is>
       </c>
-      <c r="B534" s="3" t="inlineStr">
+      <c r="B533" s="3" t="inlineStr">
         <is>
           <t>CCI-001453</t>
         </is>
       </c>
-      <c r="C534" s="3" t="inlineStr">
+      <c r="C533" s="3" t="inlineStr">
         <is>
           <t>SRG-OS-000250-GPOS-00093</t>
         </is>
       </c>
-      <c r="D534" s="3" t="inlineStr">
+      <c r="D533" s="3" t="inlineStr">
         <is>
           <t>CCE-83448-1</t>
         </is>
       </c>
-      <c r="E534" s="3" t="inlineStr">
+      <c r="E533" s="3" t="inlineStr">
         <is>
           <t>The operating system must implement cryptography to protect the integrity of remote access sessions.</t>
         </is>
       </c>
-      <c r="F534" s="3" t="inlineStr">
+      <c r="F533" s="3" t="inlineStr">
         <is>
           <t>Red Hat Enterprise Linux 9 Must Implement Cryptography To Protect The Integrity Of Remote Access Sessions.</t>
         </is>
       </c>
-      <c r="G534" s="3" t="inlineStr">
+      <c r="G533" s="3" t="inlineStr">
         <is>
           <t>Without cryptographic integrity protections, information can be altered by unauthorized users without detection.
 Remote access (e.g., RDP) is access to DoD nonpublic information systems by an authorized user (or an information system) communicating through an external, non-organization-controlled network. Remote access methods include, for example, dial-up, broadband, and wireless.
 Cryptographic mechanisms used for protecting the integrity of information include, for example, signed hash functions using asymmetric cryptography enabling distribution of the public key to verify the hash information while maintaining the confidentiality of the secret key used to generate the hash.</t>
         </is>
       </c>
-      <c r="H534" s="3" t="inlineStr">
+      <c r="H533" s="3" t="inlineStr">
         <is>
           <t>Without cryptographic integrity protections, information can be altered by
 unauthorized users without detection.</t>
         </is>
       </c>
-      <c r="I534" s="3" t="inlineStr">
-        <is>
-          <t>Applicable - Configurable</t>
-        </is>
-      </c>
-      <c r="J534" s="3" t="inlineStr">
+      <c r="I533" s="3" t="inlineStr">
+        <is>
+          <t>Applicable - Configurable</t>
+        </is>
+      </c>
+      <c r="J533" s="3" t="inlineStr">
         <is>
           <t>Verify the operating system implements cryptography to protect the integrity of remote access sessions. If it does not, this is a finding.</t>
         </is>
       </c>
-      <c r="K534" s="3" t="inlineStr">
+      <c r="K533" s="3" t="inlineStr">
         <is>
           <t>To verify if the OpenSSL uses defined TLS Crypto Policy, run:
  $ grep -P '^(TLS\.)?MinProtocol' /etc/crypto-policies/back-ends/opensslcnf.config 
@@ -42732,6 +42657,78 @@
 If cryptographic policy for openssl is not configured or is configured incorrectly, then this is a finding.</t>
         </is>
       </c>
+      <c r="L533" s="3" t="n"/>
+      <c r="M533" s="3" t="inlineStr"/>
+      <c r="N533" s="3" t="inlineStr">
+        <is>
+          <t>CAT II</t>
+        </is>
+      </c>
+      <c r="O533" s="3" t="n"/>
+      <c r="P533" s="3" t="n"/>
+      <c r="Q533" s="3" t="n"/>
+    </row>
+    <row r="534" ht="130" customHeight="1">
+      <c r="A534" s="3" t="inlineStr">
+        <is>
+          <t>AC-17 (2)</t>
+        </is>
+      </c>
+      <c r="B534" s="3" t="inlineStr">
+        <is>
+          <t>CCI-001453</t>
+        </is>
+      </c>
+      <c r="C534" s="3" t="inlineStr">
+        <is>
+          <t>SRG-OS-000250-GPOS-00093</t>
+        </is>
+      </c>
+      <c r="D534" s="3" t="inlineStr">
+        <is>
+          <t>CCE-83445-7</t>
+        </is>
+      </c>
+      <c r="E534" s="3" t="inlineStr">
+        <is>
+          <t>The operating system must implement cryptography to protect the integrity of remote access sessions.</t>
+        </is>
+      </c>
+      <c r="F534" s="3" t="inlineStr">
+        <is>
+          <t>Red Hat Enterprise Linux 9 Must Implement Cryptography To Protect The Integrity Of Remote Access Sessions.</t>
+        </is>
+      </c>
+      <c r="G534" s="3" t="inlineStr">
+        <is>
+          <t>Without cryptographic integrity protections, information can be altered by unauthorized users without detection.
+Remote access (e.g., RDP) is access to DoD nonpublic information systems by an authorized user (or an information system) communicating through an external, non-organization-controlled network. Remote access methods include, for example, dial-up, broadband, and wireless.
+Cryptographic mechanisms used for protecting the integrity of information include, for example, signed hash functions using asymmetric cryptography enabling distribution of the public key to verify the hash information while maintaining the confidentiality of the secret key used to generate the hash.</t>
+        </is>
+      </c>
+      <c r="H534" s="3" t="inlineStr">
+        <is>
+          <t>Overriding the system crypto policy makes the behavior of the SSH service violate expectations,
+and makes system configuration more fragmented.</t>
+        </is>
+      </c>
+      <c r="I534" s="3" t="inlineStr">
+        <is>
+          <t>Applicable - Configurable</t>
+        </is>
+      </c>
+      <c r="J534" s="3" t="inlineStr">
+        <is>
+          <t>Verify the operating system implements cryptography to protect the integrity of remote access sessions. If it does not, this is a finding.</t>
+        </is>
+      </c>
+      <c r="K534" s="3" t="inlineStr">
+        <is>
+          <t>Check that the "CRYPTO_POLICY" variable is not set or is commented in the
+"/etc/sysconfig/sshd".
+If the CRYPTO_POLICY variable is not set or is commented in the /etc/sysconfig/sshd, then this is a finding.</t>
+        </is>
+      </c>
       <c r="L534" s="3" t="n"/>
       <c r="M534" s="3" t="inlineStr"/>
       <c r="N534" s="3" t="inlineStr">
@@ -42761,7 +42758,7 @@
       </c>
       <c r="D535" s="3" t="inlineStr">
         <is>
-          <t>CCE-83445-7</t>
+          <t>CCE-90125-6</t>
         </is>
       </c>
       <c r="E535" s="3" t="inlineStr">
@@ -42782,78 +42779,6 @@
         </is>
       </c>
       <c r="H535" s="3" t="inlineStr">
-        <is>
-          <t>Overriding the system crypto policy makes the behavior of the SSH service violate expectations,
-and makes system configuration more fragmented.</t>
-        </is>
-      </c>
-      <c r="I535" s="3" t="inlineStr">
-        <is>
-          <t>Applicable - Configurable</t>
-        </is>
-      </c>
-      <c r="J535" s="3" t="inlineStr">
-        <is>
-          <t>Verify the operating system implements cryptography to protect the integrity of remote access sessions. If it does not, this is a finding.</t>
-        </is>
-      </c>
-      <c r="K535" s="3" t="inlineStr">
-        <is>
-          <t>Check that the "CRYPTO_POLICY" variable is not set or is commented in the
-"/etc/sysconfig/sshd".
-If the CRYPTO_POLICY variable is not set or is commented in the /etc/sysconfig/sshd, then this is a finding.</t>
-        </is>
-      </c>
-      <c r="L535" s="3" t="n"/>
-      <c r="M535" s="3" t="inlineStr"/>
-      <c r="N535" s="3" t="inlineStr">
-        <is>
-          <t>CAT II</t>
-        </is>
-      </c>
-      <c r="O535" s="3" t="n"/>
-      <c r="P535" s="3" t="n"/>
-      <c r="Q535" s="3" t="n"/>
-    </row>
-    <row r="536" ht="130" customHeight="1">
-      <c r="A536" s="3" t="inlineStr">
-        <is>
-          <t>AC-17 (2)</t>
-        </is>
-      </c>
-      <c r="B536" s="3" t="inlineStr">
-        <is>
-          <t>CCI-001453</t>
-        </is>
-      </c>
-      <c r="C536" s="3" t="inlineStr">
-        <is>
-          <t>SRG-OS-000250-GPOS-00093</t>
-        </is>
-      </c>
-      <c r="D536" s="3" t="inlineStr">
-        <is>
-          <t>CCE-90125-6</t>
-        </is>
-      </c>
-      <c r="E536" s="3" t="inlineStr">
-        <is>
-          <t>The operating system must implement cryptography to protect the integrity of remote access sessions.</t>
-        </is>
-      </c>
-      <c r="F536" s="3" t="inlineStr">
-        <is>
-          <t>Red Hat Enterprise Linux 9 Must Implement Cryptography To Protect The Integrity Of Remote Access Sessions.</t>
-        </is>
-      </c>
-      <c r="G536" s="3" t="inlineStr">
-        <is>
-          <t>Without cryptographic integrity protections, information can be altered by unauthorized users without detection.
-Remote access (e.g., RDP) is access to DoD nonpublic information systems by an authorized user (or an information system) communicating through an external, non-organization-controlled network. Remote access methods include, for example, dial-up, broadband, and wireless.
-Cryptographic mechanisms used for protecting the integrity of information include, for example, signed hash functions using asymmetric cryptography enabling distribution of the public key to verify the hash information while maintaining the confidentiality of the secret key used to generate the hash.</t>
-        </is>
-      </c>
-      <c r="H536" s="3" t="inlineStr">
         <is>
           <t>Overriding the system crypto policy makes the behavior of the OpenSSH client
 violate expectations, and makes system configuration more fragmented. By
@@ -42862,17 +42787,17 @@
 strongest cipher for securing SSH connections.</t>
         </is>
       </c>
-      <c r="I536" s="3" t="inlineStr">
-        <is>
-          <t>Applicable - Configurable</t>
-        </is>
-      </c>
-      <c r="J536" s="3" t="inlineStr">
+      <c r="I535" s="3" t="inlineStr">
+        <is>
+          <t>Applicable - Configurable</t>
+        </is>
+      </c>
+      <c r="J535" s="3" t="inlineStr">
         <is>
           <t>Verify the operating system implements cryptography to protect the integrity of remote access sessions. If it does not, this is a finding.</t>
         </is>
       </c>
-      <c r="K536" s="3" t="inlineStr">
+      <c r="K535" s="3" t="inlineStr">
         <is>
           <t>To verify if the OpenSSH client uses defined Cipher suite in the Crypto Policy, run:
  $ grep -i ciphers /etc/crypto-policies/back-ends/openssh.config 
@@ -42881,56 +42806,56 @@
 If Crypto Policy for OpenSSH client is not configured correctly, then this is a finding.</t>
         </is>
       </c>
-      <c r="L536" s="3" t="n"/>
-      <c r="M536" s="3" t="inlineStr"/>
-      <c r="N536" s="3" t="inlineStr">
-        <is>
-          <t>CAT II</t>
-        </is>
-      </c>
-      <c r="O536" s="3" t="n"/>
-      <c r="P536" s="3" t="n"/>
-      <c r="Q536" s="3" t="n"/>
-    </row>
-    <row r="537" ht="130" customHeight="1">
-      <c r="A537" s="3" t="inlineStr">
+      <c r="L535" s="3" t="n"/>
+      <c r="M535" s="3" t="inlineStr"/>
+      <c r="N535" s="3" t="inlineStr">
+        <is>
+          <t>CAT II</t>
+        </is>
+      </c>
+      <c r="O535" s="3" t="n"/>
+      <c r="P535" s="3" t="n"/>
+      <c r="Q535" s="3" t="n"/>
+    </row>
+    <row r="536" ht="130" customHeight="1">
+      <c r="A536" s="3" t="inlineStr">
         <is>
           <t>AC-17 (2)</t>
         </is>
       </c>
-      <c r="B537" s="3" t="inlineStr">
+      <c r="B536" s="3" t="inlineStr">
         <is>
           <t>CCI-001453</t>
         </is>
       </c>
-      <c r="C537" s="3" t="inlineStr">
+      <c r="C536" s="3" t="inlineStr">
         <is>
           <t>SRG-OS-000250-GPOS-00093</t>
         </is>
       </c>
-      <c r="D537" s="3" t="inlineStr">
+      <c r="D536" s="3" t="inlineStr">
         <is>
           <t>CCE-87332-3</t>
         </is>
       </c>
-      <c r="E537" s="3" t="inlineStr">
+      <c r="E536" s="3" t="inlineStr">
         <is>
           <t>The operating system must implement cryptography to protect the integrity of remote access sessions.</t>
         </is>
       </c>
-      <c r="F537" s="3" t="inlineStr">
+      <c r="F536" s="3" t="inlineStr">
         <is>
           <t>Red Hat Enterprise Linux 9 Must Implement Cryptography To Protect The Integrity Of Remote Access Sessions.</t>
         </is>
       </c>
-      <c r="G537" s="3" t="inlineStr">
+      <c r="G536" s="3" t="inlineStr">
         <is>
           <t>Without cryptographic integrity protections, information can be altered by unauthorized users without detection.
 Remote access (e.g., RDP) is access to DoD nonpublic information systems by an authorized user (or an information system) communicating through an external, non-organization-controlled network. Remote access methods include, for example, dial-up, broadband, and wireless.
 Cryptographic mechanisms used for protecting the integrity of information include, for example, signed hash functions using asymmetric cryptography enabling distribution of the public key to verify the hash information while maintaining the confidentiality of the secret key used to generate the hash.</t>
         </is>
       </c>
-      <c r="H537" s="3" t="inlineStr">
+      <c r="H536" s="3" t="inlineStr">
         <is>
           <t>Overriding the system crypto policy makes the behavior of the OpenSSH server
 violate expectations, and makes system configuration more fragmented. By
@@ -42939,17 +42864,17 @@
 strongest cipher for securing SSH connections.</t>
         </is>
       </c>
-      <c r="I537" s="3" t="inlineStr">
-        <is>
-          <t>Applicable - Configurable</t>
-        </is>
-      </c>
-      <c r="J537" s="3" t="inlineStr">
+      <c r="I536" s="3" t="inlineStr">
+        <is>
+          <t>Applicable - Configurable</t>
+        </is>
+      </c>
+      <c r="J536" s="3" t="inlineStr">
         <is>
           <t>Verify the operating system implements cryptography to protect the integrity of remote access sessions. If it does not, this is a finding.</t>
         </is>
       </c>
-      <c r="K537" s="3" t="inlineStr">
+      <c r="K536" s="3" t="inlineStr">
         <is>
           <t>To verify if the OpenSSH server uses defined ciphers in the Crypto Policy, run:
  $ grep -Po '(-oCiphers=\S+)' /etc/crypto-policies/back-ends/opensshserver.config 
@@ -42958,73 +42883,73 @@
 If Crypto Policy for OpenSSH Server is not configured correctly, then this is a finding.</t>
         </is>
       </c>
-      <c r="L537" s="3" t="n"/>
-      <c r="M537" s="3" t="inlineStr"/>
-      <c r="N537" s="3" t="inlineStr">
-        <is>
-          <t>CAT II</t>
-        </is>
-      </c>
-      <c r="O537" s="3" t="n"/>
-      <c r="P537" s="3" t="n"/>
-      <c r="Q537" s="3" t="n"/>
-    </row>
-    <row r="538" ht="130" customHeight="1">
-      <c r="A538" s="3" t="inlineStr">
+      <c r="L536" s="3" t="n"/>
+      <c r="M536" s="3" t="inlineStr"/>
+      <c r="N536" s="3" t="inlineStr">
+        <is>
+          <t>CAT II</t>
+        </is>
+      </c>
+      <c r="O536" s="3" t="n"/>
+      <c r="P536" s="3" t="n"/>
+      <c r="Q536" s="3" t="n"/>
+    </row>
+    <row r="537" ht="130" customHeight="1">
+      <c r="A537" s="3" t="inlineStr">
         <is>
           <t>AC-17 (2)</t>
         </is>
       </c>
-      <c r="B538" s="3" t="inlineStr">
+      <c r="B537" s="3" t="inlineStr">
         <is>
           <t>CCI-001453</t>
         </is>
       </c>
-      <c r="C538" s="3" t="inlineStr">
+      <c r="C537" s="3" t="inlineStr">
         <is>
           <t>SRG-OS-000250-GPOS-00093</t>
         </is>
       </c>
-      <c r="D538" s="3" t="inlineStr">
+      <c r="D537" s="3" t="inlineStr">
         <is>
           <t>CCE-86208-6</t>
         </is>
       </c>
-      <c r="E538" s="3" t="inlineStr">
+      <c r="E537" s="3" t="inlineStr">
         <is>
           <t>The operating system must implement cryptography to protect the integrity of remote access sessions.</t>
         </is>
       </c>
-      <c r="F538" s="3" t="inlineStr">
+      <c r="F537" s="3" t="inlineStr">
         <is>
           <t>Red Hat Enterprise Linux 9 Must Implement Cryptography To Protect The Integrity Of Remote Access Sessions.</t>
         </is>
       </c>
-      <c r="G538" s="3" t="inlineStr">
+      <c r="G537" s="3" t="inlineStr">
         <is>
           <t>Without cryptographic integrity protections, information can be altered by unauthorized users without detection.
 Remote access (e.g., RDP) is access to DoD nonpublic information systems by an authorized user (or an information system) communicating through an external, non-organization-controlled network. Remote access methods include, for example, dial-up, broadband, and wireless.
 Cryptographic mechanisms used for protecting the integrity of information include, for example, signed hash functions using asymmetric cryptography enabling distribution of the public key to verify the hash information while maintaining the confidentiality of the secret key used to generate the hash.</t>
         </is>
       </c>
-      <c r="H538" s="3" t="inlineStr">
+      <c r="H537" s="3" t="inlineStr">
         <is>
           <t>Overriding the system crypto policy makes the behavior of the OpenSSH
 client violate expectations, and makes system configuration more
 fragmented.</t>
         </is>
       </c>
-      <c r="I538" s="3" t="inlineStr">
-        <is>
-          <t>Applicable - Configurable</t>
-        </is>
-      </c>
-      <c r="J538" s="3" t="inlineStr">
+      <c r="I537" s="3" t="inlineStr">
+        <is>
+          <t>Applicable - Configurable</t>
+        </is>
+      </c>
+      <c r="J537" s="3" t="inlineStr">
         <is>
           <t>Verify the operating system implements cryptography to protect the integrity of remote access sessions. If it does not, this is a finding.</t>
         </is>
       </c>
-      <c r="K538" s="3" t="inlineStr">
+      <c r="K537" s="3" t="inlineStr">
         <is>
           <t>To verify if the OpenSSH client uses defined MACs in the Crypto Policy, run:
  $ grep -i macs /etc/crypto-policies/back-ends/openssh.config 
@@ -43033,73 +42958,73 @@
 If Crypto Policy for OpenSSH client is not configured correctly, then this is a finding.</t>
         </is>
       </c>
-      <c r="L538" s="3" t="n"/>
-      <c r="M538" s="3" t="inlineStr"/>
-      <c r="N538" s="3" t="inlineStr">
-        <is>
-          <t>CAT II</t>
-        </is>
-      </c>
-      <c r="O538" s="3" t="n"/>
-      <c r="P538" s="3" t="n"/>
-      <c r="Q538" s="3" t="n"/>
-    </row>
-    <row r="539" ht="130" customHeight="1">
-      <c r="A539" s="3" t="inlineStr">
+      <c r="L537" s="3" t="n"/>
+      <c r="M537" s="3" t="inlineStr"/>
+      <c r="N537" s="3" t="inlineStr">
+        <is>
+          <t>CAT II</t>
+        </is>
+      </c>
+      <c r="O537" s="3" t="n"/>
+      <c r="P537" s="3" t="n"/>
+      <c r="Q537" s="3" t="n"/>
+    </row>
+    <row r="538" ht="130" customHeight="1">
+      <c r="A538" s="3" t="inlineStr">
         <is>
           <t>AC-17 (2)</t>
         </is>
       </c>
-      <c r="B539" s="3" t="inlineStr">
+      <c r="B538" s="3" t="inlineStr">
         <is>
           <t>CCI-001453</t>
         </is>
       </c>
-      <c r="C539" s="3" t="inlineStr">
+      <c r="C538" s="3" t="inlineStr">
         <is>
           <t>SRG-OS-000250-GPOS-00093</t>
         </is>
       </c>
-      <c r="D539" s="3" t="inlineStr">
+      <c r="D538" s="3" t="inlineStr">
         <is>
           <t>CCE-87567-4</t>
         </is>
       </c>
-      <c r="E539" s="3" t="inlineStr">
+      <c r="E538" s="3" t="inlineStr">
         <is>
           <t>The operating system must implement cryptography to protect the integrity of remote access sessions.</t>
         </is>
       </c>
-      <c r="F539" s="3" t="inlineStr">
+      <c r="F538" s="3" t="inlineStr">
         <is>
           <t>Red Hat Enterprise Linux 9 Must Implement Cryptography To Protect The Integrity Of Remote Access Sessions.</t>
         </is>
       </c>
-      <c r="G539" s="3" t="inlineStr">
+      <c r="G538" s="3" t="inlineStr">
         <is>
           <t>Without cryptographic integrity protections, information can be altered by unauthorized users without detection.
 Remote access (e.g., RDP) is access to DoD nonpublic information systems by an authorized user (or an information system) communicating through an external, non-organization-controlled network. Remote access methods include, for example, dial-up, broadband, and wireless.
 Cryptographic mechanisms used for protecting the integrity of information include, for example, signed hash functions using asymmetric cryptography enabling distribution of the public key to verify the hash information while maintaining the confidentiality of the secret key used to generate the hash.</t>
         </is>
       </c>
-      <c r="H539" s="3" t="inlineStr">
+      <c r="H538" s="3" t="inlineStr">
         <is>
           <t>Overriding the system crypto policy makes the behavior of the OpenSSH
 server violate expectations, and makes system configuration more
 fragmented.</t>
         </is>
       </c>
-      <c r="I539" s="3" t="inlineStr">
-        <is>
-          <t>Applicable - Configurable</t>
-        </is>
-      </c>
-      <c r="J539" s="3" t="inlineStr">
+      <c r="I538" s="3" t="inlineStr">
+        <is>
+          <t>Applicable - Configurable</t>
+        </is>
+      </c>
+      <c r="J538" s="3" t="inlineStr">
         <is>
           <t>Verify the operating system implements cryptography to protect the integrity of remote access sessions. If it does not, this is a finding.</t>
         </is>
       </c>
-      <c r="K539" s="3" t="inlineStr">
+      <c r="K538" s="3" t="inlineStr">
         <is>
           <t>To verify if the OpenSSH server uses defined MACs in the Crypto Policy, run:
  $ grep -Po '(-oMACs=\S+)' /etc/crypto-policies/back-ends/opensshserver.config 
@@ -43108,16 +43033,16 @@
 If Crypto Policy for OpenSSH Server is not configured correctly, then this is a finding.</t>
         </is>
       </c>
-      <c r="L539" s="3" t="n"/>
-      <c r="M539" s="3" t="inlineStr"/>
-      <c r="N539" s="3" t="inlineStr">
-        <is>
-          <t>CAT II</t>
-        </is>
-      </c>
-      <c r="O539" s="3" t="n"/>
-      <c r="P539" s="3" t="n"/>
-      <c r="Q539" s="3" t="n"/>
+      <c r="L538" s="3" t="n"/>
+      <c r="M538" s="3" t="inlineStr"/>
+      <c r="N538" s="3" t="inlineStr">
+        <is>
+          <t>CAT II</t>
+        </is>
+      </c>
+      <c r="O538" s="3" t="n"/>
+      <c r="P538" s="3" t="n"/>
+      <c r="Q538" s="3" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Deploying to gh-pages from @ marcusburghardt/content@130668613ebed741d9b1cfdd0f343ddf6a7843d5 🚀
</commit_message>
<xml_diff>
--- a/srg_mapping/srg-mapping-rhel9.xlsx
+++ b/srg_mapping/srg-mapping-rhel9.xlsx
@@ -544,7 +544,7 @@
     <row r="2" ht="130" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>AC-7 a,AC-7 b</t>
+          <t>AC-7 b,AC-7 a</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
@@ -628,7 +628,7 @@
     <row r="3" ht="130" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>AC-7 a,AC-7 b</t>
+          <t>AC-7 b,AC-7 a</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
@@ -713,7 +713,7 @@
     <row r="4" ht="130" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>AC-7 a,AC-7 b</t>
+          <t>AC-7 b,AC-7 a</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
@@ -785,7 +785,7 @@
     <row r="5" ht="130" customHeight="1">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>AC-7 a,AC-7 b</t>
+          <t>AC-7 b,AC-7 a</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
@@ -967,7 +967,7 @@
     <row r="7" ht="130" customHeight="1">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>AU-5 a,AU-5 b</t>
+          <t>AU-5 b,AU-5 a</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
@@ -1461,7 +1461,7 @@
     <row r="13" ht="130" customHeight="1">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>AU-12 (3),AU-7 (1),AU-8 b,CM-5 (1),AU-3 (1),AU-14 (1),MA-4 (1) (a),AU-3,AU-7 a,AU-6 (4),AU-12 c,AU-7 b,AU-12 a</t>
+          <t>CM-5 (1),MA-4 (1) (a),AU-12 (3),AU-7 b,AU-8 b,AU-14 (1),AU-6 (4),AU-3,AU-3 (1),AU-12 a,AU-7 (1),AU-12 c,AU-7 a</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
@@ -1546,7 +1546,7 @@
     <row r="14" ht="130" customHeight="1">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>AU-12 (3),AU-7 (1),AU-8 b,CM-5 (1),AU-3 (1),AU-14 (1),MA-4 (1) (a),AU-3,AU-7 a,AU-6 (4),AU-12 c,AU-7 b,AU-12 a</t>
+          <t>CM-5 (1),MA-4 (1) (a),AU-12 (3),AU-7 b,AU-8 b,AU-14 (1),AU-6 (4),AU-3,AU-3 (1),AU-12 a,AU-7 (1),AU-12 c,AU-7 a</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
@@ -1621,7 +1621,7 @@
     <row r="15" ht="130" customHeight="1">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>CM-7 (5) (b),CM-7 (2)</t>
+          <t>CM-7 (2),CM-7 (5) (b)</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
@@ -1697,7 +1697,7 @@
     <row r="16" ht="130" customHeight="1">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>CM-7 (5) (b),CM-7 (2)</t>
+          <t>CM-7 (2),CM-7 (5) (b)</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
@@ -1851,7 +1851,7 @@
     <row r="18" ht="130" customHeight="1">
       <c r="A18" s="3" t="inlineStr">
         <is>
-          <t>CM-6 b,CM-7 (2)</t>
+          <t>CM-7 (2),CM-6 b</t>
         </is>
       </c>
       <c r="B18" s="3" t="inlineStr">
@@ -2221,7 +2221,7 @@
     <row r="23" ht="130" customHeight="1">
       <c r="A23" s="3" t="inlineStr">
         <is>
-          <t>CM-6 b,CM-7 (2)</t>
+          <t>CM-7 (2),CM-6 b</t>
         </is>
       </c>
       <c r="B23" s="3" t="inlineStr">
@@ -2295,7 +2295,7 @@
     <row r="24" ht="130" customHeight="1">
       <c r="A24" s="3" t="inlineStr">
         <is>
-          <t>CM-6 b,CM-7 (2)</t>
+          <t>CM-7 (2),CM-6 b</t>
         </is>
       </c>
       <c r="B24" s="3" t="inlineStr">
@@ -3339,7 +3339,7 @@
     <row r="38" ht="130" customHeight="1">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>AU-3 (1),AU-14 (1),MA-4 (1) (a),AU-3,AU-12 c,AU-12 a</t>
+          <t>MA-4 (1) (a),AU-14 (1),AU-3,AU-3 (1),AU-12 a,AU-12 c</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
@@ -3430,7 +3430,7 @@
     <row r="39" ht="130" customHeight="1">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>AU-4,AU-14 (1)</t>
+          <t>AU-14 (1),AU-4</t>
         </is>
       </c>
       <c r="B39" s="2" t="inlineStr">
@@ -3518,7 +3518,7 @@
     <row r="40" ht="130" customHeight="1">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>AU-4 (1),AU-3</t>
+          <t>AU-3,AU-4 (1)</t>
         </is>
       </c>
       <c r="B40" s="2" t="inlineStr">
@@ -4073,7 +4073,7 @@
     <row r="47" ht="130" customHeight="1">
       <c r="A47" s="2" t="inlineStr">
         <is>
-          <t>AU-8 b,AU-8 (1) (b),AU-8 (1) (a)</t>
+          <t>AU-8 (1) (b),AU-8 (1) (a),AU-8 b</t>
         </is>
       </c>
       <c r="B47" s="2" t="inlineStr">
@@ -4228,7 +4228,7 @@
     <row r="49" ht="130" customHeight="1">
       <c r="A49" s="2" t="inlineStr">
         <is>
-          <t>IA-2 (12),IA-2 (11)</t>
+          <t>IA-2 (11),IA-2 (12)</t>
         </is>
       </c>
       <c r="B49" s="2" t="inlineStr">
@@ -4314,7 +4314,7 @@
     <row r="50" ht="130" customHeight="1">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>IA-2 (12),IA-2 (1),IA-2 (11)</t>
+          <t>IA-2 (11),IA-2 (1),IA-2 (12)</t>
         </is>
       </c>
       <c r="B50" s="2" t="inlineStr">
@@ -4398,7 +4398,7 @@
     <row r="51" ht="130" customHeight="1">
       <c r="A51" s="2" t="inlineStr">
         <is>
-          <t>CM-3 (5),SI-6 d,SI-6 b</t>
+          <t>SI-6 b,CM-3 (5),SI-6 d</t>
         </is>
       </c>
       <c r="B51" s="2" t="inlineStr">
@@ -4574,7 +4574,7 @@
     <row r="53" ht="130" customHeight="1">
       <c r="A53" s="3" t="inlineStr">
         <is>
-          <t>AU-3 (1),MA-4 (1) (a),AU-3,AU-12 c,AU-12 a</t>
+          <t>MA-4 (1) (a),AU-3,AU-3 (1),AU-12 a,AU-12 c</t>
         </is>
       </c>
       <c r="B53" s="3" t="inlineStr">
@@ -4649,7 +4649,7 @@
     <row r="54" ht="130" customHeight="1">
       <c r="A54" s="3" t="inlineStr">
         <is>
-          <t>AU-3 (1),MA-4 (1) (a),AU-3,AU-12 c,AU-12 a</t>
+          <t>MA-4 (1) (a),AU-3,AU-3 (1),AU-12 a,AU-12 c</t>
         </is>
       </c>
       <c r="B54" s="3" t="inlineStr">
@@ -4724,7 +4724,7 @@
     <row r="55" ht="130" customHeight="1">
       <c r="A55" s="3" t="inlineStr">
         <is>
-          <t>AU-3 (1),MA-4 (1) (a),AU-3,AU-12 c,AU-12 a</t>
+          <t>MA-4 (1) (a),AU-3,AU-3 (1),AU-12 a,AU-12 c</t>
         </is>
       </c>
       <c r="B55" s="3" t="inlineStr">
@@ -4799,7 +4799,7 @@
     <row r="56" ht="130" customHeight="1">
       <c r="A56" s="3" t="inlineStr">
         <is>
-          <t>AU-3 (1),MA-4 (1) (a),AU-3,AU-12 c,AU-12 a</t>
+          <t>MA-4 (1) (a),AU-3,AU-3 (1),AU-12 a,AU-12 c</t>
         </is>
       </c>
       <c r="B56" s="3" t="inlineStr">
@@ -4874,7 +4874,7 @@
     <row r="57" ht="130" customHeight="1">
       <c r="A57" s="3" t="inlineStr">
         <is>
-          <t>AU-3 (1),MA-4 (1) (a),AU-3,AU-12 c,AU-12 a</t>
+          <t>MA-4 (1) (a),AU-3,AU-3 (1),AU-12 a,AU-12 c</t>
         </is>
       </c>
       <c r="B57" s="3" t="inlineStr">
@@ -4949,7 +4949,7 @@
     <row r="58" ht="130" customHeight="1">
       <c r="A58" s="3" t="inlineStr">
         <is>
-          <t>AU-3 (1),MA-4 (1) (a),AU-3,AU-12 c,AU-12 a</t>
+          <t>MA-4 (1) (a),AU-3,AU-3 (1),AU-12 a,AU-12 c</t>
         </is>
       </c>
       <c r="B58" s="3" t="inlineStr">
@@ -5024,7 +5024,7 @@
     <row r="59" ht="130" customHeight="1">
       <c r="A59" s="3" t="inlineStr">
         <is>
-          <t>AU-3 (1),MA-4 (1) (a),AU-3,AU-12 c,AU-12 a</t>
+          <t>MA-4 (1) (a),AU-3,AU-3 (1),AU-12 a,AU-12 c</t>
         </is>
       </c>
       <c r="B59" s="3" t="inlineStr">
@@ -5099,7 +5099,7 @@
     <row r="60" ht="130" customHeight="1">
       <c r="A60" s="3" t="inlineStr">
         <is>
-          <t>AU-3 (1),MA-4 (1) (a),AU-3,AU-12 c,AU-12 a</t>
+          <t>MA-4 (1) (a),AU-3,AU-3 (1),AU-12 a,AU-12 c</t>
         </is>
       </c>
       <c r="B60" s="3" t="inlineStr">
@@ -5174,7 +5174,7 @@
     <row r="61" ht="130" customHeight="1">
       <c r="A61" s="3" t="inlineStr">
         <is>
-          <t>AU-3 (1),MA-4 (1) (a),AU-3,AU-12 c,AU-12 a</t>
+          <t>MA-4 (1) (a),AU-3,AU-3 (1),AU-12 a,AU-12 c</t>
         </is>
       </c>
       <c r="B61" s="3" t="inlineStr">
@@ -5249,7 +5249,7 @@
     <row r="62" ht="130" customHeight="1">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>AU-3 (1),MA-4 (1) (a),AU-3,AU-12 c,AC-2 (4),AU-12 a</t>
+          <t>MA-4 (1) (a),AU-3,AU-3 (1),AU-12 a,AU-12 c,AC-2 (4)</t>
         </is>
       </c>
       <c r="B62" s="2" t="inlineStr">
@@ -5330,7 +5330,7 @@
     <row r="63" ht="130" customHeight="1">
       <c r="A63" s="2" t="inlineStr">
         <is>
-          <t>AU-3 (1),MA-4 (1) (a),AU-3,AU-12 c,AC-2 (4),AU-12 a</t>
+          <t>MA-4 (1) (a),AU-3,AU-3 (1),AU-12 a,AU-12 c,AC-2 (4)</t>
         </is>
       </c>
       <c r="B63" s="2" t="inlineStr">
@@ -5411,7 +5411,7 @@
     <row r="64" ht="130" customHeight="1">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>AU-3 (1),MA-4 (1) (a),AU-3,AU-12 c,AC-2 (4),AU-12 a</t>
+          <t>MA-4 (1) (a),AU-3,AU-3 (1),AU-12 a,AU-12 c,AC-2 (4)</t>
         </is>
       </c>
       <c r="B64" s="2" t="inlineStr">
@@ -5493,7 +5493,7 @@
     <row r="65" ht="130" customHeight="1">
       <c r="A65" s="2" t="inlineStr">
         <is>
-          <t>AU-3 (1),MA-4 (1) (a),AU-3,AU-12 c,AC-2 (4),AU-12 a</t>
+          <t>MA-4 (1) (a),AU-3,AU-3 (1),AU-12 a,AU-12 c,AC-2 (4)</t>
         </is>
       </c>
       <c r="B65" s="2" t="inlineStr">
@@ -5575,7 +5575,7 @@
     <row r="66" ht="130" customHeight="1">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>AU-3 (1),MA-4 (1) (a),AU-3,AU-12 c,AC-2 (4),AU-12 a</t>
+          <t>MA-4 (1) (a),AU-3,AU-3 (1),AU-12 a,AU-12 c,AC-2 (4)</t>
         </is>
       </c>
       <c r="B66" s="2" t="inlineStr">
@@ -5657,7 +5657,7 @@
     <row r="67" ht="130" customHeight="1">
       <c r="A67" s="2" t="inlineStr">
         <is>
-          <t>AU-3 (1),MA-4 (1) (a),AU-3,AU-12 c,AC-2 (4),AU-12 a</t>
+          <t>MA-4 (1) (a),AU-3,AU-3 (1),AU-12 a,AU-12 c,AC-2 (4)</t>
         </is>
       </c>
       <c r="B67" s="2" t="inlineStr">
@@ -5739,7 +5739,7 @@
     <row r="68" ht="130" customHeight="1">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>AU-3 (1),MA-4 (1) (a),AU-3,AU-12 c,AC-2 (4),AU-12 a</t>
+          <t>MA-4 (1) (a),AU-3,AU-3 (1),AU-12 a,AU-12 c,AC-2 (4)</t>
         </is>
       </c>
       <c r="B68" s="2" t="inlineStr">
@@ -5895,7 +5895,7 @@
     <row r="70" ht="130" customHeight="1">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>SI-11 b,AU-9</t>
+          <t>AU-9,SI-11 b</t>
         </is>
       </c>
       <c r="B70" s="2" t="inlineStr">
@@ -5978,7 +5978,7 @@
     <row r="71" ht="130" customHeight="1">
       <c r="A71" s="2" t="inlineStr">
         <is>
-          <t>SI-11 b,AU-9</t>
+          <t>AU-9,SI-11 b</t>
         </is>
       </c>
       <c r="B71" s="2" t="inlineStr">
@@ -6056,7 +6056,7 @@
     <row r="72" ht="130" customHeight="1">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t>SI-11 b,AU-9</t>
+          <t>AU-9,SI-11 b</t>
         </is>
       </c>
       <c r="B72" s="2" t="inlineStr">
@@ -6147,7 +6147,7 @@
     <row r="73" ht="130" customHeight="1">
       <c r="A73" s="2" t="inlineStr">
         <is>
-          <t>SI-11 b,AU-9</t>
+          <t>AU-9,SI-11 b</t>
         </is>
       </c>
       <c r="B73" s="2" t="inlineStr">
@@ -6229,7 +6229,7 @@
     <row r="74" ht="130" customHeight="1">
       <c r="A74" s="2" t="inlineStr">
         <is>
-          <t>SI-11 b,AU-9</t>
+          <t>AU-9,SI-11 b</t>
         </is>
       </c>
       <c r="B74" s="2" t="inlineStr">
@@ -6859,7 +6859,7 @@
     <row r="82" ht="130" customHeight="1">
       <c r="A82" s="3" t="inlineStr">
         <is>
-          <t>AU-3 (1),MA-4 (1) (a),AU-3,AU-12 c,AU-12 a</t>
+          <t>MA-4 (1) (a),AU-3,AU-3 (1),AU-12 a,AU-12 c</t>
         </is>
       </c>
       <c r="B82" s="3" t="inlineStr">
@@ -6933,7 +6933,7 @@
     <row r="83" ht="130" customHeight="1">
       <c r="A83" s="3" t="inlineStr">
         <is>
-          <t>AU-3 (1),MA-4 (1) (a),AU-3,AU-12 c,AU-12 a</t>
+          <t>MA-4 (1) (a),AU-3,AU-3 (1),AU-12 a,AU-12 c</t>
         </is>
       </c>
       <c r="B83" s="3" t="inlineStr">
@@ -7007,7 +7007,7 @@
     <row r="84" ht="130" customHeight="1">
       <c r="A84" s="3" t="inlineStr">
         <is>
-          <t>AU-3 (1),MA-4 (1) (a),AU-3,AU-12 c,AU-12 a</t>
+          <t>MA-4 (1) (a),AU-3,AU-3 (1),AU-12 a,AU-12 c</t>
         </is>
       </c>
       <c r="B84" s="3" t="inlineStr">
@@ -7081,7 +7081,7 @@
     <row r="85" ht="130" customHeight="1">
       <c r="A85" s="3" t="inlineStr">
         <is>
-          <t>AU-3 (1),MA-4 (1) (a),AU-3,AU-12 c,AU-12 a</t>
+          <t>MA-4 (1) (a),AU-3,AU-3 (1),AU-12 a,AU-12 c</t>
         </is>
       </c>
       <c r="B85" s="3" t="inlineStr">
@@ -7161,7 +7161,7 @@
     <row r="86" ht="130" customHeight="1">
       <c r="A86" s="3" t="inlineStr">
         <is>
-          <t>SC-13,MA-4 (6)</t>
+          <t>MA-4 (6),SC-13</t>
         </is>
       </c>
       <c r="B86" s="3" t="inlineStr">
@@ -7246,7 +7246,7 @@
     <row r="87" ht="130" customHeight="1">
       <c r="A87" s="3" t="inlineStr">
         <is>
-          <t>AC-17 (2),MA-4 (6)</t>
+          <t>MA-4 (6),AC-17 (2)</t>
         </is>
       </c>
       <c r="B87" s="3" t="inlineStr">
@@ -7322,7 +7322,7 @@
     <row r="88" ht="130" customHeight="1">
       <c r="A88" s="3" t="inlineStr">
         <is>
-          <t>SC-13,MA-4 (6)</t>
+          <t>MA-4 (6),SC-13</t>
         </is>
       </c>
       <c r="B88" s="3" t="inlineStr">
@@ -7505,7 +7505,7 @@
     <row r="90" ht="130" customHeight="1">
       <c r="A90" s="3" t="inlineStr">
         <is>
-          <t>AU-9 (3),AU-9</t>
+          <t>AU-9,AU-9 (3)</t>
         </is>
       </c>
       <c r="B90" s="3" t="inlineStr">
@@ -7581,7 +7581,7 @@
     <row r="91" ht="130" customHeight="1">
       <c r="A91" s="3" t="inlineStr">
         <is>
-          <t>AU-9 (3),AU-9</t>
+          <t>AU-9,AU-9 (3)</t>
         </is>
       </c>
       <c r="B91" s="3" t="inlineStr">
@@ -7657,7 +7657,7 @@
     <row r="92" ht="130" customHeight="1">
       <c r="A92" s="3" t="inlineStr">
         <is>
-          <t>AU-3 (1),MA-4 (1) (a),AU-3,AU-12 c,AU-12 a</t>
+          <t>MA-4 (1) (a),AU-3,AU-3 (1),AU-12 a,AU-12 c</t>
         </is>
       </c>
       <c r="B92" s="3" t="inlineStr">
@@ -7732,7 +7732,7 @@
     <row r="93" ht="130" customHeight="1">
       <c r="A93" s="3" t="inlineStr">
         <is>
-          <t>AU-3 (1),MA-4 (1) (a),AU-3,AU-12 c,AU-12 a</t>
+          <t>MA-4 (1) (a),AU-3,AU-3 (1),AU-12 a,AU-12 c</t>
         </is>
       </c>
       <c r="B93" s="3" t="inlineStr">
@@ -7807,7 +7807,7 @@
     <row r="94" ht="130" customHeight="1">
       <c r="A94" s="3" t="inlineStr">
         <is>
-          <t>AU-3 (1),MA-4 (1) (a),AU-3,AU-12 c,AU-12 a</t>
+          <t>MA-4 (1) (a),AU-3,AU-3 (1),AU-12 a,AU-12 c</t>
         </is>
       </c>
       <c r="B94" s="3" t="inlineStr">
@@ -7882,7 +7882,7 @@
     <row r="95" ht="130" customHeight="1">
       <c r="A95" s="3" t="inlineStr">
         <is>
-          <t>AU-3 (1),MA-4 (1) (a),AU-3,AU-12 c,AU-12 a</t>
+          <t>MA-4 (1) (a),AU-3,AU-3 (1),AU-12 a,AU-12 c</t>
         </is>
       </c>
       <c r="B95" s="3" t="inlineStr">
@@ -7962,7 +7962,7 @@
     <row r="96" ht="130" customHeight="1">
       <c r="A96" s="2" t="inlineStr">
         <is>
-          <t>AU-3 (1),MA-4 (1) (a),AU-3,AU-12 c,AU-12 a</t>
+          <t>MA-4 (1) (a),AU-3,AU-3 (1),AU-12 a,AU-12 c</t>
         </is>
       </c>
       <c r="B96" s="2" t="inlineStr">
@@ -8044,7 +8044,7 @@
     <row r="97" ht="130" customHeight="1">
       <c r="A97" s="2" t="inlineStr">
         <is>
-          <t>AU-3 (1),MA-4 (1) (a),AU-3,AU-12 c,AU-12 a</t>
+          <t>MA-4 (1) (a),AU-3,AU-3 (1),AU-12 a,AU-12 c</t>
         </is>
       </c>
       <c r="B97" s="2" t="inlineStr">
@@ -8126,7 +8126,7 @@
     <row r="98" ht="130" customHeight="1">
       <c r="A98" s="2" t="inlineStr">
         <is>
-          <t>AU-3 (1),MA-4 (1) (a),AU-3,AU-12 c,AU-12 a</t>
+          <t>MA-4 (1) (a),AU-3,AU-3 (1),AU-12 a,AU-12 c</t>
         </is>
       </c>
       <c r="B98" s="2" t="inlineStr">
@@ -8208,7 +8208,7 @@
     <row r="99" ht="130" customHeight="1">
       <c r="A99" s="2" t="inlineStr">
         <is>
-          <t>AU-3 (1),MA-4 (1) (a),AU-3,AU-12 c,AU-12 a</t>
+          <t>MA-4 (1) (a),AU-3,AU-3 (1),AU-12 a,AU-12 c</t>
         </is>
       </c>
       <c r="B99" s="2" t="inlineStr">
@@ -8290,7 +8290,7 @@
     <row r="100" ht="130" customHeight="1">
       <c r="A100" s="2" t="inlineStr">
         <is>
-          <t>AU-3 (1),MA-4 (1) (a),AU-3,AU-12 c,AU-12 a</t>
+          <t>MA-4 (1) (a),AU-3,AU-3 (1),AU-12 a,AU-12 c</t>
         </is>
       </c>
       <c r="B100" s="2" t="inlineStr">
@@ -8372,7 +8372,7 @@
     <row r="101" ht="130" customHeight="1">
       <c r="A101" s="3" t="inlineStr">
         <is>
-          <t>AU-3 (1),MA-4 (1) (a),AU-3,AU-12 c,AU-12 a</t>
+          <t>MA-4 (1) (a),AU-3,AU-3 (1),AU-12 a,AU-12 c</t>
         </is>
       </c>
       <c r="B101" s="3" t="inlineStr">
@@ -8452,7 +8452,7 @@
     <row r="102" ht="130" customHeight="1">
       <c r="A102" s="3" t="inlineStr">
         <is>
-          <t>AU-3 (1),MA-4 (1) (a),AU-3,AU-12 c,AU-12 a</t>
+          <t>MA-4 (1) (a),AU-3,AU-3 (1),AU-12 a,AU-12 c</t>
         </is>
       </c>
       <c r="B102" s="3" t="inlineStr">
@@ -8532,7 +8532,7 @@
     <row r="103" ht="130" customHeight="1">
       <c r="A103" s="3" t="inlineStr">
         <is>
-          <t>AU-3 (1),MA-4 (1) (a),AU-3,AU-12 c,AU-12 a</t>
+          <t>MA-4 (1) (a),AU-3,AU-3 (1),AU-12 a,AU-12 c</t>
         </is>
       </c>
       <c r="B103" s="3" t="inlineStr">
@@ -8862,7 +8862,7 @@
     <row r="107" ht="130" customHeight="1">
       <c r="A107" s="2" t="inlineStr">
         <is>
-          <t>AC-11 a,AC-11 b</t>
+          <t>AC-11 b,AC-11 a</t>
         </is>
       </c>
       <c r="B107" s="2" t="inlineStr">
@@ -8941,7 +8941,7 @@
     <row r="108" ht="130" customHeight="1">
       <c r="A108" s="2" t="inlineStr">
         <is>
-          <t>AC-11 a,AC-11 b</t>
+          <t>AC-11 b,AC-11 a</t>
         </is>
       </c>
       <c r="B108" s="2" t="inlineStr">
@@ -9028,7 +9028,7 @@
     <row r="109" ht="130" customHeight="1">
       <c r="A109" s="2" t="inlineStr">
         <is>
-          <t>AC-11 a,AC-11 b</t>
+          <t>AC-11 b,AC-11 a</t>
         </is>
       </c>
       <c r="B109" s="2" t="inlineStr">
@@ -9115,7 +9115,7 @@
     <row r="110" ht="130" customHeight="1">
       <c r="A110" s="3" t="inlineStr">
         <is>
-          <t>AC-11 a,AC-11 b</t>
+          <t>AC-11 b,AC-11 a</t>
         </is>
       </c>
       <c r="B110" s="3" t="inlineStr">
@@ -9360,7 +9360,7 @@
     <row r="113" ht="130" customHeight="1">
       <c r="A113" s="2" t="inlineStr">
         <is>
-          <t>SC-8,AC-17 (2),SC-13,MA-4 c</t>
+          <t>SC-13,SC-8,MA-4 c,AC-17 (2)</t>
         </is>
       </c>
       <c r="B113" s="2" t="inlineStr">
@@ -9442,7 +9442,7 @@
     <row r="114" ht="130" customHeight="1">
       <c r="A114" s="2" t="inlineStr">
         <is>
-          <t>MA-4 (1) (a),AU-12 c</t>
+          <t>AU-12 c,MA-4 (1) (a)</t>
         </is>
       </c>
       <c r="B114" s="2" t="inlineStr">
@@ -9520,7 +9520,7 @@
     <row r="115" ht="130" customHeight="1">
       <c r="A115" s="2" t="inlineStr">
         <is>
-          <t>AU-3 (1),MA-4 (1) (a),AU-3,AU-12 c,AU-12 a</t>
+          <t>MA-4 (1) (a),AU-3,AU-3 (1),AU-12 a,AU-12 c</t>
         </is>
       </c>
       <c r="B115" s="2" t="inlineStr">
@@ -9598,7 +9598,7 @@
     <row r="116" ht="130" customHeight="1">
       <c r="A116" s="2" t="inlineStr">
         <is>
-          <t>MA-4 (1) (a),AU-12 c</t>
+          <t>AU-12 c,MA-4 (1) (a)</t>
         </is>
       </c>
       <c r="B116" s="2" t="inlineStr">
@@ -9676,7 +9676,7 @@
     <row r="117" ht="130" customHeight="1">
       <c r="A117" s="3" t="inlineStr">
         <is>
-          <t>AU-3 (1),MA-4 (1) (a),AU-3,AU-12 c,AU-12 a</t>
+          <t>MA-4 (1) (a),AU-3,AU-3 (1),AU-12 a,AU-12 c</t>
         </is>
       </c>
       <c r="B117" s="3" t="inlineStr">
@@ -9756,7 +9756,7 @@
     <row r="118" ht="130" customHeight="1">
       <c r="A118" s="3" t="inlineStr">
         <is>
-          <t>MA-4 (1) (a),AU-12 c</t>
+          <t>AU-12 c,MA-4 (1) (a)</t>
         </is>
       </c>
       <c r="B118" s="3" t="inlineStr">
@@ -9825,7 +9825,7 @@
     <row r="119" ht="130" customHeight="1">
       <c r="A119" s="3" t="inlineStr">
         <is>
-          <t>MA-4 (1) (a),AU-12 c</t>
+          <t>AU-12 c,MA-4 (1) (a)</t>
         </is>
       </c>
       <c r="B119" s="3" t="inlineStr">
@@ -9894,7 +9894,7 @@
     <row r="120" ht="130" customHeight="1">
       <c r="A120" s="3" t="inlineStr">
         <is>
-          <t>MA-4 (1) (a),AU-12 c</t>
+          <t>AU-12 c,MA-4 (1) (a)</t>
         </is>
       </c>
       <c r="B120" s="3" t="inlineStr">
@@ -9963,7 +9963,7 @@
     <row r="121" ht="130" customHeight="1">
       <c r="A121" s="3" t="inlineStr">
         <is>
-          <t>MA-4 (1) (a),AU-12 c</t>
+          <t>AU-12 c,MA-4 (1) (a)</t>
         </is>
       </c>
       <c r="B121" s="3" t="inlineStr">
@@ -10032,7 +10032,7 @@
     <row r="122" ht="130" customHeight="1">
       <c r="A122" s="3" t="inlineStr">
         <is>
-          <t>AU-3 (1),MA-4 (1) (a),AU-3,AU-12 c,AU-12 a</t>
+          <t>MA-4 (1) (a),AU-3,AU-3 (1),AU-12 a,AU-12 c</t>
         </is>
       </c>
       <c r="B122" s="3" t="inlineStr">
@@ -10112,7 +10112,7 @@
     <row r="123" ht="130" customHeight="1">
       <c r="A123" s="2" t="inlineStr">
         <is>
-          <t>SC-28 (1),SC-28</t>
+          <t>SC-28,SC-28 (1)</t>
         </is>
       </c>
       <c r="B123" s="2" t="inlineStr">
@@ -11419,7 +11419,7 @@
     <row r="139" ht="130" customHeight="1">
       <c r="A139" s="3" t="inlineStr">
         <is>
-          <t>MA-4 (1) (a),AU-12 c</t>
+          <t>AU-12 c,MA-4 (1) (a)</t>
         </is>
       </c>
       <c r="B139" s="3" t="inlineStr">
@@ -11499,7 +11499,7 @@
     <row r="140" ht="130" customHeight="1">
       <c r="A140" s="3" t="inlineStr">
         <is>
-          <t>AU-3 (1),MA-4 (1) (a),AU-3,AU-12 c,AU-12 a</t>
+          <t>MA-4 (1) (a),AU-3,AU-3 (1),AU-12 a,AU-12 c</t>
         </is>
       </c>
       <c r="B140" s="3" t="inlineStr">
@@ -11579,7 +11579,7 @@
     <row r="141" ht="130" customHeight="1">
       <c r="A141" s="3" t="inlineStr">
         <is>
-          <t>AU-3 (1),MA-4 (1) (a),AU-3,AU-12 c,AU-12 a</t>
+          <t>MA-4 (1) (a),AU-3,AU-3 (1),AU-12 a,AU-12 c</t>
         </is>
       </c>
       <c r="B141" s="3" t="inlineStr">
@@ -11659,7 +11659,7 @@
     <row r="142" ht="130" customHeight="1">
       <c r="A142" s="3" t="inlineStr">
         <is>
-          <t>AU-3 (1),MA-4 (1) (a),AU-3,AU-12 c,AU-12 a</t>
+          <t>MA-4 (1) (a),AU-3,AU-3 (1),AU-12 a,AU-12 c</t>
         </is>
       </c>
       <c r="B142" s="3" t="inlineStr">
@@ -12442,7 +12442,7 @@
     <row r="152" ht="130" customHeight="1">
       <c r="A152" s="2" t="inlineStr">
         <is>
-          <t>IA-7,CM-6 b</t>
+          <t>CM-6 b,IA-7</t>
         </is>
       </c>
       <c r="B152" s="2" t="inlineStr">
@@ -12518,7 +12518,7 @@
     <row r="153" ht="130" customHeight="1">
       <c r="A153" s="2" t="inlineStr">
         <is>
-          <t>IA-7,CM-6 b</t>
+          <t>CM-6 b,IA-7</t>
         </is>
       </c>
       <c r="B153" s="2" t="inlineStr">
@@ -12603,7 +12603,7 @@
     <row r="154" ht="130" customHeight="1">
       <c r="A154" s="2" t="inlineStr">
         <is>
-          <t>IA-7,CM-6 b</t>
+          <t>CM-6 b,IA-7</t>
         </is>
       </c>
       <c r="B154" s="2" t="inlineStr">
@@ -12760,7 +12760,7 @@
     <row r="156" ht="130" customHeight="1">
       <c r="A156" s="2" t="inlineStr">
         <is>
-          <t>IA-7,CM-7 a</t>
+          <t>CM-7 a,IA-7</t>
         </is>
       </c>
       <c r="B156" s="2" t="inlineStr">
@@ -12839,7 +12839,7 @@
     <row r="157" ht="130" customHeight="1">
       <c r="A157" s="3" t="inlineStr">
         <is>
-          <t>AU-3 (1),MA-4 (1) (a),AU-3,AU-12 c,AU-12 a</t>
+          <t>MA-4 (1) (a),AU-3,AU-3 (1),AU-12 a,AU-12 c</t>
         </is>
       </c>
       <c r="B157" s="3" t="inlineStr">
@@ -12916,7 +12916,7 @@
     <row r="158" ht="130" customHeight="1">
       <c r="A158" s="3" t="inlineStr">
         <is>
-          <t>MA-4 (1) (a),AU-12 a,AU-12 c,AU-3</t>
+          <t>AU-12 a,AU-12 c,AU-3,MA-4 (1) (a)</t>
         </is>
       </c>
       <c r="B158" s="3" t="inlineStr">
@@ -12989,7 +12989,7 @@
     <row r="159" ht="130" customHeight="1">
       <c r="A159" s="3" t="inlineStr">
         <is>
-          <t>MA-4 (1) (a),AU-12 a,AU-12 c,AU-3</t>
+          <t>AU-12 a,AU-12 c,AU-3,MA-4 (1) (a)</t>
         </is>
       </c>
       <c r="B159" s="3" t="inlineStr">
@@ -13062,7 +13062,7 @@
     <row r="160" ht="130" customHeight="1">
       <c r="A160" s="3" t="inlineStr">
         <is>
-          <t>AU-3 (1),MA-4 (1) (a),AU-3,AU-12 c,AU-12 a</t>
+          <t>MA-4 (1) (a),AU-3,AU-3 (1),AU-12 a,AU-12 c</t>
         </is>
       </c>
       <c r="B160" s="3" t="inlineStr">
@@ -13147,7 +13147,7 @@
     <row r="161" ht="130" customHeight="1">
       <c r="A161" s="3" t="inlineStr">
         <is>
-          <t>AU-3 (1),MA-4 (1) (a),AU-3,AU-12 c,AU-12 a</t>
+          <t>MA-4 (1) (a),AU-3,AU-3 (1),AU-12 a,AU-12 c</t>
         </is>
       </c>
       <c r="B161" s="3" t="inlineStr">
@@ -13222,7 +13222,7 @@
     <row r="162" ht="130" customHeight="1">
       <c r="A162" s="3" t="inlineStr">
         <is>
-          <t>AU-3 (1),MA-4 (1) (a),AU-3,AU-12 c,AU-12 a</t>
+          <t>MA-4 (1) (a),AU-3,AU-3 (1),AU-12 a,AU-12 c</t>
         </is>
       </c>
       <c r="B162" s="3" t="inlineStr">
@@ -13297,7 +13297,7 @@
     <row r="163" ht="130" customHeight="1">
       <c r="A163" s="3" t="inlineStr">
         <is>
-          <t>AU-3 (1),MA-4 (1) (a),AU-3,AU-12 c,AU-12 a</t>
+          <t>MA-4 (1) (a),AU-3,AU-3 (1),AU-12 a,AU-12 c</t>
         </is>
       </c>
       <c r="B163" s="3" t="inlineStr">
@@ -13372,7 +13372,7 @@
     <row r="164" ht="130" customHeight="1">
       <c r="A164" s="3" t="inlineStr">
         <is>
-          <t>AU-3 (1),MA-4 (1) (a),AU-3,AU-12 c,AU-12 a</t>
+          <t>MA-4 (1) (a),AU-3,AU-3 (1),AU-12 a,AU-12 c</t>
         </is>
       </c>
       <c r="B164" s="3" t="inlineStr">
@@ -13447,7 +13447,7 @@
     <row r="165" ht="130" customHeight="1">
       <c r="A165" s="3" t="inlineStr">
         <is>
-          <t>MA-4 (1) (a),AU-12 c</t>
+          <t>AU-12 c,MA-4 (1) (a)</t>
         </is>
       </c>
       <c r="B165" s="3" t="inlineStr">
@@ -13518,7 +13518,7 @@
     <row r="166" ht="130" customHeight="1">
       <c r="A166" s="3" t="inlineStr">
         <is>
-          <t>MA-4 (1) (a),AU-12 c</t>
+          <t>AU-12 c,MA-4 (1) (a)</t>
         </is>
       </c>
       <c r="B166" s="3" t="inlineStr">
@@ -13589,7 +13589,7 @@
     <row r="167" ht="130" customHeight="1">
       <c r="A167" s="3" t="inlineStr">
         <is>
-          <t>MA-4 (1) (a),AU-12 c</t>
+          <t>AU-12 c,MA-4 (1) (a)</t>
         </is>
       </c>
       <c r="B167" s="3" t="inlineStr">
@@ -13661,7 +13661,7 @@
     <row r="168" ht="130" customHeight="1">
       <c r="A168" s="3" t="inlineStr">
         <is>
-          <t>MA-4 (1) (a),AU-12 c</t>
+          <t>AU-12 c,MA-4 (1) (a)</t>
         </is>
       </c>
       <c r="B168" s="3" t="inlineStr">
@@ -13732,7 +13732,7 @@
     <row r="169" ht="130" customHeight="1">
       <c r="A169" s="3" t="inlineStr">
         <is>
-          <t>MA-4 (1) (a),AU-12 c</t>
+          <t>AU-12 c,MA-4 (1) (a)</t>
         </is>
       </c>
       <c r="B169" s="3" t="inlineStr">
@@ -13803,7 +13803,7 @@
     <row r="170" ht="130" customHeight="1">
       <c r="A170" s="3" t="inlineStr">
         <is>
-          <t>MA-4 (1) (a),AU-12 c</t>
+          <t>AU-12 c,MA-4 (1) (a)</t>
         </is>
       </c>
       <c r="B170" s="3" t="inlineStr">
@@ -13875,7 +13875,7 @@
     <row r="171" ht="130" customHeight="1">
       <c r="A171" s="3" t="inlineStr">
         <is>
-          <t>AU-3 (1),MA-4 (1) (a),AU-3,AU-12 c,AU-12 a</t>
+          <t>MA-4 (1) (a),AU-3,AU-3 (1),AU-12 a,AU-12 c</t>
         </is>
       </c>
       <c r="B171" s="3" t="inlineStr">
@@ -13950,7 +13950,7 @@
     <row r="172" ht="130" customHeight="1">
       <c r="A172" s="3" t="inlineStr">
         <is>
-          <t>MA-4 (1) (a),AU-12 c</t>
+          <t>AU-12 c,MA-4 (1) (a)</t>
         </is>
       </c>
       <c r="B172" s="3" t="inlineStr">
@@ -14021,7 +14021,7 @@
     <row r="173" ht="130" customHeight="1">
       <c r="A173" s="3" t="inlineStr">
         <is>
-          <t>MA-4 (1) (a),AU-12 c</t>
+          <t>AU-12 c,MA-4 (1) (a)</t>
         </is>
       </c>
       <c r="B173" s="3" t="inlineStr">
@@ -14092,7 +14092,7 @@
     <row r="174" ht="130" customHeight="1">
       <c r="A174" s="3" t="inlineStr">
         <is>
-          <t>MA-4 (1) (a),AU-12 c</t>
+          <t>AU-12 c,MA-4 (1) (a)</t>
         </is>
       </c>
       <c r="B174" s="3" t="inlineStr">
@@ -14164,7 +14164,7 @@
     <row r="175" ht="130" customHeight="1">
       <c r="A175" s="3" t="inlineStr">
         <is>
-          <t>AU-3 (1),MA-4 (1) (a),AU-3,AU-12 c,AU-12 a</t>
+          <t>MA-4 (1) (a),AU-3,AU-3 (1),AU-12 a,AU-12 c</t>
         </is>
       </c>
       <c r="B175" s="3" t="inlineStr">
@@ -14239,7 +14239,7 @@
     <row r="176" ht="130" customHeight="1">
       <c r="A176" s="3" t="inlineStr">
         <is>
-          <t>AU-3 (1),MA-4 (1) (a),AU-3,AU-12 c,AU-12 a</t>
+          <t>MA-4 (1) (a),AU-3,AU-3 (1),AU-12 a,AU-12 c</t>
         </is>
       </c>
       <c r="B176" s="3" t="inlineStr">
@@ -14321,7 +14321,7 @@
     <row r="177" ht="130" customHeight="1">
       <c r="A177" s="3" t="inlineStr">
         <is>
-          <t>AU-3 (1),MA-4 (1) (a),AU-3,AU-12 c,AU-12 a</t>
+          <t>MA-4 (1) (a),AU-3,AU-3 (1),AU-12 a,AU-12 c</t>
         </is>
       </c>
       <c r="B177" s="3" t="inlineStr">
@@ -14403,7 +14403,7 @@
     <row r="178" ht="130" customHeight="1">
       <c r="A178" s="3" t="inlineStr">
         <is>
-          <t>AU-3 (1),MA-4 (1) (a),AU-3,AU-12 c,AU-12 a</t>
+          <t>MA-4 (1) (a),AU-3,AU-3 (1),AU-12 a,AU-12 c</t>
         </is>
       </c>
       <c r="B178" s="3" t="inlineStr">
@@ -14485,7 +14485,7 @@
     <row r="179" ht="130" customHeight="1">
       <c r="A179" s="3" t="inlineStr">
         <is>
-          <t>AU-3 (1),MA-4 (1) (a),AU-3</t>
+          <t>AU-3 (1),AU-3,MA-4 (1) (a)</t>
         </is>
       </c>
       <c r="B179" s="3" t="inlineStr">
@@ -14567,7 +14567,7 @@
     <row r="180" ht="130" customHeight="1">
       <c r="A180" s="3" t="inlineStr">
         <is>
-          <t>AU-3 (1),MA-4 (1) (a),AU-3,AU-12 c,AU-12 a</t>
+          <t>MA-4 (1) (a),AU-3,AU-3 (1),AU-12 a,AU-12 c</t>
         </is>
       </c>
       <c r="B180" s="3" t="inlineStr">
@@ -14649,7 +14649,7 @@
     <row r="181" ht="130" customHeight="1">
       <c r="A181" s="3" t="inlineStr">
         <is>
-          <t>AU-3 (1),MA-4 (1) (a),AU-3,AU-12 c,AU-12 a</t>
+          <t>MA-4 (1) (a),AU-3,AU-3 (1),AU-12 a,AU-12 c</t>
         </is>
       </c>
       <c r="B181" s="3" t="inlineStr">
@@ -14731,7 +14731,7 @@
     <row r="182" ht="130" customHeight="1">
       <c r="A182" s="3" t="inlineStr">
         <is>
-          <t>AU-3 (1),MA-4 (1) (a),AU-3,AU-12 c,AU-12 a</t>
+          <t>MA-4 (1) (a),AU-3,AU-3 (1),AU-12 a,AU-12 c</t>
         </is>
       </c>
       <c r="B182" s="3" t="inlineStr">
@@ -14813,7 +14813,7 @@
     <row r="183" ht="130" customHeight="1">
       <c r="A183" s="3" t="inlineStr">
         <is>
-          <t>AU-3 (1),MA-4 (1) (a),AU-3,AU-12 c,AU-12 a</t>
+          <t>MA-4 (1) (a),AU-3,AU-3 (1),AU-12 a,AU-12 c</t>
         </is>
       </c>
       <c r="B183" s="3" t="inlineStr">
@@ -14895,7 +14895,7 @@
     <row r="184" ht="130" customHeight="1">
       <c r="A184" s="3" t="inlineStr">
         <is>
-          <t>AU-3 (1),MA-4 (1) (a),AU-3,AU-12 c,AU-12 a</t>
+          <t>MA-4 (1) (a),AU-3,AU-3 (1),AU-12 a,AU-12 c</t>
         </is>
       </c>
       <c r="B184" s="3" t="inlineStr">
@@ -14977,7 +14977,7 @@
     <row r="185" ht="130" customHeight="1">
       <c r="A185" s="3" t="inlineStr">
         <is>
-          <t>AU-3 (1),MA-4 (1) (a),AU-12 c</t>
+          <t>AU-12 c,AU-3 (1),MA-4 (1) (a)</t>
         </is>
       </c>
       <c r="B185" s="3" t="inlineStr">
@@ -15055,7 +15055,7 @@
     <row r="186" ht="130" customHeight="1">
       <c r="A186" s="3" t="inlineStr">
         <is>
-          <t>AU-3 (1),MA-4 (1) (a),AU-3,AU-12 c,AU-12 a</t>
+          <t>MA-4 (1) (a),AU-3,AU-3 (1),AU-12 a,AU-12 c</t>
         </is>
       </c>
       <c r="B186" s="3" t="inlineStr">
@@ -15134,7 +15134,7 @@
     <row r="187" ht="130" customHeight="1">
       <c r="A187" s="3" t="inlineStr">
         <is>
-          <t>AU-3 (1),MA-4 (1) (a),AU-3,AU-12 c,AU-12 a</t>
+          <t>MA-4 (1) (a),AU-3,AU-3 (1),AU-12 a,AU-12 c</t>
         </is>
       </c>
       <c r="B187" s="3" t="inlineStr">
@@ -15216,7 +15216,7 @@
     <row r="188" ht="130" customHeight="1">
       <c r="A188" s="3" t="inlineStr">
         <is>
-          <t>AU-3 (1),MA-4 (1) (a),AU-3,AU-12 c,AU-12 a</t>
+          <t>MA-4 (1) (a),AU-3,AU-3 (1),AU-12 a,AU-12 c</t>
         </is>
       </c>
       <c r="B188" s="3" t="inlineStr">
@@ -15298,7 +15298,7 @@
     <row r="189" ht="130" customHeight="1">
       <c r="A189" s="3" t="inlineStr">
         <is>
-          <t>AU-3 (1),MA-4 (1) (a),AU-12 c,AU-3</t>
+          <t>AU-12 c,AU-3 (1),AU-3,MA-4 (1) (a)</t>
         </is>
       </c>
       <c r="B189" s="3" t="inlineStr">
@@ -15380,7 +15380,7 @@
     <row r="190" ht="130" customHeight="1">
       <c r="A190" s="3" t="inlineStr">
         <is>
-          <t>AU-3 (1),MA-4 (1) (a),AU-3,AU-12 c,AU-12 a</t>
+          <t>MA-4 (1) (a),AU-3,AU-3 (1),AU-12 a,AU-12 c</t>
         </is>
       </c>
       <c r="B190" s="3" t="inlineStr">
@@ -15462,7 +15462,7 @@
     <row r="191" ht="130" customHeight="1">
       <c r="A191" s="3" t="inlineStr">
         <is>
-          <t>AU-3 (1),MA-4 (1) (a),AU-3,AU-12 c,AU-12 a</t>
+          <t>MA-4 (1) (a),AU-3,AU-3 (1),AU-12 a,AU-12 c</t>
         </is>
       </c>
       <c r="B191" s="3" t="inlineStr">
@@ -15544,7 +15544,7 @@
     <row r="192" ht="130" customHeight="1">
       <c r="A192" s="3" t="inlineStr">
         <is>
-          <t>AU-3 (1),MA-4 (1) (a),AU-3,AU-12 c,AU-12 a</t>
+          <t>MA-4 (1) (a),AU-3,AU-3 (1),AU-12 a,AU-12 c</t>
         </is>
       </c>
       <c r="B192" s="3" t="inlineStr">
@@ -15626,7 +15626,7 @@
     <row r="193" ht="130" customHeight="1">
       <c r="A193" s="3" t="inlineStr">
         <is>
-          <t>AU-3 (1),MA-4 (1) (a),AU-3,AU-12 c,AU-12 a</t>
+          <t>MA-4 (1) (a),AU-3,AU-3 (1),AU-12 a,AU-12 c</t>
         </is>
       </c>
       <c r="B193" s="3" t="inlineStr">
@@ -15701,7 +15701,7 @@
     <row r="194" ht="130" customHeight="1">
       <c r="A194" s="2" t="inlineStr">
         <is>
-          <t>IA-2 (3),IA-2 (1),IA-2 (4),IA-2 (2)</t>
+          <t>IA-2 (2),IA-2 (4),IA-2 (3),IA-2 (1)</t>
         </is>
       </c>
       <c r="B194" s="2" t="inlineStr">
@@ -15788,7 +15788,7 @@
     <row r="195" ht="130" customHeight="1">
       <c r="A195" s="2" t="inlineStr">
         <is>
-          <t>IA-2 (2),IA-2,IA-2 (3),IA-2 (5),IA-2 (4)</t>
+          <t>IA-2 (2),IA-2 (4),IA-2 (3),IA-2,IA-2 (5)</t>
         </is>
       </c>
       <c r="B195" s="2" t="inlineStr">
@@ -15877,7 +15877,7 @@
     <row r="196" ht="130" customHeight="1">
       <c r="A196" s="2" t="inlineStr">
         <is>
-          <t>IA-2 (2),IA-2,IA-2 (3),IA-2 (5),IA-2 (4)</t>
+          <t>IA-2 (2),IA-2 (4),IA-2 (3),IA-2,IA-2 (5)</t>
         </is>
       </c>
       <c r="B196" s="2" t="inlineStr">
@@ -16501,7 +16501,7 @@
     <row r="204" ht="130" customHeight="1">
       <c r="A204" s="2" t="inlineStr">
         <is>
-          <t>SC-8,SC-8 (2),SC-8 (1)</t>
+          <t>SC-8,SC-8 (1),SC-8 (2)</t>
         </is>
       </c>
       <c r="B204" s="2" t="inlineStr">
@@ -16578,7 +16578,7 @@
     <row r="205" ht="130" customHeight="1">
       <c r="A205" s="2" t="inlineStr">
         <is>
-          <t>SC-8,SC-8 (2),SC-8 (1)</t>
+          <t>SC-8,SC-8 (1),SC-8 (2)</t>
         </is>
       </c>
       <c r="B205" s="2" t="inlineStr">
@@ -17092,7 +17092,7 @@
     <row r="211" ht="130" customHeight="1">
       <c r="A211" s="2" t="inlineStr">
         <is>
-          <t>IA-5 (1) (c),CM-6 b,CM-7 a</t>
+          <t>CM-6 b,CM-7 a,IA-5 (1) (c)</t>
         </is>
       </c>
       <c r="B211" s="2" t="inlineStr">
@@ -17343,7 +17343,7 @@
     <row r="214" ht="130" customHeight="1">
       <c r="A214" s="2" t="inlineStr">
         <is>
-          <t>SC-5,CM-6 b,SC-5 (2)</t>
+          <t>CM-6 b,SC-5 (2),SC-5</t>
         </is>
       </c>
       <c r="B214" s="2" t="inlineStr">
@@ -19513,44 +19513,44 @@
       <c r="Q239" s="2" t="n"/>
     </row>
     <row r="240" ht="130" customHeight="1">
-      <c r="A240" s="3" t="inlineStr">
+      <c r="A240" s="2" t="inlineStr">
         <is>
           <t>IA-5 (1) (b)</t>
         </is>
       </c>
-      <c r="B240" s="3" t="inlineStr">
+      <c r="B240" s="2" t="inlineStr">
         <is>
           <t>CCI-000195</t>
         </is>
       </c>
-      <c r="C240" s="3" t="inlineStr">
+      <c r="C240" s="2" t="inlineStr">
         <is>
           <t>SRG-OS-000072-GPOS-00040</t>
         </is>
       </c>
-      <c r="D240" s="3" t="inlineStr">
+      <c r="D240" s="2" t="inlineStr">
         <is>
           <t>CCE-83564-5</t>
         </is>
       </c>
-      <c r="E240" s="3" t="inlineStr">
+      <c r="E240" s="2" t="inlineStr">
         <is>
           <t>The operating system must require the change of at least 50% of the total number of characters when passwords are changed.</t>
         </is>
       </c>
-      <c r="F240" s="3" t="inlineStr">
+      <c r="F240" s="2" t="inlineStr">
         <is>
           <t>Red Hat Enterprise Linux 9 Must Require The Change Of At Least 50% Of The Total Number Of Characters When Passwords Are Changed.</t>
         </is>
       </c>
-      <c r="G240" s="3" t="inlineStr">
+      <c r="G240" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve"> If the operating system allows the user to consecutively reuse extensive portions of passwords, this increases the chances of password compromise by increasing the window of opportunity for attempts at guessing and brute-force attacks.
 The number of changed characters refers to the number of changes required with respect to the total number of positions in the current password. In other words, characters may be the same within the two passwords; however, the positions of the like characters must be different.
 If the password length is an odd number then number of changed characters must be rounded up.  For example, a password length of 15 characters must require the change of at least 8 characters.</t>
         </is>
       </c>
-      <c r="H240" s="3" t="inlineStr">
+      <c r="H240" s="2" t="inlineStr">
         <is>
           <t>Use of a complex password helps to increase the time and resources
 required to compromise the password. Password complexity, or strength,
@@ -19565,39 +19565,46 @@
 Note that passwords which are changed on compromised systems will still be compromised, however.</t>
         </is>
       </c>
-      <c r="I240" s="3" t="inlineStr">
-        <is>
-          <t>Applicable - Configurable</t>
-        </is>
-      </c>
-      <c r="J240" s="3" t="inlineStr">
+      <c r="I240" s="2" t="inlineStr">
+        <is>
+          <t>Applicable - Configurable</t>
+        </is>
+      </c>
+      <c r="J240" s="2" t="inlineStr">
         <is>
           <t>Verify the operating system requires the change of at least eight of the total number of characters when passwords are changed. If it does not, this is a finding.</t>
         </is>
       </c>
-      <c r="K240" s="3" t="inlineStr">
+      <c r="K240" s="2" t="inlineStr">
         <is>
           <t>To check how many characters must differ during a password change, run the following command:
- $ grep difok /etc/security/pwquality.conf 
+ $ sudo grep difok /etc/security/pwquality.conf
+difok = 8
 The "difok" parameter will indicate how many characters must differ.
-If difok is not found or not equal to or greater than the required value, then this is a finding.</t>
-        </is>
-      </c>
-      <c r="L240" s="3" t="n"/>
-      <c r="M240" s="3" t="inlineStr"/>
-      <c r="N240" s="3" t="inlineStr">
-        <is>
-          <t>CAT II</t>
-        </is>
-      </c>
-      <c r="O240" s="3" t="n"/>
-      <c r="P240" s="3" t="n"/>
-      <c r="Q240" s="3" t="n"/>
+If difok is not found or set to less than the required value, then this is a finding.</t>
+        </is>
+      </c>
+      <c r="L240" s="2" t="n"/>
+      <c r="M240" s="2" t="inlineStr">
+        <is>
+          <t>Configure Red Hat Enterprise Linux 9 to require the change of at least 8 of the total number of characters when passwords are changed by setting the "difok" option.
+Add the following line to "/etc/security/pwquality.conf" (or modify the line to have the required value):
+difok = 8</t>
+        </is>
+      </c>
+      <c r="N240" s="2" t="inlineStr">
+        <is>
+          <t>CAT II</t>
+        </is>
+      </c>
+      <c r="O240" s="2" t="n"/>
+      <c r="P240" s="2" t="n"/>
+      <c r="Q240" s="2" t="n"/>
     </row>
     <row r="241" ht="130" customHeight="1">
       <c r="A241" s="2" t="inlineStr">
         <is>
-          <t>CM-6 b,IA-5 (1) (a),IA-5 (1) (b)</t>
+          <t>CM-6 b,IA-5 (1) (b),IA-5 (1) (a)</t>
         </is>
       </c>
       <c r="B241" s="2" t="inlineStr">
@@ -19678,46 +19685,46 @@
       <c r="Q241" s="2" t="n"/>
     </row>
     <row r="242" ht="130" customHeight="1">
-      <c r="A242" s="3" t="inlineStr">
+      <c r="A242" s="2" t="inlineStr">
         <is>
           <t>IA-5 (1) (b)</t>
         </is>
       </c>
-      <c r="B242" s="3" t="inlineStr">
+      <c r="B242" s="2" t="inlineStr">
         <is>
           <t>CCI-000195</t>
         </is>
       </c>
-      <c r="C242" s="3" t="inlineStr">
+      <c r="C242" s="2" t="inlineStr">
         <is>
           <t>SRG-OS-000072-GPOS-00040</t>
         </is>
       </c>
-      <c r="D242" s="3" t="inlineStr">
+      <c r="D242" s="2" t="inlineStr">
         <is>
           <t>CCE-83575-1</t>
         </is>
       </c>
-      <c r="E242" s="3" t="inlineStr">
+      <c r="E242" s="2" t="inlineStr">
         <is>
           <t>The operating system must require the change of at least 50% of the total number of characters when passwords are changed.</t>
         </is>
       </c>
-      <c r="F242" s="3" t="inlineStr">
+      <c r="F242" s="2" t="inlineStr">
         <is>
           <t>Red Hat Enterprise Linux 9 Must Require The Change Of At Least 50% Of The Total Number Of Characters When Passwords Are Changed.</t>
         </is>
       </c>
-      <c r="G242" s="3" t="inlineStr">
+      <c r="G242" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve"> If the operating system allows the user to consecutively reuse extensive portions of passwords, this increases the chances of password compromise by increasing the window of opportunity for attempts at guessing and brute-force attacks.
 The number of changed characters refers to the number of changes required with respect to the total number of positions in the current password. In other words, characters may be the same within the two passwords; however, the positions of the like characters must be different.
 If the password length is an odd number then number of changed characters must be rounded up.  For example, a password length of 15 characters must require the change of at least 8 characters.</t>
         </is>
       </c>
-      <c r="H242" s="3" t="inlineStr">
-        <is>
-          <t>Use of a complex password helps to increase the time and resources required to comrpomise the password.
+      <c r="H242" s="2" t="inlineStr">
+        <is>
+          <t>Use of a complex password helps to increase the time and resources required to compromise the password.
 Password complexity, or strength, is a measure of the effectiveness of a password in resisting
 attempts at guessing and brute-force attacks.
 Password complexity is one factor of several that determines how long it takes to crack a password. The
@@ -19725,74 +19732,79 @@
 password is compromised.</t>
         </is>
       </c>
-      <c r="I242" s="3" t="inlineStr">
-        <is>
-          <t>Applicable - Configurable</t>
-        </is>
-      </c>
-      <c r="J242" s="3" t="inlineStr">
+      <c r="I242" s="2" t="inlineStr">
+        <is>
+          <t>Applicable - Configurable</t>
+        </is>
+      </c>
+      <c r="J242" s="2" t="inlineStr">
         <is>
           <t>Verify the operating system requires the change of at least eight of the total number of characters when passwords are changed. If it does not, this is a finding.</t>
         </is>
       </c>
-      <c r="K242" s="3" t="inlineStr">
+      <c r="K242" s="2" t="inlineStr">
         <is>
           <t>To check the value for maximum consecutive repeating characters, run the following command:
- $ grep maxclassrepeat /etc/security/pwquality.conf 
-For DoD systems, the output should show "maxclassrepeat"=4 or less but greater than zero.
-If that is not the case, then this is a finding.</t>
-        </is>
-      </c>
-      <c r="L242" s="3" t="n"/>
-      <c r="M242" s="3" t="inlineStr"/>
-      <c r="N242" s="3" t="inlineStr">
-        <is>
-          <t>CAT II</t>
-        </is>
-      </c>
-      <c r="O242" s="3" t="n"/>
-      <c r="P242" s="3" t="n"/>
-      <c r="Q242" s="3" t="n"/>
+ $ sudo grep maxclassrepeat /etc/security/pwquality.conf 
+If the value of "maxclassrepeat" is set to "0", more than "4" or is commented out, then this is a finding.</t>
+        </is>
+      </c>
+      <c r="L242" s="2" t="n"/>
+      <c r="M242" s="2" t="inlineStr">
+        <is>
+          <t>Configure Red Hat Enterprise Linux 9 to require the change of the number of repeating characters of the same character class when passwords are changed by setting the "maxclassrepeat" option.
+Add the following line to "/etc/security/pwquality.conf" conf (or modify the line to have the required value):
+maxclassrepeat = 4</t>
+        </is>
+      </c>
+      <c r="N242" s="2" t="inlineStr">
+        <is>
+          <t>CAT II</t>
+        </is>
+      </c>
+      <c r="O242" s="2" t="n"/>
+      <c r="P242" s="2" t="n"/>
+      <c r="Q242" s="2" t="n"/>
     </row>
     <row r="243" ht="130" customHeight="1">
-      <c r="A243" s="3" t="inlineStr">
+      <c r="A243" s="2" t="inlineStr">
         <is>
           <t>IA-5 (1) (b)</t>
         </is>
       </c>
-      <c r="B243" s="3" t="inlineStr">
+      <c r="B243" s="2" t="inlineStr">
         <is>
           <t>CCI-000195</t>
         </is>
       </c>
-      <c r="C243" s="3" t="inlineStr">
+      <c r="C243" s="2" t="inlineStr">
         <is>
           <t>SRG-OS-000072-GPOS-00040</t>
         </is>
       </c>
-      <c r="D243" s="3" t="inlineStr">
+      <c r="D243" s="2" t="inlineStr">
         <is>
           <t>CCE-83567-8</t>
         </is>
       </c>
-      <c r="E243" s="3" t="inlineStr">
+      <c r="E243" s="2" t="inlineStr">
         <is>
           <t>The operating system must require the change of at least 50% of the total number of characters when passwords are changed.</t>
         </is>
       </c>
-      <c r="F243" s="3" t="inlineStr">
+      <c r="F243" s="2" t="inlineStr">
         <is>
           <t>Red Hat Enterprise Linux 9 Must Require The Change Of At Least 50% Of The Total Number Of Characters When Passwords Are Changed.</t>
         </is>
       </c>
-      <c r="G243" s="3" t="inlineStr">
+      <c r="G243" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve"> If the operating system allows the user to consecutively reuse extensive portions of passwords, this increases the chances of password compromise by increasing the window of opportunity for attempts at guessing and brute-force attacks.
 The number of changed characters refers to the number of changes required with respect to the total number of positions in the current password. In other words, characters may be the same within the two passwords; however, the positions of the like characters must be different.
 If the password length is an odd number then number of changed characters must be rounded up.  For example, a password length of 15 characters must require the change of at least 8 characters.</t>
         </is>
       </c>
-      <c r="H243" s="3" t="inlineStr">
+      <c r="H243" s="2" t="inlineStr">
         <is>
           <t>Use of a complex password helps to increase the time and resources required to compromise the password.
 Password complexity, or strength, is a measure of the effectiveness of a password in resisting attempts at
@@ -19803,75 +19815,79 @@
 Passwords with excessive repeating characters may be more vulnerable to password-guessing attacks.</t>
         </is>
       </c>
-      <c r="I243" s="3" t="inlineStr">
-        <is>
-          <t>Applicable - Configurable</t>
-        </is>
-      </c>
-      <c r="J243" s="3" t="inlineStr">
+      <c r="I243" s="2" t="inlineStr">
+        <is>
+          <t>Applicable - Configurable</t>
+        </is>
+      </c>
+      <c r="J243" s="2" t="inlineStr">
         <is>
           <t>Verify the operating system requires the change of at least eight of the total number of characters when passwords are changed. If it does not, this is a finding.</t>
         </is>
       </c>
-      <c r="K243" s="3" t="inlineStr">
+      <c r="K243" s="2" t="inlineStr">
         <is>
           <t>To check the maximum value for consecutive repeating characters, run the following command:
- $ grep maxrepeat /etc/security/pwquality.conf 
-Look for the value of the "maxrepeat" parameter. The DoD requirement is 3, which would appear as
-"maxrepeat=3".
-If maxrepeat is not found or not greater than or equal to the required value, then this is a finding.</t>
-        </is>
-      </c>
-      <c r="L243" s="3" t="n"/>
-      <c r="M243" s="3" t="inlineStr"/>
-      <c r="N243" s="3" t="inlineStr">
-        <is>
-          <t>CAT II</t>
-        </is>
-      </c>
-      <c r="O243" s="3" t="n"/>
-      <c r="P243" s="3" t="n"/>
-      <c r="Q243" s="3" t="n"/>
+ $ sudo grep maxrepeat /etc/security/pwquality.conf 
+If the value of "maxrepeat" is set to more than "3" or is commented out, then this is a finding.</t>
+        </is>
+      </c>
+      <c r="L243" s="2" t="n"/>
+      <c r="M243" s="2" t="inlineStr">
+        <is>
+          <t>Configure Red Hat Enterprise Linux 9 to require the change of the number of repeating consecutive characters when passwords are changed by setting the "maxrepeat" option.
+Add the following line to "/etc/security/pwquality.conf" (or modify the line to have the required value):
+maxrepeat = 3</t>
+        </is>
+      </c>
+      <c r="N243" s="2" t="inlineStr">
+        <is>
+          <t>CAT II</t>
+        </is>
+      </c>
+      <c r="O243" s="2" t="n"/>
+      <c r="P243" s="2" t="n"/>
+      <c r="Q243" s="2" t="n"/>
     </row>
     <row r="244" ht="130" customHeight="1">
-      <c r="A244" s="3" t="inlineStr">
+      <c r="A244" s="2" t="inlineStr">
         <is>
           <t>IA-5 (1) (b)</t>
         </is>
       </c>
-      <c r="B244" s="3" t="inlineStr">
+      <c r="B244" s="2" t="inlineStr">
         <is>
           <t>CCI-000195</t>
         </is>
       </c>
-      <c r="C244" s="3" t="inlineStr">
+      <c r="C244" s="2" t="inlineStr">
         <is>
           <t>SRG-OS-000072-GPOS-00040</t>
         </is>
       </c>
-      <c r="D244" s="3" t="inlineStr">
+      <c r="D244" s="2" t="inlineStr">
         <is>
           <t>CCE-83563-7</t>
         </is>
       </c>
-      <c r="E244" s="3" t="inlineStr">
+      <c r="E244" s="2" t="inlineStr">
         <is>
           <t>The operating system must require the change of at least 50% of the total number of characters when passwords are changed.</t>
         </is>
       </c>
-      <c r="F244" s="3" t="inlineStr">
+      <c r="F244" s="2" t="inlineStr">
         <is>
           <t>Red Hat Enterprise Linux 9 Must Require The Change Of At Least 50% Of The Total Number Of Characters When Passwords Are Changed.</t>
         </is>
       </c>
-      <c r="G244" s="3" t="inlineStr">
+      <c r="G244" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve"> If the operating system allows the user to consecutively reuse extensive portions of passwords, this increases the chances of password compromise by increasing the window of opportunity for attempts at guessing and brute-force attacks.
 The number of changed characters refers to the number of changes required with respect to the total number of positions in the current password. In other words, characters may be the same within the two passwords; however, the positions of the like characters must be different.
 If the password length is an odd number then number of changed characters must be rounded up.  For example, a password length of 15 characters must require the change of at least 8 characters.</t>
         </is>
       </c>
-      <c r="H244" s="3" t="inlineStr">
+      <c r="H244" s="2" t="inlineStr">
         <is>
           <t>Use of a complex password helps to increase the time and resources required to compromise the password.
 Password complexity, or strength, is a measure of the effectiveness of a password in resisting attempts
@@ -19883,37 +19899,43 @@
 by ensuring a larger search space.</t>
         </is>
       </c>
-      <c r="I244" s="3" t="inlineStr">
-        <is>
-          <t>Applicable - Configurable</t>
-        </is>
-      </c>
-      <c r="J244" s="3" t="inlineStr">
+      <c r="I244" s="2" t="inlineStr">
+        <is>
+          <t>Applicable - Configurable</t>
+        </is>
+      </c>
+      <c r="J244" s="2" t="inlineStr">
         <is>
           <t>Verify the operating system requires the change of at least eight of the total number of characters when passwords are changed. If it does not, this is a finding.</t>
         </is>
       </c>
-      <c r="K244" s="3" t="inlineStr">
+      <c r="K244" s="2" t="inlineStr">
         <is>
           <t>To check how many categories of characters must be used in password during a password change,
 run the following command:
- $ grep minclass /etc/security/pwquality.conf 
+ $ sudo grep minclass /etc/security/pwquality.conf 
 The "minclass" parameter will indicate how many character classes must be used. If
-the requirement was for the password to contain characters from three different categories,
-then this would appear as "minclass = 3".
-If minclass is not found or not set equal to or greater than the required value, then this is a finding.</t>
-        </is>
-      </c>
-      <c r="L244" s="3" t="n"/>
-      <c r="M244" s="3" t="inlineStr"/>
-      <c r="N244" s="3" t="inlineStr">
-        <is>
-          <t>CAT II</t>
-        </is>
-      </c>
-      <c r="O244" s="3" t="n"/>
-      <c r="P244" s="3" t="n"/>
-      <c r="Q244" s="3" t="n"/>
+the requirement was for the password to contain characters from 4 different categories,
+then this would appear as "minclass = 4".
+If the value of "minclass" is set to less than "4" or is commented out, then this is a finding.</t>
+        </is>
+      </c>
+      <c r="L244" s="2" t="n"/>
+      <c r="M244" s="2" t="inlineStr">
+        <is>
+          <t>Configure Red Hat Enterprise Linux 9 to require the change of at least 4 character classes when passwords are changed by setting the "minclass" option.
+Add the following line to "/etc/security/pwquality.conf" (or modify the line to have the required value):
+minclass = 4</t>
+        </is>
+      </c>
+      <c r="N244" s="2" t="inlineStr">
+        <is>
+          <t>CAT II</t>
+        </is>
+      </c>
+      <c r="O244" s="2" t="n"/>
+      <c r="P244" s="2" t="n"/>
+      <c r="Q244" s="2" t="n"/>
     </row>
     <row r="245" ht="130" customHeight="1">
       <c r="A245" s="2" t="inlineStr">
@@ -20421,7 +20443,7 @@
     <row r="251" ht="130" customHeight="1">
       <c r="A251" s="2" t="inlineStr">
         <is>
-          <t>IA-2 (1),IA-2 (11)</t>
+          <t>IA-2 (11),IA-2 (1)</t>
         </is>
       </c>
       <c r="B251" s="2" t="inlineStr">
@@ -20510,7 +20532,7 @@
     <row r="252" ht="130" customHeight="1">
       <c r="A252" s="2" t="inlineStr">
         <is>
-          <t>IA-2 (12),IA-2 (11)</t>
+          <t>IA-2 (11),IA-2 (12)</t>
         </is>
       </c>
       <c r="B252" s="2" t="inlineStr">
@@ -21003,7 +21025,7 @@
     <row r="258" ht="130" customHeight="1">
       <c r="A258" s="3" t="inlineStr">
         <is>
-          <t>IA-2 (5),CM-6 b</t>
+          <t>CM-6 b,IA-2 (5)</t>
         </is>
       </c>
       <c r="B258" s="3" t="inlineStr">
@@ -21465,7 +21487,7 @@
     <row r="264" ht="130" customHeight="1">
       <c r="A264" s="2" t="inlineStr">
         <is>
-          <t>AU-9,AU-12 c</t>
+          <t>AU-12 c,AU-9</t>
         </is>
       </c>
       <c r="B264" s="2" t="inlineStr">
@@ -22238,7 +22260,7 @@
     <row r="273" ht="130" customHeight="1">
       <c r="A273" s="3" t="inlineStr">
         <is>
-          <t>CM-7 a,CM-6 b</t>
+          <t>CM-6 b,CM-7 a</t>
         </is>
       </c>
       <c r="B273" s="3" t="inlineStr">
@@ -22386,7 +22408,7 @@
     <row r="275" ht="130" customHeight="1">
       <c r="A275" s="2" t="inlineStr">
         <is>
-          <t>CM-7 b,CM-7 a</t>
+          <t>CM-7 a,CM-7 b</t>
         </is>
       </c>
       <c r="B275" s="2" t="inlineStr">
@@ -22466,7 +22488,7 @@
     <row r="276" ht="130" customHeight="1">
       <c r="A276" s="2" t="inlineStr">
         <is>
-          <t>CM-7 b,CM-7 a</t>
+          <t>CM-7 a,CM-7 b</t>
         </is>
       </c>
       <c r="B276" s="2" t="inlineStr">
@@ -23234,7 +23256,7 @@
     <row r="286" ht="130" customHeight="1">
       <c r="A286" s="3" t="inlineStr">
         <is>
-          <t>CM-7 a,CM-6 b</t>
+          <t>CM-6 b,CM-7 a</t>
         </is>
       </c>
       <c r="B286" s="3" t="inlineStr">
@@ -23305,7 +23327,7 @@
     <row r="287" ht="130" customHeight="1">
       <c r="A287" s="3" t="inlineStr">
         <is>
-          <t>CM-7 a,CM-6 b</t>
+          <t>CM-6 b,CM-7 a</t>
         </is>
       </c>
       <c r="B287" s="3" t="inlineStr">
@@ -23377,7 +23399,7 @@
     <row r="288" ht="130" customHeight="1">
       <c r="A288" s="3" t="inlineStr">
         <is>
-          <t>CM-7 a,CM-6 b</t>
+          <t>CM-6 b,CM-7 a</t>
         </is>
       </c>
       <c r="B288" s="3" t="inlineStr">
@@ -23619,7 +23641,7 @@
     <row r="291" ht="130" customHeight="1">
       <c r="A291" s="2" t="inlineStr">
         <is>
-          <t>AU-5 a,AU-5 (1)</t>
+          <t>AU-5 (1),AU-5 a</t>
         </is>
       </c>
       <c r="B291" s="2" t="inlineStr">
@@ -26987,7 +27009,7 @@
     <row r="336" ht="130" customHeight="1">
       <c r="A336" s="3" t="inlineStr">
         <is>
-          <t>IA-5 (1) (c),CM-6 b</t>
+          <t>CM-6 b,IA-5 (1) (c)</t>
         </is>
       </c>
       <c r="B336" s="3" t="inlineStr">
@@ -27137,7 +27159,7 @@
     <row r="338" ht="130" customHeight="1">
       <c r="A338" s="2" t="inlineStr">
         <is>
-          <t>CM-6 b,IA-2 (2)</t>
+          <t>IA-2 (2),CM-6 b</t>
         </is>
       </c>
       <c r="B338" s="2" t="inlineStr">
@@ -30262,7 +30284,7 @@
     <row r="379" ht="130" customHeight="1">
       <c r="A379" s="2" t="inlineStr">
         <is>
-          <t>CM-7 b,CM-6 b,AC-17 (1),AC-17 (9)</t>
+          <t>CM-6 b,AC-17 (1),AC-17 (9),CM-7 b</t>
         </is>
       </c>
       <c r="B379" s="2" t="inlineStr">
@@ -30340,7 +30362,7 @@
     <row r="380" ht="130" customHeight="1">
       <c r="A380" s="2" t="inlineStr">
         <is>
-          <t>CM-7 b,CM-6 b,AC-17 (1)</t>
+          <t>CM-6 b,AC-17 (1),CM-7 b</t>
         </is>
       </c>
       <c r="B380" s="2" t="inlineStr">
@@ -32839,7 +32861,7 @@
     <row r="409" ht="130" customHeight="1">
       <c r="A409" s="2" t="inlineStr">
         <is>
-          <t>CM-6 b,IA-3</t>
+          <t>IA-3,CM-6 b</t>
         </is>
       </c>
       <c r="B409" s="2" t="inlineStr">
@@ -32921,7 +32943,7 @@
     <row r="410" ht="130" customHeight="1">
       <c r="A410" s="2" t="inlineStr">
         <is>
-          <t>CM-6 b,IA-3</t>
+          <t>IA-3,CM-6 b</t>
         </is>
       </c>
       <c r="B410" s="2" t="inlineStr">
@@ -34973,7 +34995,7 @@
     <row r="436" ht="130" customHeight="1">
       <c r="A436" s="2" t="inlineStr">
         <is>
-          <t>CM-6 b,IA-3</t>
+          <t>IA-3,CM-6 b</t>
         </is>
       </c>
       <c r="B436" s="2" t="inlineStr">
@@ -35063,7 +35085,7 @@
     <row r="437" ht="130" customHeight="1">
       <c r="A437" s="2" t="inlineStr">
         <is>
-          <t>CM-6 b,IA-3</t>
+          <t>IA-3,CM-6 b</t>
         </is>
       </c>
       <c r="B437" s="2" t="inlineStr">
@@ -35458,7 +35480,7 @@
     <row r="442" ht="130" customHeight="1">
       <c r="A442" s="3" t="inlineStr">
         <is>
-          <t>SI-2 (2),CM-6 b</t>
+          <t>CM-6 b,SI-2 (2)</t>
         </is>
       </c>
       <c r="B442" s="3" t="inlineStr">
@@ -36105,7 +36127,7 @@
     <row r="451" ht="130" customHeight="1">
       <c r="A451" s="3" t="inlineStr">
         <is>
-          <t>SI-2 (2),CM-6 b</t>
+          <t>CM-6 b,SI-2 (2)</t>
         </is>
       </c>
       <c r="B451" s="3" t="inlineStr">
@@ -36396,7 +36418,7 @@
     <row r="455" ht="130" customHeight="1">
       <c r="A455" s="3" t="inlineStr">
         <is>
-          <t>SC-10,MA-4 e,AC-12,MA-4 (7)</t>
+          <t>AC-12,MA-4 e,MA-4 (7),SC-10</t>
         </is>
       </c>
       <c r="B455" s="3" t="inlineStr">
@@ -36471,7 +36493,7 @@
     <row r="456" ht="130" customHeight="1">
       <c r="A456" s="3" t="inlineStr">
         <is>
-          <t>SC-10,AC-12</t>
+          <t>AC-12,SC-10</t>
         </is>
       </c>
       <c r="B456" s="3" t="inlineStr">
@@ -36550,7 +36572,7 @@
     <row r="457" ht="130" customHeight="1">
       <c r="A457" s="3" t="inlineStr">
         <is>
-          <t>SC-10,AC-12</t>
+          <t>AC-12,SC-10</t>
         </is>
       </c>
       <c r="B457" s="3" t="inlineStr">
@@ -36626,7 +36648,7 @@
     <row r="458" ht="130" customHeight="1">
       <c r="A458" s="3" t="inlineStr">
         <is>
-          <t>SC-10,AC-11 a</t>
+          <t>AC-11 a,SC-10</t>
         </is>
       </c>
       <c r="B458" s="3" t="inlineStr">
@@ -38010,7 +38032,7 @@
     <row r="476" ht="130" customHeight="1">
       <c r="A476" s="2" t="inlineStr">
         <is>
-          <t>CM-7 b,IA-3</t>
+          <t>IA-3,CM-7 b</t>
         </is>
       </c>
       <c r="B476" s="2" t="inlineStr">
@@ -38329,7 +38351,7 @@
     <row r="480" ht="130" customHeight="1">
       <c r="A480" s="2" t="inlineStr">
         <is>
-          <t>CM-7 b,AC-17 (1)</t>
+          <t>AC-17 (1),CM-7 b</t>
         </is>
       </c>
       <c r="B480" s="2" t="inlineStr">

</xml_diff>